<commit_message>
Auto commit - 06031737
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$17</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="84">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-01  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="154">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-03  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -284,6 +284,217 @@
   </si>
   <si>
     <t>觸控螢幕校正後可正常使用</t>
+  </si>
+  <si>
+    <t>15451115060101</t>
+  </si>
+  <si>
+    <t>板橋懷仁店</t>
+  </si>
+  <si>
+    <t>新北市板橋區</t>
+  </si>
+  <si>
+    <t>2026-06-01 17:30:23</t>
+  </si>
+  <si>
+    <t>星期一</t>
+  </si>
+  <si>
+    <t>HL60</t>
+  </si>
+  <si>
+    <t>HL-LIFE-ET印票機L90</t>
+  </si>
+  <si>
+    <t>無反應，不會轉動</t>
+  </si>
+  <si>
+    <t>門市反應印票機L90亮紅燈無法排除，確認票券機仍有紙張，但機器重開紙捲重放後仍亮紅燈無反應無轉動....還請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF05451</t>
+  </si>
+  <si>
+    <t>狄澤洋</t>
+  </si>
+  <si>
+    <t>2026-06-01 17:31:47</t>
+  </si>
+  <si>
+    <t>2026-06-02 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-02 14:25:00</t>
+  </si>
+  <si>
+    <t>2026-06-02 21:31:00</t>
+  </si>
+  <si>
+    <t>票券紙無效票未撕除，排除後測試正常</t>
+  </si>
+  <si>
+    <t>服務</t>
+  </si>
+  <si>
+    <t>北縣商港店</t>
+  </si>
+  <si>
+    <t>新北市八里區</t>
+  </si>
+  <si>
+    <t>THILF02442</t>
+  </si>
+  <si>
+    <t>2026-06-02 15:15:47</t>
+  </si>
+  <si>
+    <t>2026-06-02 15:14:00</t>
+  </si>
+  <si>
+    <t>裝潢撤機完工</t>
+  </si>
+  <si>
+    <t>2026-06-02 15:19:11</t>
+  </si>
+  <si>
+    <t>2026-06-02 15:15:00</t>
+  </si>
+  <si>
+    <t>裝潢撤機</t>
+  </si>
+  <si>
+    <t>2026-06-02 15:21:11</t>
+  </si>
+  <si>
+    <t>PMQ2+EDC</t>
+  </si>
+  <si>
+    <t>板橋板豐店</t>
+  </si>
+  <si>
+    <t>THILF03551</t>
+  </si>
+  <si>
+    <t>2026-06-02 15:35:53</t>
+  </si>
+  <si>
+    <t>2026-06-02 15:20:00</t>
+  </si>
+  <si>
+    <t>2026-06-02 15:33:00</t>
+  </si>
+  <si>
+    <t>三重國隆店</t>
+  </si>
+  <si>
+    <t>THILF04804</t>
+  </si>
+  <si>
+    <t>2026-06-03 10:13:59</t>
+  </si>
+  <si>
+    <t>2026-06-03 09:47:00</t>
+  </si>
+  <si>
+    <t>2026-06-03 10:10:00</t>
+  </si>
+  <si>
+    <t>三重今大店</t>
+  </si>
+  <si>
+    <t>THILF04184</t>
+  </si>
+  <si>
+    <t>2026-06-03 10:45:47</t>
+  </si>
+  <si>
+    <t>2026-06-03 10:20:00</t>
+  </si>
+  <si>
+    <t>2026-06-03 10:41:00</t>
+  </si>
+  <si>
+    <t>桃縣富竹店</t>
+  </si>
+  <si>
+    <t>桃園市蘆竹區</t>
+  </si>
+  <si>
+    <t>THILF03880</t>
+  </si>
+  <si>
+    <t>2026-06-03 13:40:00</t>
+  </si>
+  <si>
+    <t>2026-06-03 13:10:00</t>
+  </si>
+  <si>
+    <t>2026-06-03 13:38:00</t>
+  </si>
+  <si>
+    <t>蘆竹六股埤</t>
+  </si>
+  <si>
+    <t>THILF04289</t>
+  </si>
+  <si>
+    <t>2026-06-03 14:36:04</t>
+  </si>
+  <si>
+    <t>2026-06-03 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-03 14:34:00</t>
+  </si>
+  <si>
+    <t>桃縣蘆華店</t>
+  </si>
+  <si>
+    <t>THILF03556</t>
+  </si>
+  <si>
+    <t>2026-06-03 15:31:34</t>
+  </si>
+  <si>
+    <t>2026-06-03 14:50:00</t>
+  </si>
+  <si>
+    <t>2026-06-03 15:10:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PMQ2+EDC
+</t>
+  </si>
+  <si>
+    <t>蘆竹大華店</t>
+  </si>
+  <si>
+    <t>THILF02322</t>
+  </si>
+  <si>
+    <t>2026-06-03 16:00:53</t>
+  </si>
+  <si>
+    <t>2026-06-03 15:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-03 16:00:00</t>
+  </si>
+  <si>
+    <t>板橋稚暉店</t>
+  </si>
+  <si>
+    <t>THILF04406</t>
+  </si>
+  <si>
+    <t>2026-06-03 16:13:34</t>
+  </si>
+  <si>
+    <t>2026-06-03 16:10:00</t>
+  </si>
+  <si>
+    <t>PMQ2+EDC+SC7</t>
   </si>
 </sst>
 </file>
@@ -697,7 +908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK5"/>
+  <dimension ref="A1:AK17"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -1133,7 +1344,7 @@
       <c r="O5" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="P5" s="8" t="s">
+      <c r="P5" s="9" t="s">
         <v>77</v>
       </c>
       <c r="Q5" s="7" t="s">
@@ -1170,7 +1381,7 @@
       <c r="AB5" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC5" s="8" t="s">
+      <c r="AC5" s="9" t="s">
         <v>83</v>
       </c>
       <c r="AD5" s="7"/>
@@ -1181,6 +1392,956 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
       <c r="AK5" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:37">
+      <c r="A6" s="3">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="3">
+        <v>2026060149</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="3">
+        <v>5451</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="N6" s="3">
+        <v>6003</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="P6" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q6" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="R6" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S6" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="T6" s="3">
+        <v>1</v>
+      </c>
+      <c r="U6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V6" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="W6" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="X6" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="Y6" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="Z6" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA6" s="3"/>
+      <c r="AB6" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC6" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="AD6" s="3"/>
+      <c r="AE6" s="3"/>
+      <c r="AF6" s="3"/>
+      <c r="AG6" s="3"/>
+      <c r="AH6" s="3"/>
+      <c r="AI6" s="3"/>
+      <c r="AJ6" s="3"/>
+      <c r="AK6" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:37">
+      <c r="A7" s="7">
+        <v>5</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C7" s="7">
+        <v>2026060445</v>
+      </c>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7">
+        <v>2442</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="9"/>
+      <c r="Q7" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="R7" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S7" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T7" s="7">
+        <v>1</v>
+      </c>
+      <c r="U7" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V7" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="W7" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="X7" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="Y7" s="7"/>
+      <c r="Z7" s="7">
+        <v>1.2</v>
+      </c>
+      <c r="AA7" s="7"/>
+      <c r="AB7" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC7" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="AD7" s="7"/>
+      <c r="AE7" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF7" s="7"/>
+      <c r="AG7" s="7"/>
+      <c r="AH7" s="7"/>
+      <c r="AI7" s="7"/>
+      <c r="AJ7" s="7"/>
+      <c r="AK7" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:37">
+      <c r="A8" s="3">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C8" s="3">
+        <v>2026060464</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3">
+        <v>2442</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="10"/>
+      <c r="Q8" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="R8" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S8" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T8" s="3">
+        <v>1</v>
+      </c>
+      <c r="U8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V8" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="W8" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="X8" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="Y8" s="3"/>
+      <c r="Z8" s="3">
+        <v>1.3</v>
+      </c>
+      <c r="AA8" s="3"/>
+      <c r="AB8" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC8" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="AD8" s="3"/>
+      <c r="AE8" s="3"/>
+      <c r="AF8" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG8" s="3"/>
+      <c r="AH8" s="3"/>
+      <c r="AI8" s="3"/>
+      <c r="AJ8" s="3"/>
+      <c r="AK8" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:37">
+      <c r="A9" s="7">
+        <v>7</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C9" s="7">
+        <v>2026060475</v>
+      </c>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7">
+        <v>5451</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="9"/>
+      <c r="Q9" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="R9" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="T9" s="7">
+        <v>1</v>
+      </c>
+      <c r="U9" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V9" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="W9" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="X9" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="Y9" s="7"/>
+      <c r="Z9" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA9" s="7"/>
+      <c r="AB9" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC9" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD9" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE9" s="7"/>
+      <c r="AF9" s="7"/>
+      <c r="AG9" s="7"/>
+      <c r="AH9" s="7"/>
+      <c r="AI9" s="7"/>
+      <c r="AJ9" s="7"/>
+      <c r="AK9" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:37">
+      <c r="A10" s="3">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C10" s="3">
+        <v>2026060510</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3">
+        <v>3551</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="10"/>
+      <c r="Q10" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="R10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S10" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="T10" s="3">
+        <v>1</v>
+      </c>
+      <c r="U10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V10" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="W10" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="X10" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="Y10" s="3"/>
+      <c r="Z10" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="AA10" s="3"/>
+      <c r="AB10" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC10" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD10" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE10" s="3"/>
+      <c r="AF10" s="3"/>
+      <c r="AG10" s="3"/>
+      <c r="AH10" s="3"/>
+      <c r="AI10" s="3"/>
+      <c r="AJ10" s="3"/>
+      <c r="AK10" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:37">
+      <c r="A11" s="7">
+        <v>9</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C11" s="7">
+        <v>2026060656</v>
+      </c>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7">
+        <v>4804</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="9"/>
+      <c r="Q11" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="R11" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S11" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T11" s="7">
+        <v>1</v>
+      </c>
+      <c r="U11" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V11" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="W11" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="X11" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="Y11" s="7"/>
+      <c r="Z11" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA11" s="7"/>
+      <c r="AB11" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC11" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD11" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE11" s="7"/>
+      <c r="AF11" s="7"/>
+      <c r="AG11" s="7"/>
+      <c r="AH11" s="7"/>
+      <c r="AI11" s="7"/>
+      <c r="AJ11" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK11" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:37">
+      <c r="A12" s="3">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="3">
+        <v>2026060669</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3">
+        <v>4184</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="3"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="10"/>
+      <c r="Q12" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="R12" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S12" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T12" s="3">
+        <v>1</v>
+      </c>
+      <c r="U12" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V12" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="W12" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="X12" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="Y12" s="3"/>
+      <c r="Z12" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA12" s="3"/>
+      <c r="AB12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC12" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD12" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE12" s="3"/>
+      <c r="AF12" s="3"/>
+      <c r="AG12" s="3"/>
+      <c r="AH12" s="3"/>
+      <c r="AI12" s="3"/>
+      <c r="AJ12" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK12" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:37">
+      <c r="A13" s="7">
+        <v>11</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C13" s="7">
+        <v>2026060812</v>
+      </c>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7">
+        <v>3880</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="9"/>
+      <c r="Q13" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="R13" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S13" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T13" s="7">
+        <v>1</v>
+      </c>
+      <c r="U13" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V13" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="W13" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="X13" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="Y13" s="7"/>
+      <c r="Z13" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA13" s="7"/>
+      <c r="AB13" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC13" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD13" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE13" s="7"/>
+      <c r="AF13" s="7"/>
+      <c r="AG13" s="7"/>
+      <c r="AH13" s="7"/>
+      <c r="AI13" s="7"/>
+      <c r="AJ13" s="7"/>
+      <c r="AK13" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:37">
+      <c r="A14" s="3">
+        <v>12</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C14" s="3">
+        <v>2026060827</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3">
+        <v>4289</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="3"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="10"/>
+      <c r="Q14" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="R14" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S14" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T14" s="3">
+        <v>1</v>
+      </c>
+      <c r="U14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V14" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="W14" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="X14" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="Y14" s="3"/>
+      <c r="Z14" s="3">
+        <v>0.6</v>
+      </c>
+      <c r="AA14" s="3"/>
+      <c r="AB14" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC14" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD14" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE14" s="3"/>
+      <c r="AF14" s="3"/>
+      <c r="AG14" s="3"/>
+      <c r="AH14" s="3"/>
+      <c r="AI14" s="3"/>
+      <c r="AJ14" s="3"/>
+      <c r="AK14" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" spans="1:37">
+      <c r="A15" s="7">
+        <v>13</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C15" s="7">
+        <v>2026060840</v>
+      </c>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7">
+        <v>3556</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="7"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="9"/>
+      <c r="Q15" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="R15" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S15" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T15" s="7">
+        <v>1</v>
+      </c>
+      <c r="U15" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V15" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="W15" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="X15" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="Y15" s="7"/>
+      <c r="Z15" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA15" s="7"/>
+      <c r="AB15" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC15" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="AD15" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE15" s="7"/>
+      <c r="AF15" s="7"/>
+      <c r="AG15" s="7"/>
+      <c r="AH15" s="7"/>
+      <c r="AI15" s="7"/>
+      <c r="AJ15" s="7"/>
+      <c r="AK15" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:37">
+      <c r="A16" s="3">
+        <v>14</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C16" s="3">
+        <v>2026060846</v>
+      </c>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3">
+        <v>2322</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="3"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="10"/>
+      <c r="Q16" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="R16" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S16" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T16" s="3">
+        <v>1</v>
+      </c>
+      <c r="U16" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V16" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="W16" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="X16" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="Y16" s="3"/>
+      <c r="Z16" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA16" s="3"/>
+      <c r="AB16" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC16" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="AD16" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE16" s="3"/>
+      <c r="AF16" s="3"/>
+      <c r="AG16" s="3"/>
+      <c r="AH16" s="3"/>
+      <c r="AI16" s="3"/>
+      <c r="AJ16" s="3"/>
+      <c r="AK16" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="1:37">
+      <c r="A17" s="7">
+        <v>15</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C17" s="7">
+        <v>2026060850</v>
+      </c>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7">
+        <v>4406</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="8"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="8"/>
+      <c r="P17" s="8"/>
+      <c r="Q17" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="R17" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S17" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="T17" s="7">
+        <v>1</v>
+      </c>
+      <c r="U17" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V17" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="W17" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="X17" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="Y17" s="7"/>
+      <c r="Z17" s="7">
+        <v>2.2</v>
+      </c>
+      <c r="AA17" s="7"/>
+      <c r="AB17" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC17" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="AD17" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE17" s="7"/>
+      <c r="AF17" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG17" s="7"/>
+      <c r="AH17" s="7"/>
+      <c r="AI17" s="7"/>
+      <c r="AJ17" s="7"/>
+      <c r="AK17" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06041340
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$21</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="154">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-03  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="183">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-04  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -448,6 +448,48 @@
     <t>2026-06-03 14:34:00</t>
   </si>
   <si>
+    <t>14680115060301</t>
+  </si>
+  <si>
+    <t>板橋江寧店</t>
+  </si>
+  <si>
+    <t>2026-06-03 14:54:03</t>
+  </si>
+  <si>
+    <t>星期三</t>
+  </si>
+  <si>
+    <t>HL24</t>
+  </si>
+  <si>
+    <t>HL-SC主機</t>
+  </si>
+  <si>
+    <t>當機/自動開關機</t>
+  </si>
+  <si>
+    <t>門市SC(SHUTTLE6S)SQL升級後,SC開啟的相關程式畫面如有右側,滾動條都會自動往右跑(例:關帳畫面或E網&gt;其他專區&gt;常用表單),已有請門市將鍵盤跟滑鼠電源線直接拔除後確認仍異常無法排除....還請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF04680</t>
+  </si>
+  <si>
+    <t>2026-06-03 14:57:12</t>
+  </si>
+  <si>
+    <t>2026-06-04 12:15:00</t>
+  </si>
+  <si>
+    <t>2026-06-04 13:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-04 18:57:00</t>
+  </si>
+  <si>
+    <t>電腦線路重新插拔測試正常</t>
+  </si>
+  <si>
     <t>桃縣蘆華店</t>
   </si>
   <si>
@@ -495,6 +537,51 @@
   </si>
   <si>
     <t>PMQ2+EDC+SC7</t>
+  </si>
+  <si>
+    <t>五股興珍店</t>
+  </si>
+  <si>
+    <t>新北市五股區</t>
+  </si>
+  <si>
+    <t>THILF02691</t>
+  </si>
+  <si>
+    <t>湯家瑋</t>
+  </si>
+  <si>
+    <t>2026-06-04 11:09:36</t>
+  </si>
+  <si>
+    <t>2026-06-04 10:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-04 11:00:00</t>
+  </si>
+  <si>
+    <t>五股四維店</t>
+  </si>
+  <si>
+    <t>THILF03227</t>
+  </si>
+  <si>
+    <t>2026-06-04 11:28:48</t>
+  </si>
+  <si>
+    <t>2026-06-04 11:30:00</t>
+  </si>
+  <si>
+    <t>五股更寮店</t>
+  </si>
+  <si>
+    <t>THILF05003</t>
+  </si>
+  <si>
+    <t>2026-06-04 11:51:34</t>
+  </si>
+  <si>
+    <t>2026-06-04 12:00:00</t>
   </si>
 </sst>
 </file>
@@ -908,7 +995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK17"/>
+  <dimension ref="A1:AK21"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -2117,38 +2204,58 @@
         <v>13</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C15" s="7">
-        <v>2026060840</v>
-      </c>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
+        <v>2026060831</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F15" s="7">
-        <v>3556</v>
+        <v>4680</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="8"/>
-      <c r="N15" s="7"/>
-      <c r="O15" s="8"/>
-      <c r="P15" s="9"/>
+        <v>86</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="M15" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="N15" s="7">
+        <v>2401</v>
+      </c>
+      <c r="O15" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="P15" s="9" t="s">
+        <v>145</v>
+      </c>
       <c r="Q15" s="7" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="R15" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S15" s="7" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="T15" s="7">
         <v>1</v>
@@ -2157,28 +2264,28 @@
         <v>53</v>
       </c>
       <c r="V15" s="7" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="W15" s="7" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="X15" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="Y15" s="7"/>
+        <v>149</v>
+      </c>
+      <c r="Y15" s="7" t="s">
+        <v>150</v>
+      </c>
       <c r="Z15" s="7">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="AA15" s="7"/>
       <c r="AB15" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC15" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="AD15" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="AD15" s="7"/>
       <c r="AE15" s="7"/>
       <c r="AF15" s="7"/>
       <c r="AG15" s="7"/>
@@ -2197,15 +2304,15 @@
         <v>100</v>
       </c>
       <c r="C16" s="3">
-        <v>2026060846</v>
+        <v>2026060840</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3">
-        <v>2322</v>
+        <v>3556</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>128</v>
@@ -2219,7 +2326,7 @@
       <c r="O16" s="4"/>
       <c r="P16" s="10"/>
       <c r="Q16" s="3" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="R16" s="3" t="s">
         <v>51</v>
@@ -2234,24 +2341,24 @@
         <v>53</v>
       </c>
       <c r="V16" s="3" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="W16" s="3" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="X16" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="Y16" s="3"/>
       <c r="Z16" s="3">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="AA16" s="3"/>
       <c r="AB16" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC16" s="10" t="s">
-        <v>143</v>
+        <v>157</v>
       </c>
       <c r="AD16" s="3" t="s">
         <v>60</v>
@@ -2274,18 +2381,18 @@
         <v>100</v>
       </c>
       <c r="C17" s="7">
-        <v>2026060850</v>
+        <v>2026060846</v>
       </c>
       <c r="D17" s="7"/>
       <c r="E17" s="7"/>
       <c r="F17" s="7">
-        <v>4406</v>
+        <v>2322</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>86</v>
+        <v>128</v>
       </c>
       <c r="I17" s="7"/>
       <c r="J17" s="7"/>
@@ -2294,15 +2401,15 @@
       <c r="M17" s="8"/>
       <c r="N17" s="7"/>
       <c r="O17" s="8"/>
-      <c r="P17" s="8"/>
+      <c r="P17" s="9"/>
       <c r="Q17" s="7" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="R17" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S17" s="7" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="T17" s="7">
         <v>1</v>
@@ -2311,37 +2418,351 @@
         <v>53</v>
       </c>
       <c r="V17" s="7" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="W17" s="7" t="s">
-        <v>136</v>
+        <v>161</v>
       </c>
       <c r="X17" s="7" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="Y17" s="7"/>
       <c r="Z17" s="7">
-        <v>2.2</v>
+        <v>0.5</v>
       </c>
       <c r="AA17" s="7"/>
       <c r="AB17" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC17" s="8" t="s">
-        <v>153</v>
+      <c r="AC17" s="9" t="s">
+        <v>157</v>
       </c>
       <c r="AD17" s="7" t="s">
         <v>60</v>
       </c>
       <c r="AE17" s="7"/>
-      <c r="AF17" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AF17" s="7"/>
       <c r="AG17" s="7"/>
       <c r="AH17" s="7"/>
       <c r="AI17" s="7"/>
       <c r="AJ17" s="7"/>
       <c r="AK17" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="1:37">
+      <c r="A18" s="3">
+        <v>16</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C18" s="3">
+        <v>2026060850</v>
+      </c>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3">
+        <v>4406</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="3"/>
+      <c r="O18" s="4"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="R18" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S18" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="T18" s="3">
+        <v>1</v>
+      </c>
+      <c r="U18" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V18" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="W18" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="X18" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="Y18" s="3"/>
+      <c r="Z18" s="3">
+        <v>2.2</v>
+      </c>
+      <c r="AA18" s="3"/>
+      <c r="AB18" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC18" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="AD18" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE18" s="3"/>
+      <c r="AF18" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG18" s="3"/>
+      <c r="AH18" s="3"/>
+      <c r="AI18" s="3"/>
+      <c r="AJ18" s="3"/>
+      <c r="AK18" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" spans="1:37">
+      <c r="A19" s="7">
+        <v>17</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C19" s="7">
+        <v>2026060898</v>
+      </c>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7">
+        <v>2691</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="7"/>
+      <c r="M19" s="8"/>
+      <c r="N19" s="7"/>
+      <c r="O19" s="8"/>
+      <c r="P19" s="9"/>
+      <c r="Q19" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="R19" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S19" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="T19" s="7">
+        <v>1</v>
+      </c>
+      <c r="U19" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V19" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="W19" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="X19" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y19" s="7"/>
+      <c r="Z19" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA19" s="7"/>
+      <c r="AB19" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC19" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD19" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE19" s="7"/>
+      <c r="AF19" s="7"/>
+      <c r="AG19" s="7"/>
+      <c r="AH19" s="7"/>
+      <c r="AI19" s="7"/>
+      <c r="AJ19" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK19" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:37">
+      <c r="A20" s="3">
+        <v>18</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C20" s="3">
+        <v>2026060899</v>
+      </c>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3">
+        <v>3227</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+      <c r="M20" s="4"/>
+      <c r="N20" s="3"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="10"/>
+      <c r="Q20" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="R20" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S20" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="T20" s="3">
+        <v>1</v>
+      </c>
+      <c r="U20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V20" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="W20" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="X20" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="Y20" s="3"/>
+      <c r="Z20" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA20" s="3"/>
+      <c r="AB20" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC20" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD20" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE20" s="3"/>
+      <c r="AF20" s="3"/>
+      <c r="AG20" s="3"/>
+      <c r="AH20" s="3"/>
+      <c r="AI20" s="3"/>
+      <c r="AJ20" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK20" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:37">
+      <c r="A21" s="7">
+        <v>19</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C21" s="7">
+        <v>2026060905</v>
+      </c>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7">
+        <v>5003</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="I21" s="7"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="7"/>
+      <c r="L21" s="7"/>
+      <c r="M21" s="8"/>
+      <c r="N21" s="7"/>
+      <c r="O21" s="8"/>
+      <c r="P21" s="8"/>
+      <c r="Q21" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="R21" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S21" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="T21" s="7">
+        <v>1</v>
+      </c>
+      <c r="U21" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V21" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="W21" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="X21" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="Y21" s="7"/>
+      <c r="Z21" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA21" s="7"/>
+      <c r="AB21" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC21" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD21" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE21" s="7"/>
+      <c r="AF21" s="7"/>
+      <c r="AG21" s="7"/>
+      <c r="AH21" s="7"/>
+      <c r="AI21" s="7"/>
+      <c r="AJ21" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK21" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06041729
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,14 +11,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$23</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="203">
   <si>
     <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-04  )</t>
   </si>
@@ -539,6 +539,56 @@
     <t>PMQ2+EDC+SC7</t>
   </si>
   <si>
+    <t>E4144115060401</t>
+  </si>
+  <si>
+    <t>新莊頭前店</t>
+  </si>
+  <si>
+    <t>新北市新莊區</t>
+  </si>
+  <si>
+    <t>2026-06-04 09:27:41</t>
+  </si>
+  <si>
+    <t>星期四</t>
+  </si>
+  <si>
+    <t>HL29</t>
+  </si>
+  <si>
+    <t>HL-CCD掃描器(SC)</t>
+  </si>
+  <si>
+    <t>掃描無反應或感應不良</t>
+  </si>
+  <si>
+    <t>門市反應sc ccd掃描器(CLab1070)無法刷讀，有亮燈無逼聲，請門市操作掃描器校正仍異常....須請台芝到店協助(掃描不良)</t>
+  </si>
+  <si>
+    <t>THILF04144</t>
+  </si>
+  <si>
+    <t>湯家瑋</t>
+  </si>
+  <si>
+    <t>2026-06-04 09:43:57</t>
+  </si>
+  <si>
+    <t>2026-06-04 13:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-04 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-05 13:43:00</t>
+  </si>
+  <si>
+    <t>更換手持
+換上8119011009
+換下8119009801</t>
+  </si>
+  <si>
     <t>五股興珍店</t>
   </si>
   <si>
@@ -548,9 +598,6 @@
     <t>THILF02691</t>
   </si>
   <si>
-    <t>湯家瑋</t>
-  </si>
-  <si>
     <t>2026-06-04 11:09:36</t>
   </si>
   <si>
@@ -582,6 +629,21 @@
   </si>
   <si>
     <t>2026-06-04 12:00:00</t>
+  </si>
+  <si>
+    <t>中和員山店</t>
+  </si>
+  <si>
+    <t>新北市中和區</t>
+  </si>
+  <si>
+    <t>THILF02062</t>
+  </si>
+  <si>
+    <t>2026-06-04 16:14:46</t>
+  </si>
+  <si>
+    <t>2026-06-04 16:10:00</t>
   </si>
 </sst>
 </file>
@@ -995,7 +1057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK21"/>
+  <dimension ref="A1:AK23"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -2534,38 +2596,58 @@
         <v>17</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C19" s="7">
-        <v>2026060898</v>
-      </c>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
+        <v>2026060873</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F19" s="7">
-        <v>2691</v>
+        <v>4144</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="I19" s="7"/>
-      <c r="J19" s="7"/>
-      <c r="K19" s="7"/>
-      <c r="L19" s="7"/>
-      <c r="M19" s="8"/>
-      <c r="N19" s="7"/>
-      <c r="O19" s="8"/>
-      <c r="P19" s="9"/>
+        <v>170</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="M19" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="N19" s="7">
+        <v>2901</v>
+      </c>
+      <c r="O19" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="P19" s="9" t="s">
+        <v>176</v>
+      </c>
       <c r="Q19" s="7" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="R19" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S19" s="7" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="T19" s="7">
         <v>1</v>
@@ -2574,15 +2656,17 @@
         <v>53</v>
       </c>
       <c r="V19" s="7" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="W19" s="7" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="X19" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="Y19" s="7"/>
+        <v>181</v>
+      </c>
+      <c r="Y19" s="7" t="s">
+        <v>182</v>
+      </c>
       <c r="Z19" s="7">
         <v>0.5</v>
       </c>
@@ -2591,19 +2675,15 @@
         <v>58</v>
       </c>
       <c r="AC19" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD19" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>183</v>
+      </c>
+      <c r="AD19" s="7"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
       <c r="AG19" s="7"/>
       <c r="AH19" s="7"/>
       <c r="AI19" s="7"/>
-      <c r="AJ19" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ19" s="7"/>
       <c r="AK19" s="7" t="s">
         <v>60</v>
       </c>
@@ -2616,18 +2696,18 @@
         <v>100</v>
       </c>
       <c r="C20" s="3">
-        <v>2026060899</v>
+        <v>2026060898</v>
       </c>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3">
-        <v>3227</v>
+        <v>2691</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
@@ -2638,13 +2718,13 @@
       <c r="O20" s="4"/>
       <c r="P20" s="10"/>
       <c r="Q20" s="3" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="R20" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S20" s="3" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="T20" s="3">
         <v>1</v>
@@ -2653,13 +2733,13 @@
         <v>53</v>
       </c>
       <c r="V20" s="3" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="W20" s="3" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
       <c r="X20" s="3" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="Y20" s="3"/>
       <c r="Z20" s="3">
@@ -2695,18 +2775,18 @@
         <v>100</v>
       </c>
       <c r="C21" s="7">
-        <v>2026060905</v>
+        <v>2026060899</v>
       </c>
       <c r="D21" s="7"/>
       <c r="E21" s="7"/>
       <c r="F21" s="7">
-        <v>5003</v>
+        <v>3227</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="I21" s="7"/>
       <c r="J21" s="7"/>
@@ -2715,15 +2795,15 @@
       <c r="M21" s="8"/>
       <c r="N21" s="7"/>
       <c r="O21" s="8"/>
-      <c r="P21" s="8"/>
+      <c r="P21" s="9"/>
       <c r="Q21" s="7" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="R21" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S21" s="7" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="T21" s="7">
         <v>1</v>
@@ -2732,13 +2812,13 @@
         <v>53</v>
       </c>
       <c r="V21" s="7" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="W21" s="7" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="X21" s="7" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="Y21" s="7"/>
       <c r="Z21" s="7">
@@ -2748,7 +2828,7 @@
       <c r="AB21" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC21" s="8" t="s">
+      <c r="AC21" s="9" t="s">
         <v>111</v>
       </c>
       <c r="AD21" s="7" t="s">
@@ -2763,6 +2843,164 @@
         <v>60</v>
       </c>
       <c r="AK21" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" spans="1:37">
+      <c r="A22" s="3">
+        <v>20</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C22" s="3">
+        <v>2026060905</v>
+      </c>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3">
+        <v>5003</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="3"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="10"/>
+      <c r="Q22" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="R22" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S22" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T22" s="3">
+        <v>1</v>
+      </c>
+      <c r="U22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V22" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="W22" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="X22" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="Y22" s="3"/>
+      <c r="Z22" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA22" s="3"/>
+      <c r="AB22" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC22" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD22" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE22" s="3"/>
+      <c r="AF22" s="3"/>
+      <c r="AG22" s="3"/>
+      <c r="AH22" s="3"/>
+      <c r="AI22" s="3"/>
+      <c r="AJ22" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK22" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="1:37">
+      <c r="A23" s="7">
+        <v>21</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C23" s="7">
+        <v>2026061018</v>
+      </c>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7">
+        <v>2062</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="I23" s="7"/>
+      <c r="J23" s="7"/>
+      <c r="K23" s="7"/>
+      <c r="L23" s="7"/>
+      <c r="M23" s="8"/>
+      <c r="N23" s="7"/>
+      <c r="O23" s="8"/>
+      <c r="P23" s="8"/>
+      <c r="Q23" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="R23" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S23" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T23" s="7">
+        <v>1</v>
+      </c>
+      <c r="U23" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V23" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="W23" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="X23" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="Y23" s="7"/>
+      <c r="Z23" s="7">
+        <v>2.2</v>
+      </c>
+      <c r="AA23" s="7"/>
+      <c r="AB23" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC23" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="AD23" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE23" s="7"/>
+      <c r="AF23" s="7"/>
+      <c r="AG23" s="7"/>
+      <c r="AH23" s="7"/>
+      <c r="AI23" s="7"/>
+      <c r="AJ23" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK23" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06051840
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$23</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$29</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="203">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-04  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="236">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-05  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -631,6 +631,36 @@
     <t>2026-06-04 12:00:00</t>
   </si>
   <si>
+    <t>E2566115060401</t>
+  </si>
+  <si>
+    <t>桃縣桃旺店</t>
+  </si>
+  <si>
+    <t>2026-06-04 11:32:44</t>
+  </si>
+  <si>
+    <t>MMK印票券L90異常不會轉動，確認票券績亮綠燈，但偵測後顯示異常，已有將電源關掉重開紙捲重放仍無法排除....還請台芝到店協助(和lifeet連線的印票機(高鐵票那些的)沒有作用,無法印票)</t>
+  </si>
+  <si>
+    <t>THILF02566</t>
+  </si>
+  <si>
+    <t>2026-06-04 11:52:50</t>
+  </si>
+  <si>
+    <t>2026-06-05 09:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-05 10:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-05 15:52:00</t>
+  </si>
+  <si>
+    <t>網路線脫落，接回後可正常使用</t>
+  </si>
+  <si>
     <t>中和員山店</t>
   </si>
   <si>
@@ -644,6 +674,75 @@
   </si>
   <si>
     <t>2026-06-04 16:10:00</t>
+  </si>
+  <si>
+    <t>2026-06-05 11:46:21</t>
+  </si>
+  <si>
+    <t>2026-06-05 10:50:00</t>
+  </si>
+  <si>
+    <t>2026-06-05 11:45:00</t>
+  </si>
+  <si>
+    <t>蘆竹南山店</t>
+  </si>
+  <si>
+    <t>THILF02501</t>
+  </si>
+  <si>
+    <t>2026-06-05 12:25:58</t>
+  </si>
+  <si>
+    <t>2026-06-05 12:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-05 12:24:00</t>
+  </si>
+  <si>
+    <t>蘆竹興安店</t>
+  </si>
+  <si>
+    <t>THILF03881</t>
+  </si>
+  <si>
+    <t>2026-06-05 14:09:12</t>
+  </si>
+  <si>
+    <t>2026-06-05 13:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-05 14:08:00</t>
+  </si>
+  <si>
+    <t>蘆竹君悅店</t>
+  </si>
+  <si>
+    <t>THILF02622</t>
+  </si>
+  <si>
+    <t>2026-06-05 14:42:05</t>
+  </si>
+  <si>
+    <t>2026-06-05 14:20:00</t>
+  </si>
+  <si>
+    <t>2026-06-05 14:40:00</t>
+  </si>
+  <si>
+    <t>桃縣桃科店</t>
+  </si>
+  <si>
+    <t>THILF02620</t>
+  </si>
+  <si>
+    <t>2026-06-05 15:14:52</t>
+  </si>
+  <si>
+    <t>2026-06-05 14:50:00</t>
+  </si>
+  <si>
+    <t>2026-06-05 15:10:00</t>
   </si>
 </sst>
 </file>
@@ -1057,7 +1156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK23"/>
+  <dimension ref="A1:AK29"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -2930,38 +3029,58 @@
         <v>21</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C23" s="7">
-        <v>2026061018</v>
-      </c>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
+        <v>2026060906</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F23" s="7">
-        <v>2062</v>
+        <v>2566</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="I23" s="7"/>
-      <c r="J23" s="7"/>
-      <c r="K23" s="7"/>
-      <c r="L23" s="7"/>
-      <c r="M23" s="8"/>
-      <c r="N23" s="7"/>
-      <c r="O23" s="8"/>
-      <c r="P23" s="8"/>
+        <v>128</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="M23" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="N23" s="7">
+        <v>6003</v>
+      </c>
+      <c r="O23" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="P23" s="9" t="s">
+        <v>201</v>
+      </c>
       <c r="Q23" s="7" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="R23" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S23" s="7" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="T23" s="7">
         <v>1</v>
@@ -2970,37 +3089,499 @@
         <v>53</v>
       </c>
       <c r="V23" s="7" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="W23" s="7" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
       <c r="X23" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="Y23" s="7"/>
+        <v>205</v>
+      </c>
+      <c r="Y23" s="7" t="s">
+        <v>206</v>
+      </c>
       <c r="Z23" s="7">
-        <v>2.2</v>
+        <v>1</v>
       </c>
       <c r="AA23" s="7"/>
       <c r="AB23" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC23" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="AD23" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AC23" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="AD23" s="7"/>
       <c r="AE23" s="7"/>
       <c r="AF23" s="7"/>
       <c r="AG23" s="7"/>
       <c r="AH23" s="7"/>
       <c r="AI23" s="7"/>
-      <c r="AJ23" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ23" s="7"/>
       <c r="AK23" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" spans="1:37">
+      <c r="A24" s="3">
+        <v>22</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C24" s="3">
+        <v>2026061018</v>
+      </c>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3">
+        <v>2062</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="3"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="10"/>
+      <c r="Q24" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="R24" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S24" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T24" s="3">
+        <v>1</v>
+      </c>
+      <c r="U24" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V24" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="W24" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="X24" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="Y24" s="3"/>
+      <c r="Z24" s="3">
+        <v>2.2</v>
+      </c>
+      <c r="AA24" s="3"/>
+      <c r="AB24" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC24" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="AD24" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE24" s="3"/>
+      <c r="AF24" s="3"/>
+      <c r="AG24" s="3"/>
+      <c r="AH24" s="3"/>
+      <c r="AI24" s="3"/>
+      <c r="AJ24" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK24" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="1:37">
+      <c r="A25" s="7">
+        <v>23</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C25" s="7">
+        <v>2026061123</v>
+      </c>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7">
+        <v>2566</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="7"/>
+      <c r="L25" s="7"/>
+      <c r="M25" s="8"/>
+      <c r="N25" s="7"/>
+      <c r="O25" s="8"/>
+      <c r="P25" s="9"/>
+      <c r="Q25" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="R25" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S25" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T25" s="7">
+        <v>1</v>
+      </c>
+      <c r="U25" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V25" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="W25" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="X25" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="Y25" s="7"/>
+      <c r="Z25" s="7">
+        <v>0.9</v>
+      </c>
+      <c r="AA25" s="7"/>
+      <c r="AB25" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC25" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="AD25" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE25" s="7"/>
+      <c r="AF25" s="7"/>
+      <c r="AG25" s="7"/>
+      <c r="AH25" s="7"/>
+      <c r="AI25" s="7"/>
+      <c r="AJ25" s="7"/>
+      <c r="AK25" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="26" spans="1:37">
+      <c r="A26" s="3">
+        <v>24</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C26" s="3">
+        <v>2026061129</v>
+      </c>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3">
+        <v>2501</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="4"/>
+      <c r="N26" s="3"/>
+      <c r="O26" s="4"/>
+      <c r="P26" s="10"/>
+      <c r="Q26" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="R26" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S26" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T26" s="3">
+        <v>1</v>
+      </c>
+      <c r="U26" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V26" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="W26" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="X26" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="Y26" s="3"/>
+      <c r="Z26" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA26" s="3"/>
+      <c r="AB26" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC26" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="AD26" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE26" s="3"/>
+      <c r="AF26" s="3"/>
+      <c r="AG26" s="3"/>
+      <c r="AH26" s="3"/>
+      <c r="AI26" s="3"/>
+      <c r="AJ26" s="3"/>
+      <c r="AK26" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" spans="1:37">
+      <c r="A27" s="7">
+        <v>25</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C27" s="7">
+        <v>2026061154</v>
+      </c>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7">
+        <v>3881</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I27" s="7"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="7"/>
+      <c r="L27" s="7"/>
+      <c r="M27" s="8"/>
+      <c r="N27" s="7"/>
+      <c r="O27" s="8"/>
+      <c r="P27" s="9"/>
+      <c r="Q27" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="R27" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S27" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T27" s="7">
+        <v>1</v>
+      </c>
+      <c r="U27" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V27" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="W27" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="X27" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="Y27" s="7"/>
+      <c r="Z27" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="AA27" s="7"/>
+      <c r="AB27" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC27" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="AD27" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE27" s="7"/>
+      <c r="AF27" s="7"/>
+      <c r="AG27" s="7"/>
+      <c r="AH27" s="7"/>
+      <c r="AI27" s="7"/>
+      <c r="AJ27" s="7"/>
+      <c r="AK27" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28" spans="1:37">
+      <c r="A28" s="3">
+        <v>26</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C28" s="3">
+        <v>2026061159</v>
+      </c>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3">
+        <v>2622</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="3"/>
+      <c r="O28" s="4"/>
+      <c r="P28" s="10"/>
+      <c r="Q28" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="R28" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S28" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T28" s="3">
+        <v>1</v>
+      </c>
+      <c r="U28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V28" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="W28" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="X28" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="Y28" s="3"/>
+      <c r="Z28" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA28" s="3"/>
+      <c r="AB28" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC28" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="AD28" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE28" s="3"/>
+      <c r="AF28" s="3"/>
+      <c r="AG28" s="3"/>
+      <c r="AH28" s="3"/>
+      <c r="AI28" s="3"/>
+      <c r="AJ28" s="3"/>
+      <c r="AK28" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="1:37">
+      <c r="A29" s="7">
+        <v>27</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C29" s="7">
+        <v>2026061169</v>
+      </c>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7">
+        <v>2620</v>
+      </c>
+      <c r="G29" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I29" s="7"/>
+      <c r="J29" s="7"/>
+      <c r="K29" s="7"/>
+      <c r="L29" s="7"/>
+      <c r="M29" s="8"/>
+      <c r="N29" s="7"/>
+      <c r="O29" s="8"/>
+      <c r="P29" s="8"/>
+      <c r="Q29" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="R29" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S29" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T29" s="7">
+        <v>1</v>
+      </c>
+      <c r="U29" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V29" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="W29" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="X29" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="Y29" s="7"/>
+      <c r="Z29" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA29" s="7"/>
+      <c r="AB29" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC29" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="AD29" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE29" s="7"/>
+      <c r="AF29" s="7"/>
+      <c r="AG29" s="7"/>
+      <c r="AH29" s="7"/>
+      <c r="AI29" s="7"/>
+      <c r="AJ29" s="7"/>
+      <c r="AK29" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06081724
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$29</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$40</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="236">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-05  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="339">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-08  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -676,6 +676,49 @@
     <t>2026-06-04 16:10:00</t>
   </si>
   <si>
+    <t>E4541115060501</t>
+  </si>
+  <si>
+    <t>淡水海天店</t>
+  </si>
+  <si>
+    <t>新北市淡水區</t>
+  </si>
+  <si>
+    <t>2026-06-05 07:24:46</t>
+  </si>
+  <si>
+    <t>凌晨</t>
+  </si>
+  <si>
+    <t>滑鼠故障無作用</t>
+  </si>
+  <si>
+    <t>門市反應SC滑鼠點左健會變右鍵有時候點擊會沒反應，門市已重新拔插線路仍異常....須請台芝到店協助(滑鼠按鍵異常,按第一次沒有反應)
+2026/6/5 (週五) 上午 09:53 MAIL總公司
+06/05 09:24 致電區經理...廖  
+06/05 09:01.09:19 門市電話未接..廖
+06/05 09:55 總公司宸宇來電告知會請部主管聯繫請門市進電叫修中心</t>
+  </si>
+  <si>
+    <t>THILF04541</t>
+  </si>
+  <si>
+    <t>2026-06-05 10:02:33</t>
+  </si>
+  <si>
+    <t>2026-06-08 10:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-08 11:05:00</t>
+  </si>
+  <si>
+    <t>2026-06-08 14:02:00</t>
+  </si>
+  <si>
+    <t>更換滑鼠</t>
+  </si>
+  <si>
     <t>2026-06-05 11:46:21</t>
   </si>
   <si>
@@ -730,6 +773,47 @@
     <t>2026-06-05 14:40:00</t>
   </si>
   <si>
+    <t>14845115060501</t>
+  </si>
+  <si>
+    <t>石門海角店</t>
+  </si>
+  <si>
+    <t>新北市石門區</t>
+  </si>
+  <si>
+    <t>2026-06-05 14:49:39</t>
+  </si>
+  <si>
+    <t>HL59</t>
+  </si>
+  <si>
+    <t>HL-LIFE-ET熱感機T70II</t>
+  </si>
+  <si>
+    <t>門市反應LIFE ET熱感機(T70II)無法列印、亮error橘燈，LIFE ET畫面顯示無法使用印表機，已嘗試重啟MMK與熱感機、並重裝紙捲仍異常...需請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF04845</t>
+  </si>
+  <si>
+    <t>2026-06-05 14:53:07</t>
+  </si>
+  <si>
+    <t>2026-06-08 12:16:00</t>
+  </si>
+  <si>
+    <t>2026-06-08 12:46:00</t>
+  </si>
+  <si>
+    <t>2026-06-08 18:53:00</t>
+  </si>
+  <si>
+    <t>更換出單機
+換下8138002751
+換上8138003163</t>
+  </si>
+  <si>
     <t>桃縣桃科店</t>
   </si>
   <si>
@@ -743,6 +827,246 @@
   </si>
   <si>
     <t>2026-06-05 15:10:00</t>
+  </si>
+  <si>
+    <t>14788115060601</t>
+  </si>
+  <si>
+    <t>急修件</t>
+  </si>
+  <si>
+    <t>淡水國家店</t>
+  </si>
+  <si>
+    <t>2026-06-06 09:33:07</t>
+  </si>
+  <si>
+    <t>星期六</t>
+  </si>
+  <si>
+    <t>檔案損毀(更換硬碟)</t>
+  </si>
+  <si>
+    <t>06/06 09:32啟動緊急叫修:門市SC(SHUTTLE6S)點選HISHOP、e網、訂貨3.0都會出現【捷徑\'HISHOP.lnk\'參照的磁碟機或網路連線無法使用。請確定插入的磁碟正確，而且網路資源可以使用，然後重試。】，重啟SC仍異常。因開啟[訂貨3.0][HiShop][E網]出現捷徑異常訊息，請更換第二顆硬碟不備份還原，並攜帶主機隨行檢測...請台芝到店協助 PS.若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對) 與門市確認帳務做到06/05，與通訊嘉芳確認缺少tm1.2電子存根聯</t>
+  </si>
+  <si>
+    <t>THILF04788</t>
+  </si>
+  <si>
+    <t>2026-06-06 09:40:40</t>
+  </si>
+  <si>
+    <t>2026-06-06 12:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-06 14:56:00</t>
+  </si>
+  <si>
+    <t>2026-06-06 15:40:00</t>
+  </si>
+  <si>
+    <t>更換第二顆硬碟不備份還原完工
+更換Sata線*2</t>
+  </si>
+  <si>
+    <t>12622115060701</t>
+  </si>
+  <si>
+    <t>2026-06-07 10:58:22</t>
+  </si>
+  <si>
+    <t>HL34</t>
+  </si>
+  <si>
+    <t>HL-HUB</t>
+  </si>
+  <si>
+    <t>不能開機</t>
+  </si>
+  <si>
+    <t>06/07 10:58啟動緊急叫修:門市反應店內無網路，PING全店僅90通，查看網管主線為綠燈，請門市查看HUB(DES121028)未過電，已有重新拔插線路、更換至白色插座仍異常....請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-06-07 11:03:20</t>
+  </si>
+  <si>
+    <t>2026-06-07 13:50:00</t>
+  </si>
+  <si>
+    <t>2026-06-07 14:39:00</t>
+  </si>
+  <si>
+    <t>2026-06-07 17:03:00</t>
+  </si>
+  <si>
+    <t>因為前陣子跳電所造成UPS沒電，重新開啟後所有網路皆為正常</t>
+  </si>
+  <si>
+    <t>E4819115060701</t>
+  </si>
+  <si>
+    <t>五股凌雲店</t>
+  </si>
+  <si>
+    <t>2026-06-07 12:13:25</t>
+  </si>
+  <si>
+    <t>06/07 12:10 萊爾富百大門市啟動緊急叫修:門市反應 MMK 四代機 熱感機T70II列印小白單無反應，燈號為綠燈，已有重啟熱感機+MMK仍異常...請台芝到店協助(無法列印)</t>
+  </si>
+  <si>
+    <t>THILF04819</t>
+  </si>
+  <si>
+    <t>2026-06-07 12:19:52</t>
+  </si>
+  <si>
+    <t>2026-06-07 15:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-07 16:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-07 18:19:00</t>
+  </si>
+  <si>
+    <t>因出單機驅動程式跑掉，重灌MMK系統，且更換出單機
+更換出單機
+換下8138001530
+換上8138001718</t>
+  </si>
+  <si>
+    <t>ED070115060801</t>
+  </si>
+  <si>
+    <t>D070</t>
+  </si>
+  <si>
+    <t>三重重新店</t>
+  </si>
+  <si>
+    <t>2026-06-08 06:48:26</t>
+  </si>
+  <si>
+    <t>鍵盤按鍵不良或無反應</t>
+  </si>
+  <si>
+    <t>門市反應SC(SHUTTLE7S)鍵盤數字鍵無反應，已有重新拔插線路仍異常...請台芝到店協助(鍵盤數字鍵無法使用)</t>
+  </si>
+  <si>
+    <t>THILF0D070</t>
+  </si>
+  <si>
+    <t>2026-06-08 09:02:02</t>
+  </si>
+  <si>
+    <t>2026-06-08 10:35:00</t>
+  </si>
+  <si>
+    <t>2026-06-09 13:02:00</t>
+  </si>
+  <si>
+    <t>取消叫修</t>
+  </si>
+  <si>
+    <t>E4483115060701</t>
+  </si>
+  <si>
+    <t>林口築夢店</t>
+  </si>
+  <si>
+    <t>新北市林口區</t>
+  </si>
+  <si>
+    <t>2026-06-07 20:12:35</t>
+  </si>
+  <si>
+    <t>夜間</t>
+  </si>
+  <si>
+    <t>HLF2</t>
+  </si>
+  <si>
+    <t>HL-CCD掃描器(TM)</t>
+  </si>
+  <si>
+    <t>F201</t>
+  </si>
+  <si>
+    <t>門市反應tm1 ccd掃描器(HC56IITR)黑色膠條脫落擋到刷讀的地方..請台芝到店協助(感應不良尤其是寄包裹條碼)
+06/08 09:04  門市話不通...廖</t>
+  </si>
+  <si>
+    <t>THILF04483</t>
+  </si>
+  <si>
+    <t>2026-06-08 09:14:41</t>
+  </si>
+  <si>
+    <t>2026-06-08 14:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-08 15:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-09 13:14:00</t>
+  </si>
+  <si>
+    <t>更換掃描槍
+換下8119006974
+換上8119012936</t>
+  </si>
+  <si>
+    <t>14483115060801</t>
+  </si>
+  <si>
+    <t>2026-06-08 09:14:06</t>
+  </si>
+  <si>
+    <t>門市反應tm2 ccd掃描器(HC56IITR)黑色膠條脫落擋到刷讀的地方..請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-06-08 09:14:59</t>
+  </si>
+  <si>
+    <t>2026-06-09 13:15:00</t>
+  </si>
+  <si>
+    <t>更換掃描槍
+換下8119006975
+換上8119012491</t>
+  </si>
+  <si>
+    <t>北縣五泰店</t>
+  </si>
+  <si>
+    <t>THILF02325</t>
+  </si>
+  <si>
+    <t>2026-06-08 12:26:49</t>
+  </si>
+  <si>
+    <t>2026-06-08 12:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-08 12:30:00</t>
+  </si>
+  <si>
+    <t>五股成州店</t>
+  </si>
+  <si>
+    <t>THILF04801</t>
+  </si>
+  <si>
+    <t>2026-06-08 12:51:53</t>
+  </si>
+  <si>
+    <t>2026-06-08 13:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-08 13:22:05</t>
+  </si>
+  <si>
+    <t>2026-06-08 13:30:00</t>
   </si>
 </sst>
 </file>
@@ -1156,7 +1480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK29"/>
+  <dimension ref="A1:AK40"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -3205,32 +3529,52 @@
         <v>23</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C25" s="7">
-        <v>2026061123</v>
-      </c>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
+        <v>2026061086</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F25" s="7">
-        <v>2566</v>
+        <v>4541</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>199</v>
+        <v>214</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="I25" s="7"/>
-      <c r="J25" s="7"/>
-      <c r="K25" s="7"/>
-      <c r="L25" s="7"/>
-      <c r="M25" s="8"/>
-      <c r="N25" s="7"/>
-      <c r="O25" s="8"/>
-      <c r="P25" s="9"/>
+        <v>215</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="M25" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="N25" s="7">
+        <v>2403</v>
+      </c>
+      <c r="O25" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="P25" s="9" t="s">
+        <v>219</v>
+      </c>
       <c r="Q25" s="7" t="s">
-        <v>202</v>
+        <v>220</v>
       </c>
       <c r="R25" s="7" t="s">
         <v>51</v>
@@ -3245,28 +3589,28 @@
         <v>53</v>
       </c>
       <c r="V25" s="7" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="W25" s="7" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="X25" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="Y25" s="7"/>
+        <v>223</v>
+      </c>
+      <c r="Y25" s="7" t="s">
+        <v>224</v>
+      </c>
       <c r="Z25" s="7">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="AA25" s="7"/>
       <c r="AB25" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC25" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="AD25" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>225</v>
+      </c>
+      <c r="AD25" s="7"/>
       <c r="AE25" s="7"/>
       <c r="AF25" s="7"/>
       <c r="AG25" s="7"/>
@@ -3285,15 +3629,15 @@
         <v>100</v>
       </c>
       <c r="C26" s="3">
-        <v>2026061129</v>
+        <v>2026061123</v>
       </c>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
       <c r="F26" s="3">
-        <v>2501</v>
+        <v>2566</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>216</v>
+        <v>199</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>128</v>
@@ -3307,7 +3651,7 @@
       <c r="O26" s="4"/>
       <c r="P26" s="10"/>
       <c r="Q26" s="3" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="R26" s="3" t="s">
         <v>51</v>
@@ -3322,17 +3666,17 @@
         <v>53</v>
       </c>
       <c r="V26" s="3" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="W26" s="3" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="X26" s="3" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="Y26" s="3"/>
       <c r="Z26" s="3">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
       <c r="AA26" s="3"/>
       <c r="AB26" s="3" t="s">
@@ -3362,15 +3706,15 @@
         <v>100</v>
       </c>
       <c r="C27" s="7">
-        <v>2026061154</v>
+        <v>2026061129</v>
       </c>
       <c r="D27" s="7"/>
       <c r="E27" s="7"/>
       <c r="F27" s="7">
-        <v>3881</v>
+        <v>2501</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="H27" s="7" t="s">
         <v>128</v>
@@ -3384,7 +3728,7 @@
       <c r="O27" s="8"/>
       <c r="P27" s="9"/>
       <c r="Q27" s="7" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="R27" s="7" t="s">
         <v>51</v>
@@ -3399,17 +3743,17 @@
         <v>53</v>
       </c>
       <c r="V27" s="7" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="W27" s="7" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="X27" s="7" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="Y27" s="7"/>
       <c r="Z27" s="7">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="AA27" s="7"/>
       <c r="AB27" s="7" t="s">
@@ -3439,15 +3783,15 @@
         <v>100</v>
       </c>
       <c r="C28" s="3">
-        <v>2026061159</v>
+        <v>2026061154</v>
       </c>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
       <c r="F28" s="3">
-        <v>2622</v>
+        <v>3881</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>128</v>
@@ -3461,7 +3805,7 @@
       <c r="O28" s="4"/>
       <c r="P28" s="10"/>
       <c r="Q28" s="3" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="R28" s="3" t="s">
         <v>51</v>
@@ -3476,17 +3820,17 @@
         <v>53</v>
       </c>
       <c r="V28" s="3" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="W28" s="3" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="X28" s="3" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="Y28" s="3"/>
       <c r="Z28" s="3">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="AA28" s="3"/>
       <c r="AB28" s="3" t="s">
@@ -3516,15 +3860,15 @@
         <v>100</v>
       </c>
       <c r="C29" s="7">
-        <v>2026061169</v>
+        <v>2026061159</v>
       </c>
       <c r="D29" s="7"/>
       <c r="E29" s="7"/>
       <c r="F29" s="7">
-        <v>2620</v>
+        <v>2622</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="H29" s="7" t="s">
         <v>128</v>
@@ -3536,9 +3880,9 @@
       <c r="M29" s="8"/>
       <c r="N29" s="7"/>
       <c r="O29" s="8"/>
-      <c r="P29" s="8"/>
+      <c r="P29" s="9"/>
       <c r="Q29" s="7" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="R29" s="7" t="s">
         <v>51</v>
@@ -3553,13 +3897,13 @@
         <v>53</v>
       </c>
       <c r="V29" s="7" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="W29" s="7" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="X29" s="7" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="Y29" s="7"/>
       <c r="Z29" s="7">
@@ -3569,7 +3913,7 @@
       <c r="AB29" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC29" s="8" t="s">
+      <c r="AC29" s="9" t="s">
         <v>157</v>
       </c>
       <c r="AD29" s="7" t="s">
@@ -3582,6 +3926,999 @@
       <c r="AI29" s="7"/>
       <c r="AJ29" s="7"/>
       <c r="AK29" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30" spans="1:37">
+      <c r="A30" s="3">
+        <v>28</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C30" s="3">
+        <v>2026061163</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F30" s="3">
+        <v>4845</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K30" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L30" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="M30" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="N30" s="3">
+        <v>5903</v>
+      </c>
+      <c r="O30" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="P30" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="Q30" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="R30" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S30" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T30" s="3">
+        <v>1</v>
+      </c>
+      <c r="U30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V30" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="W30" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="X30" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="Y30" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="Z30" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA30" s="3"/>
+      <c r="AB30" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC30" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="AD30" s="3"/>
+      <c r="AE30" s="3"/>
+      <c r="AF30" s="3"/>
+      <c r="AG30" s="3"/>
+      <c r="AH30" s="3"/>
+      <c r="AI30" s="3"/>
+      <c r="AJ30" s="3"/>
+      <c r="AK30" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31" spans="1:37">
+      <c r="A31" s="7">
+        <v>29</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C31" s="7">
+        <v>2026061169</v>
+      </c>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7">
+        <v>2620</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I31" s="7"/>
+      <c r="J31" s="7"/>
+      <c r="K31" s="7"/>
+      <c r="L31" s="7"/>
+      <c r="M31" s="8"/>
+      <c r="N31" s="7"/>
+      <c r="O31" s="8"/>
+      <c r="P31" s="9"/>
+      <c r="Q31" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="R31" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S31" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T31" s="7">
+        <v>1</v>
+      </c>
+      <c r="U31" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V31" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="W31" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="X31" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="Y31" s="7"/>
+      <c r="Z31" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA31" s="7"/>
+      <c r="AB31" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC31" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="AD31" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE31" s="7"/>
+      <c r="AF31" s="7"/>
+      <c r="AG31" s="7"/>
+      <c r="AH31" s="7"/>
+      <c r="AI31" s="7"/>
+      <c r="AJ31" s="7"/>
+      <c r="AK31" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32" spans="1:37">
+      <c r="A32" s="3">
+        <v>30</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C32" s="3">
+        <v>2026061206</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="F32" s="3">
+        <v>4788</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="I32" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="J32" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="K32" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L32" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="M32" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="N32" s="3">
+        <v>2405</v>
+      </c>
+      <c r="O32" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="P32" s="10" t="s">
+        <v>268</v>
+      </c>
+      <c r="Q32" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="R32" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S32" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T32" s="3">
+        <v>1</v>
+      </c>
+      <c r="U32" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V32" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="W32" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="X32" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="Y32" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="Z32" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="AA32" s="3"/>
+      <c r="AB32" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC32" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="AD32" s="3"/>
+      <c r="AE32" s="3"/>
+      <c r="AF32" s="3"/>
+      <c r="AG32" s="3"/>
+      <c r="AH32" s="3"/>
+      <c r="AI32" s="3"/>
+      <c r="AJ32" s="3"/>
+      <c r="AK32" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="33" spans="1:37">
+      <c r="A33" s="7">
+        <v>31</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C33" s="7">
+        <v>2026061218</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="F33" s="7">
+        <v>2622</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="J33" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="K33" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L33" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="M33" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="N33" s="7">
+        <v>3401</v>
+      </c>
+      <c r="O33" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="P33" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="Q33" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="R33" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S33" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T33" s="7">
+        <v>1</v>
+      </c>
+      <c r="U33" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V33" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="W33" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="X33" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="Y33" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="Z33" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="AA33" s="7"/>
+      <c r="AB33" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC33" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="AD33" s="7"/>
+      <c r="AE33" s="7"/>
+      <c r="AF33" s="7"/>
+      <c r="AG33" s="7"/>
+      <c r="AH33" s="7"/>
+      <c r="AI33" s="7"/>
+      <c r="AJ33" s="7"/>
+      <c r="AK33" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="34" spans="1:37">
+      <c r="A34" s="3">
+        <v>32</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C34" s="3">
+        <v>2026061219</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="F34" s="3">
+        <v>4819</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="I34" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="J34" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L34" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="M34" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="N34" s="3">
+        <v>5903</v>
+      </c>
+      <c r="O34" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="P34" s="10" t="s">
+        <v>289</v>
+      </c>
+      <c r="Q34" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="R34" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S34" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T34" s="3">
+        <v>1</v>
+      </c>
+      <c r="U34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V34" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="W34" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="X34" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="Y34" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="Z34" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA34" s="3"/>
+      <c r="AB34" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC34" s="10" t="s">
+        <v>295</v>
+      </c>
+      <c r="AD34" s="3"/>
+      <c r="AE34" s="3"/>
+      <c r="AF34" s="3"/>
+      <c r="AG34" s="3"/>
+      <c r="AH34" s="3"/>
+      <c r="AI34" s="3"/>
+      <c r="AJ34" s="3"/>
+      <c r="AK34" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="35" spans="1:37">
+      <c r="A35" s="7">
+        <v>33</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C35" s="7">
+        <v>2026061226</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="J35" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K35" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="L35" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="M35" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="N35" s="7">
+        <v>2402</v>
+      </c>
+      <c r="O35" s="8" t="s">
+        <v>300</v>
+      </c>
+      <c r="P35" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="Q35" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="R35" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S35" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T35" s="7">
+        <v>1</v>
+      </c>
+      <c r="U35" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V35" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="W35" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="X35" s="7" t="s">
+        <v>304</v>
+      </c>
+      <c r="Y35" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="Z35" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="AA35" s="7"/>
+      <c r="AB35" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="AC35" s="9" t="s">
+        <v>306</v>
+      </c>
+      <c r="AD35" s="7"/>
+      <c r="AE35" s="7"/>
+      <c r="AF35" s="7"/>
+      <c r="AG35" s="7"/>
+      <c r="AH35" s="7"/>
+      <c r="AI35" s="7"/>
+      <c r="AJ35" s="7"/>
+      <c r="AK35" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="36" spans="1:37">
+      <c r="A36" s="3">
+        <v>34</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C36" s="3">
+        <v>2026061233</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F36" s="3">
+        <v>4483</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="J36" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="L36" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="M36" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="N36" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="O36" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="P36" s="10" t="s">
+        <v>315</v>
+      </c>
+      <c r="Q36" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="R36" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S36" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T36" s="3">
+        <v>1</v>
+      </c>
+      <c r="U36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V36" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="W36" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="X36" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="Y36" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="Z36" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA36" s="3"/>
+      <c r="AB36" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC36" s="10" t="s">
+        <v>321</v>
+      </c>
+      <c r="AD36" s="3"/>
+      <c r="AE36" s="3"/>
+      <c r="AF36" s="3"/>
+      <c r="AG36" s="3"/>
+      <c r="AH36" s="3"/>
+      <c r="AI36" s="3"/>
+      <c r="AJ36" s="3"/>
+      <c r="AK36" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="37" spans="1:37">
+      <c r="A37" s="7">
+        <v>35</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C37" s="7">
+        <v>2026061234</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>322</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F37" s="7">
+        <v>4483</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="I37" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="J37" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K37" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L37" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="M37" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="N37" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="O37" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="P37" s="9" t="s">
+        <v>324</v>
+      </c>
+      <c r="Q37" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="R37" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S37" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T37" s="7">
+        <v>1</v>
+      </c>
+      <c r="U37" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V37" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="W37" s="7" t="s">
+        <v>318</v>
+      </c>
+      <c r="X37" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="Y37" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="Z37" s="7">
+        <v>1</v>
+      </c>
+      <c r="AA37" s="7"/>
+      <c r="AB37" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC37" s="9" t="s">
+        <v>327</v>
+      </c>
+      <c r="AD37" s="7"/>
+      <c r="AE37" s="7"/>
+      <c r="AF37" s="7"/>
+      <c r="AG37" s="7"/>
+      <c r="AH37" s="7"/>
+      <c r="AI37" s="7"/>
+      <c r="AJ37" s="7"/>
+      <c r="AK37" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="38" spans="1:37">
+      <c r="A38" s="3">
+        <v>36</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C38" s="3">
+        <v>2026061273</v>
+      </c>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3">
+        <v>2325</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
+      <c r="K38" s="3"/>
+      <c r="L38" s="3"/>
+      <c r="M38" s="4"/>
+      <c r="N38" s="3"/>
+      <c r="O38" s="4"/>
+      <c r="P38" s="10"/>
+      <c r="Q38" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="R38" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S38" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T38" s="3">
+        <v>1</v>
+      </c>
+      <c r="U38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V38" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="W38" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="X38" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="Y38" s="3"/>
+      <c r="Z38" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA38" s="3"/>
+      <c r="AB38" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC38" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD38" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE38" s="3"/>
+      <c r="AF38" s="3"/>
+      <c r="AG38" s="3"/>
+      <c r="AH38" s="3"/>
+      <c r="AI38" s="3"/>
+      <c r="AJ38" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK38" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="39" spans="1:37">
+      <c r="A39" s="7">
+        <v>37</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C39" s="7">
+        <v>2026061276</v>
+      </c>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7">
+        <v>4801</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I39" s="7"/>
+      <c r="J39" s="7"/>
+      <c r="K39" s="7"/>
+      <c r="L39" s="7"/>
+      <c r="M39" s="8"/>
+      <c r="N39" s="7"/>
+      <c r="O39" s="8"/>
+      <c r="P39" s="9"/>
+      <c r="Q39" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="R39" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S39" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T39" s="7">
+        <v>1</v>
+      </c>
+      <c r="U39" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V39" s="7" t="s">
+        <v>335</v>
+      </c>
+      <c r="W39" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="X39" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="Y39" s="7"/>
+      <c r="Z39" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA39" s="7"/>
+      <c r="AB39" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC39" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD39" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE39" s="7"/>
+      <c r="AF39" s="7"/>
+      <c r="AG39" s="7"/>
+      <c r="AH39" s="7"/>
+      <c r="AI39" s="7"/>
+      <c r="AJ39" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK39" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="40" spans="1:37">
+      <c r="A40" s="3">
+        <v>38</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C40" s="3">
+        <v>2026061283</v>
+      </c>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3">
+        <v>4819</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="I40" s="3"/>
+      <c r="J40" s="3"/>
+      <c r="K40" s="3"/>
+      <c r="L40" s="3"/>
+      <c r="M40" s="4"/>
+      <c r="N40" s="3"/>
+      <c r="O40" s="4"/>
+      <c r="P40" s="4"/>
+      <c r="Q40" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="R40" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S40" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T40" s="3">
+        <v>1</v>
+      </c>
+      <c r="U40" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V40" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="W40" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="X40" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="Y40" s="3"/>
+      <c r="Z40" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA40" s="3"/>
+      <c r="AB40" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC40" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD40" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE40" s="3"/>
+      <c r="AF40" s="3"/>
+      <c r="AG40" s="3"/>
+      <c r="AH40" s="3"/>
+      <c r="AI40" s="3"/>
+      <c r="AJ40" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK40" s="3" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06091720
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$45</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="339">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-08  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="374">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-09  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -935,6 +935,50 @@
 換上8138001718</t>
   </si>
   <si>
+    <t>1D349115060701</t>
+  </si>
+  <si>
+    <t>D349</t>
+  </si>
+  <si>
+    <t>板橋成都店</t>
+  </si>
+  <si>
+    <t>2026-06-07 15:49:33</t>
+  </si>
+  <si>
+    <t>HLD3</t>
+  </si>
+  <si>
+    <t>HL-熱感發票機</t>
+  </si>
+  <si>
+    <t>D303</t>
+  </si>
+  <si>
+    <t>TM1(TCX800)熱感發票機(BSC10)門市反應TM1頻繁出現請檢察熱感機電源是否開啟或USB插頭沒接上，門市已將紙捲重裝重啟後及檢查後線路拔插，但當下重啟發票機後可正常，但交易幾筆後又會再次出現..請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF0D349</t>
+  </si>
+  <si>
+    <t>2026-06-07 15:56:50</t>
+  </si>
+  <si>
+    <t>2026-06-09 11:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-09 11:37:00</t>
+  </si>
+  <si>
+    <t>2026-06-09 13:00:00</t>
+  </si>
+  <si>
+    <t>更換發票機
+換上：8155004462
+換下：8155002869</t>
+  </si>
+  <si>
     <t>ED070115060801</t>
   </si>
   <si>
@@ -1036,6 +1080,39 @@
 換上8119012491</t>
   </si>
   <si>
+    <t>14917115060801</t>
+  </si>
+  <si>
+    <t>板橋翠華店</t>
+  </si>
+  <si>
+    <t>2026-06-08 10:40:59</t>
+  </si>
+  <si>
+    <t>抽屜無法正常開關</t>
+  </si>
+  <si>
+    <t>門市反應tm1(TCX800)抽屜打不開，已請門市發票機重啟測試點餐紙正常但仍打不開抽屜無彈出聲，抽屜外觀黑色/鑰匙孔中間/無鑰匙孔編號...須請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF04917</t>
+  </si>
+  <si>
+    <t>2026-06-08 10:43:01</t>
+  </si>
+  <si>
+    <t>2026-06-09 11:50:00</t>
+  </si>
+  <si>
+    <t>2026-06-09 12:15:00</t>
+  </si>
+  <si>
+    <t>2026-06-09 14:43:00</t>
+  </si>
+  <si>
+    <t>線路重新插拔測試正常</t>
+  </si>
+  <si>
     <t>北縣五泰店</t>
   </si>
   <si>
@@ -1067,6 +1144,36 @@
   </si>
   <si>
     <t>2026-06-08 13:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-09 12:20:37</t>
+  </si>
+  <si>
+    <t>新莊棒球場</t>
+  </si>
+  <si>
+    <t>THILF03358</t>
+  </si>
+  <si>
+    <t>2026-06-09 14:17:48</t>
+  </si>
+  <si>
+    <t>2026-06-09 14:00:00</t>
+  </si>
+  <si>
+    <t>中和景德店</t>
+  </si>
+  <si>
+    <t>THILF04536</t>
+  </si>
+  <si>
+    <t>2026-06-09 16:02:27</t>
+  </si>
+  <si>
+    <t>2026-06-09 13:40:00</t>
+  </si>
+  <si>
+    <t>2026-06-09 16:00:00</t>
   </si>
 </sst>
 </file>
@@ -1480,7 +1587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK40"/>
+  <dimension ref="A1:AK45"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -4402,7 +4509,7 @@
         <v>38</v>
       </c>
       <c r="C35" s="7">
-        <v>2026061226</v>
+        <v>2026061222</v>
       </c>
       <c r="D35" s="7" t="s">
         <v>296</v>
@@ -4417,40 +4524,40 @@
         <v>298</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>42</v>
+        <v>86</v>
       </c>
       <c r="I35" s="7" t="s">
         <v>299</v>
       </c>
       <c r="J35" s="7" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="K35" s="7" t="s">
-        <v>217</v>
+        <v>45</v>
       </c>
       <c r="L35" s="7" t="s">
-        <v>142</v>
+        <v>300</v>
       </c>
       <c r="M35" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="N35" s="7">
-        <v>2402</v>
+        <v>301</v>
+      </c>
+      <c r="N35" s="7" t="s">
+        <v>302</v>
       </c>
       <c r="O35" s="8" t="s">
-        <v>300</v>
+        <v>91</v>
       </c>
       <c r="P35" s="9" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="Q35" s="7" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="R35" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S35" s="7" t="s">
-        <v>52</v>
+        <v>94</v>
       </c>
       <c r="T35" s="7">
         <v>1</v>
@@ -4459,26 +4566,26 @@
         <v>53</v>
       </c>
       <c r="V35" s="7" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="W35" s="7" t="s">
-        <v>222</v>
+        <v>306</v>
       </c>
       <c r="X35" s="7" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="Y35" s="7" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="Z35" s="7">
-        <v>0.1</v>
+        <v>0.6</v>
       </c>
       <c r="AA35" s="7"/>
       <c r="AB35" s="7" t="s">
-        <v>306</v>
+        <v>58</v>
       </c>
       <c r="AC35" s="9" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="AD35" s="7"/>
       <c r="AE35" s="7"/>
@@ -4499,43 +4606,43 @@
         <v>38</v>
       </c>
       <c r="C36" s="3">
-        <v>2026061233</v>
+        <v>2026061226</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F36" s="3">
-        <v>4483</v>
+      <c r="F36" s="3" t="s">
+        <v>311</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>309</v>
+        <v>42</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>311</v>
+        <v>217</v>
       </c>
       <c r="L36" s="3" t="s">
-        <v>312</v>
+        <v>142</v>
       </c>
       <c r="M36" s="4" t="s">
-        <v>313</v>
-      </c>
-      <c r="N36" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="N36" s="3">
+        <v>2402</v>
+      </c>
+      <c r="O36" s="4" t="s">
         <v>314</v>
-      </c>
-      <c r="O36" s="4" t="s">
-        <v>175</v>
       </c>
       <c r="P36" s="10" t="s">
         <v>315</v>
@@ -4547,7 +4654,7 @@
         <v>51</v>
       </c>
       <c r="S36" s="3" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="T36" s="3">
         <v>1</v>
@@ -4559,23 +4666,23 @@
         <v>317</v>
       </c>
       <c r="W36" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="X36" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="X36" s="3" t="s">
+      <c r="Y36" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="Y36" s="3" t="s">
-        <v>320</v>
-      </c>
       <c r="Z36" s="3">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="AA36" s="3"/>
       <c r="AB36" s="3" t="s">
-        <v>58</v>
+        <v>320</v>
       </c>
       <c r="AC36" s="10" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AD36" s="3"/>
       <c r="AE36" s="3"/>
@@ -4596,10 +4703,10 @@
         <v>38</v>
       </c>
       <c r="C37" s="7">
-        <v>2026061234</v>
+        <v>2026061233</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E37" s="7" t="s">
         <v>40</v>
@@ -4608,37 +4715,37 @@
         <v>4483</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>308</v>
+        <v>322</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>309</v>
+        <v>323</v>
       </c>
       <c r="I37" s="7" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="J37" s="7" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="K37" s="7" t="s">
-        <v>65</v>
+        <v>325</v>
       </c>
       <c r="L37" s="7" t="s">
-        <v>312</v>
+        <v>326</v>
       </c>
       <c r="M37" s="8" t="s">
-        <v>313</v>
+        <v>327</v>
       </c>
       <c r="N37" s="7" t="s">
-        <v>314</v>
+        <v>328</v>
       </c>
       <c r="O37" s="8" t="s">
         <v>175</v>
       </c>
       <c r="P37" s="9" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="Q37" s="7" t="s">
-        <v>316</v>
+        <v>330</v>
       </c>
       <c r="R37" s="7" t="s">
         <v>51</v>
@@ -4653,16 +4760,16 @@
         <v>53</v>
       </c>
       <c r="V37" s="7" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="W37" s="7" t="s">
-        <v>318</v>
+        <v>332</v>
       </c>
       <c r="X37" s="7" t="s">
-        <v>319</v>
+        <v>333</v>
       </c>
       <c r="Y37" s="7" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="Z37" s="7">
         <v>1</v>
@@ -4672,7 +4779,7 @@
         <v>58</v>
       </c>
       <c r="AC37" s="9" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="AD37" s="7"/>
       <c r="AE37" s="7"/>
@@ -4690,38 +4797,58 @@
         <v>36</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C38" s="3">
-        <v>2026061273</v>
-      </c>
-      <c r="D38" s="3"/>
-      <c r="E38" s="3"/>
+        <v>2026061234</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="F38" s="3">
-        <v>2325</v>
+        <v>4483</v>
       </c>
       <c r="G38" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L38" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="M38" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="N38" s="3" t="s">
         <v>328</v>
       </c>
-      <c r="H38" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="I38" s="3"/>
-      <c r="J38" s="3"/>
-      <c r="K38" s="3"/>
-      <c r="L38" s="3"/>
-      <c r="M38" s="4"/>
-      <c r="N38" s="3"/>
-      <c r="O38" s="4"/>
-      <c r="P38" s="10"/>
+      <c r="O38" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="P38" s="10" t="s">
+        <v>338</v>
+      </c>
       <c r="Q38" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="R38" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S38" s="3" t="s">
-        <v>178</v>
+        <v>79</v>
       </c>
       <c r="T38" s="3">
         <v>1</v>
@@ -4730,36 +4857,34 @@
         <v>53</v>
       </c>
       <c r="V38" s="3" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
       <c r="W38" s="3" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="X38" s="3" t="s">
-        <v>332</v>
-      </c>
-      <c r="Y38" s="3"/>
+        <v>333</v>
+      </c>
+      <c r="Y38" s="3" t="s">
+        <v>340</v>
+      </c>
       <c r="Z38" s="3">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="AA38" s="3"/>
       <c r="AB38" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC38" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD38" s="3" t="s">
-        <v>60</v>
-      </c>
+        <v>341</v>
+      </c>
+      <c r="AD38" s="3"/>
       <c r="AE38" s="3"/>
       <c r="AF38" s="3"/>
       <c r="AG38" s="3"/>
       <c r="AH38" s="3"/>
       <c r="AI38" s="3"/>
-      <c r="AJ38" s="3" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ38" s="3"/>
       <c r="AK38" s="3" t="s">
         <v>60</v>
       </c>
@@ -4769,38 +4894,58 @@
         <v>37</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C39" s="7">
-        <v>2026061276</v>
-      </c>
-      <c r="D39" s="7"/>
-      <c r="E39" s="7"/>
+        <v>2026061260</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F39" s="7">
-        <v>4801</v>
+        <v>4917</v>
       </c>
       <c r="G39" s="7" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="I39" s="7"/>
-      <c r="J39" s="7"/>
-      <c r="K39" s="7"/>
-      <c r="L39" s="7"/>
-      <c r="M39" s="8"/>
-      <c r="N39" s="7"/>
-      <c r="O39" s="8"/>
-      <c r="P39" s="9"/>
+        <v>86</v>
+      </c>
+      <c r="I39" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="J39" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K39" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L39" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M39" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="N39" s="7">
+        <v>2305</v>
+      </c>
+      <c r="O39" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="P39" s="9" t="s">
+        <v>346</v>
+      </c>
       <c r="Q39" s="7" t="s">
-        <v>334</v>
+        <v>347</v>
       </c>
       <c r="R39" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S39" s="7" t="s">
-        <v>178</v>
+        <v>94</v>
       </c>
       <c r="T39" s="7">
         <v>1</v>
@@ -4809,36 +4954,34 @@
         <v>53</v>
       </c>
       <c r="V39" s="7" t="s">
-        <v>335</v>
+        <v>348</v>
       </c>
       <c r="W39" s="7" t="s">
-        <v>332</v>
+        <v>349</v>
       </c>
       <c r="X39" s="7" t="s">
-        <v>336</v>
-      </c>
-      <c r="Y39" s="7"/>
+        <v>350</v>
+      </c>
+      <c r="Y39" s="7" t="s">
+        <v>351</v>
+      </c>
       <c r="Z39" s="7">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="AA39" s="7"/>
       <c r="AB39" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC39" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD39" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>352</v>
+      </c>
+      <c r="AD39" s="7"/>
       <c r="AE39" s="7"/>
       <c r="AF39" s="7"/>
       <c r="AG39" s="7"/>
       <c r="AH39" s="7"/>
       <c r="AI39" s="7"/>
-      <c r="AJ39" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ39" s="7"/>
       <c r="AK39" s="7" t="s">
         <v>60</v>
       </c>
@@ -4851,15 +4994,15 @@
         <v>100</v>
       </c>
       <c r="C40" s="3">
-        <v>2026061283</v>
+        <v>2026061273</v>
       </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
       <c r="F40" s="3">
-        <v>4819</v>
+        <v>2325</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>287</v>
+        <v>353</v>
       </c>
       <c r="H40" s="3" t="s">
         <v>185</v>
@@ -4871,9 +5014,9 @@
       <c r="M40" s="4"/>
       <c r="N40" s="3"/>
       <c r="O40" s="4"/>
-      <c r="P40" s="4"/>
+      <c r="P40" s="10"/>
       <c r="Q40" s="3" t="s">
-        <v>290</v>
+        <v>354</v>
       </c>
       <c r="R40" s="3" t="s">
         <v>51</v>
@@ -4888,13 +5031,13 @@
         <v>53</v>
       </c>
       <c r="V40" s="3" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="W40" s="3" t="s">
-        <v>336</v>
+        <v>356</v>
       </c>
       <c r="X40" s="3" t="s">
-        <v>338</v>
+        <v>357</v>
       </c>
       <c r="Y40" s="3"/>
       <c r="Z40" s="3">
@@ -4904,7 +5047,7 @@
       <c r="AB40" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="AC40" s="4" t="s">
+      <c r="AC40" s="10" t="s">
         <v>111</v>
       </c>
       <c r="AD40" s="3" t="s">
@@ -4919,6 +5062,397 @@
         <v>60</v>
       </c>
       <c r="AK40" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="41" spans="1:37">
+      <c r="A41" s="7">
+        <v>39</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C41" s="7">
+        <v>2026061276</v>
+      </c>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="7">
+        <v>4801</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I41" s="7"/>
+      <c r="J41" s="7"/>
+      <c r="K41" s="7"/>
+      <c r="L41" s="7"/>
+      <c r="M41" s="8"/>
+      <c r="N41" s="7"/>
+      <c r="O41" s="8"/>
+      <c r="P41" s="9"/>
+      <c r="Q41" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="R41" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S41" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T41" s="7">
+        <v>1</v>
+      </c>
+      <c r="U41" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V41" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="W41" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="X41" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="Y41" s="7"/>
+      <c r="Z41" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA41" s="7"/>
+      <c r="AB41" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC41" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD41" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE41" s="7"/>
+      <c r="AF41" s="7"/>
+      <c r="AG41" s="7"/>
+      <c r="AH41" s="7"/>
+      <c r="AI41" s="7"/>
+      <c r="AJ41" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK41" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="42" spans="1:37">
+      <c r="A42" s="3">
+        <v>40</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C42" s="3">
+        <v>2026061283</v>
+      </c>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3">
+        <v>4819</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="3"/>
+      <c r="L42" s="3"/>
+      <c r="M42" s="4"/>
+      <c r="N42" s="3"/>
+      <c r="O42" s="4"/>
+      <c r="P42" s="10"/>
+      <c r="Q42" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="R42" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S42" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T42" s="3">
+        <v>1</v>
+      </c>
+      <c r="U42" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V42" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="W42" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="X42" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="Y42" s="3"/>
+      <c r="Z42" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA42" s="3"/>
+      <c r="AB42" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC42" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD42" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE42" s="3"/>
+      <c r="AF42" s="3"/>
+      <c r="AG42" s="3"/>
+      <c r="AH42" s="3"/>
+      <c r="AI42" s="3"/>
+      <c r="AJ42" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK42" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="43" spans="1:37">
+      <c r="A43" s="7">
+        <v>41</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C43" s="7">
+        <v>2026061529</v>
+      </c>
+      <c r="D43" s="7"/>
+      <c r="E43" s="7"/>
+      <c r="F43" s="7">
+        <v>4917</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="H43" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I43" s="7"/>
+      <c r="J43" s="7"/>
+      <c r="K43" s="7"/>
+      <c r="L43" s="7"/>
+      <c r="M43" s="8"/>
+      <c r="N43" s="7"/>
+      <c r="O43" s="8"/>
+      <c r="P43" s="9"/>
+      <c r="Q43" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="R43" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S43" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="T43" s="7">
+        <v>1</v>
+      </c>
+      <c r="U43" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V43" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="W43" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="X43" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="Y43" s="7"/>
+      <c r="Z43" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA43" s="7"/>
+      <c r="AB43" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC43" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD43" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE43" s="7"/>
+      <c r="AF43" s="7"/>
+      <c r="AG43" s="7"/>
+      <c r="AH43" s="7"/>
+      <c r="AI43" s="7"/>
+      <c r="AJ43" s="7"/>
+      <c r="AK43" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="44" spans="1:37">
+      <c r="A44" s="3">
+        <v>42</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C44" s="3">
+        <v>2026061539</v>
+      </c>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3">
+        <v>3358</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="I44" s="3"/>
+      <c r="J44" s="3"/>
+      <c r="K44" s="3"/>
+      <c r="L44" s="3"/>
+      <c r="M44" s="4"/>
+      <c r="N44" s="3"/>
+      <c r="O44" s="4"/>
+      <c r="P44" s="10"/>
+      <c r="Q44" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="R44" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S44" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T44" s="3">
+        <v>1</v>
+      </c>
+      <c r="U44" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V44" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="W44" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="X44" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="Y44" s="3"/>
+      <c r="Z44" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA44" s="3"/>
+      <c r="AB44" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC44" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="AD44" s="3"/>
+      <c r="AE44" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF44" s="3"/>
+      <c r="AG44" s="3"/>
+      <c r="AH44" s="3"/>
+      <c r="AI44" s="3"/>
+      <c r="AJ44" s="3"/>
+      <c r="AK44" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="45" spans="1:37">
+      <c r="A45" s="7">
+        <v>43</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C45" s="7">
+        <v>2026061569</v>
+      </c>
+      <c r="D45" s="7"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7">
+        <v>4536</v>
+      </c>
+      <c r="G45" s="7" t="s">
+        <v>369</v>
+      </c>
+      <c r="H45" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="I45" s="7"/>
+      <c r="J45" s="7"/>
+      <c r="K45" s="7"/>
+      <c r="L45" s="7"/>
+      <c r="M45" s="8"/>
+      <c r="N45" s="7"/>
+      <c r="O45" s="8"/>
+      <c r="P45" s="8"/>
+      <c r="Q45" s="7" t="s">
+        <v>370</v>
+      </c>
+      <c r="R45" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S45" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T45" s="7">
+        <v>1</v>
+      </c>
+      <c r="U45" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V45" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="W45" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="X45" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="Y45" s="7"/>
+      <c r="Z45" s="7">
+        <v>2.3</v>
+      </c>
+      <c r="AA45" s="7"/>
+      <c r="AB45" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC45" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="AD45" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE45" s="7"/>
+      <c r="AF45" s="7"/>
+      <c r="AG45" s="7"/>
+      <c r="AH45" s="7"/>
+      <c r="AI45" s="7"/>
+      <c r="AJ45" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK45" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06111805
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$45</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$65</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="374">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-10  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="496">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-11  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -1174,6 +1174,380 @@
   </si>
   <si>
     <t>2026-06-09 16:00:00</t>
+  </si>
+  <si>
+    <t>E2209115060901</t>
+  </si>
+  <si>
+    <t>2026-06-09 16:50:01</t>
+  </si>
+  <si>
+    <t>星期二</t>
+  </si>
+  <si>
+    <t>門市反應TM2(TCX800)上方會員的地方需要點很多次才有反應，確認無貼透明塑膠墊及文宣，客服協助執行觸控校正仍異常，門市告知已反應多次，5/14工程師到店重新整理排線.執行觸控校正，6/1工程師到店更換主機仍無改善..請台芝到店協助(2號機無法按會員)</t>
+  </si>
+  <si>
+    <t>2026-06-09 17:03:25</t>
+  </si>
+  <si>
+    <t>2026-06-10 10:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-10 12:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-10 21:03:00</t>
+  </si>
+  <si>
+    <t>換下8185002320.換上8185000786</t>
+  </si>
+  <si>
+    <t>1D767115061001</t>
+  </si>
+  <si>
+    <t>D767</t>
+  </si>
+  <si>
+    <t>板橋寶翠店</t>
+  </si>
+  <si>
+    <t>2026-06-10 09:24:23</t>
+  </si>
+  <si>
+    <t>門市反應tm1 ccd掃描器(HC56II-TR、HC76-TR	)刷讀所有條碼常常都感應不到有亮燈有逼聲，門市告知校正表單第二段、第三段刷不過去....請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF0D767</t>
+  </si>
+  <si>
+    <t>2026-06-10 09:25:33</t>
+  </si>
+  <si>
+    <t>2026-06-11 12:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 12:40:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 13:25:00</t>
+  </si>
+  <si>
+    <t>更換掃槍
+換上：8119012471
+換下：8119008154</t>
+  </si>
+  <si>
+    <t>1C216115061001</t>
+  </si>
+  <si>
+    <t>C216</t>
+  </si>
+  <si>
+    <t>中和南勢店</t>
+  </si>
+  <si>
+    <t>2026-06-10 10:27:59</t>
+  </si>
+  <si>
+    <t>SC升級SQL2019更新失敗，發現更新檔案損壞，SC型號：SHUTTLE7S 請到店更換SC第一顆硬碟，資料不備份、不還原。(到店時需先進線騰雲確認銷售資料是否已傳回萊爾富總公司)</t>
+  </si>
+  <si>
+    <t>THILF0C216</t>
+  </si>
+  <si>
+    <t>2026-06-10 10:32:42</t>
+  </si>
+  <si>
+    <t>2026-06-11 10:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 12:27:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 14:32:00</t>
+  </si>
+  <si>
+    <t>更換第一顆硬碟不備份還原. 已跟店家告知回報代收會計</t>
+  </si>
+  <si>
+    <t>龜山復恆店</t>
+  </si>
+  <si>
+    <t>THILF04503</t>
+  </si>
+  <si>
+    <t>2026-06-10 12:09:16</t>
+  </si>
+  <si>
+    <t>2026-06-10 11:00:00</t>
+  </si>
+  <si>
+    <t>L533</t>
+  </si>
+  <si>
+    <t>田倉復興店</t>
+  </si>
+  <si>
+    <t>THILF0L533</t>
+  </si>
+  <si>
+    <t>2026-06-10 12:27:18</t>
+  </si>
+  <si>
+    <t>2026-06-10 12:10:00</t>
+  </si>
+  <si>
+    <t>2026-06-10 12:25:00</t>
+  </si>
+  <si>
+    <t>PMQ2</t>
+  </si>
+  <si>
+    <t>龜山文化七</t>
+  </si>
+  <si>
+    <t>THILF05031</t>
+  </si>
+  <si>
+    <t>2026-06-10 12:54:49</t>
+  </si>
+  <si>
+    <t>2026-06-10 12:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-10 12:50:00</t>
+  </si>
+  <si>
+    <t>龜山頂湖店</t>
+  </si>
+  <si>
+    <t>THILF03692</t>
+  </si>
+  <si>
+    <t>2026-06-10 14:13:14</t>
+  </si>
+  <si>
+    <t>2026-06-10 13:10:00</t>
+  </si>
+  <si>
+    <t>2026-06-10 13:40:00</t>
+  </si>
+  <si>
+    <t>E4422115061001</t>
+  </si>
+  <si>
+    <t>板橋合安店</t>
+  </si>
+  <si>
+    <t>2026-06-10 14:00:34</t>
+  </si>
+  <si>
+    <t>門市反應tm1(TCX800) ccd掃描器(HC76TR)刷讀生生喝鮮乳和店內商品掃描條碼感應不良，有亮燈有逼聲兩台tm都無法刷讀已有操作掃描器校正仍異常....須請台芝到店協助(感應不良  機一 兌換卷第二條無法刷取  基二  兩個兌換條碼常感應不良)</t>
+  </si>
+  <si>
+    <t>THILF04422</t>
+  </si>
+  <si>
+    <t>2026-06-10 14:20:48</t>
+  </si>
+  <si>
+    <t>2026-06-11 12:50:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 13:55:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 18:20:00</t>
+  </si>
+  <si>
+    <t>更換發票機
+換上：8155005860
+換下：8155003127</t>
+  </si>
+  <si>
+    <t>14422115061001</t>
+  </si>
+  <si>
+    <t>2026-06-10 14:20:46</t>
+  </si>
+  <si>
+    <t>門市反應tm2(TCX800) ccd掃描器(HC76TR)刷讀生生喝鮮乳和店內商品掃描條碼感應不良，有亮燈有逼聲兩台tm都無法刷讀已有操作掃描器校正仍異常....須請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-06-10 14:21:17</t>
+  </si>
+  <si>
+    <t>2026-06-11 13:54:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 18:21:00</t>
+  </si>
+  <si>
+    <t>更換發票機
+換上：8155005859
+換下：8155003532</t>
+  </si>
+  <si>
+    <t>桃縣桃燿店</t>
+  </si>
+  <si>
+    <t>THILF02763</t>
+  </si>
+  <si>
+    <t>2026-06-10 14:45:38</t>
+  </si>
+  <si>
+    <t>2026-06-10 13:50:00</t>
+  </si>
+  <si>
+    <t>2026-06-10 14:20:00</t>
+  </si>
+  <si>
+    <t>蘆竹南工店</t>
+  </si>
+  <si>
+    <t>THILF02401</t>
+  </si>
+  <si>
+    <t>2026-06-10 15:33:25</t>
+  </si>
+  <si>
+    <t>2026-06-10 15:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-10 15:30:00</t>
+  </si>
+  <si>
+    <t>蘆竹蘆興店</t>
+  </si>
+  <si>
+    <t>THILF02988</t>
+  </si>
+  <si>
+    <t>2026-06-10 16:03:16</t>
+  </si>
+  <si>
+    <t>2026-06-10 15:35:00</t>
+  </si>
+  <si>
+    <t>2026-06-10 16:01:00</t>
+  </si>
+  <si>
+    <t>13811115061001</t>
+  </si>
+  <si>
+    <t>三重碧華公園</t>
+  </si>
+  <si>
+    <t>2026-06-10 16:12:26</t>
+  </si>
+  <si>
+    <t>HLF6</t>
+  </si>
+  <si>
+    <t>HL-多卡機QP3000E</t>
+  </si>
+  <si>
+    <t>F604</t>
+  </si>
+  <si>
+    <t>無電源反應</t>
+  </si>
+  <si>
+    <t>門市反應TM1(TCX800)多卡機(QP3000E)無電源反應黑屏，後方線路雜亂無法重新拔插....須請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF03811</t>
+  </si>
+  <si>
+    <t>2026-06-10 16:13:50</t>
+  </si>
+  <si>
+    <t>2026-06-11 17:15:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 17:34:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 20:13:00</t>
+  </si>
+  <si>
+    <t>重接線路測試正常</t>
+  </si>
+  <si>
+    <t>13811115061002</t>
+  </si>
+  <si>
+    <t>2026-06-10 16:13:54</t>
+  </si>
+  <si>
+    <t>門市反應TM2(TCX800)多卡機(QP3000E)無電源反應黑屏，後方線路雜亂無法重新拔插....須請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-06-10 16:14:30</t>
+  </si>
+  <si>
+    <t>2026-06-11 17:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 20:14:00</t>
+  </si>
+  <si>
+    <t>龜山慧敏店</t>
+  </si>
+  <si>
+    <t>THILF05248</t>
+  </si>
+  <si>
+    <t>2026-06-11 11:14:11</t>
+  </si>
+  <si>
+    <t>2026-06-11 10:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 11:00:00</t>
+  </si>
+  <si>
+    <t>協助撤店 現場無店章</t>
+  </si>
+  <si>
+    <t>2026-06-11 11:15:23</t>
+  </si>
+  <si>
+    <t>PMQ2+EDC
+現場無印章</t>
+  </si>
+  <si>
+    <t>2026-06-11 11:15:30</t>
+  </si>
+  <si>
+    <t>裝潢撤機完工
+現場無印章</t>
+  </si>
+  <si>
+    <t>2026-06-11 12:43:32</t>
+  </si>
+  <si>
+    <t>2026-06-11 13:58:38</t>
+  </si>
+  <si>
+    <t>2026-06-11 13:15:00</t>
+  </si>
+  <si>
+    <t>中和霸氣店</t>
+  </si>
+  <si>
+    <t>THILF04748</t>
+  </si>
+  <si>
+    <t>2026-06-11 15:53:10</t>
+  </si>
+  <si>
+    <t>2026-06-11 13:50:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 15:50:00</t>
   </si>
 </sst>
 </file>
@@ -1587,7 +1961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK45"/>
+  <dimension ref="A1:AK65"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -5405,7 +5779,7 @@
       <c r="M45" s="8"/>
       <c r="N45" s="7"/>
       <c r="O45" s="8"/>
-      <c r="P45" s="8"/>
+      <c r="P45" s="9"/>
       <c r="Q45" s="7" t="s">
         <v>370</v>
       </c>
@@ -5438,7 +5812,7 @@
       <c r="AB45" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC45" s="8" t="s">
+      <c r="AC45" s="9" t="s">
         <v>167</v>
       </c>
       <c r="AD45" s="7" t="s">
@@ -5453,6 +5827,1688 @@
         <v>60</v>
       </c>
       <c r="AK45" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="46" spans="1:37">
+      <c r="A46" s="3">
+        <v>44</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C46" s="3">
+        <v>2026061588</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F46" s="3">
+        <v>2209</v>
+      </c>
+      <c r="G46" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H46" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I46" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="J46" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="K46" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L46" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M46" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="N46" s="3">
+        <v>2307</v>
+      </c>
+      <c r="O46" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="P46" s="10" t="s">
+        <v>377</v>
+      </c>
+      <c r="Q46" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="R46" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S46" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T46" s="3">
+        <v>1</v>
+      </c>
+      <c r="U46" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V46" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="W46" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="X46" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="Y46" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="Z46" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="AA46" s="3"/>
+      <c r="AB46" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC46" s="10" t="s">
+        <v>382</v>
+      </c>
+      <c r="AD46" s="3"/>
+      <c r="AE46" s="3"/>
+      <c r="AF46" s="3"/>
+      <c r="AG46" s="3"/>
+      <c r="AH46" s="3"/>
+      <c r="AI46" s="3"/>
+      <c r="AJ46" s="3"/>
+      <c r="AK46" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="47" spans="1:37">
+      <c r="A47" s="7">
+        <v>45</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C47" s="7">
+        <v>2026061598</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="G47" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="H47" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I47" s="7" t="s">
+        <v>386</v>
+      </c>
+      <c r="J47" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="K47" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L47" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="M47" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="N47" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="O47" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="P47" s="9" t="s">
+        <v>387</v>
+      </c>
+      <c r="Q47" s="7" t="s">
+        <v>388</v>
+      </c>
+      <c r="R47" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S47" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="T47" s="7">
+        <v>1</v>
+      </c>
+      <c r="U47" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V47" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="W47" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="X47" s="7" t="s">
+        <v>391</v>
+      </c>
+      <c r="Y47" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="Z47" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="AA47" s="7"/>
+      <c r="AB47" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC47" s="9" t="s">
+        <v>393</v>
+      </c>
+      <c r="AD47" s="7"/>
+      <c r="AE47" s="7"/>
+      <c r="AF47" s="7"/>
+      <c r="AG47" s="7"/>
+      <c r="AH47" s="7"/>
+      <c r="AI47" s="7"/>
+      <c r="AJ47" s="7"/>
+      <c r="AK47" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="48" spans="1:37">
+      <c r="A48" s="3">
+        <v>46</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C48" s="3">
+        <v>2026061643</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="G48" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="I48" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="J48" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="K48" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L48" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="M48" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="N48" s="3">
+        <v>2405</v>
+      </c>
+      <c r="O48" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="P48" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="Q48" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="R48" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S48" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T48" s="3">
+        <v>1</v>
+      </c>
+      <c r="U48" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V48" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="W48" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="X48" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="Y48" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="Z48" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="AA48" s="3"/>
+      <c r="AB48" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC48" s="10" t="s">
+        <v>404</v>
+      </c>
+      <c r="AD48" s="3"/>
+      <c r="AE48" s="3"/>
+      <c r="AF48" s="3"/>
+      <c r="AG48" s="3"/>
+      <c r="AH48" s="3"/>
+      <c r="AI48" s="3"/>
+      <c r="AJ48" s="3"/>
+      <c r="AK48" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="49" spans="1:37">
+      <c r="A49" s="7">
+        <v>47</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C49" s="7">
+        <v>2026061674</v>
+      </c>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7">
+        <v>4503</v>
+      </c>
+      <c r="G49" s="7" t="s">
+        <v>405</v>
+      </c>
+      <c r="H49" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="I49" s="7"/>
+      <c r="J49" s="7"/>
+      <c r="K49" s="7"/>
+      <c r="L49" s="7"/>
+      <c r="M49" s="8"/>
+      <c r="N49" s="7"/>
+      <c r="O49" s="8"/>
+      <c r="P49" s="9"/>
+      <c r="Q49" s="7" t="s">
+        <v>406</v>
+      </c>
+      <c r="R49" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S49" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T49" s="7">
+        <v>1</v>
+      </c>
+      <c r="U49" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V49" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="W49" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="X49" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="Y49" s="7"/>
+      <c r="Z49" s="7">
+        <v>1</v>
+      </c>
+      <c r="AA49" s="7"/>
+      <c r="AB49" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC49" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD49" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE49" s="7"/>
+      <c r="AF49" s="7"/>
+      <c r="AG49" s="7"/>
+      <c r="AH49" s="7"/>
+      <c r="AI49" s="7"/>
+      <c r="AJ49" s="7"/>
+      <c r="AK49" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="50" spans="1:37">
+      <c r="A50" s="3">
+        <v>48</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C50" s="3">
+        <v>2026061675</v>
+      </c>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="H50" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I50" s="3"/>
+      <c r="J50" s="3"/>
+      <c r="K50" s="3"/>
+      <c r="L50" s="3"/>
+      <c r="M50" s="4"/>
+      <c r="N50" s="3"/>
+      <c r="O50" s="4"/>
+      <c r="P50" s="10"/>
+      <c r="Q50" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="R50" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S50" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T50" s="3">
+        <v>1</v>
+      </c>
+      <c r="U50" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V50" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="W50" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="X50" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="Y50" s="3"/>
+      <c r="Z50" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA50" s="3"/>
+      <c r="AB50" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC50" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="AD50" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE50" s="3"/>
+      <c r="AF50" s="3"/>
+      <c r="AG50" s="3"/>
+      <c r="AH50" s="3"/>
+      <c r="AI50" s="3"/>
+      <c r="AJ50" s="3"/>
+      <c r="AK50" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="51" spans="1:37">
+      <c r="A51" s="7">
+        <v>49</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C51" s="7">
+        <v>2026061677</v>
+      </c>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7">
+        <v>5031</v>
+      </c>
+      <c r="G51" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="H51" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="I51" s="7"/>
+      <c r="J51" s="7"/>
+      <c r="K51" s="7"/>
+      <c r="L51" s="7"/>
+      <c r="M51" s="8"/>
+      <c r="N51" s="7"/>
+      <c r="O51" s="8"/>
+      <c r="P51" s="9"/>
+      <c r="Q51" s="7" t="s">
+        <v>417</v>
+      </c>
+      <c r="R51" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S51" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T51" s="7">
+        <v>1</v>
+      </c>
+      <c r="U51" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V51" s="7" t="s">
+        <v>418</v>
+      </c>
+      <c r="W51" s="7" t="s">
+        <v>419</v>
+      </c>
+      <c r="X51" s="7" t="s">
+        <v>420</v>
+      </c>
+      <c r="Y51" s="7"/>
+      <c r="Z51" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA51" s="7"/>
+      <c r="AB51" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC51" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD51" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE51" s="7"/>
+      <c r="AF51" s="7"/>
+      <c r="AG51" s="7"/>
+      <c r="AH51" s="7"/>
+      <c r="AI51" s="7"/>
+      <c r="AJ51" s="7"/>
+      <c r="AK51" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="52" spans="1:37">
+      <c r="A52" s="3">
+        <v>50</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C52" s="3">
+        <v>2026061686</v>
+      </c>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3">
+        <v>3692</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="H52" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I52" s="3"/>
+      <c r="J52" s="3"/>
+      <c r="K52" s="3"/>
+      <c r="L52" s="3"/>
+      <c r="M52" s="4"/>
+      <c r="N52" s="3"/>
+      <c r="O52" s="4"/>
+      <c r="P52" s="10"/>
+      <c r="Q52" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="R52" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S52" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T52" s="3">
+        <v>1</v>
+      </c>
+      <c r="U52" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V52" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="W52" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="X52" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="Y52" s="3"/>
+      <c r="Z52" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA52" s="3"/>
+      <c r="AB52" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC52" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD52" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE52" s="3"/>
+      <c r="AF52" s="3"/>
+      <c r="AG52" s="3"/>
+      <c r="AH52" s="3"/>
+      <c r="AI52" s="3"/>
+      <c r="AJ52" s="3"/>
+      <c r="AK52" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="53" spans="1:37">
+      <c r="A53" s="7">
+        <v>51</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C53" s="7">
+        <v>2026061688</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>426</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F53" s="7">
+        <v>4422</v>
+      </c>
+      <c r="G53" s="7" t="s">
+        <v>427</v>
+      </c>
+      <c r="H53" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I53" s="7" t="s">
+        <v>428</v>
+      </c>
+      <c r="J53" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="K53" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L53" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="M53" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="N53" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="O53" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="P53" s="9" t="s">
+        <v>429</v>
+      </c>
+      <c r="Q53" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="R53" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S53" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="T53" s="7">
+        <v>1</v>
+      </c>
+      <c r="U53" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V53" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="W53" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="X53" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="Y53" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="Z53" s="7">
+        <v>1.1</v>
+      </c>
+      <c r="AA53" s="7"/>
+      <c r="AB53" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC53" s="9" t="s">
+        <v>435</v>
+      </c>
+      <c r="AD53" s="7"/>
+      <c r="AE53" s="7"/>
+      <c r="AF53" s="7"/>
+      <c r="AG53" s="7"/>
+      <c r="AH53" s="7"/>
+      <c r="AI53" s="7"/>
+      <c r="AJ53" s="7"/>
+      <c r="AK53" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="54" spans="1:37">
+      <c r="A54" s="3">
+        <v>52</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C54" s="3">
+        <v>2026061689</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F54" s="3">
+        <v>4422</v>
+      </c>
+      <c r="G54" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="H54" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I54" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="J54" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="K54" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L54" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="M54" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="N54" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="O54" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="P54" s="10" t="s">
+        <v>438</v>
+      </c>
+      <c r="Q54" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="R54" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S54" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="T54" s="3">
+        <v>1</v>
+      </c>
+      <c r="U54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V54" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="W54" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="X54" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="Y54" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="Z54" s="3">
+        <v>1.1</v>
+      </c>
+      <c r="AA54" s="3"/>
+      <c r="AB54" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC54" s="10" t="s">
+        <v>442</v>
+      </c>
+      <c r="AD54" s="3"/>
+      <c r="AE54" s="3"/>
+      <c r="AF54" s="3"/>
+      <c r="AG54" s="3"/>
+      <c r="AH54" s="3"/>
+      <c r="AI54" s="3"/>
+      <c r="AJ54" s="3"/>
+      <c r="AK54" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="55" spans="1:37">
+      <c r="A55" s="7">
+        <v>53</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C55" s="7">
+        <v>2026061749</v>
+      </c>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="7">
+        <v>2763</v>
+      </c>
+      <c r="G55" s="7" t="s">
+        <v>443</v>
+      </c>
+      <c r="H55" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="I55" s="7"/>
+      <c r="J55" s="7"/>
+      <c r="K55" s="7"/>
+      <c r="L55" s="7"/>
+      <c r="M55" s="8"/>
+      <c r="N55" s="7"/>
+      <c r="O55" s="8"/>
+      <c r="P55" s="9"/>
+      <c r="Q55" s="7" t="s">
+        <v>444</v>
+      </c>
+      <c r="R55" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S55" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T55" s="7">
+        <v>1</v>
+      </c>
+      <c r="U55" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V55" s="7" t="s">
+        <v>445</v>
+      </c>
+      <c r="W55" s="7" t="s">
+        <v>446</v>
+      </c>
+      <c r="X55" s="7" t="s">
+        <v>447</v>
+      </c>
+      <c r="Y55" s="7"/>
+      <c r="Z55" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA55" s="7"/>
+      <c r="AB55" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC55" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD55" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE55" s="7"/>
+      <c r="AF55" s="7"/>
+      <c r="AG55" s="7"/>
+      <c r="AH55" s="7"/>
+      <c r="AI55" s="7"/>
+      <c r="AJ55" s="7"/>
+      <c r="AK55" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="56" spans="1:37">
+      <c r="A56" s="3">
+        <v>54</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C56" s="3">
+        <v>2026061761</v>
+      </c>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="3">
+        <v>2401</v>
+      </c>
+      <c r="G56" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="I56" s="3"/>
+      <c r="J56" s="3"/>
+      <c r="K56" s="3"/>
+      <c r="L56" s="3"/>
+      <c r="M56" s="4"/>
+      <c r="N56" s="3"/>
+      <c r="O56" s="4"/>
+      <c r="P56" s="10"/>
+      <c r="Q56" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="R56" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S56" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T56" s="3">
+        <v>1</v>
+      </c>
+      <c r="U56" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V56" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="W56" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="X56" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="Y56" s="3"/>
+      <c r="Z56" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA56" s="3"/>
+      <c r="AB56" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC56" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD56" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE56" s="3"/>
+      <c r="AF56" s="3"/>
+      <c r="AG56" s="3"/>
+      <c r="AH56" s="3"/>
+      <c r="AI56" s="3"/>
+      <c r="AJ56" s="3"/>
+      <c r="AK56" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="57" spans="1:37">
+      <c r="A57" s="7">
+        <v>55</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C57" s="7">
+        <v>2026061769</v>
+      </c>
+      <c r="D57" s="7"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="7">
+        <v>2988</v>
+      </c>
+      <c r="G57" s="7" t="s">
+        <v>453</v>
+      </c>
+      <c r="H57" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I57" s="7"/>
+      <c r="J57" s="7"/>
+      <c r="K57" s="7"/>
+      <c r="L57" s="7"/>
+      <c r="M57" s="8"/>
+      <c r="N57" s="7"/>
+      <c r="O57" s="8"/>
+      <c r="P57" s="9"/>
+      <c r="Q57" s="7" t="s">
+        <v>454</v>
+      </c>
+      <c r="R57" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S57" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T57" s="7">
+        <v>1</v>
+      </c>
+      <c r="U57" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V57" s="7" t="s">
+        <v>455</v>
+      </c>
+      <c r="W57" s="7" t="s">
+        <v>456</v>
+      </c>
+      <c r="X57" s="7" t="s">
+        <v>457</v>
+      </c>
+      <c r="Y57" s="7"/>
+      <c r="Z57" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA57" s="7"/>
+      <c r="AB57" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC57" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="AD57" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE57" s="7"/>
+      <c r="AF57" s="7"/>
+      <c r="AG57" s="7"/>
+      <c r="AH57" s="7"/>
+      <c r="AI57" s="7"/>
+      <c r="AJ57" s="7"/>
+      <c r="AK57" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="58" spans="1:37">
+      <c r="A58" s="3">
+        <v>56</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C58" s="3">
+        <v>2026061770</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F58" s="3">
+        <v>3811</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I58" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="J58" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="K58" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L58" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="M58" s="4" t="s">
+        <v>462</v>
+      </c>
+      <c r="N58" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="O58" s="4" t="s">
+        <v>464</v>
+      </c>
+      <c r="P58" s="10" t="s">
+        <v>465</v>
+      </c>
+      <c r="Q58" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="R58" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S58" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T58" s="3">
+        <v>1</v>
+      </c>
+      <c r="U58" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V58" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="W58" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="X58" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Y58" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="Z58" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA58" s="3"/>
+      <c r="AB58" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC58" s="10" t="s">
+        <v>471</v>
+      </c>
+      <c r="AD58" s="3"/>
+      <c r="AE58" s="3"/>
+      <c r="AF58" s="3"/>
+      <c r="AG58" s="3"/>
+      <c r="AH58" s="3"/>
+      <c r="AI58" s="3"/>
+      <c r="AJ58" s="3"/>
+      <c r="AK58" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="59" spans="1:37">
+      <c r="A59" s="7">
+        <v>57</v>
+      </c>
+      <c r="B59" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C59" s="7">
+        <v>2026061773</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>472</v>
+      </c>
+      <c r="E59" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F59" s="7">
+        <v>3811</v>
+      </c>
+      <c r="G59" s="7" t="s">
+        <v>459</v>
+      </c>
+      <c r="H59" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I59" s="7" t="s">
+        <v>473</v>
+      </c>
+      <c r="J59" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="K59" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L59" s="7" t="s">
+        <v>461</v>
+      </c>
+      <c r="M59" s="8" t="s">
+        <v>462</v>
+      </c>
+      <c r="N59" s="7" t="s">
+        <v>463</v>
+      </c>
+      <c r="O59" s="8" t="s">
+        <v>464</v>
+      </c>
+      <c r="P59" s="9" t="s">
+        <v>474</v>
+      </c>
+      <c r="Q59" s="7" t="s">
+        <v>466</v>
+      </c>
+      <c r="R59" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S59" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T59" s="7">
+        <v>1</v>
+      </c>
+      <c r="U59" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V59" s="7" t="s">
+        <v>475</v>
+      </c>
+      <c r="W59" s="7" t="s">
+        <v>476</v>
+      </c>
+      <c r="X59" s="7" t="s">
+        <v>468</v>
+      </c>
+      <c r="Y59" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="Z59" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA59" s="7"/>
+      <c r="AB59" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC59" s="9" t="s">
+        <v>471</v>
+      </c>
+      <c r="AD59" s="7"/>
+      <c r="AE59" s="7"/>
+      <c r="AF59" s="7"/>
+      <c r="AG59" s="7"/>
+      <c r="AH59" s="7"/>
+      <c r="AI59" s="7"/>
+      <c r="AJ59" s="7"/>
+      <c r="AK59" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="60" spans="1:37">
+      <c r="A60" s="3">
+        <v>58</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C60" s="3">
+        <v>2026061829</v>
+      </c>
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
+      <c r="F60" s="3">
+        <v>5248</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="H60" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I60" s="3"/>
+      <c r="J60" s="3"/>
+      <c r="K60" s="3"/>
+      <c r="L60" s="3"/>
+      <c r="M60" s="4"/>
+      <c r="N60" s="3"/>
+      <c r="O60" s="4"/>
+      <c r="P60" s="10"/>
+      <c r="Q60" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="R60" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S60" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T60" s="3">
+        <v>1</v>
+      </c>
+      <c r="U60" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V60" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="W60" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="X60" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="Y60" s="3"/>
+      <c r="Z60" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA60" s="3"/>
+      <c r="AB60" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC60" s="10" t="s">
+        <v>483</v>
+      </c>
+      <c r="AD60" s="3"/>
+      <c r="AE60" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF60" s="3"/>
+      <c r="AG60" s="3"/>
+      <c r="AH60" s="3"/>
+      <c r="AI60" s="3"/>
+      <c r="AJ60" s="3"/>
+      <c r="AK60" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="61" spans="1:37">
+      <c r="A61" s="7">
+        <v>59</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C61" s="7">
+        <v>2026061830</v>
+      </c>
+      <c r="D61" s="7"/>
+      <c r="E61" s="7"/>
+      <c r="F61" s="7">
+        <v>5248</v>
+      </c>
+      <c r="G61" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="H61" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="I61" s="7"/>
+      <c r="J61" s="7"/>
+      <c r="K61" s="7"/>
+      <c r="L61" s="7"/>
+      <c r="M61" s="8"/>
+      <c r="N61" s="7"/>
+      <c r="O61" s="8"/>
+      <c r="P61" s="9"/>
+      <c r="Q61" s="7" t="s">
+        <v>479</v>
+      </c>
+      <c r="R61" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S61" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T61" s="7">
+        <v>1</v>
+      </c>
+      <c r="U61" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V61" s="7" t="s">
+        <v>484</v>
+      </c>
+      <c r="W61" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="X61" s="7" t="s">
+        <v>481</v>
+      </c>
+      <c r="Y61" s="7"/>
+      <c r="Z61" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA61" s="7"/>
+      <c r="AB61" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC61" s="9" t="s">
+        <v>485</v>
+      </c>
+      <c r="AD61" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE61" s="7"/>
+      <c r="AF61" s="7"/>
+      <c r="AG61" s="7"/>
+      <c r="AH61" s="7"/>
+      <c r="AI61" s="7"/>
+      <c r="AJ61" s="7"/>
+      <c r="AK61" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:37">
+      <c r="A62" s="3">
+        <v>60</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C62" s="3">
+        <v>2026061831</v>
+      </c>
+      <c r="D62" s="3"/>
+      <c r="E62" s="3"/>
+      <c r="F62" s="3">
+        <v>5248</v>
+      </c>
+      <c r="G62" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="H62" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I62" s="3"/>
+      <c r="J62" s="3"/>
+      <c r="K62" s="3"/>
+      <c r="L62" s="3"/>
+      <c r="M62" s="4"/>
+      <c r="N62" s="3"/>
+      <c r="O62" s="4"/>
+      <c r="P62" s="10"/>
+      <c r="Q62" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="R62" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S62" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T62" s="3">
+        <v>1</v>
+      </c>
+      <c r="U62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V62" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="W62" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="X62" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="Y62" s="3"/>
+      <c r="Z62" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA62" s="3"/>
+      <c r="AB62" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC62" s="10" t="s">
+        <v>487</v>
+      </c>
+      <c r="AD62" s="3"/>
+      <c r="AE62" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF62" s="3"/>
+      <c r="AG62" s="3"/>
+      <c r="AH62" s="3"/>
+      <c r="AI62" s="3"/>
+      <c r="AJ62" s="3"/>
+      <c r="AK62" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="63" spans="1:37">
+      <c r="A63" s="7">
+        <v>61</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C63" s="7">
+        <v>2026061839</v>
+      </c>
+      <c r="D63" s="7"/>
+      <c r="E63" s="7"/>
+      <c r="F63" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="G63" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="H63" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I63" s="7"/>
+      <c r="J63" s="7"/>
+      <c r="K63" s="7"/>
+      <c r="L63" s="7"/>
+      <c r="M63" s="8"/>
+      <c r="N63" s="7"/>
+      <c r="O63" s="8"/>
+      <c r="P63" s="9"/>
+      <c r="Q63" s="7" t="s">
+        <v>388</v>
+      </c>
+      <c r="R63" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S63" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="T63" s="7">
+        <v>1</v>
+      </c>
+      <c r="U63" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V63" s="7" t="s">
+        <v>488</v>
+      </c>
+      <c r="W63" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="X63" s="7" t="s">
+        <v>391</v>
+      </c>
+      <c r="Y63" s="7"/>
+      <c r="Z63" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="AA63" s="7"/>
+      <c r="AB63" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC63" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD63" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE63" s="7"/>
+      <c r="AF63" s="7"/>
+      <c r="AG63" s="7"/>
+      <c r="AH63" s="7"/>
+      <c r="AI63" s="7"/>
+      <c r="AJ63" s="7"/>
+      <c r="AK63" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="64" spans="1:37">
+      <c r="A64" s="3">
+        <v>62</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C64" s="3">
+        <v>2026061850</v>
+      </c>
+      <c r="D64" s="3"/>
+      <c r="E64" s="3"/>
+      <c r="F64" s="3">
+        <v>4422</v>
+      </c>
+      <c r="G64" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="H64" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I64" s="3"/>
+      <c r="J64" s="3"/>
+      <c r="K64" s="3"/>
+      <c r="L64" s="3"/>
+      <c r="M64" s="4"/>
+      <c r="N64" s="3"/>
+      <c r="O64" s="4"/>
+      <c r="P64" s="10"/>
+      <c r="Q64" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="R64" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S64" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="T64" s="3">
+        <v>1</v>
+      </c>
+      <c r="U64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V64" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="W64" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="X64" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="Y64" s="3"/>
+      <c r="Z64" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA64" s="3"/>
+      <c r="AB64" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC64" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD64" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE64" s="3"/>
+      <c r="AF64" s="3"/>
+      <c r="AG64" s="3"/>
+      <c r="AH64" s="3"/>
+      <c r="AI64" s="3"/>
+      <c r="AJ64" s="3"/>
+      <c r="AK64" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="65" spans="1:37">
+      <c r="A65" s="7">
+        <v>63</v>
+      </c>
+      <c r="B65" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C65" s="7">
+        <v>2026061879</v>
+      </c>
+      <c r="D65" s="7"/>
+      <c r="E65" s="7"/>
+      <c r="F65" s="7">
+        <v>4748</v>
+      </c>
+      <c r="G65" s="7" t="s">
+        <v>491</v>
+      </c>
+      <c r="H65" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="I65" s="7"/>
+      <c r="J65" s="7"/>
+      <c r="K65" s="7"/>
+      <c r="L65" s="7"/>
+      <c r="M65" s="8"/>
+      <c r="N65" s="7"/>
+      <c r="O65" s="8"/>
+      <c r="P65" s="8"/>
+      <c r="Q65" s="7" t="s">
+        <v>492</v>
+      </c>
+      <c r="R65" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S65" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T65" s="7">
+        <v>1</v>
+      </c>
+      <c r="U65" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V65" s="7" t="s">
+        <v>493</v>
+      </c>
+      <c r="W65" s="7" t="s">
+        <v>494</v>
+      </c>
+      <c r="X65" s="7" t="s">
+        <v>495</v>
+      </c>
+      <c r="Y65" s="7"/>
+      <c r="Z65" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA65" s="7"/>
+      <c r="AB65" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC65" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="AD65" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE65" s="7"/>
+      <c r="AF65" s="7"/>
+      <c r="AG65" s="7"/>
+      <c r="AH65" s="7"/>
+      <c r="AI65" s="7"/>
+      <c r="AJ65" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK65" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06121710
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$65</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$80</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="496">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-11  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="585">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-12  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -1238,6 +1238,42 @@
 換下：8119008154</t>
   </si>
   <si>
+    <t>1D350115061001</t>
+  </si>
+  <si>
+    <t>D350</t>
+  </si>
+  <si>
+    <t>三重徐匯站</t>
+  </si>
+  <si>
+    <t>2026-06-10 10:28:20</t>
+  </si>
+  <si>
+    <t>SC升級SQL2019更新失敗，發現更新檔案損壞，SC型號：SHUTTLE7S 請到店更換SC第一顆硬碟，資料不備份、不還原。(到店時需先進線騰雲確認銷售資料是否已傳回萊爾富總公司)</t>
+  </si>
+  <si>
+    <t>THILF0D350</t>
+  </si>
+  <si>
+    <t>2026-06-10 10:29:54</t>
+  </si>
+  <si>
+    <t>2026-06-12 11:35:00</t>
+  </si>
+  <si>
+    <t>2026-06-12 13:32:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 14:29:00</t>
+  </si>
+  <si>
+    <t>23小時3分鐘</t>
+  </si>
+  <si>
+    <t>更換第一顆硬碟不備份還原.等已跟店家告知回報代收會計</t>
+  </si>
+  <si>
     <t>1C216115061001</t>
   </si>
   <si>
@@ -1250,9 +1286,6 @@
     <t>2026-06-10 10:27:59</t>
   </si>
   <si>
-    <t>SC升級SQL2019更新失敗，發現更新檔案損壞，SC型號：SHUTTLE7S 請到店更換SC第一顆硬碟，資料不備份、不還原。(到店時需先進線騰雲確認銷售資料是否已傳回萊爾富總公司)</t>
-  </si>
-  <si>
     <t>THILF0C216</t>
   </si>
   <si>
@@ -1269,6 +1302,37 @@
   </si>
   <si>
     <t>更換第一顆硬碟不備份還原. 已跟店家告知回報代收會計</t>
+  </si>
+  <si>
+    <t>14341115061001</t>
+  </si>
+  <si>
+    <t>新莊莊美店</t>
+  </si>
+  <si>
+    <t>2026-06-10 10:33:52</t>
+  </si>
+  <si>
+    <t>THILF04341</t>
+  </si>
+  <si>
+    <t>2026-06-10 10:36:20</t>
+  </si>
+  <si>
+    <t>2026-06-12 13:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-12 15:15:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 14:36:00</t>
+  </si>
+  <si>
+    <t>24小時39分鐘</t>
+  </si>
+  <si>
+    <t>更換第一顆硬碟不備份還原
+並告知黃小姐更換硬碟注意事項</t>
   </si>
   <si>
     <t>龜山復恆店</t>
@@ -1548,6 +1612,210 @@
   </si>
   <si>
     <t>2026-06-11 15:50:00</t>
+  </si>
+  <si>
+    <t>D022</t>
+  </si>
+  <si>
+    <t>三重溪尾店</t>
+  </si>
+  <si>
+    <t>THILF0D022</t>
+  </si>
+  <si>
+    <t>2026-06-12 10:15:45</t>
+  </si>
+  <si>
+    <t>2026-06-12 09:45:00</t>
+  </si>
+  <si>
+    <t>2026-06-12 10:07:00</t>
+  </si>
+  <si>
+    <t>D057</t>
+  </si>
+  <si>
+    <t>北縣溪尾二店</t>
+  </si>
+  <si>
+    <t>THILF0D057</t>
+  </si>
+  <si>
+    <t>2026-06-12 10:42:19</t>
+  </si>
+  <si>
+    <t>2026-06-12 10:18:00</t>
+  </si>
+  <si>
+    <t>2026-06-12 10:40:00</t>
+  </si>
+  <si>
+    <t>蘆洲鴻悅店</t>
+  </si>
+  <si>
+    <t>新北市蘆洲區</t>
+  </si>
+  <si>
+    <t>THILF05197</t>
+  </si>
+  <si>
+    <t>2026-06-12 10:45:39</t>
+  </si>
+  <si>
+    <t>2026-06-12 10:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-12 10:50:00</t>
+  </si>
+  <si>
+    <t>北縣蘆旺店</t>
+  </si>
+  <si>
+    <t>THILF02958</t>
+  </si>
+  <si>
+    <t>2026-06-12 11:02:17</t>
+  </si>
+  <si>
+    <t>2026-06-12 11:10:00</t>
+  </si>
+  <si>
+    <t>三重仁美店</t>
+  </si>
+  <si>
+    <t>THILF04098</t>
+  </si>
+  <si>
+    <t>2026-06-12 11:09:42</t>
+  </si>
+  <si>
+    <t>2026-06-12 10:49:00</t>
+  </si>
+  <si>
+    <t>板橋互助店</t>
+  </si>
+  <si>
+    <t>THILF03853</t>
+  </si>
+  <si>
+    <t>2026-06-12 11:31:14</t>
+  </si>
+  <si>
+    <t>2026-06-12 10:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-12 11:00:00</t>
+  </si>
+  <si>
+    <t>板橋民生站</t>
+  </si>
+  <si>
+    <t>THILF05384</t>
+  </si>
+  <si>
+    <t>2026-06-12 13:04:55</t>
+  </si>
+  <si>
+    <t>2026-06-12 12:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-12 13:00:00</t>
+  </si>
+  <si>
+    <t>三重福仁店</t>
+  </si>
+  <si>
+    <t>THILF03957</t>
+  </si>
+  <si>
+    <t>2026-06-12 14:54:49</t>
+  </si>
+  <si>
+    <t>2026-06-12 14:10:00</t>
+  </si>
+  <si>
+    <t>2026-06-12 14:35:00</t>
+  </si>
+  <si>
+    <t>板橋民治店</t>
+  </si>
+  <si>
+    <t>THILF03965</t>
+  </si>
+  <si>
+    <t>2026-06-12 15:08:22</t>
+  </si>
+  <si>
+    <t>2026-06-12 14:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-12 15:00:00</t>
+  </si>
+  <si>
+    <t>D195</t>
+  </si>
+  <si>
+    <t>三重車路頭</t>
+  </si>
+  <si>
+    <t>THILF0D195</t>
+  </si>
+  <si>
+    <t>2026-06-12 15:29:26</t>
+  </si>
+  <si>
+    <t>2026-06-12 14:50:00</t>
+  </si>
+  <si>
+    <t>2026-06-12 15:18:00</t>
+  </si>
+  <si>
+    <t>板橋板莊店</t>
+  </si>
+  <si>
+    <t>THILF02154</t>
+  </si>
+  <si>
+    <t>2026-06-12 15:36:57</t>
+  </si>
+  <si>
+    <t>2026-06-12 15:10:00</t>
+  </si>
+  <si>
+    <t>2026-06-12 15:30:00</t>
+  </si>
+  <si>
+    <t>三重護山店</t>
+  </si>
+  <si>
+    <t>THILF05245</t>
+  </si>
+  <si>
+    <t>2026-06-12 16:06:52</t>
+  </si>
+  <si>
+    <t>2026-06-12 15:35:00</t>
+  </si>
+  <si>
+    <t>2026-06-12 16:00:00</t>
+  </si>
+  <si>
+    <t>D072</t>
+  </si>
+  <si>
+    <t>板橋僑福店</t>
+  </si>
+  <si>
+    <t>THILF0D072</t>
+  </si>
+  <si>
+    <t>2026-06-12 16:45:17</t>
+  </si>
+  <si>
+    <t>2026-06-12 04:10:00</t>
+  </si>
+  <si>
+    <t>2026-06-12 16:40:00</t>
   </si>
 </sst>
 </file>
@@ -1961,7 +2229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK65"/>
+  <dimension ref="A1:AK80"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -6032,7 +6300,7 @@
         <v>38</v>
       </c>
       <c r="C48" s="3">
-        <v>2026061643</v>
+        <v>2026061633</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>394</v>
@@ -6047,7 +6315,7 @@
         <v>396</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>209</v>
+        <v>42</v>
       </c>
       <c r="I48" s="3" t="s">
         <v>397</v>
@@ -6101,14 +6369,16 @@
         <v>403</v>
       </c>
       <c r="Z48" s="3">
-        <v>2.5</v>
-      </c>
-      <c r="AA48" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="AA48" s="3" t="s">
+        <v>404</v>
+      </c>
       <c r="AB48" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC48" s="10" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="AD48" s="3"/>
       <c r="AE48" s="3"/>
@@ -6126,38 +6396,58 @@
         <v>47</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C49" s="7">
-        <v>2026061674</v>
-      </c>
-      <c r="D49" s="7"/>
-      <c r="E49" s="7"/>
-      <c r="F49" s="7">
-        <v>4503</v>
+        <v>2026061643</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>406</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>407</v>
       </c>
       <c r="G49" s="7" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="I49" s="7"/>
-      <c r="J49" s="7"/>
-      <c r="K49" s="7"/>
-      <c r="L49" s="7"/>
-      <c r="M49" s="8"/>
-      <c r="N49" s="7"/>
-      <c r="O49" s="8"/>
-      <c r="P49" s="9"/>
+        <v>209</v>
+      </c>
+      <c r="I49" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="J49" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="K49" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L49" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="M49" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="N49" s="7">
+        <v>2405</v>
+      </c>
+      <c r="O49" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="P49" s="9" t="s">
+        <v>398</v>
+      </c>
       <c r="Q49" s="7" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="R49" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S49" s="7" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="T49" s="7">
         <v>1</v>
@@ -6166,28 +6456,28 @@
         <v>53</v>
       </c>
       <c r="V49" s="7" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="W49" s="7" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="X49" s="7" t="s">
-        <v>380</v>
-      </c>
-      <c r="Y49" s="7"/>
+        <v>413</v>
+      </c>
+      <c r="Y49" s="7" t="s">
+        <v>414</v>
+      </c>
       <c r="Z49" s="7">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="AA49" s="7"/>
       <c r="AB49" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC49" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD49" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>415</v>
+      </c>
+      <c r="AD49" s="7"/>
       <c r="AE49" s="7"/>
       <c r="AF49" s="7"/>
       <c r="AG49" s="7"/>
@@ -6203,38 +6493,58 @@
         <v>48</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C50" s="3">
-        <v>2026061675</v>
-      </c>
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
-      <c r="F50" s="3" t="s">
-        <v>409</v>
+        <v>2026061647</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F50" s="3">
+        <v>4341</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="I50" s="3"/>
-      <c r="J50" s="3"/>
-      <c r="K50" s="3"/>
-      <c r="L50" s="3"/>
-      <c r="M50" s="4"/>
-      <c r="N50" s="3"/>
-      <c r="O50" s="4"/>
-      <c r="P50" s="10"/>
+        <v>170</v>
+      </c>
+      <c r="I50" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="J50" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="K50" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L50" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="M50" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="N50" s="3">
+        <v>2405</v>
+      </c>
+      <c r="O50" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="P50" s="10" t="s">
+        <v>398</v>
+      </c>
       <c r="Q50" s="3" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="R50" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S50" s="3" t="s">
-        <v>79</v>
+        <v>178</v>
       </c>
       <c r="T50" s="3">
         <v>1</v>
@@ -6243,28 +6553,30 @@
         <v>53</v>
       </c>
       <c r="V50" s="3" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="W50" s="3" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
       <c r="X50" s="3" t="s">
-        <v>414</v>
-      </c>
-      <c r="Y50" s="3"/>
+        <v>422</v>
+      </c>
+      <c r="Y50" s="3" t="s">
+        <v>423</v>
+      </c>
       <c r="Z50" s="3">
-        <v>0.3</v>
-      </c>
-      <c r="AA50" s="3"/>
+        <v>1.8</v>
+      </c>
+      <c r="AA50" s="3" t="s">
+        <v>424</v>
+      </c>
       <c r="AB50" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC50" s="10" t="s">
-        <v>415</v>
-      </c>
-      <c r="AD50" s="3" t="s">
-        <v>60</v>
-      </c>
+        <v>425</v>
+      </c>
+      <c r="AD50" s="3"/>
       <c r="AE50" s="3"/>
       <c r="AF50" s="3"/>
       <c r="AG50" s="3"/>
@@ -6283,15 +6595,15 @@
         <v>100</v>
       </c>
       <c r="C51" s="7">
-        <v>2026061677</v>
+        <v>2026061674</v>
       </c>
       <c r="D51" s="7"/>
       <c r="E51" s="7"/>
       <c r="F51" s="7">
-        <v>5031</v>
+        <v>4503</v>
       </c>
       <c r="G51" s="7" t="s">
-        <v>416</v>
+        <v>426</v>
       </c>
       <c r="H51" s="7" t="s">
         <v>75</v>
@@ -6305,7 +6617,7 @@
       <c r="O51" s="8"/>
       <c r="P51" s="9"/>
       <c r="Q51" s="7" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
       <c r="R51" s="7" t="s">
         <v>51</v>
@@ -6320,17 +6632,17 @@
         <v>53</v>
       </c>
       <c r="V51" s="7" t="s">
-        <v>418</v>
+        <v>428</v>
       </c>
       <c r="W51" s="7" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="X51" s="7" t="s">
-        <v>420</v>
+        <v>380</v>
       </c>
       <c r="Y51" s="7"/>
       <c r="Z51" s="7">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="AA51" s="7"/>
       <c r="AB51" s="7" t="s">
@@ -6360,15 +6672,15 @@
         <v>100</v>
       </c>
       <c r="C52" s="3">
-        <v>2026061686</v>
+        <v>2026061675</v>
       </c>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
-      <c r="F52" s="3">
-        <v>3692</v>
+      <c r="F52" s="3" t="s">
+        <v>430</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>421</v>
+        <v>431</v>
       </c>
       <c r="H52" s="3" t="s">
         <v>75</v>
@@ -6382,7 +6694,7 @@
       <c r="O52" s="4"/>
       <c r="P52" s="10"/>
       <c r="Q52" s="3" t="s">
-        <v>422</v>
+        <v>432</v>
       </c>
       <c r="R52" s="3" t="s">
         <v>51</v>
@@ -6397,24 +6709,24 @@
         <v>53</v>
       </c>
       <c r="V52" s="3" t="s">
-        <v>423</v>
+        <v>433</v>
       </c>
       <c r="W52" s="3" t="s">
-        <v>424</v>
+        <v>434</v>
       </c>
       <c r="X52" s="3" t="s">
-        <v>425</v>
+        <v>435</v>
       </c>
       <c r="Y52" s="3"/>
       <c r="Z52" s="3">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="AA52" s="3"/>
       <c r="AB52" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC52" s="10" t="s">
-        <v>111</v>
+        <v>436</v>
       </c>
       <c r="AD52" s="3" t="s">
         <v>60</v>
@@ -6434,58 +6746,38 @@
         <v>51</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C53" s="7">
-        <v>2026061688</v>
-      </c>
-      <c r="D53" s="7" t="s">
-        <v>426</v>
-      </c>
-      <c r="E53" s="7" t="s">
-        <v>40</v>
-      </c>
+        <v>2026061677</v>
+      </c>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
       <c r="F53" s="7">
-        <v>4422</v>
+        <v>5031</v>
       </c>
       <c r="G53" s="7" t="s">
-        <v>427</v>
+        <v>437</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="I53" s="7" t="s">
-        <v>428</v>
-      </c>
-      <c r="J53" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="K53" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="L53" s="7" t="s">
-        <v>326</v>
-      </c>
-      <c r="M53" s="8" t="s">
-        <v>327</v>
-      </c>
-      <c r="N53" s="7" t="s">
-        <v>328</v>
-      </c>
-      <c r="O53" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="P53" s="9" t="s">
-        <v>429</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="I53" s="7"/>
+      <c r="J53" s="7"/>
+      <c r="K53" s="7"/>
+      <c r="L53" s="7"/>
+      <c r="M53" s="8"/>
+      <c r="N53" s="7"/>
+      <c r="O53" s="8"/>
+      <c r="P53" s="9"/>
       <c r="Q53" s="7" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="R53" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S53" s="7" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="T53" s="7">
         <v>1</v>
@@ -6494,28 +6786,28 @@
         <v>53</v>
       </c>
       <c r="V53" s="7" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="W53" s="7" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
       <c r="X53" s="7" t="s">
-        <v>433</v>
-      </c>
-      <c r="Y53" s="7" t="s">
-        <v>434</v>
-      </c>
+        <v>441</v>
+      </c>
+      <c r="Y53" s="7"/>
       <c r="Z53" s="7">
-        <v>1.1</v>
+        <v>0.3</v>
       </c>
       <c r="AA53" s="7"/>
       <c r="AB53" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC53" s="9" t="s">
-        <v>435</v>
-      </c>
-      <c r="AD53" s="7"/>
+        <v>111</v>
+      </c>
+      <c r="AD53" s="7" t="s">
+        <v>60</v>
+      </c>
       <c r="AE53" s="7"/>
       <c r="AF53" s="7"/>
       <c r="AG53" s="7"/>
@@ -6531,58 +6823,38 @@
         <v>52</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C54" s="3">
-        <v>2026061689</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>436</v>
-      </c>
-      <c r="E54" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>2026061686</v>
+      </c>
+      <c r="D54" s="3"/>
+      <c r="E54" s="3"/>
       <c r="F54" s="3">
-        <v>4422</v>
+        <v>3692</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>427</v>
+        <v>442</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="I54" s="3" t="s">
-        <v>437</v>
-      </c>
-      <c r="J54" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="K54" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="L54" s="3" t="s">
-        <v>326</v>
-      </c>
-      <c r="M54" s="4" t="s">
-        <v>327</v>
-      </c>
-      <c r="N54" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="O54" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="P54" s="10" t="s">
-        <v>438</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="I54" s="3"/>
+      <c r="J54" s="3"/>
+      <c r="K54" s="3"/>
+      <c r="L54" s="3"/>
+      <c r="M54" s="4"/>
+      <c r="N54" s="3"/>
+      <c r="O54" s="4"/>
+      <c r="P54" s="10"/>
       <c r="Q54" s="3" t="s">
-        <v>430</v>
+        <v>443</v>
       </c>
       <c r="R54" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S54" s="3" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="T54" s="3">
         <v>1</v>
@@ -6591,28 +6863,28 @@
         <v>53</v>
       </c>
       <c r="V54" s="3" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
       <c r="W54" s="3" t="s">
-        <v>432</v>
+        <v>445</v>
       </c>
       <c r="X54" s="3" t="s">
-        <v>440</v>
-      </c>
-      <c r="Y54" s="3" t="s">
-        <v>441</v>
-      </c>
+        <v>446</v>
+      </c>
+      <c r="Y54" s="3"/>
       <c r="Z54" s="3">
-        <v>1.1</v>
+        <v>0.5</v>
       </c>
       <c r="AA54" s="3"/>
       <c r="AB54" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC54" s="10" t="s">
-        <v>442</v>
-      </c>
-      <c r="AD54" s="3"/>
+        <v>111</v>
+      </c>
+      <c r="AD54" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="AE54" s="3"/>
       <c r="AF54" s="3"/>
       <c r="AG54" s="3"/>
@@ -6628,38 +6900,58 @@
         <v>53</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C55" s="7">
-        <v>2026061749</v>
-      </c>
-      <c r="D55" s="7"/>
-      <c r="E55" s="7"/>
+        <v>2026061688</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>447</v>
+      </c>
+      <c r="E55" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F55" s="7">
-        <v>2763</v>
+        <v>4422</v>
       </c>
       <c r="G55" s="7" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="I55" s="7"/>
-      <c r="J55" s="7"/>
-      <c r="K55" s="7"/>
-      <c r="L55" s="7"/>
-      <c r="M55" s="8"/>
-      <c r="N55" s="7"/>
-      <c r="O55" s="8"/>
-      <c r="P55" s="9"/>
+        <v>86</v>
+      </c>
+      <c r="I55" s="7" t="s">
+        <v>449</v>
+      </c>
+      <c r="J55" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="K55" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L55" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="M55" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="N55" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="O55" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="P55" s="9" t="s">
+        <v>450</v>
+      </c>
       <c r="Q55" s="7" t="s">
-        <v>444</v>
+        <v>451</v>
       </c>
       <c r="R55" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S55" s="7" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="T55" s="7">
         <v>1</v>
@@ -6668,28 +6960,28 @@
         <v>53</v>
       </c>
       <c r="V55" s="7" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
       <c r="W55" s="7" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="X55" s="7" t="s">
-        <v>447</v>
-      </c>
-      <c r="Y55" s="7"/>
+        <v>454</v>
+      </c>
+      <c r="Y55" s="7" t="s">
+        <v>455</v>
+      </c>
       <c r="Z55" s="7">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
       <c r="AA55" s="7"/>
       <c r="AB55" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC55" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD55" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>456</v>
+      </c>
+      <c r="AD55" s="7"/>
       <c r="AE55" s="7"/>
       <c r="AF55" s="7"/>
       <c r="AG55" s="7"/>
@@ -6705,38 +6997,58 @@
         <v>54</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C56" s="3">
-        <v>2026061761</v>
-      </c>
-      <c r="D56" s="3"/>
-      <c r="E56" s="3"/>
+        <v>2026061689</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="F56" s="3">
-        <v>2401</v>
+        <v>4422</v>
       </c>
       <c r="G56" s="3" t="s">
         <v>448</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="I56" s="3"/>
-      <c r="J56" s="3"/>
-      <c r="K56" s="3"/>
-      <c r="L56" s="3"/>
-      <c r="M56" s="4"/>
-      <c r="N56" s="3"/>
-      <c r="O56" s="4"/>
-      <c r="P56" s="10"/>
+        <v>86</v>
+      </c>
+      <c r="I56" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="J56" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="K56" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L56" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="M56" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="N56" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="O56" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="P56" s="10" t="s">
+        <v>459</v>
+      </c>
       <c r="Q56" s="3" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="R56" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S56" s="3" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="T56" s="3">
         <v>1</v>
@@ -6745,28 +7057,28 @@
         <v>53</v>
       </c>
       <c r="V56" s="3" t="s">
-        <v>450</v>
+        <v>460</v>
       </c>
       <c r="W56" s="3" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="X56" s="3" t="s">
-        <v>452</v>
-      </c>
-      <c r="Y56" s="3"/>
+        <v>461</v>
+      </c>
+      <c r="Y56" s="3" t="s">
+        <v>462</v>
+      </c>
       <c r="Z56" s="3">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
       <c r="AA56" s="3"/>
       <c r="AB56" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC56" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD56" s="3" t="s">
-        <v>60</v>
-      </c>
+        <v>463</v>
+      </c>
+      <c r="AD56" s="3"/>
       <c r="AE56" s="3"/>
       <c r="AF56" s="3"/>
       <c r="AG56" s="3"/>
@@ -6785,18 +7097,18 @@
         <v>100</v>
       </c>
       <c r="C57" s="7">
-        <v>2026061769</v>
+        <v>2026061749</v>
       </c>
       <c r="D57" s="7"/>
       <c r="E57" s="7"/>
       <c r="F57" s="7">
-        <v>2988</v>
+        <v>2763</v>
       </c>
       <c r="G57" s="7" t="s">
-        <v>453</v>
+        <v>464</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>128</v>
+        <v>75</v>
       </c>
       <c r="I57" s="7"/>
       <c r="J57" s="7"/>
@@ -6807,7 +7119,7 @@
       <c r="O57" s="8"/>
       <c r="P57" s="9"/>
       <c r="Q57" s="7" t="s">
-        <v>454</v>
+        <v>465</v>
       </c>
       <c r="R57" s="7" t="s">
         <v>51</v>
@@ -6822,24 +7134,24 @@
         <v>53</v>
       </c>
       <c r="V57" s="7" t="s">
-        <v>455</v>
+        <v>466</v>
       </c>
       <c r="W57" s="7" t="s">
-        <v>456</v>
+        <v>467</v>
       </c>
       <c r="X57" s="7" t="s">
-        <v>457</v>
+        <v>468</v>
       </c>
       <c r="Y57" s="7"/>
       <c r="Z57" s="7">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="AA57" s="7"/>
       <c r="AB57" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC57" s="9" t="s">
-        <v>157</v>
+        <v>111</v>
       </c>
       <c r="AD57" s="7" t="s">
         <v>60</v>
@@ -6859,58 +7171,38 @@
         <v>56</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C58" s="3">
-        <v>2026061770</v>
-      </c>
-      <c r="D58" s="3" t="s">
-        <v>458</v>
-      </c>
-      <c r="E58" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>2026061761</v>
+      </c>
+      <c r="D58" s="3"/>
+      <c r="E58" s="3"/>
       <c r="F58" s="3">
-        <v>3811</v>
+        <v>2401</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>459</v>
+        <v>469</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I58" s="3" t="s">
-        <v>460</v>
-      </c>
-      <c r="J58" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="K58" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="L58" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="M58" s="4" t="s">
-        <v>462</v>
-      </c>
-      <c r="N58" s="3" t="s">
-        <v>463</v>
-      </c>
-      <c r="O58" s="4" t="s">
-        <v>464</v>
-      </c>
-      <c r="P58" s="10" t="s">
-        <v>465</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="I58" s="3"/>
+      <c r="J58" s="3"/>
+      <c r="K58" s="3"/>
+      <c r="L58" s="3"/>
+      <c r="M58" s="4"/>
+      <c r="N58" s="3"/>
+      <c r="O58" s="4"/>
+      <c r="P58" s="10"/>
       <c r="Q58" s="3" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="R58" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S58" s="3" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="T58" s="3">
         <v>1</v>
@@ -6919,28 +7211,28 @@
         <v>53</v>
       </c>
       <c r="V58" s="3" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="W58" s="3" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="X58" s="3" t="s">
-        <v>469</v>
-      </c>
-      <c r="Y58" s="3" t="s">
-        <v>470</v>
-      </c>
+        <v>473</v>
+      </c>
+      <c r="Y58" s="3"/>
       <c r="Z58" s="3">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="AA58" s="3"/>
       <c r="AB58" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC58" s="10" t="s">
-        <v>471</v>
-      </c>
-      <c r="AD58" s="3"/>
+        <v>111</v>
+      </c>
+      <c r="AD58" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="AE58" s="3"/>
       <c r="AF58" s="3"/>
       <c r="AG58" s="3"/>
@@ -6956,58 +7248,38 @@
         <v>57</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C59" s="7">
-        <v>2026061773</v>
-      </c>
-      <c r="D59" s="7" t="s">
-        <v>472</v>
-      </c>
-      <c r="E59" s="7" t="s">
-        <v>40</v>
-      </c>
+        <v>2026061769</v>
+      </c>
+      <c r="D59" s="7"/>
+      <c r="E59" s="7"/>
       <c r="F59" s="7">
-        <v>3811</v>
+        <v>2988</v>
       </c>
       <c r="G59" s="7" t="s">
-        <v>459</v>
+        <v>474</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="I59" s="7" t="s">
-        <v>473</v>
-      </c>
-      <c r="J59" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="K59" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="L59" s="7" t="s">
-        <v>461</v>
-      </c>
-      <c r="M59" s="8" t="s">
-        <v>462</v>
-      </c>
-      <c r="N59" s="7" t="s">
-        <v>463</v>
-      </c>
-      <c r="O59" s="8" t="s">
-        <v>464</v>
-      </c>
-      <c r="P59" s="9" t="s">
-        <v>474</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="I59" s="7"/>
+      <c r="J59" s="7"/>
+      <c r="K59" s="7"/>
+      <c r="L59" s="7"/>
+      <c r="M59" s="8"/>
+      <c r="N59" s="7"/>
+      <c r="O59" s="8"/>
+      <c r="P59" s="9"/>
       <c r="Q59" s="7" t="s">
-        <v>466</v>
+        <v>475</v>
       </c>
       <c r="R59" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S59" s="7" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="T59" s="7">
         <v>1</v>
@@ -7016,28 +7288,28 @@
         <v>53</v>
       </c>
       <c r="V59" s="7" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="W59" s="7" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="X59" s="7" t="s">
-        <v>468</v>
-      </c>
-      <c r="Y59" s="7" t="s">
-        <v>477</v>
-      </c>
+        <v>478</v>
+      </c>
+      <c r="Y59" s="7"/>
       <c r="Z59" s="7">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="AA59" s="7"/>
       <c r="AB59" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC59" s="9" t="s">
-        <v>471</v>
-      </c>
-      <c r="AD59" s="7"/>
+        <v>157</v>
+      </c>
+      <c r="AD59" s="7" t="s">
+        <v>60</v>
+      </c>
       <c r="AE59" s="7"/>
       <c r="AF59" s="7"/>
       <c r="AG59" s="7"/>
@@ -7053,38 +7325,58 @@
         <v>58</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C60" s="3">
-        <v>2026061829</v>
-      </c>
-      <c r="D60" s="3"/>
-      <c r="E60" s="3"/>
+        <v>2026061770</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="F60" s="3">
-        <v>5248</v>
+        <v>3811</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="I60" s="3"/>
-      <c r="J60" s="3"/>
-      <c r="K60" s="3"/>
-      <c r="L60" s="3"/>
-      <c r="M60" s="4"/>
-      <c r="N60" s="3"/>
-      <c r="O60" s="4"/>
-      <c r="P60" s="10"/>
+        <v>42</v>
+      </c>
+      <c r="I60" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="J60" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="K60" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L60" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="M60" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="N60" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="O60" s="4" t="s">
+        <v>485</v>
+      </c>
+      <c r="P60" s="10" t="s">
+        <v>486</v>
+      </c>
       <c r="Q60" s="3" t="s">
-        <v>479</v>
+        <v>487</v>
       </c>
       <c r="R60" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S60" s="3" t="s">
-        <v>178</v>
+        <v>52</v>
       </c>
       <c r="T60" s="3">
         <v>1</v>
@@ -7093,29 +7385,29 @@
         <v>53</v>
       </c>
       <c r="V60" s="3" t="s">
-        <v>480</v>
+        <v>488</v>
       </c>
       <c r="W60" s="3" t="s">
-        <v>481</v>
+        <v>489</v>
       </c>
       <c r="X60" s="3" t="s">
-        <v>482</v>
-      </c>
-      <c r="Y60" s="3"/>
+        <v>490</v>
+      </c>
+      <c r="Y60" s="3" t="s">
+        <v>491</v>
+      </c>
       <c r="Z60" s="3">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="AA60" s="3"/>
       <c r="AB60" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC60" s="10" t="s">
-        <v>483</v>
+        <v>492</v>
       </c>
       <c r="AD60" s="3"/>
-      <c r="AE60" s="3" t="s">
-        <v>60</v>
-      </c>
+      <c r="AE60" s="3"/>
       <c r="AF60" s="3"/>
       <c r="AG60" s="3"/>
       <c r="AH60" s="3"/>
@@ -7130,38 +7422,58 @@
         <v>59</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C61" s="7">
-        <v>2026061830</v>
-      </c>
-      <c r="D61" s="7"/>
-      <c r="E61" s="7"/>
+        <v>2026061773</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>493</v>
+      </c>
+      <c r="E61" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F61" s="7">
-        <v>5248</v>
+        <v>3811</v>
       </c>
       <c r="G61" s="7" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="I61" s="7"/>
-      <c r="J61" s="7"/>
-      <c r="K61" s="7"/>
-      <c r="L61" s="7"/>
-      <c r="M61" s="8"/>
-      <c r="N61" s="7"/>
-      <c r="O61" s="8"/>
-      <c r="P61" s="9"/>
+        <v>42</v>
+      </c>
+      <c r="I61" s="7" t="s">
+        <v>494</v>
+      </c>
+      <c r="J61" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="K61" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L61" s="7" t="s">
+        <v>482</v>
+      </c>
+      <c r="M61" s="8" t="s">
+        <v>483</v>
+      </c>
+      <c r="N61" s="7" t="s">
+        <v>484</v>
+      </c>
+      <c r="O61" s="8" t="s">
+        <v>485</v>
+      </c>
+      <c r="P61" s="9" t="s">
+        <v>495</v>
+      </c>
       <c r="Q61" s="7" t="s">
-        <v>479</v>
+        <v>487</v>
       </c>
       <c r="R61" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S61" s="7" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="T61" s="7">
         <v>1</v>
@@ -7170,28 +7482,28 @@
         <v>53</v>
       </c>
       <c r="V61" s="7" t="s">
-        <v>484</v>
+        <v>496</v>
       </c>
       <c r="W61" s="7" t="s">
-        <v>401</v>
+        <v>497</v>
       </c>
       <c r="X61" s="7" t="s">
-        <v>481</v>
-      </c>
-      <c r="Y61" s="7"/>
+        <v>489</v>
+      </c>
+      <c r="Y61" s="7" t="s">
+        <v>498</v>
+      </c>
       <c r="Z61" s="7">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="AA61" s="7"/>
       <c r="AB61" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC61" s="9" t="s">
-        <v>485</v>
-      </c>
-      <c r="AD61" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>492</v>
+      </c>
+      <c r="AD61" s="7"/>
       <c r="AE61" s="7"/>
       <c r="AF61" s="7"/>
       <c r="AG61" s="7"/>
@@ -7210,7 +7522,7 @@
         <v>100</v>
       </c>
       <c r="C62" s="3">
-        <v>2026061831</v>
+        <v>2026061829</v>
       </c>
       <c r="D62" s="3"/>
       <c r="E62" s="3"/>
@@ -7218,7 +7530,7 @@
         <v>5248</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>478</v>
+        <v>499</v>
       </c>
       <c r="H62" s="3" t="s">
         <v>75</v>
@@ -7232,13 +7544,13 @@
       <c r="O62" s="4"/>
       <c r="P62" s="10"/>
       <c r="Q62" s="3" t="s">
-        <v>479</v>
+        <v>500</v>
       </c>
       <c r="R62" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S62" s="3" t="s">
-        <v>79</v>
+        <v>178</v>
       </c>
       <c r="T62" s="3">
         <v>1</v>
@@ -7247,13 +7559,13 @@
         <v>53</v>
       </c>
       <c r="V62" s="3" t="s">
-        <v>486</v>
+        <v>501</v>
       </c>
       <c r="W62" s="3" t="s">
-        <v>481</v>
+        <v>502</v>
       </c>
       <c r="X62" s="3" t="s">
-        <v>482</v>
+        <v>503</v>
       </c>
       <c r="Y62" s="3"/>
       <c r="Z62" s="3">
@@ -7264,7 +7576,7 @@
         <v>58</v>
       </c>
       <c r="AC62" s="10" t="s">
-        <v>487</v>
+        <v>504</v>
       </c>
       <c r="AD62" s="3"/>
       <c r="AE62" s="3" t="s">
@@ -7287,18 +7599,18 @@
         <v>100</v>
       </c>
       <c r="C63" s="7">
-        <v>2026061839</v>
+        <v>2026061830</v>
       </c>
       <c r="D63" s="7"/>
       <c r="E63" s="7"/>
-      <c r="F63" s="7" t="s">
-        <v>384</v>
+      <c r="F63" s="7">
+        <v>5248</v>
       </c>
       <c r="G63" s="7" t="s">
-        <v>385</v>
+        <v>499</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="I63" s="7"/>
       <c r="J63" s="7"/>
@@ -7309,13 +7621,13 @@
       <c r="O63" s="8"/>
       <c r="P63" s="9"/>
       <c r="Q63" s="7" t="s">
-        <v>388</v>
+        <v>500</v>
       </c>
       <c r="R63" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S63" s="7" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="T63" s="7">
         <v>1</v>
@@ -7324,24 +7636,24 @@
         <v>53</v>
       </c>
       <c r="V63" s="7" t="s">
-        <v>488</v>
+        <v>505</v>
       </c>
       <c r="W63" s="7" t="s">
-        <v>390</v>
+        <v>412</v>
       </c>
       <c r="X63" s="7" t="s">
-        <v>391</v>
+        <v>502</v>
       </c>
       <c r="Y63" s="7"/>
       <c r="Z63" s="7">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="AA63" s="7"/>
       <c r="AB63" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC63" s="9" t="s">
-        <v>111</v>
+        <v>506</v>
       </c>
       <c r="AD63" s="7" t="s">
         <v>60</v>
@@ -7364,18 +7676,18 @@
         <v>100</v>
       </c>
       <c r="C64" s="3">
-        <v>2026061850</v>
+        <v>2026061831</v>
       </c>
       <c r="D64" s="3"/>
       <c r="E64" s="3"/>
       <c r="F64" s="3">
-        <v>4422</v>
+        <v>5248</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>427</v>
+        <v>499</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="I64" s="3"/>
       <c r="J64" s="3"/>
@@ -7386,13 +7698,13 @@
       <c r="O64" s="4"/>
       <c r="P64" s="10"/>
       <c r="Q64" s="3" t="s">
-        <v>430</v>
+        <v>500</v>
       </c>
       <c r="R64" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S64" s="3" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="T64" s="3">
         <v>1</v>
@@ -7401,29 +7713,29 @@
         <v>53</v>
       </c>
       <c r="V64" s="3" t="s">
-        <v>489</v>
+        <v>507</v>
       </c>
       <c r="W64" s="3" t="s">
-        <v>432</v>
+        <v>502</v>
       </c>
       <c r="X64" s="3" t="s">
-        <v>490</v>
+        <v>503</v>
       </c>
       <c r="Y64" s="3"/>
       <c r="Z64" s="3">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="AA64" s="3"/>
       <c r="AB64" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC64" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD64" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AE64" s="3"/>
+        <v>508</v>
+      </c>
+      <c r="AD64" s="3"/>
+      <c r="AE64" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="AF64" s="3"/>
       <c r="AG64" s="3"/>
       <c r="AH64" s="3"/>
@@ -7441,18 +7753,18 @@
         <v>100</v>
       </c>
       <c r="C65" s="7">
-        <v>2026061879</v>
+        <v>2026061839</v>
       </c>
       <c r="D65" s="7"/>
       <c r="E65" s="7"/>
-      <c r="F65" s="7">
-        <v>4748</v>
+      <c r="F65" s="7" t="s">
+        <v>384</v>
       </c>
       <c r="G65" s="7" t="s">
-        <v>491</v>
+        <v>385</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>209</v>
+        <v>86</v>
       </c>
       <c r="I65" s="7"/>
       <c r="J65" s="7"/>
@@ -7461,15 +7773,15 @@
       <c r="M65" s="8"/>
       <c r="N65" s="7"/>
       <c r="O65" s="8"/>
-      <c r="P65" s="8"/>
+      <c r="P65" s="9"/>
       <c r="Q65" s="7" t="s">
-        <v>492</v>
+        <v>388</v>
       </c>
       <c r="R65" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S65" s="7" t="s">
-        <v>52</v>
+        <v>94</v>
       </c>
       <c r="T65" s="7">
         <v>1</v>
@@ -7478,24 +7790,24 @@
         <v>53</v>
       </c>
       <c r="V65" s="7" t="s">
-        <v>493</v>
+        <v>509</v>
       </c>
       <c r="W65" s="7" t="s">
-        <v>494</v>
+        <v>390</v>
       </c>
       <c r="X65" s="7" t="s">
-        <v>495</v>
+        <v>391</v>
       </c>
       <c r="Y65" s="7"/>
       <c r="Z65" s="7">
-        <v>2</v>
+        <v>0.2</v>
       </c>
       <c r="AA65" s="7"/>
       <c r="AB65" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC65" s="8" t="s">
-        <v>167</v>
+      <c r="AC65" s="9" t="s">
+        <v>111</v>
       </c>
       <c r="AD65" s="7" t="s">
         <v>60</v>
@@ -7505,10 +7817,1181 @@
       <c r="AG65" s="7"/>
       <c r="AH65" s="7"/>
       <c r="AI65" s="7"/>
-      <c r="AJ65" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ65" s="7"/>
       <c r="AK65" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="66" spans="1:37">
+      <c r="A66" s="3">
+        <v>64</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C66" s="3">
+        <v>2026061850</v>
+      </c>
+      <c r="D66" s="3"/>
+      <c r="E66" s="3"/>
+      <c r="F66" s="3">
+        <v>4422</v>
+      </c>
+      <c r="G66" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="H66" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I66" s="3"/>
+      <c r="J66" s="3"/>
+      <c r="K66" s="3"/>
+      <c r="L66" s="3"/>
+      <c r="M66" s="4"/>
+      <c r="N66" s="3"/>
+      <c r="O66" s="4"/>
+      <c r="P66" s="10"/>
+      <c r="Q66" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="R66" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S66" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="T66" s="3">
+        <v>1</v>
+      </c>
+      <c r="U66" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V66" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="W66" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="X66" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="Y66" s="3"/>
+      <c r="Z66" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA66" s="3"/>
+      <c r="AB66" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC66" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD66" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE66" s="3"/>
+      <c r="AF66" s="3"/>
+      <c r="AG66" s="3"/>
+      <c r="AH66" s="3"/>
+      <c r="AI66" s="3"/>
+      <c r="AJ66" s="3"/>
+      <c r="AK66" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="67" spans="1:37">
+      <c r="A67" s="7">
+        <v>65</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C67" s="7">
+        <v>2026061879</v>
+      </c>
+      <c r="D67" s="7"/>
+      <c r="E67" s="7"/>
+      <c r="F67" s="7">
+        <v>4748</v>
+      </c>
+      <c r="G67" s="7" t="s">
+        <v>512</v>
+      </c>
+      <c r="H67" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="I67" s="7"/>
+      <c r="J67" s="7"/>
+      <c r="K67" s="7"/>
+      <c r="L67" s="7"/>
+      <c r="M67" s="8"/>
+      <c r="N67" s="7"/>
+      <c r="O67" s="8"/>
+      <c r="P67" s="9"/>
+      <c r="Q67" s="7" t="s">
+        <v>513</v>
+      </c>
+      <c r="R67" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S67" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T67" s="7">
+        <v>1</v>
+      </c>
+      <c r="U67" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V67" s="7" t="s">
+        <v>514</v>
+      </c>
+      <c r="W67" s="7" t="s">
+        <v>515</v>
+      </c>
+      <c r="X67" s="7" t="s">
+        <v>516</v>
+      </c>
+      <c r="Y67" s="7"/>
+      <c r="Z67" s="7">
+        <v>2</v>
+      </c>
+      <c r="AA67" s="7"/>
+      <c r="AB67" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC67" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="AD67" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE67" s="7"/>
+      <c r="AF67" s="7"/>
+      <c r="AG67" s="7"/>
+      <c r="AH67" s="7"/>
+      <c r="AI67" s="7"/>
+      <c r="AJ67" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK67" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="68" spans="1:37">
+      <c r="A68" s="3">
+        <v>66</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C68" s="3">
+        <v>2026061916</v>
+      </c>
+      <c r="D68" s="3"/>
+      <c r="E68" s="3"/>
+      <c r="F68" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="G68" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="H68" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I68" s="3"/>
+      <c r="J68" s="3"/>
+      <c r="K68" s="3"/>
+      <c r="L68" s="3"/>
+      <c r="M68" s="4"/>
+      <c r="N68" s="3"/>
+      <c r="O68" s="4"/>
+      <c r="P68" s="10"/>
+      <c r="Q68" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="R68" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S68" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T68" s="3">
+        <v>1</v>
+      </c>
+      <c r="U68" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V68" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="W68" s="3" t="s">
+        <v>521</v>
+      </c>
+      <c r="X68" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="Y68" s="3"/>
+      <c r="Z68" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA68" s="3"/>
+      <c r="AB68" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC68" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD68" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE68" s="3"/>
+      <c r="AF68" s="3"/>
+      <c r="AG68" s="3"/>
+      <c r="AH68" s="3"/>
+      <c r="AI68" s="3"/>
+      <c r="AJ68" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK68" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="69" spans="1:37">
+      <c r="A69" s="7">
+        <v>67</v>
+      </c>
+      <c r="B69" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C69" s="7">
+        <v>2026061920</v>
+      </c>
+      <c r="D69" s="7"/>
+      <c r="E69" s="7"/>
+      <c r="F69" s="7" t="s">
+        <v>523</v>
+      </c>
+      <c r="G69" s="7" t="s">
+        <v>524</v>
+      </c>
+      <c r="H69" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I69" s="7"/>
+      <c r="J69" s="7"/>
+      <c r="K69" s="7"/>
+      <c r="L69" s="7"/>
+      <c r="M69" s="8"/>
+      <c r="N69" s="7"/>
+      <c r="O69" s="8"/>
+      <c r="P69" s="9"/>
+      <c r="Q69" s="7" t="s">
+        <v>525</v>
+      </c>
+      <c r="R69" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S69" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T69" s="7">
+        <v>1</v>
+      </c>
+      <c r="U69" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V69" s="7" t="s">
+        <v>526</v>
+      </c>
+      <c r="W69" s="7" t="s">
+        <v>527</v>
+      </c>
+      <c r="X69" s="7" t="s">
+        <v>528</v>
+      </c>
+      <c r="Y69" s="7"/>
+      <c r="Z69" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA69" s="7"/>
+      <c r="AB69" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC69" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD69" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE69" s="7"/>
+      <c r="AF69" s="7"/>
+      <c r="AG69" s="7"/>
+      <c r="AH69" s="7"/>
+      <c r="AI69" s="7"/>
+      <c r="AJ69" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK69" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="70" spans="1:37">
+      <c r="A70" s="3">
+        <v>68</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C70" s="3">
+        <v>2026061921</v>
+      </c>
+      <c r="D70" s="3"/>
+      <c r="E70" s="3"/>
+      <c r="F70" s="3">
+        <v>5197</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="H70" s="3" t="s">
+        <v>530</v>
+      </c>
+      <c r="I70" s="3"/>
+      <c r="J70" s="3"/>
+      <c r="K70" s="3"/>
+      <c r="L70" s="3"/>
+      <c r="M70" s="4"/>
+      <c r="N70" s="3"/>
+      <c r="O70" s="4"/>
+      <c r="P70" s="10"/>
+      <c r="Q70" s="3" t="s">
+        <v>531</v>
+      </c>
+      <c r="R70" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S70" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T70" s="3">
+        <v>1</v>
+      </c>
+      <c r="U70" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V70" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="W70" s="3" t="s">
+        <v>533</v>
+      </c>
+      <c r="X70" s="3" t="s">
+        <v>534</v>
+      </c>
+      <c r="Y70" s="3"/>
+      <c r="Z70" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA70" s="3"/>
+      <c r="AB70" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC70" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD70" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE70" s="3"/>
+      <c r="AF70" s="3"/>
+      <c r="AG70" s="3"/>
+      <c r="AH70" s="3"/>
+      <c r="AI70" s="3"/>
+      <c r="AJ70" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK70" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="71" spans="1:37">
+      <c r="A71" s="7">
+        <v>69</v>
+      </c>
+      <c r="B71" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C71" s="7">
+        <v>2026061926</v>
+      </c>
+      <c r="D71" s="7"/>
+      <c r="E71" s="7"/>
+      <c r="F71" s="7">
+        <v>2958</v>
+      </c>
+      <c r="G71" s="7" t="s">
+        <v>535</v>
+      </c>
+      <c r="H71" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="I71" s="7"/>
+      <c r="J71" s="7"/>
+      <c r="K71" s="7"/>
+      <c r="L71" s="7"/>
+      <c r="M71" s="8"/>
+      <c r="N71" s="7"/>
+      <c r="O71" s="8"/>
+      <c r="P71" s="9"/>
+      <c r="Q71" s="7" t="s">
+        <v>536</v>
+      </c>
+      <c r="R71" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S71" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T71" s="7">
+        <v>1</v>
+      </c>
+      <c r="U71" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V71" s="7" t="s">
+        <v>537</v>
+      </c>
+      <c r="W71" s="7" t="s">
+        <v>534</v>
+      </c>
+      <c r="X71" s="7" t="s">
+        <v>538</v>
+      </c>
+      <c r="Y71" s="7"/>
+      <c r="Z71" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA71" s="7"/>
+      <c r="AB71" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC71" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD71" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE71" s="7"/>
+      <c r="AF71" s="7"/>
+      <c r="AG71" s="7"/>
+      <c r="AH71" s="7"/>
+      <c r="AI71" s="7"/>
+      <c r="AJ71" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK71" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="72" spans="1:37">
+      <c r="A72" s="3">
+        <v>70</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C72" s="3">
+        <v>2026061928</v>
+      </c>
+      <c r="D72" s="3"/>
+      <c r="E72" s="3"/>
+      <c r="F72" s="3">
+        <v>4098</v>
+      </c>
+      <c r="G72" s="3" t="s">
+        <v>539</v>
+      </c>
+      <c r="H72" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I72" s="3"/>
+      <c r="J72" s="3"/>
+      <c r="K72" s="3"/>
+      <c r="L72" s="3"/>
+      <c r="M72" s="4"/>
+      <c r="N72" s="3"/>
+      <c r="O72" s="4"/>
+      <c r="P72" s="10"/>
+      <c r="Q72" s="3" t="s">
+        <v>540</v>
+      </c>
+      <c r="R72" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S72" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T72" s="3">
+        <v>1</v>
+      </c>
+      <c r="U72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V72" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="W72" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="X72" s="3" t="s">
+        <v>538</v>
+      </c>
+      <c r="Y72" s="3"/>
+      <c r="Z72" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA72" s="3"/>
+      <c r="AB72" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC72" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD72" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE72" s="3"/>
+      <c r="AF72" s="3"/>
+      <c r="AG72" s="3"/>
+      <c r="AH72" s="3"/>
+      <c r="AI72" s="3"/>
+      <c r="AJ72" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK72" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="73" spans="1:37">
+      <c r="A73" s="7">
+        <v>71</v>
+      </c>
+      <c r="B73" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C73" s="7">
+        <v>2026061931</v>
+      </c>
+      <c r="D73" s="7"/>
+      <c r="E73" s="7"/>
+      <c r="F73" s="7">
+        <v>3853</v>
+      </c>
+      <c r="G73" s="7" t="s">
+        <v>543</v>
+      </c>
+      <c r="H73" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I73" s="7"/>
+      <c r="J73" s="7"/>
+      <c r="K73" s="7"/>
+      <c r="L73" s="7"/>
+      <c r="M73" s="8"/>
+      <c r="N73" s="7"/>
+      <c r="O73" s="8"/>
+      <c r="P73" s="9"/>
+      <c r="Q73" s="7" t="s">
+        <v>544</v>
+      </c>
+      <c r="R73" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S73" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T73" s="7">
+        <v>1</v>
+      </c>
+      <c r="U73" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V73" s="7" t="s">
+        <v>545</v>
+      </c>
+      <c r="W73" s="7" t="s">
+        <v>546</v>
+      </c>
+      <c r="X73" s="7" t="s">
+        <v>547</v>
+      </c>
+      <c r="Y73" s="7"/>
+      <c r="Z73" s="7">
+        <v>1</v>
+      </c>
+      <c r="AA73" s="7"/>
+      <c r="AB73" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC73" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="AD73" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE73" s="7"/>
+      <c r="AF73" s="7"/>
+      <c r="AG73" s="7"/>
+      <c r="AH73" s="7"/>
+      <c r="AI73" s="7"/>
+      <c r="AJ73" s="7"/>
+      <c r="AK73" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="74" spans="1:37">
+      <c r="A74" s="3">
+        <v>72</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C74" s="3">
+        <v>2026061963</v>
+      </c>
+      <c r="D74" s="3"/>
+      <c r="E74" s="3"/>
+      <c r="F74" s="3">
+        <v>5384</v>
+      </c>
+      <c r="G74" s="3" t="s">
+        <v>548</v>
+      </c>
+      <c r="H74" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I74" s="3"/>
+      <c r="J74" s="3"/>
+      <c r="K74" s="3"/>
+      <c r="L74" s="3"/>
+      <c r="M74" s="4"/>
+      <c r="N74" s="3"/>
+      <c r="O74" s="4"/>
+      <c r="P74" s="10"/>
+      <c r="Q74" s="3" t="s">
+        <v>549</v>
+      </c>
+      <c r="R74" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S74" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T74" s="3">
+        <v>1</v>
+      </c>
+      <c r="U74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V74" s="3" t="s">
+        <v>550</v>
+      </c>
+      <c r="W74" s="3" t="s">
+        <v>551</v>
+      </c>
+      <c r="X74" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="Y74" s="3"/>
+      <c r="Z74" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA74" s="3"/>
+      <c r="AB74" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC74" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="AD74" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE74" s="3"/>
+      <c r="AF74" s="3"/>
+      <c r="AG74" s="3"/>
+      <c r="AH74" s="3"/>
+      <c r="AI74" s="3"/>
+      <c r="AJ74" s="3"/>
+      <c r="AK74" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="75" spans="1:37">
+      <c r="A75" s="7">
+        <v>73</v>
+      </c>
+      <c r="B75" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C75" s="7">
+        <v>2026061971</v>
+      </c>
+      <c r="D75" s="7"/>
+      <c r="E75" s="7"/>
+      <c r="F75" s="7">
+        <v>3957</v>
+      </c>
+      <c r="G75" s="7" t="s">
+        <v>553</v>
+      </c>
+      <c r="H75" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I75" s="7"/>
+      <c r="J75" s="7"/>
+      <c r="K75" s="7"/>
+      <c r="L75" s="7"/>
+      <c r="M75" s="8"/>
+      <c r="N75" s="7"/>
+      <c r="O75" s="8"/>
+      <c r="P75" s="9"/>
+      <c r="Q75" s="7" t="s">
+        <v>554</v>
+      </c>
+      <c r="R75" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S75" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T75" s="7">
+        <v>1</v>
+      </c>
+      <c r="U75" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V75" s="7" t="s">
+        <v>555</v>
+      </c>
+      <c r="W75" s="7" t="s">
+        <v>556</v>
+      </c>
+      <c r="X75" s="7" t="s">
+        <v>557</v>
+      </c>
+      <c r="Y75" s="7"/>
+      <c r="Z75" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA75" s="7"/>
+      <c r="AB75" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC75" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD75" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE75" s="7"/>
+      <c r="AF75" s="7"/>
+      <c r="AG75" s="7"/>
+      <c r="AH75" s="7"/>
+      <c r="AI75" s="7"/>
+      <c r="AJ75" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK75" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="76" spans="1:37">
+      <c r="A76" s="3">
+        <v>74</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C76" s="3">
+        <v>2026061977</v>
+      </c>
+      <c r="D76" s="3"/>
+      <c r="E76" s="3"/>
+      <c r="F76" s="3">
+        <v>3965</v>
+      </c>
+      <c r="G76" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="H76" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I76" s="3"/>
+      <c r="J76" s="3"/>
+      <c r="K76" s="3"/>
+      <c r="L76" s="3"/>
+      <c r="M76" s="4"/>
+      <c r="N76" s="3"/>
+      <c r="O76" s="4"/>
+      <c r="P76" s="10"/>
+      <c r="Q76" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="R76" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S76" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T76" s="3">
+        <v>1</v>
+      </c>
+      <c r="U76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V76" s="3" t="s">
+        <v>560</v>
+      </c>
+      <c r="W76" s="3" t="s">
+        <v>561</v>
+      </c>
+      <c r="X76" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="Y76" s="3"/>
+      <c r="Z76" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA76" s="3"/>
+      <c r="AB76" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC76" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD76" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE76" s="3"/>
+      <c r="AF76" s="3"/>
+      <c r="AG76" s="3"/>
+      <c r="AH76" s="3"/>
+      <c r="AI76" s="3"/>
+      <c r="AJ76" s="3"/>
+      <c r="AK76" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="77" spans="1:37">
+      <c r="A77" s="7">
+        <v>75</v>
+      </c>
+      <c r="B77" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C77" s="7">
+        <v>2026061983</v>
+      </c>
+      <c r="D77" s="7"/>
+      <c r="E77" s="7"/>
+      <c r="F77" s="7" t="s">
+        <v>563</v>
+      </c>
+      <c r="G77" s="7" t="s">
+        <v>564</v>
+      </c>
+      <c r="H77" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I77" s="7"/>
+      <c r="J77" s="7"/>
+      <c r="K77" s="7"/>
+      <c r="L77" s="7"/>
+      <c r="M77" s="8"/>
+      <c r="N77" s="7"/>
+      <c r="O77" s="8"/>
+      <c r="P77" s="9"/>
+      <c r="Q77" s="7" t="s">
+        <v>565</v>
+      </c>
+      <c r="R77" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S77" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T77" s="7">
+        <v>1</v>
+      </c>
+      <c r="U77" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V77" s="7" t="s">
+        <v>566</v>
+      </c>
+      <c r="W77" s="7" t="s">
+        <v>567</v>
+      </c>
+      <c r="X77" s="7" t="s">
+        <v>568</v>
+      </c>
+      <c r="Y77" s="7"/>
+      <c r="Z77" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA77" s="7"/>
+      <c r="AB77" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC77" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD77" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE77" s="7"/>
+      <c r="AF77" s="7"/>
+      <c r="AG77" s="7"/>
+      <c r="AH77" s="7"/>
+      <c r="AI77" s="7"/>
+      <c r="AJ77" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK77" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="78" spans="1:37">
+      <c r="A78" s="3">
+        <v>76</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C78" s="3">
+        <v>2026061986</v>
+      </c>
+      <c r="D78" s="3"/>
+      <c r="E78" s="3"/>
+      <c r="F78" s="3">
+        <v>2154</v>
+      </c>
+      <c r="G78" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="H78" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I78" s="3"/>
+      <c r="J78" s="3"/>
+      <c r="K78" s="3"/>
+      <c r="L78" s="3"/>
+      <c r="M78" s="4"/>
+      <c r="N78" s="3"/>
+      <c r="O78" s="4"/>
+      <c r="P78" s="10"/>
+      <c r="Q78" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="R78" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S78" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T78" s="3">
+        <v>1</v>
+      </c>
+      <c r="U78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V78" s="3" t="s">
+        <v>571</v>
+      </c>
+      <c r="W78" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="X78" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="Y78" s="3"/>
+      <c r="Z78" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA78" s="3"/>
+      <c r="AB78" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC78" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD78" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE78" s="3"/>
+      <c r="AF78" s="3"/>
+      <c r="AG78" s="3"/>
+      <c r="AH78" s="3"/>
+      <c r="AI78" s="3"/>
+      <c r="AJ78" s="3"/>
+      <c r="AK78" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="79" spans="1:37">
+      <c r="A79" s="7">
+        <v>77</v>
+      </c>
+      <c r="B79" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C79" s="7">
+        <v>2026062001</v>
+      </c>
+      <c r="D79" s="7"/>
+      <c r="E79" s="7"/>
+      <c r="F79" s="7">
+        <v>5245</v>
+      </c>
+      <c r="G79" s="7" t="s">
+        <v>574</v>
+      </c>
+      <c r="H79" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I79" s="7"/>
+      <c r="J79" s="7"/>
+      <c r="K79" s="7"/>
+      <c r="L79" s="7"/>
+      <c r="M79" s="8"/>
+      <c r="N79" s="7"/>
+      <c r="O79" s="8"/>
+      <c r="P79" s="9"/>
+      <c r="Q79" s="7" t="s">
+        <v>575</v>
+      </c>
+      <c r="R79" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S79" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T79" s="7">
+        <v>1</v>
+      </c>
+      <c r="U79" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V79" s="7" t="s">
+        <v>576</v>
+      </c>
+      <c r="W79" s="7" t="s">
+        <v>577</v>
+      </c>
+      <c r="X79" s="7" t="s">
+        <v>578</v>
+      </c>
+      <c r="Y79" s="7"/>
+      <c r="Z79" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA79" s="7"/>
+      <c r="AB79" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC79" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD79" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE79" s="7"/>
+      <c r="AF79" s="7"/>
+      <c r="AG79" s="7"/>
+      <c r="AH79" s="7"/>
+      <c r="AI79" s="7"/>
+      <c r="AJ79" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK79" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="80" spans="1:37">
+      <c r="A80" s="3">
+        <v>78</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C80" s="3">
+        <v>2026062007</v>
+      </c>
+      <c r="D80" s="3"/>
+      <c r="E80" s="3"/>
+      <c r="F80" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="G80" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="H80" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I80" s="3"/>
+      <c r="J80" s="3"/>
+      <c r="K80" s="3"/>
+      <c r="L80" s="3"/>
+      <c r="M80" s="4"/>
+      <c r="N80" s="3"/>
+      <c r="O80" s="4"/>
+      <c r="P80" s="4"/>
+      <c r="Q80" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="R80" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S80" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T80" s="3">
+        <v>1</v>
+      </c>
+      <c r="U80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V80" s="3" t="s">
+        <v>582</v>
+      </c>
+      <c r="W80" s="3" t="s">
+        <v>583</v>
+      </c>
+      <c r="X80" s="3" t="s">
+        <v>584</v>
+      </c>
+      <c r="Y80" s="3"/>
+      <c r="Z80" s="3">
+        <v>12.5</v>
+      </c>
+      <c r="AA80" s="3"/>
+      <c r="AB80" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC80" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD80" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE80" s="3"/>
+      <c r="AF80" s="3"/>
+      <c r="AG80" s="3"/>
+      <c r="AH80" s="3"/>
+      <c r="AI80" s="3"/>
+      <c r="AJ80" s="3"/>
+      <c r="AK80" s="3" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06151802
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$80</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$95</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="585">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-12  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="667">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-15  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -1274,6 +1274,36 @@
     <t>更換第一顆硬碟不備份還原.等已跟店家告知回報代收會計</t>
   </si>
   <si>
+    <t>12482115061001</t>
+  </si>
+  <si>
+    <t>蘆竹光明店</t>
+  </si>
+  <si>
+    <t>2026-06-10 10:14:20</t>
+  </si>
+  <si>
+    <t>THILF02482</t>
+  </si>
+  <si>
+    <t>2026-06-10 10:32:24</t>
+  </si>
+  <si>
+    <t>2026-06-15 10:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-15 12:21:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 14:32:00</t>
+  </si>
+  <si>
+    <t>93小時49分鐘</t>
+  </si>
+  <si>
+    <t>更換第一顆硬碟不備份還原完成</t>
+  </si>
+  <si>
     <t>1C216115061001</t>
   </si>
   <si>
@@ -1298,10 +1328,44 @@
     <t>2026-06-11 12:27:00</t>
   </si>
   <si>
-    <t>2026-06-11 14:32:00</t>
-  </si>
-  <si>
     <t>更換第一顆硬碟不備份還原. 已跟店家告知回報代收會計</t>
+  </si>
+  <si>
+    <t>15341115061001</t>
+  </si>
+  <si>
+    <t>蘆洲切仔麵</t>
+  </si>
+  <si>
+    <t>新北市蘆洲區</t>
+  </si>
+  <si>
+    <t>2026-06-10 09:57:56</t>
+  </si>
+  <si>
+    <t>SC升級SQL2019更新失敗，發現更新檔案損壞，SC型號：SHUTTLE6S 請到店更換SC第一顆硬碟，資料不備份、不還原。(到店時需先進線騰雲確認銷售資料是否已傳回萊爾富總公司)</t>
+  </si>
+  <si>
+    <t>THILF05341</t>
+  </si>
+  <si>
+    <t>2026-06-10 10:33:05</t>
+  </si>
+  <si>
+    <t>2026-06-15 13:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-15 15:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-11 14:33:00</t>
+  </si>
+  <si>
+    <t>96小時27分鐘</t>
+  </si>
+  <si>
+    <t>更換第一顆硬碟不備份還原
+並告知曾小姐更換硬碟注意事項</t>
   </si>
   <si>
     <t>14341115061001</t>
@@ -1653,9 +1717,6 @@
     <t>蘆洲鴻悅店</t>
   </si>
   <si>
-    <t>新北市蘆洲區</t>
-  </si>
-  <si>
     <t>THILF05197</t>
   </si>
   <si>
@@ -1816,6 +1877,196 @@
   </si>
   <si>
     <t>2026-06-12 16:40:00</t>
+  </si>
+  <si>
+    <t>E5430115061201</t>
+  </si>
+  <si>
+    <t>蘆洲河上洲</t>
+  </si>
+  <si>
+    <t>2026-06-12 23:17:10</t>
+  </si>
+  <si>
+    <t>F603</t>
+  </si>
+  <si>
+    <t>無法連線</t>
+  </si>
+  <si>
+    <t>門市反應tm1多卡機(QP3000E)無法使用悠遊卡/一卡通，已協助版本更新後悠遊卡機開機顯示通訊逾時，一卡通重開也顯示0801一卡通機異常...請台芝到店協助(櫃台操作 多卡機無反應 1號機)</t>
+  </si>
+  <si>
+    <t>THILF05430</t>
+  </si>
+  <si>
+    <t>2026-06-13 09:24:13</t>
+  </si>
+  <si>
+    <t>2026-06-15 09:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-16 13:00:00</t>
+  </si>
+  <si>
+    <t>重接排線 版本更新正常 測試正常</t>
+  </si>
+  <si>
+    <t>E4035115061401</t>
+  </si>
+  <si>
+    <t>龜山南上店</t>
+  </si>
+  <si>
+    <t>2026-06-14 09:04:01</t>
+  </si>
+  <si>
+    <t>門市反應TM1 CCD掃描器(HC56II-TR)前方膠條已破損且刷讀所有條碼都很難刷，已有執行校正仍異常，門市告知已造成困擾需求更換新掃描器...請台芝到店協助(掃描器感應不良 以校正過需更換新的掃描器2支 機1機2新品費用由加盟主自行吸收)</t>
+  </si>
+  <si>
+    <t>THILF04035</t>
+  </si>
+  <si>
+    <t>2026-06-14 09:25:13</t>
+  </si>
+  <si>
+    <t>2026-06-15 12:50:00</t>
+  </si>
+  <si>
+    <t>2026-06-15 13:20:00</t>
+  </si>
+  <si>
+    <t>更換掃描槍
+換下8119008446
+換上8119013784</t>
+  </si>
+  <si>
+    <t>14035115061401</t>
+  </si>
+  <si>
+    <t>2026-06-14 09:25:15</t>
+  </si>
+  <si>
+    <t>門市反應TM2 CCD掃描器(HC56II-TR)前方膠條已破損且刷讀所有條碼都很難刷，已有執行校正仍異常，門市告知已造成困擾需求更換新掃描器...請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-06-14 09:25:44</t>
+  </si>
+  <si>
+    <t>更換掃描槍
+換下8119006381
+換上8119013995</t>
+  </si>
+  <si>
+    <t>三重三文店</t>
+  </si>
+  <si>
+    <t>THILF04586</t>
+  </si>
+  <si>
+    <t>2026-06-15 10:02:34</t>
+  </si>
+  <si>
+    <t>2026-06-15 09:35:00</t>
+  </si>
+  <si>
+    <t>2026-06-15 09:57:00</t>
+  </si>
+  <si>
+    <t>D028</t>
+  </si>
+  <si>
+    <t>三重正義北店</t>
+  </si>
+  <si>
+    <t>THILF0D028</t>
+  </si>
+  <si>
+    <t>2026-06-15 10:48:31</t>
+  </si>
+  <si>
+    <t>2026-06-15 10:16:00</t>
+  </si>
+  <si>
+    <t>2026-06-15 10:38:00</t>
+  </si>
+  <si>
+    <t>2026-06-15 11:01:45</t>
+  </si>
+  <si>
+    <t>2026-06-15 11:00:00</t>
+  </si>
+  <si>
+    <t>蘆洲水湳店</t>
+  </si>
+  <si>
+    <t>THILF05082</t>
+  </si>
+  <si>
+    <t>2026-06-15 11:22:14</t>
+  </si>
+  <si>
+    <t>2026-06-15 11:30:00</t>
+  </si>
+  <si>
+    <t>三重重陽店</t>
+  </si>
+  <si>
+    <t>THILF05352</t>
+  </si>
+  <si>
+    <t>2026-06-15 11:28:25</t>
+  </si>
+  <si>
+    <t>2026-06-15 10:53:00</t>
+  </si>
+  <si>
+    <t>2026-06-15 11:20:00</t>
+  </si>
+  <si>
+    <t>三重自強店</t>
+  </si>
+  <si>
+    <t>THILF03623</t>
+  </si>
+  <si>
+    <t>2026-06-15 11:54:35</t>
+  </si>
+  <si>
+    <t>2026-06-15 11:55:00</t>
+  </si>
+  <si>
+    <t>2026-06-15 15:21:29</t>
+  </si>
+  <si>
+    <t>2026-06-15 15:30:00</t>
+  </si>
+  <si>
+    <t>C742</t>
+  </si>
+  <si>
+    <t>中和景安站</t>
+  </si>
+  <si>
+    <t>THILF0C742</t>
+  </si>
+  <si>
+    <t>2026-06-15 15:45:06</t>
+  </si>
+  <si>
+    <t>2026-06-15 15:42:00</t>
+  </si>
+  <si>
+    <t>裝潢撤機完成</t>
+  </si>
+  <si>
+    <t>2026-06-15 15:52:20</t>
+  </si>
+  <si>
+    <t>2026-06-15 15:50:00</t>
+  </si>
+  <si>
+    <t>改裝撤店</t>
   </si>
 </sst>
 </file>
@@ -2229,7 +2480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK80"/>
+  <dimension ref="A1:AK95"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -6399,7 +6650,7 @@
         <v>38</v>
       </c>
       <c r="C49" s="7">
-        <v>2026061643</v>
+        <v>2026061642</v>
       </c>
       <c r="D49" s="7" t="s">
         <v>406</v>
@@ -6407,17 +6658,17 @@
       <c r="E49" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="F49" s="7" t="s">
+      <c r="F49" s="7">
+        <v>2482</v>
+      </c>
+      <c r="G49" s="7" t="s">
         <v>407</v>
       </c>
-      <c r="G49" s="7" t="s">
+      <c r="H49" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I49" s="7" t="s">
         <v>408</v>
-      </c>
-      <c r="H49" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="I49" s="7" t="s">
-        <v>409</v>
       </c>
       <c r="J49" s="7" t="s">
         <v>141</v>
@@ -6441,13 +6692,13 @@
         <v>398</v>
       </c>
       <c r="Q49" s="7" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="R49" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S49" s="7" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="T49" s="7">
         <v>1</v>
@@ -6456,21 +6707,23 @@
         <v>53</v>
       </c>
       <c r="V49" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="W49" s="7" t="s">
         <v>411</v>
       </c>
-      <c r="W49" s="7" t="s">
+      <c r="X49" s="7" t="s">
         <v>412</v>
       </c>
-      <c r="X49" s="7" t="s">
+      <c r="Y49" s="7" t="s">
         <v>413</v>
       </c>
-      <c r="Y49" s="7" t="s">
+      <c r="Z49" s="7">
+        <v>1.9</v>
+      </c>
+      <c r="AA49" s="7" t="s">
         <v>414</v>
       </c>
-      <c r="Z49" s="7">
-        <v>2.5</v>
-      </c>
-      <c r="AA49" s="7"/>
       <c r="AB49" s="7" t="s">
         <v>58</v>
       </c>
@@ -6496,7 +6749,7 @@
         <v>38</v>
       </c>
       <c r="C50" s="3">
-        <v>2026061647</v>
+        <v>2026061643</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>416</v>
@@ -6504,17 +6757,17 @@
       <c r="E50" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F50" s="3">
-        <v>4341</v>
+      <c r="F50" s="3" t="s">
+        <v>417</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>170</v>
+        <v>209</v>
       </c>
       <c r="I50" s="3" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="J50" s="3" t="s">
         <v>141</v>
@@ -6538,13 +6791,13 @@
         <v>398</v>
       </c>
       <c r="Q50" s="3" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="R50" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S50" s="3" t="s">
-        <v>178</v>
+        <v>52</v>
       </c>
       <c r="T50" s="3">
         <v>1</v>
@@ -6553,28 +6806,26 @@
         <v>53</v>
       </c>
       <c r="V50" s="3" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="W50" s="3" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="X50" s="3" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="Y50" s="3" t="s">
-        <v>423</v>
+        <v>413</v>
       </c>
       <c r="Z50" s="3">
-        <v>1.8</v>
-      </c>
-      <c r="AA50" s="3" t="s">
-        <v>424</v>
-      </c>
+        <v>2.5</v>
+      </c>
+      <c r="AA50" s="3"/>
       <c r="AB50" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC50" s="10" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="AD50" s="3"/>
       <c r="AE50" s="3"/>
@@ -6592,38 +6843,58 @@
         <v>49</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C51" s="7">
-        <v>2026061674</v>
-      </c>
-      <c r="D51" s="7"/>
-      <c r="E51" s="7"/>
+        <v>2026061644</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>425</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F51" s="7">
-        <v>4503</v>
+        <v>5341</v>
       </c>
       <c r="G51" s="7" t="s">
         <v>426</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="I51" s="7"/>
-      <c r="J51" s="7"/>
-      <c r="K51" s="7"/>
-      <c r="L51" s="7"/>
-      <c r="M51" s="8"/>
-      <c r="N51" s="7"/>
-      <c r="O51" s="8"/>
-      <c r="P51" s="9"/>
+        <v>427</v>
+      </c>
+      <c r="I51" s="7" t="s">
+        <v>428</v>
+      </c>
+      <c r="J51" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="K51" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L51" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="M51" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="N51" s="7">
+        <v>2405</v>
+      </c>
+      <c r="O51" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="P51" s="9" t="s">
+        <v>429</v>
+      </c>
       <c r="Q51" s="7" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="R51" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S51" s="7" t="s">
-        <v>79</v>
+        <v>178</v>
       </c>
       <c r="T51" s="7">
         <v>1</v>
@@ -6632,28 +6903,30 @@
         <v>53</v>
       </c>
       <c r="V51" s="7" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="W51" s="7" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="X51" s="7" t="s">
-        <v>380</v>
-      </c>
-      <c r="Y51" s="7"/>
+        <v>433</v>
+      </c>
+      <c r="Y51" s="7" t="s">
+        <v>434</v>
+      </c>
       <c r="Z51" s="7">
-        <v>1</v>
-      </c>
-      <c r="AA51" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="AA51" s="7" t="s">
+        <v>435</v>
+      </c>
       <c r="AB51" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC51" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD51" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>436</v>
+      </c>
+      <c r="AD51" s="7"/>
       <c r="AE51" s="7"/>
       <c r="AF51" s="7"/>
       <c r="AG51" s="7"/>
@@ -6669,38 +6942,58 @@
         <v>50</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C52" s="3">
-        <v>2026061675</v>
-      </c>
-      <c r="D52" s="3"/>
-      <c r="E52" s="3"/>
-      <c r="F52" s="3" t="s">
-        <v>430</v>
+        <v>2026061647</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F52" s="3">
+        <v>4341</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="I52" s="3"/>
-      <c r="J52" s="3"/>
-      <c r="K52" s="3"/>
-      <c r="L52" s="3"/>
-      <c r="M52" s="4"/>
-      <c r="N52" s="3"/>
-      <c r="O52" s="4"/>
-      <c r="P52" s="10"/>
+        <v>170</v>
+      </c>
+      <c r="I52" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="J52" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="K52" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L52" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="M52" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="N52" s="3">
+        <v>2405</v>
+      </c>
+      <c r="O52" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="P52" s="10" t="s">
+        <v>398</v>
+      </c>
       <c r="Q52" s="3" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
       <c r="R52" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S52" s="3" t="s">
-        <v>79</v>
+        <v>178</v>
       </c>
       <c r="T52" s="3">
         <v>1</v>
@@ -6709,28 +7002,30 @@
         <v>53</v>
       </c>
       <c r="V52" s="3" t="s">
-        <v>433</v>
+        <v>441</v>
       </c>
       <c r="W52" s="3" t="s">
-        <v>434</v>
+        <v>442</v>
       </c>
       <c r="X52" s="3" t="s">
-        <v>435</v>
-      </c>
-      <c r="Y52" s="3"/>
+        <v>443</v>
+      </c>
+      <c r="Y52" s="3" t="s">
+        <v>444</v>
+      </c>
       <c r="Z52" s="3">
-        <v>0.3</v>
-      </c>
-      <c r="AA52" s="3"/>
+        <v>1.8</v>
+      </c>
+      <c r="AA52" s="3" t="s">
+        <v>445</v>
+      </c>
       <c r="AB52" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC52" s="10" t="s">
-        <v>436</v>
-      </c>
-      <c r="AD52" s="3" t="s">
-        <v>60</v>
-      </c>
+        <v>446</v>
+      </c>
+      <c r="AD52" s="3"/>
       <c r="AE52" s="3"/>
       <c r="AF52" s="3"/>
       <c r="AG52" s="3"/>
@@ -6749,15 +7044,15 @@
         <v>100</v>
       </c>
       <c r="C53" s="7">
-        <v>2026061677</v>
+        <v>2026061674</v>
       </c>
       <c r="D53" s="7"/>
       <c r="E53" s="7"/>
       <c r="F53" s="7">
-        <v>5031</v>
+        <v>4503</v>
       </c>
       <c r="G53" s="7" t="s">
-        <v>437</v>
+        <v>447</v>
       </c>
       <c r="H53" s="7" t="s">
         <v>75</v>
@@ -6771,7 +7066,7 @@
       <c r="O53" s="8"/>
       <c r="P53" s="9"/>
       <c r="Q53" s="7" t="s">
-        <v>438</v>
+        <v>448</v>
       </c>
       <c r="R53" s="7" t="s">
         <v>51</v>
@@ -6786,17 +7081,17 @@
         <v>53</v>
       </c>
       <c r="V53" s="7" t="s">
-        <v>439</v>
+        <v>449</v>
       </c>
       <c r="W53" s="7" t="s">
-        <v>440</v>
+        <v>450</v>
       </c>
       <c r="X53" s="7" t="s">
-        <v>441</v>
+        <v>380</v>
       </c>
       <c r="Y53" s="7"/>
       <c r="Z53" s="7">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="AA53" s="7"/>
       <c r="AB53" s="7" t="s">
@@ -6826,15 +7121,15 @@
         <v>100</v>
       </c>
       <c r="C54" s="3">
-        <v>2026061686</v>
+        <v>2026061675</v>
       </c>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
-      <c r="F54" s="3">
-        <v>3692</v>
+      <c r="F54" s="3" t="s">
+        <v>451</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>442</v>
+        <v>452</v>
       </c>
       <c r="H54" s="3" t="s">
         <v>75</v>
@@ -6848,7 +7143,7 @@
       <c r="O54" s="4"/>
       <c r="P54" s="10"/>
       <c r="Q54" s="3" t="s">
-        <v>443</v>
+        <v>453</v>
       </c>
       <c r="R54" s="3" t="s">
         <v>51</v>
@@ -6863,24 +7158,24 @@
         <v>53</v>
       </c>
       <c r="V54" s="3" t="s">
-        <v>444</v>
+        <v>454</v>
       </c>
       <c r="W54" s="3" t="s">
-        <v>445</v>
+        <v>455</v>
       </c>
       <c r="X54" s="3" t="s">
-        <v>446</v>
+        <v>456</v>
       </c>
       <c r="Y54" s="3"/>
       <c r="Z54" s="3">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="AA54" s="3"/>
       <c r="AB54" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC54" s="10" t="s">
-        <v>111</v>
+        <v>457</v>
       </c>
       <c r="AD54" s="3" t="s">
         <v>60</v>
@@ -6900,58 +7195,38 @@
         <v>53</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C55" s="7">
-        <v>2026061688</v>
-      </c>
-      <c r="D55" s="7" t="s">
-        <v>447</v>
-      </c>
-      <c r="E55" s="7" t="s">
-        <v>40</v>
-      </c>
+        <v>2026061677</v>
+      </c>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
       <c r="F55" s="7">
-        <v>4422</v>
+        <v>5031</v>
       </c>
       <c r="G55" s="7" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="I55" s="7" t="s">
-        <v>449</v>
-      </c>
-      <c r="J55" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="K55" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="L55" s="7" t="s">
-        <v>326</v>
-      </c>
-      <c r="M55" s="8" t="s">
-        <v>327</v>
-      </c>
-      <c r="N55" s="7" t="s">
-        <v>328</v>
-      </c>
-      <c r="O55" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="P55" s="9" t="s">
-        <v>450</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="I55" s="7"/>
+      <c r="J55" s="7"/>
+      <c r="K55" s="7"/>
+      <c r="L55" s="7"/>
+      <c r="M55" s="8"/>
+      <c r="N55" s="7"/>
+      <c r="O55" s="8"/>
+      <c r="P55" s="9"/>
       <c r="Q55" s="7" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
       <c r="R55" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S55" s="7" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="T55" s="7">
         <v>1</v>
@@ -6960,28 +7235,28 @@
         <v>53</v>
       </c>
       <c r="V55" s="7" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
       <c r="W55" s="7" t="s">
-        <v>453</v>
+        <v>461</v>
       </c>
       <c r="X55" s="7" t="s">
-        <v>454</v>
-      </c>
-      <c r="Y55" s="7" t="s">
-        <v>455</v>
-      </c>
+        <v>462</v>
+      </c>
+      <c r="Y55" s="7"/>
       <c r="Z55" s="7">
-        <v>1.1</v>
+        <v>0.3</v>
       </c>
       <c r="AA55" s="7"/>
       <c r="AB55" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC55" s="9" t="s">
-        <v>456</v>
-      </c>
-      <c r="AD55" s="7"/>
+        <v>111</v>
+      </c>
+      <c r="AD55" s="7" t="s">
+        <v>60</v>
+      </c>
       <c r="AE55" s="7"/>
       <c r="AF55" s="7"/>
       <c r="AG55" s="7"/>
@@ -6997,58 +7272,38 @@
         <v>54</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C56" s="3">
-        <v>2026061689</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>457</v>
-      </c>
-      <c r="E56" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>2026061686</v>
+      </c>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
       <c r="F56" s="3">
-        <v>4422</v>
+        <v>3692</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>448</v>
+        <v>463</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="I56" s="3" t="s">
-        <v>458</v>
-      </c>
-      <c r="J56" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="K56" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="L56" s="3" t="s">
-        <v>326</v>
-      </c>
-      <c r="M56" s="4" t="s">
-        <v>327</v>
-      </c>
-      <c r="N56" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="O56" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="P56" s="10" t="s">
-        <v>459</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="I56" s="3"/>
+      <c r="J56" s="3"/>
+      <c r="K56" s="3"/>
+      <c r="L56" s="3"/>
+      <c r="M56" s="4"/>
+      <c r="N56" s="3"/>
+      <c r="O56" s="4"/>
+      <c r="P56" s="10"/>
       <c r="Q56" s="3" t="s">
-        <v>451</v>
+        <v>464</v>
       </c>
       <c r="R56" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S56" s="3" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="T56" s="3">
         <v>1</v>
@@ -7057,28 +7312,28 @@
         <v>53</v>
       </c>
       <c r="V56" s="3" t="s">
-        <v>460</v>
+        <v>465</v>
       </c>
       <c r="W56" s="3" t="s">
-        <v>453</v>
+        <v>466</v>
       </c>
       <c r="X56" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="Y56" s="3" t="s">
-        <v>462</v>
-      </c>
+        <v>467</v>
+      </c>
+      <c r="Y56" s="3"/>
       <c r="Z56" s="3">
-        <v>1.1</v>
+        <v>0.5</v>
       </c>
       <c r="AA56" s="3"/>
       <c r="AB56" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC56" s="10" t="s">
-        <v>463</v>
-      </c>
-      <c r="AD56" s="3"/>
+        <v>111</v>
+      </c>
+      <c r="AD56" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="AE56" s="3"/>
       <c r="AF56" s="3"/>
       <c r="AG56" s="3"/>
@@ -7094,38 +7349,58 @@
         <v>55</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C57" s="7">
-        <v>2026061749</v>
-      </c>
-      <c r="D57" s="7"/>
-      <c r="E57" s="7"/>
+        <v>2026061688</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>468</v>
+      </c>
+      <c r="E57" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F57" s="7">
-        <v>2763</v>
+        <v>4422</v>
       </c>
       <c r="G57" s="7" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="I57" s="7"/>
-      <c r="J57" s="7"/>
-      <c r="K57" s="7"/>
-      <c r="L57" s="7"/>
-      <c r="M57" s="8"/>
-      <c r="N57" s="7"/>
-      <c r="O57" s="8"/>
-      <c r="P57" s="9"/>
+        <v>86</v>
+      </c>
+      <c r="I57" s="7" t="s">
+        <v>470</v>
+      </c>
+      <c r="J57" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="K57" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L57" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="M57" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="N57" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="O57" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="P57" s="9" t="s">
+        <v>471</v>
+      </c>
       <c r="Q57" s="7" t="s">
-        <v>465</v>
+        <v>472</v>
       </c>
       <c r="R57" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S57" s="7" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="T57" s="7">
         <v>1</v>
@@ -7134,28 +7409,28 @@
         <v>53</v>
       </c>
       <c r="V57" s="7" t="s">
-        <v>466</v>
+        <v>473</v>
       </c>
       <c r="W57" s="7" t="s">
-        <v>467</v>
+        <v>474</v>
       </c>
       <c r="X57" s="7" t="s">
-        <v>468</v>
-      </c>
-      <c r="Y57" s="7"/>
+        <v>475</v>
+      </c>
+      <c r="Y57" s="7" t="s">
+        <v>476</v>
+      </c>
       <c r="Z57" s="7">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
       <c r="AA57" s="7"/>
       <c r="AB57" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC57" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD57" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>477</v>
+      </c>
+      <c r="AD57" s="7"/>
       <c r="AE57" s="7"/>
       <c r="AF57" s="7"/>
       <c r="AG57" s="7"/>
@@ -7171,38 +7446,58 @@
         <v>56</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C58" s="3">
-        <v>2026061761</v>
-      </c>
-      <c r="D58" s="3"/>
-      <c r="E58" s="3"/>
+        <v>2026061689</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="F58" s="3">
-        <v>2401</v>
+        <v>4422</v>
       </c>
       <c r="G58" s="3" t="s">
         <v>469</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="I58" s="3"/>
-      <c r="J58" s="3"/>
-      <c r="K58" s="3"/>
-      <c r="L58" s="3"/>
-      <c r="M58" s="4"/>
-      <c r="N58" s="3"/>
-      <c r="O58" s="4"/>
-      <c r="P58" s="10"/>
+        <v>86</v>
+      </c>
+      <c r="I58" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="J58" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="K58" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L58" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="M58" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="N58" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="O58" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="P58" s="10" t="s">
+        <v>480</v>
+      </c>
       <c r="Q58" s="3" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="R58" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S58" s="3" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="T58" s="3">
         <v>1</v>
@@ -7211,28 +7506,28 @@
         <v>53</v>
       </c>
       <c r="V58" s="3" t="s">
-        <v>471</v>
+        <v>481</v>
       </c>
       <c r="W58" s="3" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="X58" s="3" t="s">
-        <v>473</v>
-      </c>
-      <c r="Y58" s="3"/>
+        <v>482</v>
+      </c>
+      <c r="Y58" s="3" t="s">
+        <v>483</v>
+      </c>
       <c r="Z58" s="3">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
       <c r="AA58" s="3"/>
       <c r="AB58" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC58" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD58" s="3" t="s">
-        <v>60</v>
-      </c>
+        <v>484</v>
+      </c>
+      <c r="AD58" s="3"/>
       <c r="AE58" s="3"/>
       <c r="AF58" s="3"/>
       <c r="AG58" s="3"/>
@@ -7251,18 +7546,18 @@
         <v>100</v>
       </c>
       <c r="C59" s="7">
-        <v>2026061769</v>
+        <v>2026061749</v>
       </c>
       <c r="D59" s="7"/>
       <c r="E59" s="7"/>
       <c r="F59" s="7">
-        <v>2988</v>
+        <v>2763</v>
       </c>
       <c r="G59" s="7" t="s">
-        <v>474</v>
+        <v>485</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>128</v>
+        <v>75</v>
       </c>
       <c r="I59" s="7"/>
       <c r="J59" s="7"/>
@@ -7273,7 +7568,7 @@
       <c r="O59" s="8"/>
       <c r="P59" s="9"/>
       <c r="Q59" s="7" t="s">
-        <v>475</v>
+        <v>486</v>
       </c>
       <c r="R59" s="7" t="s">
         <v>51</v>
@@ -7288,24 +7583,24 @@
         <v>53</v>
       </c>
       <c r="V59" s="7" t="s">
-        <v>476</v>
+        <v>487</v>
       </c>
       <c r="W59" s="7" t="s">
-        <v>477</v>
+        <v>488</v>
       </c>
       <c r="X59" s="7" t="s">
-        <v>478</v>
+        <v>489</v>
       </c>
       <c r="Y59" s="7"/>
       <c r="Z59" s="7">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="AA59" s="7"/>
       <c r="AB59" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC59" s="9" t="s">
-        <v>157</v>
+        <v>111</v>
       </c>
       <c r="AD59" s="7" t="s">
         <v>60</v>
@@ -7325,58 +7620,38 @@
         <v>58</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C60" s="3">
-        <v>2026061770</v>
-      </c>
-      <c r="D60" s="3" t="s">
-        <v>479</v>
-      </c>
-      <c r="E60" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>2026061761</v>
+      </c>
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
       <c r="F60" s="3">
-        <v>3811</v>
+        <v>2401</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I60" s="3" t="s">
-        <v>481</v>
-      </c>
-      <c r="J60" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="K60" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="L60" s="3" t="s">
-        <v>482</v>
-      </c>
-      <c r="M60" s="4" t="s">
-        <v>483</v>
-      </c>
-      <c r="N60" s="3" t="s">
-        <v>484</v>
-      </c>
-      <c r="O60" s="4" t="s">
-        <v>485</v>
-      </c>
-      <c r="P60" s="10" t="s">
-        <v>486</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="I60" s="3"/>
+      <c r="J60" s="3"/>
+      <c r="K60" s="3"/>
+      <c r="L60" s="3"/>
+      <c r="M60" s="4"/>
+      <c r="N60" s="3"/>
+      <c r="O60" s="4"/>
+      <c r="P60" s="10"/>
       <c r="Q60" s="3" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="R60" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S60" s="3" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="T60" s="3">
         <v>1</v>
@@ -7385,28 +7660,28 @@
         <v>53</v>
       </c>
       <c r="V60" s="3" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="W60" s="3" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="X60" s="3" t="s">
-        <v>490</v>
-      </c>
-      <c r="Y60" s="3" t="s">
-        <v>491</v>
-      </c>
+        <v>494</v>
+      </c>
+      <c r="Y60" s="3"/>
       <c r="Z60" s="3">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="AA60" s="3"/>
       <c r="AB60" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC60" s="10" t="s">
-        <v>492</v>
-      </c>
-      <c r="AD60" s="3"/>
+        <v>111</v>
+      </c>
+      <c r="AD60" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="AE60" s="3"/>
       <c r="AF60" s="3"/>
       <c r="AG60" s="3"/>
@@ -7422,58 +7697,38 @@
         <v>59</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C61" s="7">
-        <v>2026061773</v>
-      </c>
-      <c r="D61" s="7" t="s">
-        <v>493</v>
-      </c>
-      <c r="E61" s="7" t="s">
-        <v>40</v>
-      </c>
+        <v>2026061769</v>
+      </c>
+      <c r="D61" s="7"/>
+      <c r="E61" s="7"/>
       <c r="F61" s="7">
-        <v>3811</v>
+        <v>2988</v>
       </c>
       <c r="G61" s="7" t="s">
-        <v>480</v>
+        <v>495</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="I61" s="7" t="s">
-        <v>494</v>
-      </c>
-      <c r="J61" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="K61" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="L61" s="7" t="s">
-        <v>482</v>
-      </c>
-      <c r="M61" s="8" t="s">
-        <v>483</v>
-      </c>
-      <c r="N61" s="7" t="s">
-        <v>484</v>
-      </c>
-      <c r="O61" s="8" t="s">
-        <v>485</v>
-      </c>
-      <c r="P61" s="9" t="s">
-        <v>495</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="I61" s="7"/>
+      <c r="J61" s="7"/>
+      <c r="K61" s="7"/>
+      <c r="L61" s="7"/>
+      <c r="M61" s="8"/>
+      <c r="N61" s="7"/>
+      <c r="O61" s="8"/>
+      <c r="P61" s="9"/>
       <c r="Q61" s="7" t="s">
-        <v>487</v>
+        <v>496</v>
       </c>
       <c r="R61" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S61" s="7" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="T61" s="7">
         <v>1</v>
@@ -7482,28 +7737,28 @@
         <v>53</v>
       </c>
       <c r="V61" s="7" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="W61" s="7" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="X61" s="7" t="s">
-        <v>489</v>
-      </c>
-      <c r="Y61" s="7" t="s">
-        <v>498</v>
-      </c>
+        <v>499</v>
+      </c>
+      <c r="Y61" s="7"/>
       <c r="Z61" s="7">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="AA61" s="7"/>
       <c r="AB61" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC61" s="9" t="s">
-        <v>492</v>
-      </c>
-      <c r="AD61" s="7"/>
+        <v>157</v>
+      </c>
+      <c r="AD61" s="7" t="s">
+        <v>60</v>
+      </c>
       <c r="AE61" s="7"/>
       <c r="AF61" s="7"/>
       <c r="AG61" s="7"/>
@@ -7519,38 +7774,58 @@
         <v>60</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C62" s="3">
-        <v>2026061829</v>
-      </c>
-      <c r="D62" s="3"/>
-      <c r="E62" s="3"/>
+        <v>2026061770</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>500</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="F62" s="3">
-        <v>5248</v>
+        <v>3811</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="I62" s="3"/>
-      <c r="J62" s="3"/>
-      <c r="K62" s="3"/>
-      <c r="L62" s="3"/>
-      <c r="M62" s="4"/>
-      <c r="N62" s="3"/>
-      <c r="O62" s="4"/>
-      <c r="P62" s="10"/>
+        <v>42</v>
+      </c>
+      <c r="I62" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="J62" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="K62" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L62" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="M62" s="4" t="s">
+        <v>504</v>
+      </c>
+      <c r="N62" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="O62" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="P62" s="10" t="s">
+        <v>507</v>
+      </c>
       <c r="Q62" s="3" t="s">
-        <v>500</v>
+        <v>508</v>
       </c>
       <c r="R62" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S62" s="3" t="s">
-        <v>178</v>
+        <v>52</v>
       </c>
       <c r="T62" s="3">
         <v>1</v>
@@ -7559,29 +7834,29 @@
         <v>53</v>
       </c>
       <c r="V62" s="3" t="s">
-        <v>501</v>
+        <v>509</v>
       </c>
       <c r="W62" s="3" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="X62" s="3" t="s">
-        <v>503</v>
-      </c>
-      <c r="Y62" s="3"/>
+        <v>511</v>
+      </c>
+      <c r="Y62" s="3" t="s">
+        <v>512</v>
+      </c>
       <c r="Z62" s="3">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="AA62" s="3"/>
       <c r="AB62" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC62" s="10" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="AD62" s="3"/>
-      <c r="AE62" s="3" t="s">
-        <v>60</v>
-      </c>
+      <c r="AE62" s="3"/>
       <c r="AF62" s="3"/>
       <c r="AG62" s="3"/>
       <c r="AH62" s="3"/>
@@ -7596,38 +7871,58 @@
         <v>61</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C63" s="7">
-        <v>2026061830</v>
-      </c>
-      <c r="D63" s="7"/>
-      <c r="E63" s="7"/>
+        <v>2026061773</v>
+      </c>
+      <c r="D63" s="7" t="s">
+        <v>514</v>
+      </c>
+      <c r="E63" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F63" s="7">
-        <v>5248</v>
+        <v>3811</v>
       </c>
       <c r="G63" s="7" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="I63" s="7"/>
-      <c r="J63" s="7"/>
-      <c r="K63" s="7"/>
-      <c r="L63" s="7"/>
-      <c r="M63" s="8"/>
-      <c r="N63" s="7"/>
-      <c r="O63" s="8"/>
-      <c r="P63" s="9"/>
+        <v>42</v>
+      </c>
+      <c r="I63" s="7" t="s">
+        <v>515</v>
+      </c>
+      <c r="J63" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="K63" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L63" s="7" t="s">
+        <v>503</v>
+      </c>
+      <c r="M63" s="8" t="s">
+        <v>504</v>
+      </c>
+      <c r="N63" s="7" t="s">
+        <v>505</v>
+      </c>
+      <c r="O63" s="8" t="s">
+        <v>506</v>
+      </c>
+      <c r="P63" s="9" t="s">
+        <v>516</v>
+      </c>
       <c r="Q63" s="7" t="s">
-        <v>500</v>
+        <v>508</v>
       </c>
       <c r="R63" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S63" s="7" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="T63" s="7">
         <v>1</v>
@@ -7636,28 +7931,28 @@
         <v>53</v>
       </c>
       <c r="V63" s="7" t="s">
-        <v>505</v>
+        <v>517</v>
       </c>
       <c r="W63" s="7" t="s">
-        <v>412</v>
+        <v>518</v>
       </c>
       <c r="X63" s="7" t="s">
-        <v>502</v>
-      </c>
-      <c r="Y63" s="7"/>
+        <v>510</v>
+      </c>
+      <c r="Y63" s="7" t="s">
+        <v>519</v>
+      </c>
       <c r="Z63" s="7">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="AA63" s="7"/>
       <c r="AB63" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC63" s="9" t="s">
-        <v>506</v>
-      </c>
-      <c r="AD63" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>513</v>
+      </c>
+      <c r="AD63" s="7"/>
       <c r="AE63" s="7"/>
       <c r="AF63" s="7"/>
       <c r="AG63" s="7"/>
@@ -7676,7 +7971,7 @@
         <v>100</v>
       </c>
       <c r="C64" s="3">
-        <v>2026061831</v>
+        <v>2026061829</v>
       </c>
       <c r="D64" s="3"/>
       <c r="E64" s="3"/>
@@ -7684,7 +7979,7 @@
         <v>5248</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>499</v>
+        <v>520</v>
       </c>
       <c r="H64" s="3" t="s">
         <v>75</v>
@@ -7698,13 +7993,13 @@
       <c r="O64" s="4"/>
       <c r="P64" s="10"/>
       <c r="Q64" s="3" t="s">
-        <v>500</v>
+        <v>521</v>
       </c>
       <c r="R64" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S64" s="3" t="s">
-        <v>79</v>
+        <v>178</v>
       </c>
       <c r="T64" s="3">
         <v>1</v>
@@ -7713,13 +8008,13 @@
         <v>53</v>
       </c>
       <c r="V64" s="3" t="s">
-        <v>507</v>
+        <v>522</v>
       </c>
       <c r="W64" s="3" t="s">
-        <v>502</v>
+        <v>523</v>
       </c>
       <c r="X64" s="3" t="s">
-        <v>503</v>
+        <v>524</v>
       </c>
       <c r="Y64" s="3"/>
       <c r="Z64" s="3">
@@ -7730,7 +8025,7 @@
         <v>58</v>
       </c>
       <c r="AC64" s="10" t="s">
-        <v>508</v>
+        <v>525</v>
       </c>
       <c r="AD64" s="3"/>
       <c r="AE64" s="3" t="s">
@@ -7753,18 +8048,18 @@
         <v>100</v>
       </c>
       <c r="C65" s="7">
-        <v>2026061839</v>
+        <v>2026061830</v>
       </c>
       <c r="D65" s="7"/>
       <c r="E65" s="7"/>
-      <c r="F65" s="7" t="s">
-        <v>384</v>
+      <c r="F65" s="7">
+        <v>5248</v>
       </c>
       <c r="G65" s="7" t="s">
-        <v>385</v>
+        <v>520</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="I65" s="7"/>
       <c r="J65" s="7"/>
@@ -7775,13 +8070,13 @@
       <c r="O65" s="8"/>
       <c r="P65" s="9"/>
       <c r="Q65" s="7" t="s">
-        <v>388</v>
+        <v>521</v>
       </c>
       <c r="R65" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S65" s="7" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="T65" s="7">
         <v>1</v>
@@ -7790,24 +8085,24 @@
         <v>53</v>
       </c>
       <c r="V65" s="7" t="s">
-        <v>509</v>
+        <v>526</v>
       </c>
       <c r="W65" s="7" t="s">
-        <v>390</v>
+        <v>422</v>
       </c>
       <c r="X65" s="7" t="s">
-        <v>391</v>
+        <v>523</v>
       </c>
       <c r="Y65" s="7"/>
       <c r="Z65" s="7">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="AA65" s="7"/>
       <c r="AB65" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC65" s="9" t="s">
-        <v>111</v>
+        <v>527</v>
       </c>
       <c r="AD65" s="7" t="s">
         <v>60</v>
@@ -7830,18 +8125,18 @@
         <v>100</v>
       </c>
       <c r="C66" s="3">
-        <v>2026061850</v>
+        <v>2026061831</v>
       </c>
       <c r="D66" s="3"/>
       <c r="E66" s="3"/>
       <c r="F66" s="3">
-        <v>4422</v>
+        <v>5248</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>448</v>
+        <v>520</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="I66" s="3"/>
       <c r="J66" s="3"/>
@@ -7852,13 +8147,13 @@
       <c r="O66" s="4"/>
       <c r="P66" s="10"/>
       <c r="Q66" s="3" t="s">
-        <v>451</v>
+        <v>521</v>
       </c>
       <c r="R66" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S66" s="3" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="T66" s="3">
         <v>1</v>
@@ -7867,29 +8162,29 @@
         <v>53</v>
       </c>
       <c r="V66" s="3" t="s">
-        <v>510</v>
+        <v>528</v>
       </c>
       <c r="W66" s="3" t="s">
-        <v>453</v>
+        <v>523</v>
       </c>
       <c r="X66" s="3" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="Y66" s="3"/>
       <c r="Z66" s="3">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="AA66" s="3"/>
       <c r="AB66" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC66" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD66" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AE66" s="3"/>
+        <v>529</v>
+      </c>
+      <c r="AD66" s="3"/>
+      <c r="AE66" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="AF66" s="3"/>
       <c r="AG66" s="3"/>
       <c r="AH66" s="3"/>
@@ -7907,18 +8202,18 @@
         <v>100</v>
       </c>
       <c r="C67" s="7">
-        <v>2026061879</v>
+        <v>2026061839</v>
       </c>
       <c r="D67" s="7"/>
       <c r="E67" s="7"/>
-      <c r="F67" s="7">
-        <v>4748</v>
+      <c r="F67" s="7" t="s">
+        <v>384</v>
       </c>
       <c r="G67" s="7" t="s">
-        <v>512</v>
+        <v>385</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>209</v>
+        <v>86</v>
       </c>
       <c r="I67" s="7"/>
       <c r="J67" s="7"/>
@@ -7929,13 +8224,13 @@
       <c r="O67" s="8"/>
       <c r="P67" s="9"/>
       <c r="Q67" s="7" t="s">
-        <v>513</v>
+        <v>388</v>
       </c>
       <c r="R67" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S67" s="7" t="s">
-        <v>52</v>
+        <v>94</v>
       </c>
       <c r="T67" s="7">
         <v>1</v>
@@ -7944,24 +8239,24 @@
         <v>53</v>
       </c>
       <c r="V67" s="7" t="s">
-        <v>514</v>
+        <v>530</v>
       </c>
       <c r="W67" s="7" t="s">
-        <v>515</v>
+        <v>390</v>
       </c>
       <c r="X67" s="7" t="s">
-        <v>516</v>
+        <v>391</v>
       </c>
       <c r="Y67" s="7"/>
       <c r="Z67" s="7">
-        <v>2</v>
+        <v>0.2</v>
       </c>
       <c r="AA67" s="7"/>
       <c r="AB67" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC67" s="9" t="s">
-        <v>167</v>
+        <v>111</v>
       </c>
       <c r="AD67" s="7" t="s">
         <v>60</v>
@@ -7971,9 +8266,7 @@
       <c r="AG67" s="7"/>
       <c r="AH67" s="7"/>
       <c r="AI67" s="7"/>
-      <c r="AJ67" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ67" s="7"/>
       <c r="AK67" s="7" t="s">
         <v>60</v>
       </c>
@@ -7986,18 +8279,18 @@
         <v>100</v>
       </c>
       <c r="C68" s="3">
-        <v>2026061916</v>
+        <v>2026061850</v>
       </c>
       <c r="D68" s="3"/>
       <c r="E68" s="3"/>
-      <c r="F68" s="3" t="s">
-        <v>517</v>
+      <c r="F68" s="3">
+        <v>4422</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>518</v>
+        <v>469</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>42</v>
+        <v>86</v>
       </c>
       <c r="I68" s="3"/>
       <c r="J68" s="3"/>
@@ -8008,13 +8301,13 @@
       <c r="O68" s="4"/>
       <c r="P68" s="10"/>
       <c r="Q68" s="3" t="s">
-        <v>519</v>
+        <v>472</v>
       </c>
       <c r="R68" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S68" s="3" t="s">
-        <v>52</v>
+        <v>94</v>
       </c>
       <c r="T68" s="3">
         <v>1</v>
@@ -8023,13 +8316,13 @@
         <v>53</v>
       </c>
       <c r="V68" s="3" t="s">
-        <v>520</v>
+        <v>531</v>
       </c>
       <c r="W68" s="3" t="s">
-        <v>521</v>
+        <v>474</v>
       </c>
       <c r="X68" s="3" t="s">
-        <v>522</v>
+        <v>532</v>
       </c>
       <c r="Y68" s="3"/>
       <c r="Z68" s="3">
@@ -8050,9 +8343,7 @@
       <c r="AG68" s="3"/>
       <c r="AH68" s="3"/>
       <c r="AI68" s="3"/>
-      <c r="AJ68" s="3" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ68" s="3"/>
       <c r="AK68" s="3" t="s">
         <v>60</v>
       </c>
@@ -8065,18 +8356,18 @@
         <v>100</v>
       </c>
       <c r="C69" s="7">
-        <v>2026061920</v>
+        <v>2026061879</v>
       </c>
       <c r="D69" s="7"/>
       <c r="E69" s="7"/>
-      <c r="F69" s="7" t="s">
-        <v>523</v>
+      <c r="F69" s="7">
+        <v>4748</v>
       </c>
       <c r="G69" s="7" t="s">
-        <v>524</v>
+        <v>533</v>
       </c>
       <c r="H69" s="7" t="s">
-        <v>42</v>
+        <v>209</v>
       </c>
       <c r="I69" s="7"/>
       <c r="J69" s="7"/>
@@ -8087,7 +8378,7 @@
       <c r="O69" s="8"/>
       <c r="P69" s="9"/>
       <c r="Q69" s="7" t="s">
-        <v>525</v>
+        <v>534</v>
       </c>
       <c r="R69" s="7" t="s">
         <v>51</v>
@@ -8102,24 +8393,24 @@
         <v>53</v>
       </c>
       <c r="V69" s="7" t="s">
-        <v>526</v>
+        <v>535</v>
       </c>
       <c r="W69" s="7" t="s">
-        <v>527</v>
+        <v>536</v>
       </c>
       <c r="X69" s="7" t="s">
-        <v>528</v>
+        <v>537</v>
       </c>
       <c r="Y69" s="7"/>
       <c r="Z69" s="7">
-        <v>0.4</v>
+        <v>2</v>
       </c>
       <c r="AA69" s="7"/>
       <c r="AB69" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC69" s="9" t="s">
-        <v>111</v>
+        <v>167</v>
       </c>
       <c r="AD69" s="7" t="s">
         <v>60</v>
@@ -8144,18 +8435,18 @@
         <v>100</v>
       </c>
       <c r="C70" s="3">
-        <v>2026061921</v>
+        <v>2026061916</v>
       </c>
       <c r="D70" s="3"/>
       <c r="E70" s="3"/>
-      <c r="F70" s="3">
-        <v>5197</v>
+      <c r="F70" s="3" t="s">
+        <v>538</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>529</v>
+        <v>539</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>530</v>
+        <v>42</v>
       </c>
       <c r="I70" s="3"/>
       <c r="J70" s="3"/>
@@ -8166,13 +8457,13 @@
       <c r="O70" s="4"/>
       <c r="P70" s="10"/>
       <c r="Q70" s="3" t="s">
-        <v>531</v>
+        <v>540</v>
       </c>
       <c r="R70" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S70" s="3" t="s">
-        <v>178</v>
+        <v>52</v>
       </c>
       <c r="T70" s="3">
         <v>1</v>
@@ -8181,17 +8472,17 @@
         <v>53</v>
       </c>
       <c r="V70" s="3" t="s">
-        <v>532</v>
+        <v>541</v>
       </c>
       <c r="W70" s="3" t="s">
-        <v>533</v>
+        <v>542</v>
       </c>
       <c r="X70" s="3" t="s">
-        <v>534</v>
+        <v>543</v>
       </c>
       <c r="Y70" s="3"/>
       <c r="Z70" s="3">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="AA70" s="3"/>
       <c r="AB70" s="3" t="s">
@@ -8223,18 +8514,18 @@
         <v>100</v>
       </c>
       <c r="C71" s="7">
-        <v>2026061926</v>
+        <v>2026061920</v>
       </c>
       <c r="D71" s="7"/>
       <c r="E71" s="7"/>
-      <c r="F71" s="7">
-        <v>2958</v>
+      <c r="F71" s="7" t="s">
+        <v>544</v>
       </c>
       <c r="G71" s="7" t="s">
-        <v>535</v>
+        <v>545</v>
       </c>
       <c r="H71" s="7" t="s">
-        <v>530</v>
+        <v>42</v>
       </c>
       <c r="I71" s="7"/>
       <c r="J71" s="7"/>
@@ -8245,13 +8536,13 @@
       <c r="O71" s="8"/>
       <c r="P71" s="9"/>
       <c r="Q71" s="7" t="s">
-        <v>536</v>
+        <v>546</v>
       </c>
       <c r="R71" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S71" s="7" t="s">
-        <v>178</v>
+        <v>52</v>
       </c>
       <c r="T71" s="7">
         <v>1</v>
@@ -8260,17 +8551,17 @@
         <v>53</v>
       </c>
       <c r="V71" s="7" t="s">
-        <v>537</v>
+        <v>547</v>
       </c>
       <c r="W71" s="7" t="s">
-        <v>534</v>
+        <v>548</v>
       </c>
       <c r="X71" s="7" t="s">
-        <v>538</v>
+        <v>549</v>
       </c>
       <c r="Y71" s="7"/>
       <c r="Z71" s="7">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="AA71" s="7"/>
       <c r="AB71" s="7" t="s">
@@ -8302,18 +8593,18 @@
         <v>100</v>
       </c>
       <c r="C72" s="3">
-        <v>2026061928</v>
+        <v>2026061921</v>
       </c>
       <c r="D72" s="3"/>
       <c r="E72" s="3"/>
       <c r="F72" s="3">
-        <v>4098</v>
+        <v>5197</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>42</v>
+        <v>427</v>
       </c>
       <c r="I72" s="3"/>
       <c r="J72" s="3"/>
@@ -8324,13 +8615,13 @@
       <c r="O72" s="4"/>
       <c r="P72" s="10"/>
       <c r="Q72" s="3" t="s">
-        <v>540</v>
+        <v>551</v>
       </c>
       <c r="R72" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S72" s="3" t="s">
-        <v>52</v>
+        <v>178</v>
       </c>
       <c r="T72" s="3">
         <v>1</v>
@@ -8339,17 +8630,17 @@
         <v>53</v>
       </c>
       <c r="V72" s="3" t="s">
-        <v>541</v>
+        <v>552</v>
       </c>
       <c r="W72" s="3" t="s">
-        <v>542</v>
+        <v>553</v>
       </c>
       <c r="X72" s="3" t="s">
-        <v>538</v>
+        <v>554</v>
       </c>
       <c r="Y72" s="3"/>
       <c r="Z72" s="3">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="AA72" s="3"/>
       <c r="AB72" s="3" t="s">
@@ -8381,18 +8672,18 @@
         <v>100</v>
       </c>
       <c r="C73" s="7">
-        <v>2026061931</v>
+        <v>2026061926</v>
       </c>
       <c r="D73" s="7"/>
       <c r="E73" s="7"/>
       <c r="F73" s="7">
-        <v>3853</v>
+        <v>2958</v>
       </c>
       <c r="G73" s="7" t="s">
-        <v>543</v>
+        <v>555</v>
       </c>
       <c r="H73" s="7" t="s">
-        <v>86</v>
+        <v>427</v>
       </c>
       <c r="I73" s="7"/>
       <c r="J73" s="7"/>
@@ -8403,13 +8694,13 @@
       <c r="O73" s="8"/>
       <c r="P73" s="9"/>
       <c r="Q73" s="7" t="s">
-        <v>544</v>
+        <v>556</v>
       </c>
       <c r="R73" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S73" s="7" t="s">
-        <v>79</v>
+        <v>178</v>
       </c>
       <c r="T73" s="7">
         <v>1</v>
@@ -8418,24 +8709,24 @@
         <v>53</v>
       </c>
       <c r="V73" s="7" t="s">
-        <v>545</v>
+        <v>557</v>
       </c>
       <c r="W73" s="7" t="s">
-        <v>546</v>
+        <v>554</v>
       </c>
       <c r="X73" s="7" t="s">
-        <v>547</v>
+        <v>558</v>
       </c>
       <c r="Y73" s="7"/>
       <c r="Z73" s="7">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="AA73" s="7"/>
       <c r="AB73" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC73" s="9" t="s">
-        <v>157</v>
+        <v>111</v>
       </c>
       <c r="AD73" s="7" t="s">
         <v>60</v>
@@ -8445,7 +8736,9 @@
       <c r="AG73" s="7"/>
       <c r="AH73" s="7"/>
       <c r="AI73" s="7"/>
-      <c r="AJ73" s="7"/>
+      <c r="AJ73" s="7" t="s">
+        <v>60</v>
+      </c>
       <c r="AK73" s="7" t="s">
         <v>60</v>
       </c>
@@ -8458,18 +8751,18 @@
         <v>100</v>
       </c>
       <c r="C74" s="3">
-        <v>2026061963</v>
+        <v>2026061928</v>
       </c>
       <c r="D74" s="3"/>
       <c r="E74" s="3"/>
       <c r="F74" s="3">
-        <v>5384</v>
+        <v>4098</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>548</v>
+        <v>559</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="I74" s="3"/>
       <c r="J74" s="3"/>
@@ -8480,13 +8773,13 @@
       <c r="O74" s="4"/>
       <c r="P74" s="10"/>
       <c r="Q74" s="3" t="s">
-        <v>549</v>
+        <v>560</v>
       </c>
       <c r="R74" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S74" s="3" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="T74" s="3">
         <v>1</v>
@@ -8495,24 +8788,24 @@
         <v>53</v>
       </c>
       <c r="V74" s="3" t="s">
-        <v>550</v>
+        <v>561</v>
       </c>
       <c r="W74" s="3" t="s">
-        <v>551</v>
+        <v>562</v>
       </c>
       <c r="X74" s="3" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="Y74" s="3"/>
       <c r="Z74" s="3">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="AA74" s="3"/>
       <c r="AB74" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC74" s="10" t="s">
-        <v>157</v>
+        <v>111</v>
       </c>
       <c r="AD74" s="3" t="s">
         <v>60</v>
@@ -8522,7 +8815,9 @@
       <c r="AG74" s="3"/>
       <c r="AH74" s="3"/>
       <c r="AI74" s="3"/>
-      <c r="AJ74" s="3"/>
+      <c r="AJ74" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="AK74" s="3" t="s">
         <v>60</v>
       </c>
@@ -8535,18 +8830,18 @@
         <v>100</v>
       </c>
       <c r="C75" s="7">
-        <v>2026061971</v>
+        <v>2026061931</v>
       </c>
       <c r="D75" s="7"/>
       <c r="E75" s="7"/>
       <c r="F75" s="7">
-        <v>3957</v>
+        <v>3853</v>
       </c>
       <c r="G75" s="7" t="s">
-        <v>553</v>
+        <v>563</v>
       </c>
       <c r="H75" s="7" t="s">
-        <v>42</v>
+        <v>86</v>
       </c>
       <c r="I75" s="7"/>
       <c r="J75" s="7"/>
@@ -8557,13 +8852,13 @@
       <c r="O75" s="8"/>
       <c r="P75" s="9"/>
       <c r="Q75" s="7" t="s">
-        <v>554</v>
+        <v>564</v>
       </c>
       <c r="R75" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S75" s="7" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="T75" s="7">
         <v>1</v>
@@ -8572,24 +8867,24 @@
         <v>53</v>
       </c>
       <c r="V75" s="7" t="s">
-        <v>555</v>
+        <v>565</v>
       </c>
       <c r="W75" s="7" t="s">
-        <v>556</v>
+        <v>566</v>
       </c>
       <c r="X75" s="7" t="s">
-        <v>557</v>
+        <v>567</v>
       </c>
       <c r="Y75" s="7"/>
       <c r="Z75" s="7">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="AA75" s="7"/>
       <c r="AB75" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC75" s="9" t="s">
-        <v>111</v>
+        <v>157</v>
       </c>
       <c r="AD75" s="7" t="s">
         <v>60</v>
@@ -8599,9 +8894,7 @@
       <c r="AG75" s="7"/>
       <c r="AH75" s="7"/>
       <c r="AI75" s="7"/>
-      <c r="AJ75" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ75" s="7"/>
       <c r="AK75" s="7" t="s">
         <v>60</v>
       </c>
@@ -8614,15 +8907,15 @@
         <v>100</v>
       </c>
       <c r="C76" s="3">
-        <v>2026061977</v>
+        <v>2026061963</v>
       </c>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3">
-        <v>3965</v>
+        <v>5384</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>558</v>
+        <v>568</v>
       </c>
       <c r="H76" s="3" t="s">
         <v>86</v>
@@ -8636,7 +8929,7 @@
       <c r="O76" s="4"/>
       <c r="P76" s="10"/>
       <c r="Q76" s="3" t="s">
-        <v>559</v>
+        <v>569</v>
       </c>
       <c r="R76" s="3" t="s">
         <v>51</v>
@@ -8651,24 +8944,24 @@
         <v>53</v>
       </c>
       <c r="V76" s="3" t="s">
-        <v>560</v>
+        <v>570</v>
       </c>
       <c r="W76" s="3" t="s">
-        <v>561</v>
+        <v>571</v>
       </c>
       <c r="X76" s="3" t="s">
-        <v>562</v>
+        <v>572</v>
       </c>
       <c r="Y76" s="3"/>
       <c r="Z76" s="3">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="AA76" s="3"/>
       <c r="AB76" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC76" s="10" t="s">
-        <v>111</v>
+        <v>157</v>
       </c>
       <c r="AD76" s="3" t="s">
         <v>60</v>
@@ -8691,15 +8984,15 @@
         <v>100</v>
       </c>
       <c r="C77" s="7">
-        <v>2026061983</v>
+        <v>2026061971</v>
       </c>
       <c r="D77" s="7"/>
       <c r="E77" s="7"/>
-      <c r="F77" s="7" t="s">
-        <v>563</v>
+      <c r="F77" s="7">
+        <v>3957</v>
       </c>
       <c r="G77" s="7" t="s">
-        <v>564</v>
+        <v>573</v>
       </c>
       <c r="H77" s="7" t="s">
         <v>42</v>
@@ -8713,7 +9006,7 @@
       <c r="O77" s="8"/>
       <c r="P77" s="9"/>
       <c r="Q77" s="7" t="s">
-        <v>565</v>
+        <v>574</v>
       </c>
       <c r="R77" s="7" t="s">
         <v>51</v>
@@ -8728,17 +9021,17 @@
         <v>53</v>
       </c>
       <c r="V77" s="7" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="W77" s="7" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="X77" s="7" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="Y77" s="7"/>
       <c r="Z77" s="7">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="AA77" s="7"/>
       <c r="AB77" s="7" t="s">
@@ -8770,15 +9063,15 @@
         <v>100</v>
       </c>
       <c r="C78" s="3">
-        <v>2026061986</v>
+        <v>2026061977</v>
       </c>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3">
-        <v>2154</v>
+        <v>3965</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>86</v>
@@ -8792,7 +9085,7 @@
       <c r="O78" s="4"/>
       <c r="P78" s="10"/>
       <c r="Q78" s="3" t="s">
-        <v>570</v>
+        <v>579</v>
       </c>
       <c r="R78" s="3" t="s">
         <v>51</v>
@@ -8807,17 +9100,17 @@
         <v>53</v>
       </c>
       <c r="V78" s="3" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="W78" s="3" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="X78" s="3" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
       <c r="Y78" s="3"/>
       <c r="Z78" s="3">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="AA78" s="3"/>
       <c r="AB78" s="3" t="s">
@@ -8847,15 +9140,15 @@
         <v>100</v>
       </c>
       <c r="C79" s="7">
-        <v>2026062001</v>
+        <v>2026061983</v>
       </c>
       <c r="D79" s="7"/>
       <c r="E79" s="7"/>
-      <c r="F79" s="7">
-        <v>5245</v>
+      <c r="F79" s="7" t="s">
+        <v>583</v>
       </c>
       <c r="G79" s="7" t="s">
-        <v>574</v>
+        <v>584</v>
       </c>
       <c r="H79" s="7" t="s">
         <v>42</v>
@@ -8869,7 +9162,7 @@
       <c r="O79" s="8"/>
       <c r="P79" s="9"/>
       <c r="Q79" s="7" t="s">
-        <v>575</v>
+        <v>585</v>
       </c>
       <c r="R79" s="7" t="s">
         <v>51</v>
@@ -8884,17 +9177,17 @@
         <v>53</v>
       </c>
       <c r="V79" s="7" t="s">
-        <v>576</v>
+        <v>586</v>
       </c>
       <c r="W79" s="7" t="s">
-        <v>577</v>
+        <v>587</v>
       </c>
       <c r="X79" s="7" t="s">
-        <v>578</v>
+        <v>588</v>
       </c>
       <c r="Y79" s="7"/>
       <c r="Z79" s="7">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="AA79" s="7"/>
       <c r="AB79" s="7" t="s">
@@ -8926,15 +9219,15 @@
         <v>100</v>
       </c>
       <c r="C80" s="3">
-        <v>2026062007</v>
+        <v>2026061986</v>
       </c>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
-      <c r="F80" s="3" t="s">
-        <v>579</v>
+      <c r="F80" s="3">
+        <v>2154</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="H80" s="3" t="s">
         <v>86</v>
@@ -8946,9 +9239,9 @@
       <c r="M80" s="4"/>
       <c r="N80" s="3"/>
       <c r="O80" s="4"/>
-      <c r="P80" s="4"/>
+      <c r="P80" s="10"/>
       <c r="Q80" s="3" t="s">
-        <v>581</v>
+        <v>590</v>
       </c>
       <c r="R80" s="3" t="s">
         <v>51</v>
@@ -8963,23 +9256,23 @@
         <v>53</v>
       </c>
       <c r="V80" s="3" t="s">
-        <v>582</v>
+        <v>591</v>
       </c>
       <c r="W80" s="3" t="s">
-        <v>583</v>
+        <v>592</v>
       </c>
       <c r="X80" s="3" t="s">
-        <v>584</v>
+        <v>593</v>
       </c>
       <c r="Y80" s="3"/>
       <c r="Z80" s="3">
-        <v>12.5</v>
+        <v>0.3</v>
       </c>
       <c r="AA80" s="3"/>
       <c r="AB80" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="AC80" s="4" t="s">
+      <c r="AC80" s="10" t="s">
         <v>111</v>
       </c>
       <c r="AD80" s="3" t="s">
@@ -8992,6 +9285,1257 @@
       <c r="AI80" s="3"/>
       <c r="AJ80" s="3"/>
       <c r="AK80" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="81" spans="1:37">
+      <c r="A81" s="7">
+        <v>79</v>
+      </c>
+      <c r="B81" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C81" s="7">
+        <v>2026062001</v>
+      </c>
+      <c r="D81" s="7"/>
+      <c r="E81" s="7"/>
+      <c r="F81" s="7">
+        <v>5245</v>
+      </c>
+      <c r="G81" s="7" t="s">
+        <v>594</v>
+      </c>
+      <c r="H81" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I81" s="7"/>
+      <c r="J81" s="7"/>
+      <c r="K81" s="7"/>
+      <c r="L81" s="7"/>
+      <c r="M81" s="8"/>
+      <c r="N81" s="7"/>
+      <c r="O81" s="8"/>
+      <c r="P81" s="9"/>
+      <c r="Q81" s="7" t="s">
+        <v>595</v>
+      </c>
+      <c r="R81" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S81" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T81" s="7">
+        <v>1</v>
+      </c>
+      <c r="U81" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V81" s="7" t="s">
+        <v>596</v>
+      </c>
+      <c r="W81" s="7" t="s">
+        <v>597</v>
+      </c>
+      <c r="X81" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="Y81" s="7"/>
+      <c r="Z81" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA81" s="7"/>
+      <c r="AB81" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC81" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD81" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE81" s="7"/>
+      <c r="AF81" s="7"/>
+      <c r="AG81" s="7"/>
+      <c r="AH81" s="7"/>
+      <c r="AI81" s="7"/>
+      <c r="AJ81" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK81" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="82" spans="1:37">
+      <c r="A82" s="3">
+        <v>80</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C82" s="3">
+        <v>2026062007</v>
+      </c>
+      <c r="D82" s="3"/>
+      <c r="E82" s="3"/>
+      <c r="F82" s="3" t="s">
+        <v>599</v>
+      </c>
+      <c r="G82" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="H82" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I82" s="3"/>
+      <c r="J82" s="3"/>
+      <c r="K82" s="3"/>
+      <c r="L82" s="3"/>
+      <c r="M82" s="4"/>
+      <c r="N82" s="3"/>
+      <c r="O82" s="4"/>
+      <c r="P82" s="10"/>
+      <c r="Q82" s="3" t="s">
+        <v>601</v>
+      </c>
+      <c r="R82" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S82" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T82" s="3">
+        <v>1</v>
+      </c>
+      <c r="U82" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V82" s="3" t="s">
+        <v>602</v>
+      </c>
+      <c r="W82" s="3" t="s">
+        <v>603</v>
+      </c>
+      <c r="X82" s="3" t="s">
+        <v>604</v>
+      </c>
+      <c r="Y82" s="3"/>
+      <c r="Z82" s="3">
+        <v>12.5</v>
+      </c>
+      <c r="AA82" s="3"/>
+      <c r="AB82" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC82" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD82" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE82" s="3"/>
+      <c r="AF82" s="3"/>
+      <c r="AG82" s="3"/>
+      <c r="AH82" s="3"/>
+      <c r="AI82" s="3"/>
+      <c r="AJ82" s="3"/>
+      <c r="AK82" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="83" spans="1:37">
+      <c r="A83" s="7">
+        <v>81</v>
+      </c>
+      <c r="B83" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C83" s="7">
+        <v>2026062020</v>
+      </c>
+      <c r="D83" s="7" t="s">
+        <v>605</v>
+      </c>
+      <c r="E83" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F83" s="7">
+        <v>5430</v>
+      </c>
+      <c r="G83" s="7" t="s">
+        <v>606</v>
+      </c>
+      <c r="H83" s="7" t="s">
+        <v>427</v>
+      </c>
+      <c r="I83" s="7" t="s">
+        <v>607</v>
+      </c>
+      <c r="J83" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="K83" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="L83" s="7" t="s">
+        <v>503</v>
+      </c>
+      <c r="M83" s="8" t="s">
+        <v>504</v>
+      </c>
+      <c r="N83" s="7" t="s">
+        <v>608</v>
+      </c>
+      <c r="O83" s="8" t="s">
+        <v>609</v>
+      </c>
+      <c r="P83" s="9" t="s">
+        <v>610</v>
+      </c>
+      <c r="Q83" s="7" t="s">
+        <v>611</v>
+      </c>
+      <c r="R83" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S83" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T83" s="7">
+        <v>1</v>
+      </c>
+      <c r="U83" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V83" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="W83" s="7" t="s">
+        <v>613</v>
+      </c>
+      <c r="X83" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="Y83" s="7" t="s">
+        <v>614</v>
+      </c>
+      <c r="Z83" s="7">
+        <v>1</v>
+      </c>
+      <c r="AA83" s="7"/>
+      <c r="AB83" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC83" s="9" t="s">
+        <v>615</v>
+      </c>
+      <c r="AD83" s="7"/>
+      <c r="AE83" s="7"/>
+      <c r="AF83" s="7"/>
+      <c r="AG83" s="7"/>
+      <c r="AH83" s="7"/>
+      <c r="AI83" s="7"/>
+      <c r="AJ83" s="7"/>
+      <c r="AK83" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="84" spans="1:37">
+      <c r="A84" s="3">
+        <v>82</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C84" s="3">
+        <v>2026062032</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>616</v>
+      </c>
+      <c r="E84" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F84" s="3">
+        <v>4035</v>
+      </c>
+      <c r="G84" s="3" t="s">
+        <v>617</v>
+      </c>
+      <c r="H84" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I84" s="3" t="s">
+        <v>618</v>
+      </c>
+      <c r="J84" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="K84" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L84" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="M84" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="N84" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="O84" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="P84" s="10" t="s">
+        <v>619</v>
+      </c>
+      <c r="Q84" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="R84" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S84" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T84" s="3">
+        <v>1</v>
+      </c>
+      <c r="U84" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V84" s="3" t="s">
+        <v>621</v>
+      </c>
+      <c r="W84" s="3" t="s">
+        <v>622</v>
+      </c>
+      <c r="X84" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="Y84" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="Z84" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA84" s="3"/>
+      <c r="AB84" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC84" s="10" t="s">
+        <v>624</v>
+      </c>
+      <c r="AD84" s="3"/>
+      <c r="AE84" s="3"/>
+      <c r="AF84" s="3"/>
+      <c r="AG84" s="3"/>
+      <c r="AH84" s="3"/>
+      <c r="AI84" s="3"/>
+      <c r="AJ84" s="3"/>
+      <c r="AK84" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="85" spans="1:37">
+      <c r="A85" s="7">
+        <v>83</v>
+      </c>
+      <c r="B85" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C85" s="7">
+        <v>2026062032</v>
+      </c>
+      <c r="D85" s="7" t="s">
+        <v>616</v>
+      </c>
+      <c r="E85" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F85" s="7">
+        <v>4035</v>
+      </c>
+      <c r="G85" s="7" t="s">
+        <v>617</v>
+      </c>
+      <c r="H85" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="I85" s="7" t="s">
+        <v>618</v>
+      </c>
+      <c r="J85" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="K85" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L85" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="M85" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="N85" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="O85" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="P85" s="9" t="s">
+        <v>619</v>
+      </c>
+      <c r="Q85" s="7" t="s">
+        <v>620</v>
+      </c>
+      <c r="R85" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S85" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T85" s="7">
+        <v>2</v>
+      </c>
+      <c r="U85" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V85" s="7" t="s">
+        <v>621</v>
+      </c>
+      <c r="W85" s="7" t="s">
+        <v>622</v>
+      </c>
+      <c r="X85" s="7" t="s">
+        <v>623</v>
+      </c>
+      <c r="Y85" s="7" t="s">
+        <v>614</v>
+      </c>
+      <c r="Z85" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA85" s="7"/>
+      <c r="AB85" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC85" s="9" t="s">
+        <v>624</v>
+      </c>
+      <c r="AD85" s="7"/>
+      <c r="AE85" s="7"/>
+      <c r="AF85" s="7"/>
+      <c r="AG85" s="7"/>
+      <c r="AH85" s="7"/>
+      <c r="AI85" s="7"/>
+      <c r="AJ85" s="7"/>
+      <c r="AK85" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="86" spans="1:37">
+      <c r="A86" s="3">
+        <v>84</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C86" s="3">
+        <v>2026062033</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="E86" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F86" s="3">
+        <v>4035</v>
+      </c>
+      <c r="G86" s="3" t="s">
+        <v>617</v>
+      </c>
+      <c r="H86" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I86" s="3" t="s">
+        <v>626</v>
+      </c>
+      <c r="J86" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="K86" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L86" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="M86" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="N86" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="O86" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="P86" s="10" t="s">
+        <v>627</v>
+      </c>
+      <c r="Q86" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="R86" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S86" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T86" s="3">
+        <v>1</v>
+      </c>
+      <c r="U86" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V86" s="3" t="s">
+        <v>628</v>
+      </c>
+      <c r="W86" s="3" t="s">
+        <v>622</v>
+      </c>
+      <c r="X86" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="Y86" s="3" t="s">
+        <v>614</v>
+      </c>
+      <c r="Z86" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA86" s="3"/>
+      <c r="AB86" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC86" s="10" t="s">
+        <v>629</v>
+      </c>
+      <c r="AD86" s="3"/>
+      <c r="AE86" s="3"/>
+      <c r="AF86" s="3"/>
+      <c r="AG86" s="3"/>
+      <c r="AH86" s="3"/>
+      <c r="AI86" s="3"/>
+      <c r="AJ86" s="3"/>
+      <c r="AK86" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="87" spans="1:37">
+      <c r="A87" s="7">
+        <v>85</v>
+      </c>
+      <c r="B87" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C87" s="7">
+        <v>2026062058</v>
+      </c>
+      <c r="D87" s="7"/>
+      <c r="E87" s="7"/>
+      <c r="F87" s="7">
+        <v>4586</v>
+      </c>
+      <c r="G87" s="7" t="s">
+        <v>630</v>
+      </c>
+      <c r="H87" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I87" s="7"/>
+      <c r="J87" s="7"/>
+      <c r="K87" s="7"/>
+      <c r="L87" s="7"/>
+      <c r="M87" s="8"/>
+      <c r="N87" s="7"/>
+      <c r="O87" s="8"/>
+      <c r="P87" s="9"/>
+      <c r="Q87" s="7" t="s">
+        <v>631</v>
+      </c>
+      <c r="R87" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S87" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T87" s="7">
+        <v>1</v>
+      </c>
+      <c r="U87" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V87" s="7" t="s">
+        <v>632</v>
+      </c>
+      <c r="W87" s="7" t="s">
+        <v>633</v>
+      </c>
+      <c r="X87" s="7" t="s">
+        <v>634</v>
+      </c>
+      <c r="Y87" s="7"/>
+      <c r="Z87" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA87" s="7"/>
+      <c r="AB87" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC87" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD87" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE87" s="7"/>
+      <c r="AF87" s="7"/>
+      <c r="AG87" s="7"/>
+      <c r="AH87" s="7"/>
+      <c r="AI87" s="7"/>
+      <c r="AJ87" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK87" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="88" spans="1:37">
+      <c r="A88" s="3">
+        <v>86</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C88" s="3">
+        <v>2026062063</v>
+      </c>
+      <c r="D88" s="3"/>
+      <c r="E88" s="3"/>
+      <c r="F88" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="G88" s="3" t="s">
+        <v>636</v>
+      </c>
+      <c r="H88" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I88" s="3"/>
+      <c r="J88" s="3"/>
+      <c r="K88" s="3"/>
+      <c r="L88" s="3"/>
+      <c r="M88" s="4"/>
+      <c r="N88" s="3"/>
+      <c r="O88" s="4"/>
+      <c r="P88" s="10"/>
+      <c r="Q88" s="3" t="s">
+        <v>637</v>
+      </c>
+      <c r="R88" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S88" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T88" s="3">
+        <v>1</v>
+      </c>
+      <c r="U88" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V88" s="3" t="s">
+        <v>638</v>
+      </c>
+      <c r="W88" s="3" t="s">
+        <v>639</v>
+      </c>
+      <c r="X88" s="3" t="s">
+        <v>640</v>
+      </c>
+      <c r="Y88" s="3"/>
+      <c r="Z88" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA88" s="3"/>
+      <c r="AB88" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC88" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD88" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE88" s="3"/>
+      <c r="AF88" s="3"/>
+      <c r="AG88" s="3"/>
+      <c r="AH88" s="3"/>
+      <c r="AI88" s="3"/>
+      <c r="AJ88" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK88" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="89" spans="1:37">
+      <c r="A89" s="7">
+        <v>87</v>
+      </c>
+      <c r="B89" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C89" s="7">
+        <v>2026062067</v>
+      </c>
+      <c r="D89" s="7"/>
+      <c r="E89" s="7"/>
+      <c r="F89" s="7">
+        <v>5430</v>
+      </c>
+      <c r="G89" s="7" t="s">
+        <v>606</v>
+      </c>
+      <c r="H89" s="7" t="s">
+        <v>427</v>
+      </c>
+      <c r="I89" s="7"/>
+      <c r="J89" s="7"/>
+      <c r="K89" s="7"/>
+      <c r="L89" s="7"/>
+      <c r="M89" s="8"/>
+      <c r="N89" s="7"/>
+      <c r="O89" s="8"/>
+      <c r="P89" s="9"/>
+      <c r="Q89" s="7" t="s">
+        <v>611</v>
+      </c>
+      <c r="R89" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S89" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T89" s="7">
+        <v>1</v>
+      </c>
+      <c r="U89" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V89" s="7" t="s">
+        <v>641</v>
+      </c>
+      <c r="W89" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="X89" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="Y89" s="7"/>
+      <c r="Z89" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA89" s="7"/>
+      <c r="AB89" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC89" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD89" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE89" s="7"/>
+      <c r="AF89" s="7"/>
+      <c r="AG89" s="7"/>
+      <c r="AH89" s="7"/>
+      <c r="AI89" s="7"/>
+      <c r="AJ89" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK89" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="90" spans="1:37">
+      <c r="A90" s="3">
+        <v>88</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C90" s="3">
+        <v>2026062072</v>
+      </c>
+      <c r="D90" s="3"/>
+      <c r="E90" s="3"/>
+      <c r="F90" s="3">
+        <v>5082</v>
+      </c>
+      <c r="G90" s="3" t="s">
+        <v>643</v>
+      </c>
+      <c r="H90" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="I90" s="3"/>
+      <c r="J90" s="3"/>
+      <c r="K90" s="3"/>
+      <c r="L90" s="3"/>
+      <c r="M90" s="4"/>
+      <c r="N90" s="3"/>
+      <c r="O90" s="4"/>
+      <c r="P90" s="10"/>
+      <c r="Q90" s="3" t="s">
+        <v>644</v>
+      </c>
+      <c r="R90" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S90" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T90" s="3">
+        <v>1</v>
+      </c>
+      <c r="U90" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V90" s="3" t="s">
+        <v>645</v>
+      </c>
+      <c r="W90" s="3" t="s">
+        <v>642</v>
+      </c>
+      <c r="X90" s="3" t="s">
+        <v>646</v>
+      </c>
+      <c r="Y90" s="3"/>
+      <c r="Z90" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA90" s="3"/>
+      <c r="AB90" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC90" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD90" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE90" s="3"/>
+      <c r="AF90" s="3"/>
+      <c r="AG90" s="3"/>
+      <c r="AH90" s="3"/>
+      <c r="AI90" s="3"/>
+      <c r="AJ90" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK90" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="91" spans="1:37">
+      <c r="A91" s="7">
+        <v>89</v>
+      </c>
+      <c r="B91" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C91" s="7">
+        <v>2026062076</v>
+      </c>
+      <c r="D91" s="7"/>
+      <c r="E91" s="7"/>
+      <c r="F91" s="7">
+        <v>5352</v>
+      </c>
+      <c r="G91" s="7" t="s">
+        <v>647</v>
+      </c>
+      <c r="H91" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I91" s="7"/>
+      <c r="J91" s="7"/>
+      <c r="K91" s="7"/>
+      <c r="L91" s="7"/>
+      <c r="M91" s="8"/>
+      <c r="N91" s="7"/>
+      <c r="O91" s="8"/>
+      <c r="P91" s="9"/>
+      <c r="Q91" s="7" t="s">
+        <v>648</v>
+      </c>
+      <c r="R91" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S91" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T91" s="7">
+        <v>1</v>
+      </c>
+      <c r="U91" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V91" s="7" t="s">
+        <v>649</v>
+      </c>
+      <c r="W91" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="X91" s="7" t="s">
+        <v>651</v>
+      </c>
+      <c r="Y91" s="7"/>
+      <c r="Z91" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA91" s="7"/>
+      <c r="AB91" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC91" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD91" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE91" s="7"/>
+      <c r="AF91" s="7"/>
+      <c r="AG91" s="7"/>
+      <c r="AH91" s="7"/>
+      <c r="AI91" s="7"/>
+      <c r="AJ91" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK91" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="92" spans="1:37">
+      <c r="A92" s="3">
+        <v>90</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C92" s="3">
+        <v>2026062082</v>
+      </c>
+      <c r="D92" s="3"/>
+      <c r="E92" s="3"/>
+      <c r="F92" s="3">
+        <v>3623</v>
+      </c>
+      <c r="G92" s="3" t="s">
+        <v>652</v>
+      </c>
+      <c r="H92" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I92" s="3"/>
+      <c r="J92" s="3"/>
+      <c r="K92" s="3"/>
+      <c r="L92" s="3"/>
+      <c r="M92" s="4"/>
+      <c r="N92" s="3"/>
+      <c r="O92" s="4"/>
+      <c r="P92" s="10"/>
+      <c r="Q92" s="3" t="s">
+        <v>653</v>
+      </c>
+      <c r="R92" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S92" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T92" s="3">
+        <v>1</v>
+      </c>
+      <c r="U92" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V92" s="3" t="s">
+        <v>654</v>
+      </c>
+      <c r="W92" s="3" t="s">
+        <v>646</v>
+      </c>
+      <c r="X92" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="Y92" s="3"/>
+      <c r="Z92" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA92" s="3"/>
+      <c r="AB92" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC92" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD92" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE92" s="3"/>
+      <c r="AF92" s="3"/>
+      <c r="AG92" s="3"/>
+      <c r="AH92" s="3"/>
+      <c r="AI92" s="3"/>
+      <c r="AJ92" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK92" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="93" spans="1:37">
+      <c r="A93" s="7">
+        <v>91</v>
+      </c>
+      <c r="B93" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C93" s="7">
+        <v>2026062105</v>
+      </c>
+      <c r="D93" s="7"/>
+      <c r="E93" s="7"/>
+      <c r="F93" s="7">
+        <v>5341</v>
+      </c>
+      <c r="G93" s="7" t="s">
+        <v>426</v>
+      </c>
+      <c r="H93" s="7" t="s">
+        <v>427</v>
+      </c>
+      <c r="I93" s="7"/>
+      <c r="J93" s="7"/>
+      <c r="K93" s="7"/>
+      <c r="L93" s="7"/>
+      <c r="M93" s="8"/>
+      <c r="N93" s="7"/>
+      <c r="O93" s="8"/>
+      <c r="P93" s="9"/>
+      <c r="Q93" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="R93" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S93" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T93" s="7">
+        <v>1</v>
+      </c>
+      <c r="U93" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V93" s="7" t="s">
+        <v>656</v>
+      </c>
+      <c r="W93" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="X93" s="7" t="s">
+        <v>657</v>
+      </c>
+      <c r="Y93" s="7"/>
+      <c r="Z93" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA93" s="7"/>
+      <c r="AB93" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC93" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD93" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE93" s="7"/>
+      <c r="AF93" s="7"/>
+      <c r="AG93" s="7"/>
+      <c r="AH93" s="7"/>
+      <c r="AI93" s="7"/>
+      <c r="AJ93" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK93" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="94" spans="1:37">
+      <c r="A94" s="3">
+        <v>92</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C94" s="3">
+        <v>2026062115</v>
+      </c>
+      <c r="D94" s="3"/>
+      <c r="E94" s="3"/>
+      <c r="F94" s="3" t="s">
+        <v>658</v>
+      </c>
+      <c r="G94" s="3" t="s">
+        <v>659</v>
+      </c>
+      <c r="H94" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="I94" s="3"/>
+      <c r="J94" s="3"/>
+      <c r="K94" s="3"/>
+      <c r="L94" s="3"/>
+      <c r="M94" s="4"/>
+      <c r="N94" s="3"/>
+      <c r="O94" s="4"/>
+      <c r="P94" s="10"/>
+      <c r="Q94" s="3" t="s">
+        <v>660</v>
+      </c>
+      <c r="R94" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S94" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T94" s="3">
+        <v>1</v>
+      </c>
+      <c r="U94" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V94" s="3" t="s">
+        <v>661</v>
+      </c>
+      <c r="W94" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="X94" s="3" t="s">
+        <v>662</v>
+      </c>
+      <c r="Y94" s="3"/>
+      <c r="Z94" s="3">
+        <v>0.7</v>
+      </c>
+      <c r="AA94" s="3"/>
+      <c r="AB94" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC94" s="10" t="s">
+        <v>663</v>
+      </c>
+      <c r="AD94" s="3"/>
+      <c r="AE94" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF94" s="3"/>
+      <c r="AG94" s="3"/>
+      <c r="AH94" s="3"/>
+      <c r="AI94" s="3"/>
+      <c r="AJ94" s="3"/>
+      <c r="AK94" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="95" spans="1:37">
+      <c r="A95" s="7">
+        <v>93</v>
+      </c>
+      <c r="B95" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C95" s="7">
+        <v>2026062119</v>
+      </c>
+      <c r="D95" s="7"/>
+      <c r="E95" s="7"/>
+      <c r="F95" s="7" t="s">
+        <v>658</v>
+      </c>
+      <c r="G95" s="7" t="s">
+        <v>659</v>
+      </c>
+      <c r="H95" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="I95" s="7"/>
+      <c r="J95" s="7"/>
+      <c r="K95" s="7"/>
+      <c r="L95" s="7"/>
+      <c r="M95" s="8"/>
+      <c r="N95" s="7"/>
+      <c r="O95" s="8"/>
+      <c r="P95" s="8"/>
+      <c r="Q95" s="7" t="s">
+        <v>660</v>
+      </c>
+      <c r="R95" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S95" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T95" s="7">
+        <v>1</v>
+      </c>
+      <c r="U95" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V95" s="7" t="s">
+        <v>664</v>
+      </c>
+      <c r="W95" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="X95" s="7" t="s">
+        <v>665</v>
+      </c>
+      <c r="Y95" s="7"/>
+      <c r="Z95" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="AA95" s="7"/>
+      <c r="AB95" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC95" s="8" t="s">
+        <v>666</v>
+      </c>
+      <c r="AD95" s="7"/>
+      <c r="AE95" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF95" s="7"/>
+      <c r="AG95" s="7"/>
+      <c r="AH95" s="7"/>
+      <c r="AI95" s="7"/>
+      <c r="AJ95" s="7"/>
+      <c r="AK95" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06181718
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$116</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$121</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="803">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-17  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="836">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-18  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -2357,9 +2357,6 @@
     <t>THILF03941</t>
   </si>
   <si>
-    <t>未完工</t>
-  </si>
-  <si>
     <t>2026-06-16 17:51:19</t>
   </si>
   <si>
@@ -2381,6 +2378,18 @@
     <t>2026-06-17 12:38:00</t>
   </si>
   <si>
+    <t>2026-06-18 09:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-18 15:28:00</t>
+  </si>
+  <si>
+    <t>17小時37分鐘</t>
+  </si>
+  <si>
+    <t>更換一二顆硬碟不備份還原.已跟店長告知回報代收會計</t>
+  </si>
+  <si>
     <t>13606115061701</t>
   </si>
   <si>
@@ -2484,6 +2493,98 @@
   </si>
   <si>
     <t>2026-06-17 14:50:00</t>
+  </si>
+  <si>
+    <t>12222115061701</t>
+  </si>
+  <si>
+    <t>三重義天店</t>
+  </si>
+  <si>
+    <t>2026-06-17 19:47:00</t>
+  </si>
+  <si>
+    <t>HL58</t>
+  </si>
+  <si>
+    <t>HL-LIFE-ET主機</t>
+  </si>
+  <si>
+    <t>門市反應MMK四代機無法連線，有跳出小視窗，門市依序點選1.重新設定&gt;2.偵測網路後顯示網路異常，重新開機後仍無法連線，ping60不通、與門市確認MMK後方網路線無鬆脫，查看HUB孔位燈號正常、重新插拔7PORT仍無法連線...需請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF02222</t>
+  </si>
+  <si>
+    <t>2026-06-17 19:50:54</t>
+  </si>
+  <si>
+    <t>2026-06-18 16:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-18 16:24:00</t>
+  </si>
+  <si>
+    <t>2026-06-18 23:50:00</t>
+  </si>
+  <si>
+    <t>重新插拔網路線重新偵測</t>
+  </si>
+  <si>
+    <t>龜山茶專店</t>
+  </si>
+  <si>
+    <t>THILF05162</t>
+  </si>
+  <si>
+    <t>2026-06-18 11:03:34</t>
+  </si>
+  <si>
+    <t>2026-06-18 10:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-18 11:00:00</t>
+  </si>
+  <si>
+    <t>協助撤店</t>
+  </si>
+  <si>
+    <t>2026-06-18 11:05:44</t>
+  </si>
+  <si>
+    <t>2026-06-18 11:04:00</t>
+  </si>
+  <si>
+    <t>撤店完成</t>
+  </si>
+  <si>
+    <t>E4856115061801</t>
+  </si>
+  <si>
+    <t>新莊小胖店</t>
+  </si>
+  <si>
+    <t>2026-06-18 14:12:38</t>
+  </si>
+  <si>
+    <t>門市反應tm2收銀機(TCX800)(抽屜顏色:米白色、鑰匙孔位子(中)、鎖頭編號:5001)鑰匙可以插進去但無法轉動....需請台芝到店協助(機台二抽屜使用鑰匙後無法正常彈開)</t>
+  </si>
+  <si>
+    <t>THILF04856</t>
+  </si>
+  <si>
+    <t>2026-06-18 14:16:58</t>
+  </si>
+  <si>
+    <t>2026-06-18 15:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-22 18:16:00</t>
+  </si>
+  <si>
+    <t>更換錢箱
+換上81Z1004771
+換下81Z1001056</t>
   </si>
 </sst>
 </file>
@@ -2897,7 +2998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK116"/>
+  <dimension ref="A1:AK121"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -12149,19 +12250,19 @@
         <v>1</v>
       </c>
       <c r="U109" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V109" s="7" t="s">
         <v>760</v>
       </c>
-      <c r="V109" s="7" t="s">
+      <c r="W109" s="7" t="s">
         <v>761</v>
       </c>
-      <c r="W109" s="7" t="s">
+      <c r="X109" s="7" t="s">
         <v>762</v>
       </c>
-      <c r="X109" s="7" t="s">
+      <c r="Y109" s="7" t="s">
         <v>763</v>
-      </c>
-      <c r="Y109" s="7" t="s">
-        <v>764</v>
       </c>
       <c r="Z109" s="7">
         <v>0.5</v>
@@ -12171,7 +12272,7 @@
         <v>58</v>
       </c>
       <c r="AC109" s="9" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="AD109" s="7"/>
       <c r="AE109" s="7"/>
@@ -12246,19 +12347,19 @@
         <v>2</v>
       </c>
       <c r="U110" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V110" s="3" t="s">
         <v>760</v>
       </c>
-      <c r="V110" s="3" t="s">
-        <v>761</v>
-      </c>
       <c r="W110" s="3" t="s">
+        <v>765</v>
+      </c>
+      <c r="X110" s="3" t="s">
         <v>766</v>
       </c>
-      <c r="X110" s="3" t="s">
-        <v>767</v>
-      </c>
       <c r="Y110" s="3" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="Z110" s="3">
         <v>0.5</v>
@@ -12268,7 +12369,7 @@
         <v>58</v>
       </c>
       <c r="AC110" s="10" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="AD110" s="3"/>
       <c r="AE110" s="3"/>
@@ -12289,83 +12390,85 @@
         <v>38</v>
       </c>
       <c r="C111" s="7">
-        <v>2026062263</v>
+        <v>2026062256</v>
       </c>
       <c r="D111" s="7" t="s">
-        <v>768</v>
+        <v>754</v>
       </c>
       <c r="E111" s="7" t="s">
         <v>40</v>
       </c>
       <c r="F111" s="7">
-        <v>3606</v>
+        <v>3941</v>
       </c>
       <c r="G111" s="7" t="s">
-        <v>769</v>
+        <v>755</v>
       </c>
       <c r="H111" s="7" t="s">
-        <v>770</v>
+        <v>756</v>
       </c>
       <c r="I111" s="7" t="s">
-        <v>771</v>
+        <v>757</v>
       </c>
       <c r="J111" s="7" t="s">
-        <v>141</v>
+        <v>376</v>
       </c>
       <c r="K111" s="7" t="s">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="L111" s="7" t="s">
-        <v>46</v>
+        <v>142</v>
       </c>
       <c r="M111" s="8" t="s">
-        <v>47</v>
+        <v>143</v>
       </c>
       <c r="N111" s="7">
-        <v>2307</v>
+        <v>2405</v>
       </c>
       <c r="O111" s="8" t="s">
-        <v>48</v>
+        <v>267</v>
       </c>
       <c r="P111" s="9" t="s">
-        <v>772</v>
+        <v>758</v>
       </c>
       <c r="Q111" s="7" t="s">
-        <v>773</v>
+        <v>759</v>
       </c>
       <c r="R111" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S111" s="7" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="T111" s="7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U111" s="7" t="s">
         <v>53</v>
       </c>
       <c r="V111" s="7" t="s">
-        <v>774</v>
+        <v>760</v>
       </c>
       <c r="W111" s="7" t="s">
-        <v>775</v>
+        <v>767</v>
       </c>
       <c r="X111" s="7" t="s">
-        <v>776</v>
+        <v>768</v>
       </c>
       <c r="Y111" s="7" t="s">
-        <v>777</v>
+        <v>763</v>
       </c>
       <c r="Z111" s="7">
-        <v>1</v>
-      </c>
-      <c r="AA111" s="7"/>
+        <v>6.5</v>
+      </c>
+      <c r="AA111" s="7" t="s">
+        <v>769</v>
+      </c>
       <c r="AB111" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC111" s="9" t="s">
-        <v>778</v>
+        <v>770</v>
       </c>
       <c r="AD111" s="7"/>
       <c r="AE111" s="7"/>
@@ -12383,32 +12486,52 @@
         <v>110</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C112" s="3">
-        <v>2026062310</v>
-      </c>
-      <c r="D112" s="3"/>
-      <c r="E112" s="3"/>
-      <c r="F112" s="3" t="s">
-        <v>779</v>
+        <v>2026062263</v>
+      </c>
+      <c r="D112" s="3" t="s">
+        <v>771</v>
+      </c>
+      <c r="E112" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F112" s="3">
+        <v>3606</v>
       </c>
       <c r="G112" s="3" t="s">
-        <v>780</v>
+        <v>772</v>
       </c>
       <c r="H112" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="I112" s="3"/>
-      <c r="J112" s="3"/>
-      <c r="K112" s="3"/>
-      <c r="L112" s="3"/>
-      <c r="M112" s="4"/>
-      <c r="N112" s="3"/>
-      <c r="O112" s="4"/>
-      <c r="P112" s="10"/>
+        <v>773</v>
+      </c>
+      <c r="I112" s="3" t="s">
+        <v>774</v>
+      </c>
+      <c r="J112" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="K112" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L112" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M112" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="N112" s="3">
+        <v>2307</v>
+      </c>
+      <c r="O112" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="P112" s="10" t="s">
+        <v>775</v>
+      </c>
       <c r="Q112" s="3" t="s">
-        <v>781</v>
+        <v>776</v>
       </c>
       <c r="R112" s="3" t="s">
         <v>51</v>
@@ -12423,28 +12546,28 @@
         <v>53</v>
       </c>
       <c r="V112" s="3" t="s">
-        <v>782</v>
+        <v>777</v>
       </c>
       <c r="W112" s="3" t="s">
-        <v>783</v>
+        <v>778</v>
       </c>
       <c r="X112" s="3" t="s">
-        <v>784</v>
-      </c>
-      <c r="Y112" s="3"/>
+        <v>779</v>
+      </c>
+      <c r="Y112" s="3" t="s">
+        <v>780</v>
+      </c>
       <c r="Z112" s="3">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="AA112" s="3"/>
       <c r="AB112" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC112" s="10" t="s">
-        <v>476</v>
-      </c>
-      <c r="AD112" s="3" t="s">
-        <v>60</v>
-      </c>
+        <v>781</v>
+      </c>
+      <c r="AD112" s="3"/>
       <c r="AE112" s="3"/>
       <c r="AF112" s="3"/>
       <c r="AG112" s="3"/>
@@ -12463,15 +12586,15 @@
         <v>100</v>
       </c>
       <c r="C113" s="7">
-        <v>2026062311</v>
+        <v>2026062310</v>
       </c>
       <c r="D113" s="7"/>
       <c r="E113" s="7"/>
-      <c r="F113" s="7">
-        <v>5496</v>
+      <c r="F113" s="7" t="s">
+        <v>782</v>
       </c>
       <c r="G113" s="7" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="H113" s="7" t="s">
         <v>86</v>
@@ -12485,7 +12608,7 @@
       <c r="O113" s="8"/>
       <c r="P113" s="9"/>
       <c r="Q113" s="7" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
       <c r="R113" s="7" t="s">
         <v>51</v>
@@ -12500,24 +12623,24 @@
         <v>53</v>
       </c>
       <c r="V113" s="7" t="s">
+        <v>785</v>
+      </c>
+      <c r="W113" s="7" t="s">
+        <v>786</v>
+      </c>
+      <c r="X113" s="7" t="s">
         <v>787</v>
-      </c>
-      <c r="W113" s="7" t="s">
-        <v>788</v>
-      </c>
-      <c r="X113" s="7" t="s">
-        <v>789</v>
       </c>
       <c r="Y113" s="7"/>
       <c r="Z113" s="7">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="AA113" s="7"/>
       <c r="AB113" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC113" s="9" t="s">
-        <v>157</v>
+        <v>476</v>
       </c>
       <c r="AD113" s="7" t="s">
         <v>60</v>
@@ -12540,15 +12663,15 @@
         <v>100</v>
       </c>
       <c r="C114" s="3">
-        <v>2026062314</v>
+        <v>2026062311</v>
       </c>
       <c r="D114" s="3"/>
       <c r="E114" s="3"/>
-      <c r="F114" s="3" t="s">
-        <v>297</v>
+      <c r="F114" s="3">
+        <v>5496</v>
       </c>
       <c r="G114" s="3" t="s">
-        <v>298</v>
+        <v>788</v>
       </c>
       <c r="H114" s="3" t="s">
         <v>86</v>
@@ -12562,7 +12685,7 @@
       <c r="O114" s="4"/>
       <c r="P114" s="10"/>
       <c r="Q114" s="3" t="s">
-        <v>304</v>
+        <v>789</v>
       </c>
       <c r="R114" s="3" t="s">
         <v>51</v>
@@ -12587,7 +12710,7 @@
       </c>
       <c r="Y114" s="3"/>
       <c r="Z114" s="3">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="AA114" s="3"/>
       <c r="AB114" s="3" t="s">
@@ -12617,15 +12740,15 @@
         <v>100</v>
       </c>
       <c r="C115" s="7">
-        <v>2026062317</v>
+        <v>2026062314</v>
       </c>
       <c r="D115" s="7"/>
       <c r="E115" s="7"/>
-      <c r="F115" s="7">
-        <v>2995</v>
+      <c r="F115" s="7" t="s">
+        <v>297</v>
       </c>
       <c r="G115" s="7" t="s">
-        <v>793</v>
+        <v>298</v>
       </c>
       <c r="H115" s="7" t="s">
         <v>86</v>
@@ -12639,7 +12762,7 @@
       <c r="O115" s="8"/>
       <c r="P115" s="9"/>
       <c r="Q115" s="7" t="s">
-        <v>794</v>
+        <v>304</v>
       </c>
       <c r="R115" s="7" t="s">
         <v>51</v>
@@ -12654,24 +12777,24 @@
         <v>53</v>
       </c>
       <c r="V115" s="7" t="s">
+        <v>793</v>
+      </c>
+      <c r="W115" s="7" t="s">
+        <v>794</v>
+      </c>
+      <c r="X115" s="7" t="s">
         <v>795</v>
-      </c>
-      <c r="W115" s="7" t="s">
-        <v>796</v>
-      </c>
-      <c r="X115" s="7" t="s">
-        <v>797</v>
       </c>
       <c r="Y115" s="7"/>
       <c r="Z115" s="7">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="AA115" s="7"/>
       <c r="AB115" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC115" s="9" t="s">
-        <v>111</v>
+        <v>157</v>
       </c>
       <c r="AD115" s="7" t="s">
         <v>60</v>
@@ -12694,15 +12817,15 @@
         <v>100</v>
       </c>
       <c r="C116" s="3">
-        <v>2026062318</v>
+        <v>2026062317</v>
       </c>
       <c r="D116" s="3"/>
       <c r="E116" s="3"/>
       <c r="F116" s="3">
-        <v>2422</v>
+        <v>2995</v>
       </c>
       <c r="G116" s="3" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="H116" s="3" t="s">
         <v>86</v>
@@ -12714,9 +12837,9 @@
       <c r="M116" s="4"/>
       <c r="N116" s="3"/>
       <c r="O116" s="4"/>
-      <c r="P116" s="4"/>
+      <c r="P116" s="10"/>
       <c r="Q116" s="3" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
       <c r="R116" s="3" t="s">
         <v>51</v>
@@ -12731,23 +12854,23 @@
         <v>53</v>
       </c>
       <c r="V116" s="3" t="s">
+        <v>798</v>
+      </c>
+      <c r="W116" s="3" t="s">
+        <v>799</v>
+      </c>
+      <c r="X116" s="3" t="s">
         <v>800</v>
-      </c>
-      <c r="W116" s="3" t="s">
-        <v>801</v>
-      </c>
-      <c r="X116" s="3" t="s">
-        <v>802</v>
       </c>
       <c r="Y116" s="3"/>
       <c r="Z116" s="3">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="AA116" s="3"/>
       <c r="AB116" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="AC116" s="4" t="s">
+      <c r="AC116" s="10" t="s">
         <v>111</v>
       </c>
       <c r="AD116" s="3" t="s">
@@ -12760,6 +12883,431 @@
       <c r="AI116" s="3"/>
       <c r="AJ116" s="3"/>
       <c r="AK116" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="117" spans="1:37">
+      <c r="A117" s="7">
+        <v>115</v>
+      </c>
+      <c r="B117" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C117" s="7">
+        <v>2026062318</v>
+      </c>
+      <c r="D117" s="7"/>
+      <c r="E117" s="7"/>
+      <c r="F117" s="7">
+        <v>2422</v>
+      </c>
+      <c r="G117" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="H117" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I117" s="7"/>
+      <c r="J117" s="7"/>
+      <c r="K117" s="7"/>
+      <c r="L117" s="7"/>
+      <c r="M117" s="8"/>
+      <c r="N117" s="7"/>
+      <c r="O117" s="8"/>
+      <c r="P117" s="9"/>
+      <c r="Q117" s="7" t="s">
+        <v>802</v>
+      </c>
+      <c r="R117" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S117" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T117" s="7">
+        <v>1</v>
+      </c>
+      <c r="U117" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V117" s="7" t="s">
+        <v>803</v>
+      </c>
+      <c r="W117" s="7" t="s">
+        <v>804</v>
+      </c>
+      <c r="X117" s="7" t="s">
+        <v>805</v>
+      </c>
+      <c r="Y117" s="7"/>
+      <c r="Z117" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA117" s="7"/>
+      <c r="AB117" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC117" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD117" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE117" s="7"/>
+      <c r="AF117" s="7"/>
+      <c r="AG117" s="7"/>
+      <c r="AH117" s="7"/>
+      <c r="AI117" s="7"/>
+      <c r="AJ117" s="7"/>
+      <c r="AK117" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="118" spans="1:37">
+      <c r="A118" s="3">
+        <v>116</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C118" s="3">
+        <v>2026062346</v>
+      </c>
+      <c r="D118" s="3" t="s">
+        <v>806</v>
+      </c>
+      <c r="E118" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F118" s="3">
+        <v>2222</v>
+      </c>
+      <c r="G118" s="3" t="s">
+        <v>807</v>
+      </c>
+      <c r="H118" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I118" s="3" t="s">
+        <v>808</v>
+      </c>
+      <c r="J118" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="K118" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="L118" s="3" t="s">
+        <v>809</v>
+      </c>
+      <c r="M118" s="4" t="s">
+        <v>810</v>
+      </c>
+      <c r="N118" s="3">
+        <v>5804</v>
+      </c>
+      <c r="O118" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="P118" s="10" t="s">
+        <v>811</v>
+      </c>
+      <c r="Q118" s="3" t="s">
+        <v>812</v>
+      </c>
+      <c r="R118" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S118" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T118" s="3">
+        <v>1</v>
+      </c>
+      <c r="U118" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V118" s="3" t="s">
+        <v>813</v>
+      </c>
+      <c r="W118" s="3" t="s">
+        <v>814</v>
+      </c>
+      <c r="X118" s="3" t="s">
+        <v>815</v>
+      </c>
+      <c r="Y118" s="3" t="s">
+        <v>816</v>
+      </c>
+      <c r="Z118" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA118" s="3"/>
+      <c r="AB118" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC118" s="10" t="s">
+        <v>817</v>
+      </c>
+      <c r="AD118" s="3"/>
+      <c r="AE118" s="3"/>
+      <c r="AF118" s="3"/>
+      <c r="AG118" s="3"/>
+      <c r="AH118" s="3"/>
+      <c r="AI118" s="3"/>
+      <c r="AJ118" s="3"/>
+      <c r="AK118" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="119" spans="1:37">
+      <c r="A119" s="7">
+        <v>117</v>
+      </c>
+      <c r="B119" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C119" s="7">
+        <v>2026062387</v>
+      </c>
+      <c r="D119" s="7"/>
+      <c r="E119" s="7"/>
+      <c r="F119" s="7">
+        <v>5162</v>
+      </c>
+      <c r="G119" s="7" t="s">
+        <v>818</v>
+      </c>
+      <c r="H119" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="I119" s="7"/>
+      <c r="J119" s="7"/>
+      <c r="K119" s="7"/>
+      <c r="L119" s="7"/>
+      <c r="M119" s="8"/>
+      <c r="N119" s="7"/>
+      <c r="O119" s="8"/>
+      <c r="P119" s="9"/>
+      <c r="Q119" s="7" t="s">
+        <v>819</v>
+      </c>
+      <c r="R119" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S119" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T119" s="7">
+        <v>1</v>
+      </c>
+      <c r="U119" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V119" s="7" t="s">
+        <v>820</v>
+      </c>
+      <c r="W119" s="7" t="s">
+        <v>821</v>
+      </c>
+      <c r="X119" s="7" t="s">
+        <v>822</v>
+      </c>
+      <c r="Y119" s="7"/>
+      <c r="Z119" s="7">
+        <v>1</v>
+      </c>
+      <c r="AA119" s="7"/>
+      <c r="AB119" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC119" s="9" t="s">
+        <v>823</v>
+      </c>
+      <c r="AD119" s="7"/>
+      <c r="AE119" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF119" s="7"/>
+      <c r="AG119" s="7"/>
+      <c r="AH119" s="7"/>
+      <c r="AI119" s="7"/>
+      <c r="AJ119" s="7"/>
+      <c r="AK119" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="120" spans="1:37">
+      <c r="A120" s="3">
+        <v>118</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C120" s="3">
+        <v>2026062388</v>
+      </c>
+      <c r="D120" s="3"/>
+      <c r="E120" s="3"/>
+      <c r="F120" s="3">
+        <v>5162</v>
+      </c>
+      <c r="G120" s="3" t="s">
+        <v>818</v>
+      </c>
+      <c r="H120" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I120" s="3"/>
+      <c r="J120" s="3"/>
+      <c r="K120" s="3"/>
+      <c r="L120" s="3"/>
+      <c r="M120" s="4"/>
+      <c r="N120" s="3"/>
+      <c r="O120" s="4"/>
+      <c r="P120" s="10"/>
+      <c r="Q120" s="3" t="s">
+        <v>819</v>
+      </c>
+      <c r="R120" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S120" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T120" s="3">
+        <v>1</v>
+      </c>
+      <c r="U120" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V120" s="3" t="s">
+        <v>824</v>
+      </c>
+      <c r="W120" s="3" t="s">
+        <v>821</v>
+      </c>
+      <c r="X120" s="3" t="s">
+        <v>825</v>
+      </c>
+      <c r="Y120" s="3"/>
+      <c r="Z120" s="3">
+        <v>1.1</v>
+      </c>
+      <c r="AA120" s="3"/>
+      <c r="AB120" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC120" s="10" t="s">
+        <v>826</v>
+      </c>
+      <c r="AD120" s="3"/>
+      <c r="AE120" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF120" s="3"/>
+      <c r="AG120" s="3"/>
+      <c r="AH120" s="3"/>
+      <c r="AI120" s="3"/>
+      <c r="AJ120" s="3"/>
+      <c r="AK120" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="121" spans="1:37">
+      <c r="A121" s="7">
+        <v>119</v>
+      </c>
+      <c r="B121" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C121" s="7">
+        <v>2026062443</v>
+      </c>
+      <c r="D121" s="7" t="s">
+        <v>827</v>
+      </c>
+      <c r="E121" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F121" s="7">
+        <v>4856</v>
+      </c>
+      <c r="G121" s="7" t="s">
+        <v>828</v>
+      </c>
+      <c r="H121" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="I121" s="7" t="s">
+        <v>829</v>
+      </c>
+      <c r="J121" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="K121" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L121" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M121" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="N121" s="7">
+        <v>2305</v>
+      </c>
+      <c r="O121" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="P121" s="8" t="s">
+        <v>830</v>
+      </c>
+      <c r="Q121" s="7" t="s">
+        <v>831</v>
+      </c>
+      <c r="R121" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S121" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T121" s="7">
+        <v>1</v>
+      </c>
+      <c r="U121" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V121" s="7" t="s">
+        <v>832</v>
+      </c>
+      <c r="W121" s="7" t="s">
+        <v>833</v>
+      </c>
+      <c r="X121" s="7" t="s">
+        <v>814</v>
+      </c>
+      <c r="Y121" s="7" t="s">
+        <v>834</v>
+      </c>
+      <c r="Z121" s="7">
+        <v>1</v>
+      </c>
+      <c r="AA121" s="7"/>
+      <c r="AB121" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC121" s="8" t="s">
+        <v>835</v>
+      </c>
+      <c r="AD121" s="7"/>
+      <c r="AE121" s="7"/>
+      <c r="AF121" s="7"/>
+      <c r="AG121" s="7"/>
+      <c r="AH121" s="7"/>
+      <c r="AI121" s="7"/>
+      <c r="AJ121" s="7"/>
+      <c r="AK121" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06231719
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$121</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$144</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="836">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-18  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1009">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-23  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -2585,6 +2585,535 @@
     <t>更換錢箱
 換上81Z1004771
 換下81Z1001056</t>
+  </si>
+  <si>
+    <t>永和樂華夜市</t>
+  </si>
+  <si>
+    <t>THILF02380</t>
+  </si>
+  <si>
+    <t>2026-06-18 21:27:53</t>
+  </si>
+  <si>
+    <t>2026-06-18 17:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-18 21:00:00</t>
+  </si>
+  <si>
+    <t>E3458115061901</t>
+  </si>
+  <si>
+    <t>八里龍米店</t>
+  </si>
+  <si>
+    <t>2026-06-19 09:50:42</t>
+  </si>
+  <si>
+    <t>門市反應tm2 ccd掃描器(HC56II-TR)刷讀所有條碼都很難刷，已有執行校正仍異常....請台芝到店協助(很難刷 又刷不進去 機台2的手握掃描器)</t>
+  </si>
+  <si>
+    <t>THILF03458</t>
+  </si>
+  <si>
+    <t>2026-06-19 09:59:11</t>
+  </si>
+  <si>
+    <t>2026-06-22 14:37:00</t>
+  </si>
+  <si>
+    <t>2026-06-22 15:10:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 13:00:00</t>
+  </si>
+  <si>
+    <t>更換掃描槍
+換下8119006826
+換上8119011356</t>
+  </si>
+  <si>
+    <t>E2380115062001</t>
+  </si>
+  <si>
+    <t>2026-06-20 12:44:29</t>
+  </si>
+  <si>
+    <t>門市6/18專案更換SC主機，更換主機後舊鍵盤無法使用於新主機，工程師有借用一個鍵盤在門市，並請門市在叫修....須請台芝協助(...)</t>
+  </si>
+  <si>
+    <t>2026-06-20 12:52:39</t>
+  </si>
+  <si>
+    <t>2026-06-22 10:50:00</t>
+  </si>
+  <si>
+    <t>2026-06-22 11:10:00</t>
+  </si>
+  <si>
+    <t>更換鍵盤</t>
+  </si>
+  <si>
+    <t>ED620115062101</t>
+  </si>
+  <si>
+    <t>D620</t>
+  </si>
+  <si>
+    <t>三重福隆店</t>
+  </si>
+  <si>
+    <t>2026-06-21 09:32:19</t>
+  </si>
+  <si>
+    <t>HL25</t>
+  </si>
+  <si>
+    <t>HL-SC螢幕</t>
+  </si>
+  <si>
+    <t>螢幕畫面閃爍頻繁或無畫面</t>
+  </si>
+  <si>
+    <t>門市反應SC螢幕(LCD)有許多小線條，PING1通VNC畫面正常，請門市重新拔插後方線路仍異常..請台芝到店協助(螢幕一直出現橫條一開始一小條，現在已經快半個畫面了)
+06/21  09:21  請門市拔插線路，稍晚聯繫...廖</t>
+  </si>
+  <si>
+    <t>THILF0D620</t>
+  </si>
+  <si>
+    <t>2026-06-21 10:11:41</t>
+  </si>
+  <si>
+    <t>2026-06-22 12:40:00</t>
+  </si>
+  <si>
+    <t>2026-06-22 12:55:00</t>
+  </si>
+  <si>
+    <t>換下8133000526.換上8133003218</t>
+  </si>
+  <si>
+    <t>13929115062101</t>
+  </si>
+  <si>
+    <t>2026-06-21 14:18:16</t>
+  </si>
+  <si>
+    <t>錢匣損壞</t>
+  </si>
+  <si>
+    <t>門市反應TM2收銀機(TCX800)(抽屜顏色:白、鑰匙孔位子(右)、鎖頭編號:713)抽屜內彈簧不見一個...請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-06-21 14:22:56</t>
+  </si>
+  <si>
+    <t>2026-06-22 11:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-22 12:00:00</t>
+  </si>
+  <si>
+    <t>調整彈簧</t>
+  </si>
+  <si>
+    <t>14529115062201</t>
+  </si>
+  <si>
+    <t>淡水新洲店</t>
+  </si>
+  <si>
+    <t>2026-06-22 09:16:56</t>
+  </si>
+  <si>
+    <t xml:space="preserve">門市反應TM2(TCX800)多卡機QP3000E無電源反應，已有重新拔插線路仍異常....請台芝到店協助	</t>
+  </si>
+  <si>
+    <t>THILF04529</t>
+  </si>
+  <si>
+    <t>2026-06-22 09:17:57</t>
+  </si>
+  <si>
+    <t>2026-06-22 11:41:00</t>
+  </si>
+  <si>
+    <t>2026-06-22 12:11:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 13:17:00</t>
+  </si>
+  <si>
+    <t>E2995115062201</t>
+  </si>
+  <si>
+    <t>2026-06-22 09:12:43</t>
+  </si>
+  <si>
+    <t>06/22 09:20 萊爾富百大門市啟動緊急叫修: 門市反應LIFE-ET4顯示無網路，重啟MMK後跳出偵測網路小視窗，依序點選後仍異常，ping60不通....請台芝到店協助(顯示無網路，按疑難排除一樣\'網路纜線未接好或是可能已經損毀。)</t>
+  </si>
+  <si>
+    <t>2026-06-22 09:24:23</t>
+  </si>
+  <si>
+    <t>2026-06-22 12:45:00</t>
+  </si>
+  <si>
+    <t>2026-06-22 15:24:00</t>
+  </si>
+  <si>
+    <t>重開數據機 HUB MMK</t>
+  </si>
+  <si>
+    <t>14093115062201</t>
+  </si>
+  <si>
+    <t>淡水新市一</t>
+  </si>
+  <si>
+    <t>2026-06-22 09:26:26</t>
+  </si>
+  <si>
+    <t>THILF04093</t>
+  </si>
+  <si>
+    <t>2026-06-22 09:27:11</t>
+  </si>
+  <si>
+    <t>2026-06-22 15:46:00</t>
+  </si>
+  <si>
+    <t>2026-06-22 16:16:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 13:27:00</t>
+  </si>
+  <si>
+    <t>更換多卡機
+換下8183002077
+換上8183001858</t>
+  </si>
+  <si>
+    <t>蘆洲希望店</t>
+  </si>
+  <si>
+    <t>THILF05354</t>
+  </si>
+  <si>
+    <t>2026-06-22 11:16:58</t>
+  </si>
+  <si>
+    <t>2026-06-22 11:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-22 11:25:00</t>
+  </si>
+  <si>
+    <t>1C894115062201</t>
+  </si>
+  <si>
+    <t>C894</t>
+  </si>
+  <si>
+    <t>中和遠東店</t>
+  </si>
+  <si>
+    <t>2026-06-22 11:59:34</t>
+  </si>
+  <si>
+    <t>門市反應TM2 CCD掃描器(HC56II-TR、HC76-TR)條碼很難刷，代收刷第一段條碼刷過但第二段常常感應不到，已有進行條碼校正仍無改善...還請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF0C894</t>
+  </si>
+  <si>
+    <t>2026-06-22 12:19:48</t>
+  </si>
+  <si>
+    <t>2026-06-23 15:50:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 16:15:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 16:19:00</t>
+  </si>
+  <si>
+    <t>換下H811908653. 換上H811913996</t>
+  </si>
+  <si>
+    <t>2026-06-22 13:23:24</t>
+  </si>
+  <si>
+    <t>2026-06-22 12:50:00</t>
+  </si>
+  <si>
+    <t>2026-06-22 13:15:00</t>
+  </si>
+  <si>
+    <t>三重仁義店</t>
+  </si>
+  <si>
+    <t>THILF04241</t>
+  </si>
+  <si>
+    <t>2026-06-22 13:54:52</t>
+  </si>
+  <si>
+    <t>2026-06-22 13:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-22 13:52:00</t>
+  </si>
+  <si>
+    <t>蘆洲鷺江店</t>
+  </si>
+  <si>
+    <t>THILF02890</t>
+  </si>
+  <si>
+    <t>2026-06-22 14:29:46</t>
+  </si>
+  <si>
+    <t>2026-06-22 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-22 14:30:00</t>
+  </si>
+  <si>
+    <t>L517</t>
+  </si>
+  <si>
+    <t>車麗屋蘆洲店</t>
+  </si>
+  <si>
+    <t>THILF0L517</t>
+  </si>
+  <si>
+    <t>2026-06-22 14:49:07</t>
+  </si>
+  <si>
+    <t>2026-06-22 14:50:00</t>
+  </si>
+  <si>
+    <t>12349115062201</t>
+  </si>
+  <si>
+    <t>三重永福店</t>
+  </si>
+  <si>
+    <t>2026-06-22 15:47:45</t>
+  </si>
+  <si>
+    <t>無電源反應、無紅光</t>
+  </si>
+  <si>
+    <t>門市反應sc ccd掃描器(AT20B)無電源反應無亮紅光，已有重新拔插線路仍異常....請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF02349</t>
+  </si>
+  <si>
+    <t>2026-06-22 15:49:04</t>
+  </si>
+  <si>
+    <t>2026-06-23 13:25:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 13:45:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 19:49:00</t>
+  </si>
+  <si>
+    <t>重新插拔掃槍端USB端正常</t>
+  </si>
+  <si>
+    <t>12422115062201</t>
+  </si>
+  <si>
+    <t>2026-06-22 16:57:50</t>
+  </si>
+  <si>
+    <t>D301</t>
+  </si>
+  <si>
+    <t>發票切刀卡紙，切紙不正常</t>
+  </si>
+  <si>
+    <t>門市反應TM1熱感發票機(BSC10II)裁切不正常，已嘗試重啟設備+重裝紙捲仍異常..請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-06-22 17:00:28</t>
+  </si>
+  <si>
+    <t>2026-06-23 11:10:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 11:37:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 21:00:00</t>
+  </si>
+  <si>
+    <t>排除發票機內部異物測試正常</t>
+  </si>
+  <si>
+    <t>14025115062301</t>
+  </si>
+  <si>
+    <t>新莊祐信店</t>
+  </si>
+  <si>
+    <t>2026-06-23 08:51:06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">門市反應在E網檯帳專區檯帳圖查詢點選任何檯帳區域無法開啟檔案，已有重啟SC跟重開E網皆無法排除。
+2026/6/23 (週二) 上午 08:49 總公司明翰mail:有關 4025新莊祐信店出現SC(SHUTTLE6S)硬碟損壞，請儘速到店更換SC第二顆硬碟，資料不要備份。請協助緊急派工，到店更換SC第二顆硬碟，資料不備份，謝謝。
+PS.若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對)																																
+與門市確認帳務做到06/22，與通訊健誌副理確認有收到06/22的銷售																																
+</t>
+  </si>
+  <si>
+    <t>THILF04025</t>
+  </si>
+  <si>
+    <t>2026-06-23 09:01:28</t>
+  </si>
+  <si>
+    <t>2026-06-23 09:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 10:45:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 15:01:00</t>
+  </si>
+  <si>
+    <t>更換第二顆硬碟不備份還原 並告知更換硬碟注意事項</t>
+  </si>
+  <si>
+    <t>E4196115062301</t>
+  </si>
+  <si>
+    <t>三重蝶愛店</t>
+  </si>
+  <si>
+    <t>2026-06-23 09:20:27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">門市反應TM1(UPOS211K)抽屜開關都會卡卡的，抽屜外觀米白/鑰匙孔位置中間/鑰匙孔編號5001.....須請台芝到店協助(收銀機抽屜會卡住)
+</t>
+  </si>
+  <si>
+    <t>THILF04196</t>
+  </si>
+  <si>
+    <t>2026-06-23 09:32:04</t>
+  </si>
+  <si>
+    <t>2026-06-23 13:50:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 14:15:00</t>
+  </si>
+  <si>
+    <t>2026-06-24 13:32:00</t>
+  </si>
+  <si>
+    <t>清潔軌道測試正常</t>
+  </si>
+  <si>
+    <t>14196115062301</t>
+  </si>
+  <si>
+    <t>2026-06-23 09:32:00</t>
+  </si>
+  <si>
+    <t>門市反應TM2(UPOS211K)抽屜彈開只會是手掌寬度，都需要手動拉開，抽屜外觀米白/鑰匙孔位置中間/鑰匙孔編號5001.....須請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-06-23 09:33:28</t>
+  </si>
+  <si>
+    <t>2026-06-23 14:40:00</t>
+  </si>
+  <si>
+    <t>2026-06-24 13:33:00</t>
+  </si>
+  <si>
+    <t>換下81Z1000933. 換上81Z1004948</t>
+  </si>
+  <si>
+    <t>北縣醒吾店</t>
+  </si>
+  <si>
+    <t>THILF03243</t>
+  </si>
+  <si>
+    <t>2026-06-23 11:09:28</t>
+  </si>
+  <si>
+    <t>2026-06-23 10:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 11:07:00</t>
+  </si>
+  <si>
+    <t>閉店撤機完成</t>
+  </si>
+  <si>
+    <t>板橋漢江店</t>
+  </si>
+  <si>
+    <t>THILF03818</t>
+  </si>
+  <si>
+    <t>2026-06-23 12:16:36</t>
+  </si>
+  <si>
+    <t>2026-06-23 10:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 11:50:00</t>
+  </si>
+  <si>
+    <t>閉店撤機已完工</t>
+  </si>
+  <si>
+    <t>林口捷韻店</t>
+  </si>
+  <si>
+    <t>THILF04715</t>
+  </si>
+  <si>
+    <t>2026-06-23 16:27:14</t>
+  </si>
+  <si>
+    <t>2026-06-23 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 16:24:00</t>
+  </si>
+  <si>
+    <t>SC7</t>
+  </si>
+  <si>
+    <t>中和世紀店</t>
+  </si>
+  <si>
+    <t>THILF05399</t>
+  </si>
+  <si>
+    <t>2026-06-23 16:40:16</t>
+  </si>
+  <si>
+    <t>2026-06-23 16:20:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 16:40:00</t>
   </si>
 </sst>
 </file>
@@ -2998,7 +3527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK121"/>
+  <dimension ref="A1:AK144"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -13260,7 +13789,7 @@
       <c r="O121" s="8" t="s">
         <v>345</v>
       </c>
-      <c r="P121" s="8" t="s">
+      <c r="P121" s="9" t="s">
         <v>830</v>
       </c>
       <c r="Q121" s="7" t="s">
@@ -13297,7 +13826,7 @@
       <c r="AB121" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC121" s="8" t="s">
+      <c r="AC121" s="9" t="s">
         <v>835</v>
       </c>
       <c r="AD121" s="7"/>
@@ -13308,6 +13837,2051 @@
       <c r="AI121" s="7"/>
       <c r="AJ121" s="7"/>
       <c r="AK121" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="122" spans="1:37">
+      <c r="A122" s="3">
+        <v>120</v>
+      </c>
+      <c r="B122" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C122" s="3">
+        <v>2026062505</v>
+      </c>
+      <c r="D122" s="3"/>
+      <c r="E122" s="3"/>
+      <c r="F122" s="3">
+        <v>2380</v>
+      </c>
+      <c r="G122" s="3" t="s">
+        <v>836</v>
+      </c>
+      <c r="H122" s="3" t="s">
+        <v>756</v>
+      </c>
+      <c r="I122" s="3"/>
+      <c r="J122" s="3"/>
+      <c r="K122" s="3"/>
+      <c r="L122" s="3"/>
+      <c r="M122" s="4"/>
+      <c r="N122" s="3"/>
+      <c r="O122" s="4"/>
+      <c r="P122" s="10"/>
+      <c r="Q122" s="3" t="s">
+        <v>837</v>
+      </c>
+      <c r="R122" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S122" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T122" s="3">
+        <v>1</v>
+      </c>
+      <c r="U122" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V122" s="3" t="s">
+        <v>838</v>
+      </c>
+      <c r="W122" s="3" t="s">
+        <v>839</v>
+      </c>
+      <c r="X122" s="3" t="s">
+        <v>840</v>
+      </c>
+      <c r="Y122" s="3"/>
+      <c r="Z122" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="AA122" s="3"/>
+      <c r="AB122" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC122" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="AD122" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE122" s="3"/>
+      <c r="AF122" s="3"/>
+      <c r="AG122" s="3"/>
+      <c r="AH122" s="3"/>
+      <c r="AI122" s="3"/>
+      <c r="AJ122" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK122" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="123" spans="1:37">
+      <c r="A123" s="7">
+        <v>121</v>
+      </c>
+      <c r="B123" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C123" s="7">
+        <v>2026062506</v>
+      </c>
+      <c r="D123" s="7" t="s">
+        <v>841</v>
+      </c>
+      <c r="E123" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F123" s="7">
+        <v>3458</v>
+      </c>
+      <c r="G123" s="7" t="s">
+        <v>842</v>
+      </c>
+      <c r="H123" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="I123" s="7" t="s">
+        <v>843</v>
+      </c>
+      <c r="J123" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="K123" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L123" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="M123" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="N123" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="O123" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="P123" s="9" t="s">
+        <v>844</v>
+      </c>
+      <c r="Q123" s="7" t="s">
+        <v>845</v>
+      </c>
+      <c r="R123" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S123" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T123" s="7">
+        <v>1</v>
+      </c>
+      <c r="U123" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V123" s="7" t="s">
+        <v>846</v>
+      </c>
+      <c r="W123" s="7" t="s">
+        <v>847</v>
+      </c>
+      <c r="X123" s="7" t="s">
+        <v>848</v>
+      </c>
+      <c r="Y123" s="7" t="s">
+        <v>849</v>
+      </c>
+      <c r="Z123" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="AA123" s="7"/>
+      <c r="AB123" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC123" s="9" t="s">
+        <v>850</v>
+      </c>
+      <c r="AD123" s="7"/>
+      <c r="AE123" s="7"/>
+      <c r="AF123" s="7"/>
+      <c r="AG123" s="7"/>
+      <c r="AH123" s="7"/>
+      <c r="AI123" s="7"/>
+      <c r="AJ123" s="7"/>
+      <c r="AK123" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="124" spans="1:37">
+      <c r="A124" s="3">
+        <v>122</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C124" s="3">
+        <v>2026062514</v>
+      </c>
+      <c r="D124" s="3" t="s">
+        <v>851</v>
+      </c>
+      <c r="E124" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F124" s="3">
+        <v>2380</v>
+      </c>
+      <c r="G124" s="3" t="s">
+        <v>836</v>
+      </c>
+      <c r="H124" s="3" t="s">
+        <v>756</v>
+      </c>
+      <c r="I124" s="3" t="s">
+        <v>852</v>
+      </c>
+      <c r="J124" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="K124" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L124" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="M124" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="N124" s="3">
+        <v>2402</v>
+      </c>
+      <c r="O124" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="P124" s="10" t="s">
+        <v>853</v>
+      </c>
+      <c r="Q124" s="3" t="s">
+        <v>837</v>
+      </c>
+      <c r="R124" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S124" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T124" s="3">
+        <v>1</v>
+      </c>
+      <c r="U124" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V124" s="3" t="s">
+        <v>854</v>
+      </c>
+      <c r="W124" s="3" t="s">
+        <v>855</v>
+      </c>
+      <c r="X124" s="3" t="s">
+        <v>856</v>
+      </c>
+      <c r="Y124" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="Z124" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA124" s="3"/>
+      <c r="AB124" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC124" s="10" t="s">
+        <v>857</v>
+      </c>
+      <c r="AD124" s="3"/>
+      <c r="AE124" s="3"/>
+      <c r="AF124" s="3"/>
+      <c r="AG124" s="3"/>
+      <c r="AH124" s="3"/>
+      <c r="AI124" s="3"/>
+      <c r="AJ124" s="3"/>
+      <c r="AK124" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="125" spans="1:37">
+      <c r="A125" s="7">
+        <v>123</v>
+      </c>
+      <c r="B125" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C125" s="7">
+        <v>2026062521</v>
+      </c>
+      <c r="D125" s="7" t="s">
+        <v>858</v>
+      </c>
+      <c r="E125" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F125" s="7" t="s">
+        <v>859</v>
+      </c>
+      <c r="G125" s="7" t="s">
+        <v>860</v>
+      </c>
+      <c r="H125" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I125" s="7" t="s">
+        <v>861</v>
+      </c>
+      <c r="J125" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="K125" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L125" s="7" t="s">
+        <v>862</v>
+      </c>
+      <c r="M125" s="8" t="s">
+        <v>863</v>
+      </c>
+      <c r="N125" s="7">
+        <v>2501</v>
+      </c>
+      <c r="O125" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="P125" s="9" t="s">
+        <v>865</v>
+      </c>
+      <c r="Q125" s="7" t="s">
+        <v>866</v>
+      </c>
+      <c r="R125" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S125" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T125" s="7">
+        <v>1</v>
+      </c>
+      <c r="U125" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V125" s="7" t="s">
+        <v>867</v>
+      </c>
+      <c r="W125" s="7" t="s">
+        <v>868</v>
+      </c>
+      <c r="X125" s="7" t="s">
+        <v>869</v>
+      </c>
+      <c r="Y125" s="7" t="s">
+        <v>849</v>
+      </c>
+      <c r="Z125" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA125" s="7"/>
+      <c r="AB125" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC125" s="9" t="s">
+        <v>870</v>
+      </c>
+      <c r="AD125" s="7"/>
+      <c r="AE125" s="7"/>
+      <c r="AF125" s="7"/>
+      <c r="AG125" s="7"/>
+      <c r="AH125" s="7"/>
+      <c r="AI125" s="7"/>
+      <c r="AJ125" s="7"/>
+      <c r="AK125" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="126" spans="1:37">
+      <c r="A126" s="3">
+        <v>124</v>
+      </c>
+      <c r="B126" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C126" s="3">
+        <v>2026062525</v>
+      </c>
+      <c r="D126" s="3" t="s">
+        <v>871</v>
+      </c>
+      <c r="E126" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F126" s="3">
+        <v>3929</v>
+      </c>
+      <c r="G126" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="H126" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="I126" s="3" t="s">
+        <v>872</v>
+      </c>
+      <c r="J126" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="K126" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L126" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M126" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="N126" s="3">
+        <v>2304</v>
+      </c>
+      <c r="O126" s="4" t="s">
+        <v>873</v>
+      </c>
+      <c r="P126" s="10" t="s">
+        <v>874</v>
+      </c>
+      <c r="Q126" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="R126" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S126" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T126" s="3">
+        <v>1</v>
+      </c>
+      <c r="U126" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V126" s="3" t="s">
+        <v>875</v>
+      </c>
+      <c r="W126" s="3" t="s">
+        <v>876</v>
+      </c>
+      <c r="X126" s="3" t="s">
+        <v>877</v>
+      </c>
+      <c r="Y126" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="Z126" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA126" s="3"/>
+      <c r="AB126" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC126" s="10" t="s">
+        <v>878</v>
+      </c>
+      <c r="AD126" s="3"/>
+      <c r="AE126" s="3"/>
+      <c r="AF126" s="3"/>
+      <c r="AG126" s="3"/>
+      <c r="AH126" s="3"/>
+      <c r="AI126" s="3"/>
+      <c r="AJ126" s="3"/>
+      <c r="AK126" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="127" spans="1:37">
+      <c r="A127" s="7">
+        <v>125</v>
+      </c>
+      <c r="B127" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C127" s="7">
+        <v>2026062535</v>
+      </c>
+      <c r="D127" s="7" t="s">
+        <v>879</v>
+      </c>
+      <c r="E127" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F127" s="7">
+        <v>4529</v>
+      </c>
+      <c r="G127" s="7" t="s">
+        <v>880</v>
+      </c>
+      <c r="H127" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="I127" s="7" t="s">
+        <v>881</v>
+      </c>
+      <c r="J127" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K127" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L127" s="7" t="s">
+        <v>522</v>
+      </c>
+      <c r="M127" s="8" t="s">
+        <v>523</v>
+      </c>
+      <c r="N127" s="7" t="s">
+        <v>524</v>
+      </c>
+      <c r="O127" s="8" t="s">
+        <v>525</v>
+      </c>
+      <c r="P127" s="9" t="s">
+        <v>882</v>
+      </c>
+      <c r="Q127" s="7" t="s">
+        <v>883</v>
+      </c>
+      <c r="R127" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S127" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T127" s="7">
+        <v>1</v>
+      </c>
+      <c r="U127" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V127" s="7" t="s">
+        <v>884</v>
+      </c>
+      <c r="W127" s="7" t="s">
+        <v>885</v>
+      </c>
+      <c r="X127" s="7" t="s">
+        <v>886</v>
+      </c>
+      <c r="Y127" s="7" t="s">
+        <v>887</v>
+      </c>
+      <c r="Z127" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA127" s="7"/>
+      <c r="AB127" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="AC127" s="9" t="s">
+        <v>320</v>
+      </c>
+      <c r="AD127" s="7"/>
+      <c r="AE127" s="7"/>
+      <c r="AF127" s="7"/>
+      <c r="AG127" s="7"/>
+      <c r="AH127" s="7"/>
+      <c r="AI127" s="7"/>
+      <c r="AJ127" s="7"/>
+      <c r="AK127" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="128" spans="1:37">
+      <c r="A128" s="3">
+        <v>126</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C128" s="3">
+        <v>2026062538</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>888</v>
+      </c>
+      <c r="E128" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="F128" s="3">
+        <v>2995</v>
+      </c>
+      <c r="G128" s="3" t="s">
+        <v>796</v>
+      </c>
+      <c r="H128" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I128" s="3" t="s">
+        <v>889</v>
+      </c>
+      <c r="J128" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="K128" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L128" s="3" t="s">
+        <v>809</v>
+      </c>
+      <c r="M128" s="4" t="s">
+        <v>810</v>
+      </c>
+      <c r="N128" s="3">
+        <v>5804</v>
+      </c>
+      <c r="O128" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="P128" s="10" t="s">
+        <v>890</v>
+      </c>
+      <c r="Q128" s="3" t="s">
+        <v>797</v>
+      </c>
+      <c r="R128" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S128" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T128" s="3">
+        <v>1</v>
+      </c>
+      <c r="U128" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V128" s="3" t="s">
+        <v>891</v>
+      </c>
+      <c r="W128" s="3" t="s">
+        <v>877</v>
+      </c>
+      <c r="X128" s="3" t="s">
+        <v>892</v>
+      </c>
+      <c r="Y128" s="3" t="s">
+        <v>893</v>
+      </c>
+      <c r="Z128" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="AA128" s="3"/>
+      <c r="AB128" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC128" s="10" t="s">
+        <v>894</v>
+      </c>
+      <c r="AD128" s="3"/>
+      <c r="AE128" s="3"/>
+      <c r="AF128" s="3"/>
+      <c r="AG128" s="3"/>
+      <c r="AH128" s="3"/>
+      <c r="AI128" s="3"/>
+      <c r="AJ128" s="3"/>
+      <c r="AK128" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="129" spans="1:37">
+      <c r="A129" s="7">
+        <v>127</v>
+      </c>
+      <c r="B129" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C129" s="7">
+        <v>2026062540</v>
+      </c>
+      <c r="D129" s="7" t="s">
+        <v>895</v>
+      </c>
+      <c r="E129" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F129" s="7">
+        <v>4093</v>
+      </c>
+      <c r="G129" s="7" t="s">
+        <v>896</v>
+      </c>
+      <c r="H129" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="I129" s="7" t="s">
+        <v>897</v>
+      </c>
+      <c r="J129" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K129" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L129" s="7" t="s">
+        <v>522</v>
+      </c>
+      <c r="M129" s="8" t="s">
+        <v>523</v>
+      </c>
+      <c r="N129" s="7" t="s">
+        <v>524</v>
+      </c>
+      <c r="O129" s="8" t="s">
+        <v>525</v>
+      </c>
+      <c r="P129" s="9" t="s">
+        <v>882</v>
+      </c>
+      <c r="Q129" s="7" t="s">
+        <v>898</v>
+      </c>
+      <c r="R129" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S129" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T129" s="7">
+        <v>1</v>
+      </c>
+      <c r="U129" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V129" s="7" t="s">
+        <v>899</v>
+      </c>
+      <c r="W129" s="7" t="s">
+        <v>900</v>
+      </c>
+      <c r="X129" s="7" t="s">
+        <v>901</v>
+      </c>
+      <c r="Y129" s="7" t="s">
+        <v>902</v>
+      </c>
+      <c r="Z129" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA129" s="7"/>
+      <c r="AB129" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC129" s="9" t="s">
+        <v>903</v>
+      </c>
+      <c r="AD129" s="7"/>
+      <c r="AE129" s="7"/>
+      <c r="AF129" s="7"/>
+      <c r="AG129" s="7"/>
+      <c r="AH129" s="7"/>
+      <c r="AI129" s="7"/>
+      <c r="AJ129" s="7"/>
+      <c r="AK129" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="130" spans="1:37">
+      <c r="A130" s="3">
+        <v>128</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C130" s="3">
+        <v>2026062580</v>
+      </c>
+      <c r="D130" s="3"/>
+      <c r="E130" s="3"/>
+      <c r="F130" s="3">
+        <v>5354</v>
+      </c>
+      <c r="G130" s="3" t="s">
+        <v>904</v>
+      </c>
+      <c r="H130" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="I130" s="3"/>
+      <c r="J130" s="3"/>
+      <c r="K130" s="3"/>
+      <c r="L130" s="3"/>
+      <c r="M130" s="4"/>
+      <c r="N130" s="3"/>
+      <c r="O130" s="4"/>
+      <c r="P130" s="10"/>
+      <c r="Q130" s="3" t="s">
+        <v>905</v>
+      </c>
+      <c r="R130" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S130" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T130" s="3">
+        <v>1</v>
+      </c>
+      <c r="U130" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V130" s="3" t="s">
+        <v>906</v>
+      </c>
+      <c r="W130" s="3" t="s">
+        <v>907</v>
+      </c>
+      <c r="X130" s="3" t="s">
+        <v>908</v>
+      </c>
+      <c r="Y130" s="3"/>
+      <c r="Z130" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA130" s="3"/>
+      <c r="AB130" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC130" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD130" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE130" s="3"/>
+      <c r="AF130" s="3"/>
+      <c r="AG130" s="3"/>
+      <c r="AH130" s="3"/>
+      <c r="AI130" s="3"/>
+      <c r="AJ130" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK130" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="131" spans="1:37">
+      <c r="A131" s="7">
+        <v>129</v>
+      </c>
+      <c r="B131" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C131" s="7">
+        <v>2026062589</v>
+      </c>
+      <c r="D131" s="7" t="s">
+        <v>909</v>
+      </c>
+      <c r="E131" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F131" s="7" t="s">
+        <v>910</v>
+      </c>
+      <c r="G131" s="7" t="s">
+        <v>911</v>
+      </c>
+      <c r="H131" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="I131" s="7" t="s">
+        <v>912</v>
+      </c>
+      <c r="J131" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K131" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L131" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="M131" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="N131" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="O131" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="P131" s="9" t="s">
+        <v>913</v>
+      </c>
+      <c r="Q131" s="7" t="s">
+        <v>914</v>
+      </c>
+      <c r="R131" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S131" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T131" s="7">
+        <v>1</v>
+      </c>
+      <c r="U131" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V131" s="7" t="s">
+        <v>915</v>
+      </c>
+      <c r="W131" s="7" t="s">
+        <v>916</v>
+      </c>
+      <c r="X131" s="7" t="s">
+        <v>917</v>
+      </c>
+      <c r="Y131" s="7" t="s">
+        <v>918</v>
+      </c>
+      <c r="Z131" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA131" s="7"/>
+      <c r="AB131" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC131" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="AD131" s="7"/>
+      <c r="AE131" s="7"/>
+      <c r="AF131" s="7"/>
+      <c r="AG131" s="7"/>
+      <c r="AH131" s="7"/>
+      <c r="AI131" s="7"/>
+      <c r="AJ131" s="7"/>
+      <c r="AK131" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="132" spans="1:37">
+      <c r="A132" s="3">
+        <v>130</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C132" s="3">
+        <v>2026062597</v>
+      </c>
+      <c r="D132" s="3"/>
+      <c r="E132" s="3"/>
+      <c r="F132" s="3" t="s">
+        <v>859</v>
+      </c>
+      <c r="G132" s="3" t="s">
+        <v>860</v>
+      </c>
+      <c r="H132" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I132" s="3"/>
+      <c r="J132" s="3"/>
+      <c r="K132" s="3"/>
+      <c r="L132" s="3"/>
+      <c r="M132" s="4"/>
+      <c r="N132" s="3"/>
+      <c r="O132" s="4"/>
+      <c r="P132" s="10"/>
+      <c r="Q132" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="R132" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S132" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T132" s="3">
+        <v>1</v>
+      </c>
+      <c r="U132" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V132" s="3" t="s">
+        <v>920</v>
+      </c>
+      <c r="W132" s="3" t="s">
+        <v>921</v>
+      </c>
+      <c r="X132" s="3" t="s">
+        <v>922</v>
+      </c>
+      <c r="Y132" s="3"/>
+      <c r="Z132" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA132" s="3"/>
+      <c r="AB132" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC132" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD132" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE132" s="3"/>
+      <c r="AF132" s="3"/>
+      <c r="AG132" s="3"/>
+      <c r="AH132" s="3"/>
+      <c r="AI132" s="3"/>
+      <c r="AJ132" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK132" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="133" spans="1:37">
+      <c r="A133" s="7">
+        <v>131</v>
+      </c>
+      <c r="B133" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C133" s="7">
+        <v>2026062601</v>
+      </c>
+      <c r="D133" s="7"/>
+      <c r="E133" s="7"/>
+      <c r="F133" s="7">
+        <v>4241</v>
+      </c>
+      <c r="G133" s="7" t="s">
+        <v>923</v>
+      </c>
+      <c r="H133" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I133" s="7"/>
+      <c r="J133" s="7"/>
+      <c r="K133" s="7"/>
+      <c r="L133" s="7"/>
+      <c r="M133" s="8"/>
+      <c r="N133" s="7"/>
+      <c r="O133" s="8"/>
+      <c r="P133" s="9"/>
+      <c r="Q133" s="7" t="s">
+        <v>924</v>
+      </c>
+      <c r="R133" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S133" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T133" s="7">
+        <v>1</v>
+      </c>
+      <c r="U133" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V133" s="7" t="s">
+        <v>925</v>
+      </c>
+      <c r="W133" s="7" t="s">
+        <v>926</v>
+      </c>
+      <c r="X133" s="7" t="s">
+        <v>927</v>
+      </c>
+      <c r="Y133" s="7"/>
+      <c r="Z133" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA133" s="7"/>
+      <c r="AB133" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC133" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD133" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE133" s="7"/>
+      <c r="AF133" s="7"/>
+      <c r="AG133" s="7"/>
+      <c r="AH133" s="7"/>
+      <c r="AI133" s="7"/>
+      <c r="AJ133" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK133" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="134" spans="1:37">
+      <c r="A134" s="3">
+        <v>132</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C134" s="3">
+        <v>2026062608</v>
+      </c>
+      <c r="D134" s="3"/>
+      <c r="E134" s="3"/>
+      <c r="F134" s="3">
+        <v>2890</v>
+      </c>
+      <c r="G134" s="3" t="s">
+        <v>928</v>
+      </c>
+      <c r="H134" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="I134" s="3"/>
+      <c r="J134" s="3"/>
+      <c r="K134" s="3"/>
+      <c r="L134" s="3"/>
+      <c r="M134" s="4"/>
+      <c r="N134" s="3"/>
+      <c r="O134" s="4"/>
+      <c r="P134" s="10"/>
+      <c r="Q134" s="3" t="s">
+        <v>929</v>
+      </c>
+      <c r="R134" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S134" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T134" s="3">
+        <v>1</v>
+      </c>
+      <c r="U134" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V134" s="3" t="s">
+        <v>930</v>
+      </c>
+      <c r="W134" s="3" t="s">
+        <v>931</v>
+      </c>
+      <c r="X134" s="3" t="s">
+        <v>932</v>
+      </c>
+      <c r="Y134" s="3"/>
+      <c r="Z134" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA134" s="3"/>
+      <c r="AB134" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC134" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD134" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE134" s="3"/>
+      <c r="AF134" s="3"/>
+      <c r="AG134" s="3"/>
+      <c r="AH134" s="3"/>
+      <c r="AI134" s="3"/>
+      <c r="AJ134" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK134" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="135" spans="1:37">
+      <c r="A135" s="7">
+        <v>133</v>
+      </c>
+      <c r="B135" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C135" s="7">
+        <v>2026062615</v>
+      </c>
+      <c r="D135" s="7"/>
+      <c r="E135" s="7"/>
+      <c r="F135" s="7" t="s">
+        <v>933</v>
+      </c>
+      <c r="G135" s="7" t="s">
+        <v>934</v>
+      </c>
+      <c r="H135" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="I135" s="7"/>
+      <c r="J135" s="7"/>
+      <c r="K135" s="7"/>
+      <c r="L135" s="7"/>
+      <c r="M135" s="8"/>
+      <c r="N135" s="7"/>
+      <c r="O135" s="8"/>
+      <c r="P135" s="9"/>
+      <c r="Q135" s="7" t="s">
+        <v>935</v>
+      </c>
+      <c r="R135" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S135" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T135" s="7">
+        <v>1</v>
+      </c>
+      <c r="U135" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V135" s="7" t="s">
+        <v>936</v>
+      </c>
+      <c r="W135" s="7" t="s">
+        <v>932</v>
+      </c>
+      <c r="X135" s="7" t="s">
+        <v>937</v>
+      </c>
+      <c r="Y135" s="7"/>
+      <c r="Z135" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA135" s="7"/>
+      <c r="AB135" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC135" s="9" t="s">
+        <v>476</v>
+      </c>
+      <c r="AD135" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE135" s="7"/>
+      <c r="AF135" s="7"/>
+      <c r="AG135" s="7"/>
+      <c r="AH135" s="7"/>
+      <c r="AI135" s="7"/>
+      <c r="AJ135" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK135" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="136" spans="1:37">
+      <c r="A136" s="3">
+        <v>134</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C136" s="3">
+        <v>2026062626</v>
+      </c>
+      <c r="D136" s="3" t="s">
+        <v>938</v>
+      </c>
+      <c r="E136" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F136" s="3">
+        <v>2349</v>
+      </c>
+      <c r="G136" s="3" t="s">
+        <v>939</v>
+      </c>
+      <c r="H136" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I136" s="3" t="s">
+        <v>940</v>
+      </c>
+      <c r="J136" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="K136" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L136" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="M136" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="N136" s="3">
+        <v>2902</v>
+      </c>
+      <c r="O136" s="4" t="s">
+        <v>941</v>
+      </c>
+      <c r="P136" s="10" t="s">
+        <v>942</v>
+      </c>
+      <c r="Q136" s="3" t="s">
+        <v>943</v>
+      </c>
+      <c r="R136" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S136" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T136" s="3">
+        <v>1</v>
+      </c>
+      <c r="U136" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V136" s="3" t="s">
+        <v>944</v>
+      </c>
+      <c r="W136" s="3" t="s">
+        <v>945</v>
+      </c>
+      <c r="X136" s="3" t="s">
+        <v>946</v>
+      </c>
+      <c r="Y136" s="3" t="s">
+        <v>947</v>
+      </c>
+      <c r="Z136" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA136" s="3"/>
+      <c r="AB136" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC136" s="10" t="s">
+        <v>948</v>
+      </c>
+      <c r="AD136" s="3"/>
+      <c r="AE136" s="3"/>
+      <c r="AF136" s="3"/>
+      <c r="AG136" s="3"/>
+      <c r="AH136" s="3"/>
+      <c r="AI136" s="3"/>
+      <c r="AJ136" s="3"/>
+      <c r="AK136" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="137" spans="1:37">
+      <c r="A137" s="7">
+        <v>135</v>
+      </c>
+      <c r="B137" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C137" s="7">
+        <v>2026062655</v>
+      </c>
+      <c r="D137" s="7" t="s">
+        <v>949</v>
+      </c>
+      <c r="E137" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F137" s="7">
+        <v>2422</v>
+      </c>
+      <c r="G137" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="H137" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I137" s="7" t="s">
+        <v>950</v>
+      </c>
+      <c r="J137" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K137" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L137" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="M137" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="N137" s="7" t="s">
+        <v>951</v>
+      </c>
+      <c r="O137" s="8" t="s">
+        <v>952</v>
+      </c>
+      <c r="P137" s="9" t="s">
+        <v>953</v>
+      </c>
+      <c r="Q137" s="7" t="s">
+        <v>802</v>
+      </c>
+      <c r="R137" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S137" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="T137" s="7">
+        <v>1</v>
+      </c>
+      <c r="U137" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V137" s="7" t="s">
+        <v>954</v>
+      </c>
+      <c r="W137" s="7" t="s">
+        <v>955</v>
+      </c>
+      <c r="X137" s="7" t="s">
+        <v>956</v>
+      </c>
+      <c r="Y137" s="7" t="s">
+        <v>957</v>
+      </c>
+      <c r="Z137" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA137" s="7"/>
+      <c r="AB137" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC137" s="9" t="s">
+        <v>958</v>
+      </c>
+      <c r="AD137" s="7"/>
+      <c r="AE137" s="7"/>
+      <c r="AF137" s="7"/>
+      <c r="AG137" s="7"/>
+      <c r="AH137" s="7"/>
+      <c r="AI137" s="7"/>
+      <c r="AJ137" s="7"/>
+      <c r="AK137" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="138" spans="1:37">
+      <c r="A138" s="3">
+        <v>136</v>
+      </c>
+      <c r="B138" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C138" s="3">
+        <v>2026062684</v>
+      </c>
+      <c r="D138" s="3" t="s">
+        <v>959</v>
+      </c>
+      <c r="E138" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="F138" s="3">
+        <v>4025</v>
+      </c>
+      <c r="G138" s="3" t="s">
+        <v>960</v>
+      </c>
+      <c r="H138" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="I138" s="3" t="s">
+        <v>961</v>
+      </c>
+      <c r="J138" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="K138" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L138" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="M138" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="N138" s="3">
+        <v>2405</v>
+      </c>
+      <c r="O138" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="P138" s="10" t="s">
+        <v>962</v>
+      </c>
+      <c r="Q138" s="3" t="s">
+        <v>963</v>
+      </c>
+      <c r="R138" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S138" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T138" s="3">
+        <v>1</v>
+      </c>
+      <c r="U138" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V138" s="3" t="s">
+        <v>964</v>
+      </c>
+      <c r="W138" s="3" t="s">
+        <v>965</v>
+      </c>
+      <c r="X138" s="3" t="s">
+        <v>966</v>
+      </c>
+      <c r="Y138" s="3" t="s">
+        <v>967</v>
+      </c>
+      <c r="Z138" s="3">
+        <v>1.3</v>
+      </c>
+      <c r="AA138" s="3"/>
+      <c r="AB138" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC138" s="10" t="s">
+        <v>968</v>
+      </c>
+      <c r="AD138" s="3"/>
+      <c r="AE138" s="3"/>
+      <c r="AF138" s="3"/>
+      <c r="AG138" s="3"/>
+      <c r="AH138" s="3"/>
+      <c r="AI138" s="3"/>
+      <c r="AJ138" s="3"/>
+      <c r="AK138" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="139" spans="1:37">
+      <c r="A139" s="7">
+        <v>137</v>
+      </c>
+      <c r="B139" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C139" s="7">
+        <v>2026062706</v>
+      </c>
+      <c r="D139" s="7" t="s">
+        <v>969</v>
+      </c>
+      <c r="E139" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F139" s="7">
+        <v>4196</v>
+      </c>
+      <c r="G139" s="7" t="s">
+        <v>970</v>
+      </c>
+      <c r="H139" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I139" s="7" t="s">
+        <v>971</v>
+      </c>
+      <c r="J139" s="7" t="s">
+        <v>376</v>
+      </c>
+      <c r="K139" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L139" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M139" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="N139" s="7">
+        <v>2305</v>
+      </c>
+      <c r="O139" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="P139" s="9" t="s">
+        <v>972</v>
+      </c>
+      <c r="Q139" s="7" t="s">
+        <v>973</v>
+      </c>
+      <c r="R139" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S139" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T139" s="7">
+        <v>1</v>
+      </c>
+      <c r="U139" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V139" s="7" t="s">
+        <v>974</v>
+      </c>
+      <c r="W139" s="7" t="s">
+        <v>975</v>
+      </c>
+      <c r="X139" s="7" t="s">
+        <v>976</v>
+      </c>
+      <c r="Y139" s="7" t="s">
+        <v>977</v>
+      </c>
+      <c r="Z139" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA139" s="7"/>
+      <c r="AB139" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC139" s="9" t="s">
+        <v>978</v>
+      </c>
+      <c r="AD139" s="7"/>
+      <c r="AE139" s="7"/>
+      <c r="AF139" s="7"/>
+      <c r="AG139" s="7"/>
+      <c r="AH139" s="7"/>
+      <c r="AI139" s="7"/>
+      <c r="AJ139" s="7"/>
+      <c r="AK139" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="140" spans="1:37">
+      <c r="A140" s="3">
+        <v>138</v>
+      </c>
+      <c r="B140" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C140" s="3">
+        <v>2026062707</v>
+      </c>
+      <c r="D140" s="3" t="s">
+        <v>979</v>
+      </c>
+      <c r="E140" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F140" s="3">
+        <v>4196</v>
+      </c>
+      <c r="G140" s="3" t="s">
+        <v>970</v>
+      </c>
+      <c r="H140" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I140" s="3" t="s">
+        <v>980</v>
+      </c>
+      <c r="J140" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="K140" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L140" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M140" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="N140" s="3">
+        <v>2305</v>
+      </c>
+      <c r="O140" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="P140" s="10" t="s">
+        <v>981</v>
+      </c>
+      <c r="Q140" s="3" t="s">
+        <v>973</v>
+      </c>
+      <c r="R140" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S140" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T140" s="3">
+        <v>1</v>
+      </c>
+      <c r="U140" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V140" s="3" t="s">
+        <v>982</v>
+      </c>
+      <c r="W140" s="3" t="s">
+        <v>976</v>
+      </c>
+      <c r="X140" s="3" t="s">
+        <v>983</v>
+      </c>
+      <c r="Y140" s="3" t="s">
+        <v>984</v>
+      </c>
+      <c r="Z140" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA140" s="3"/>
+      <c r="AB140" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC140" s="10" t="s">
+        <v>985</v>
+      </c>
+      <c r="AD140" s="3"/>
+      <c r="AE140" s="3"/>
+      <c r="AF140" s="3"/>
+      <c r="AG140" s="3"/>
+      <c r="AH140" s="3"/>
+      <c r="AI140" s="3"/>
+      <c r="AJ140" s="3"/>
+      <c r="AK140" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="141" spans="1:37">
+      <c r="A141" s="7">
+        <v>139</v>
+      </c>
+      <c r="B141" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C141" s="7">
+        <v>2026062732</v>
+      </c>
+      <c r="D141" s="7"/>
+      <c r="E141" s="7"/>
+      <c r="F141" s="7">
+        <v>3243</v>
+      </c>
+      <c r="G141" s="7" t="s">
+        <v>986</v>
+      </c>
+      <c r="H141" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="I141" s="7"/>
+      <c r="J141" s="7"/>
+      <c r="K141" s="7"/>
+      <c r="L141" s="7"/>
+      <c r="M141" s="8"/>
+      <c r="N141" s="7"/>
+      <c r="O141" s="8"/>
+      <c r="P141" s="9"/>
+      <c r="Q141" s="7" t="s">
+        <v>987</v>
+      </c>
+      <c r="R141" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S141" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T141" s="7">
+        <v>1</v>
+      </c>
+      <c r="U141" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V141" s="7" t="s">
+        <v>988</v>
+      </c>
+      <c r="W141" s="7" t="s">
+        <v>989</v>
+      </c>
+      <c r="X141" s="7" t="s">
+        <v>990</v>
+      </c>
+      <c r="Y141" s="7"/>
+      <c r="Z141" s="7">
+        <v>1.1</v>
+      </c>
+      <c r="AA141" s="7"/>
+      <c r="AB141" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC141" s="9" t="s">
+        <v>991</v>
+      </c>
+      <c r="AD141" s="7"/>
+      <c r="AE141" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF141" s="7"/>
+      <c r="AG141" s="7"/>
+      <c r="AH141" s="7"/>
+      <c r="AI141" s="7"/>
+      <c r="AJ141" s="7"/>
+      <c r="AK141" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="142" spans="1:37">
+      <c r="A142" s="3">
+        <v>140</v>
+      </c>
+      <c r="B142" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C142" s="3">
+        <v>2026062748</v>
+      </c>
+      <c r="D142" s="3"/>
+      <c r="E142" s="3"/>
+      <c r="F142" s="3">
+        <v>3818</v>
+      </c>
+      <c r="G142" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="H142" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I142" s="3"/>
+      <c r="J142" s="3"/>
+      <c r="K142" s="3"/>
+      <c r="L142" s="3"/>
+      <c r="M142" s="4"/>
+      <c r="N142" s="3"/>
+      <c r="O142" s="4"/>
+      <c r="P142" s="10"/>
+      <c r="Q142" s="3" t="s">
+        <v>993</v>
+      </c>
+      <c r="R142" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S142" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="T142" s="3">
+        <v>1</v>
+      </c>
+      <c r="U142" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V142" s="3" t="s">
+        <v>994</v>
+      </c>
+      <c r="W142" s="3" t="s">
+        <v>995</v>
+      </c>
+      <c r="X142" s="3" t="s">
+        <v>996</v>
+      </c>
+      <c r="Y142" s="3"/>
+      <c r="Z142" s="3">
+        <v>1.3</v>
+      </c>
+      <c r="AA142" s="3"/>
+      <c r="AB142" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC142" s="10" t="s">
+        <v>997</v>
+      </c>
+      <c r="AD142" s="3"/>
+      <c r="AE142" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF142" s="3"/>
+      <c r="AG142" s="3"/>
+      <c r="AH142" s="3"/>
+      <c r="AI142" s="3"/>
+      <c r="AJ142" s="3"/>
+      <c r="AK142" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="143" spans="1:37">
+      <c r="A143" s="7">
+        <v>141</v>
+      </c>
+      <c r="B143" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C143" s="7">
+        <v>2026062835</v>
+      </c>
+      <c r="D143" s="7"/>
+      <c r="E143" s="7"/>
+      <c r="F143" s="7">
+        <v>4715</v>
+      </c>
+      <c r="G143" s="7" t="s">
+        <v>998</v>
+      </c>
+      <c r="H143" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="I143" s="7"/>
+      <c r="J143" s="7"/>
+      <c r="K143" s="7"/>
+      <c r="L143" s="7"/>
+      <c r="M143" s="8"/>
+      <c r="N143" s="7"/>
+      <c r="O143" s="8"/>
+      <c r="P143" s="9"/>
+      <c r="Q143" s="7" t="s">
+        <v>999</v>
+      </c>
+      <c r="R143" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S143" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T143" s="7">
+        <v>1</v>
+      </c>
+      <c r="U143" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V143" s="7" t="s">
+        <v>1000</v>
+      </c>
+      <c r="W143" s="7" t="s">
+        <v>1001</v>
+      </c>
+      <c r="X143" s="7" t="s">
+        <v>1002</v>
+      </c>
+      <c r="Y143" s="7"/>
+      <c r="Z143" s="7">
+        <v>2.4</v>
+      </c>
+      <c r="AA143" s="7"/>
+      <c r="AB143" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC143" s="9" t="s">
+        <v>1003</v>
+      </c>
+      <c r="AD143" s="7"/>
+      <c r="AE143" s="7"/>
+      <c r="AF143" s="7"/>
+      <c r="AG143" s="7"/>
+      <c r="AH143" s="7"/>
+      <c r="AI143" s="7"/>
+      <c r="AJ143" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK143" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="144" spans="1:37">
+      <c r="A144" s="3">
+        <v>142</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C144" s="3">
+        <v>2026062845</v>
+      </c>
+      <c r="D144" s="3"/>
+      <c r="E144" s="3"/>
+      <c r="F144" s="3">
+        <v>5399</v>
+      </c>
+      <c r="G144" s="3" t="s">
+        <v>1004</v>
+      </c>
+      <c r="H144" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="I144" s="3"/>
+      <c r="J144" s="3"/>
+      <c r="K144" s="3"/>
+      <c r="L144" s="3"/>
+      <c r="M144" s="4"/>
+      <c r="N144" s="3"/>
+      <c r="O144" s="4"/>
+      <c r="P144" s="4"/>
+      <c r="Q144" s="3" t="s">
+        <v>1005</v>
+      </c>
+      <c r="R144" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S144" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T144" s="3">
+        <v>1</v>
+      </c>
+      <c r="U144" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V144" s="3" t="s">
+        <v>1006</v>
+      </c>
+      <c r="W144" s="3" t="s">
+        <v>1007</v>
+      </c>
+      <c r="X144" s="3" t="s">
+        <v>1008</v>
+      </c>
+      <c r="Y144" s="3"/>
+      <c r="Z144" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA144" s="3"/>
+      <c r="AB144" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC144" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD144" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE144" s="3"/>
+      <c r="AF144" s="3"/>
+      <c r="AG144" s="3"/>
+      <c r="AH144" s="3"/>
+      <c r="AI144" s="3"/>
+      <c r="AJ144" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK144" s="3" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06241719
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$144</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$149</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1009">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-23  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1045">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-24  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -2961,6 +2961,40 @@
     <t>排除發票機內部異物測試正常</t>
   </si>
   <si>
+    <t>EC660115062201</t>
+  </si>
+  <si>
+    <t>C660</t>
+  </si>
+  <si>
+    <t>中和永安市場</t>
+  </si>
+  <si>
+    <t>2026-06-22 21:22:52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">門市反應TM1(TCX800)觸控不良、時好時壞，反應遲緩且有時候要點很多下或按很大力，與門市確認面板無張貼文宣或透明塑膠墊，已於6/20協助門市執行觸控校正，門市告知仍異常...需請台芝到店協助(機一觸控不良.很難按.麻煩工程師查修.謝謝)
+</t>
+  </si>
+  <si>
+    <t>THILF0C660</t>
+  </si>
+  <si>
+    <t>2026-06-22 21:45:44</t>
+  </si>
+  <si>
+    <t>2026-06-23 17:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-23 17:35:00</t>
+  </si>
+  <si>
+    <t>2026-06-24 01:45:00</t>
+  </si>
+  <si>
+    <t>執行觸控校正.整理排線</t>
+  </si>
+  <si>
     <t>14025115062301</t>
   </si>
   <si>
@@ -3114,6 +3148,81 @@
   </si>
   <si>
     <t>2026-06-23 16:40:00</t>
+  </si>
+  <si>
+    <t>15428115062402</t>
+  </si>
+  <si>
+    <t>三重野球魂</t>
+  </si>
+  <si>
+    <t>2026-06-24 13:58:48</t>
+  </si>
+  <si>
+    <t>門市反應MMK四代機畫面顯示網路設定介面視窗，門市依序點選1.重新設定&gt;2.偵測網路&gt;3.重新開機，重新開機後仍顯示網路設定介面小視窗，PING60不通....須請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF05428</t>
+  </si>
+  <si>
+    <t>2026-06-24 14:00:51</t>
+  </si>
+  <si>
+    <t>2026-06-24 15:03:00</t>
+  </si>
+  <si>
+    <t>2026-06-24 15:24:00</t>
+  </si>
+  <si>
+    <t>2026-06-25 18:00:00</t>
+  </si>
+  <si>
+    <t>重新插拔網路線. 重新偵測</t>
+  </si>
+  <si>
+    <t>三重鑫五華</t>
+  </si>
+  <si>
+    <t>THILF05457</t>
+  </si>
+  <si>
+    <t>2026-06-24 14:13:17</t>
+  </si>
+  <si>
+    <t>2026-06-24 13:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-24 13:54:00</t>
+  </si>
+  <si>
+    <t>三重進安店</t>
+  </si>
+  <si>
+    <t>THILF03796</t>
+  </si>
+  <si>
+    <t>2026-06-24 14:46:23</t>
+  </si>
+  <si>
+    <t>2026-06-24 14:05:00</t>
+  </si>
+  <si>
+    <t>2026-06-24 14:30:00</t>
+  </si>
+  <si>
+    <t>三重溪美店</t>
+  </si>
+  <si>
+    <t>THILF04191</t>
+  </si>
+  <si>
+    <t>2026-06-24 15:09:04</t>
+  </si>
+  <si>
+    <t>2026-06-24 14:41:00</t>
+  </si>
+  <si>
+    <t>2026-06-24 15:06:00</t>
   </si>
 </sst>
 </file>
@@ -3527,7 +3636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK144"/>
+  <dimension ref="A1:AK149"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -15292,55 +15401,55 @@
         <v>38</v>
       </c>
       <c r="C138" s="3">
-        <v>2026062684</v>
+        <v>2026062673</v>
       </c>
       <c r="D138" s="3" t="s">
         <v>959</v>
       </c>
       <c r="E138" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="F138" s="3">
-        <v>4025</v>
+        <v>40</v>
+      </c>
+      <c r="F138" s="3" t="s">
+        <v>960</v>
       </c>
       <c r="G138" s="3" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="H138" s="3" t="s">
-        <v>170</v>
+        <v>209</v>
       </c>
       <c r="I138" s="3" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="J138" s="3" t="s">
-        <v>376</v>
+        <v>88</v>
       </c>
       <c r="K138" s="3" t="s">
-        <v>65</v>
+        <v>325</v>
       </c>
       <c r="L138" s="3" t="s">
-        <v>142</v>
+        <v>46</v>
       </c>
       <c r="M138" s="4" t="s">
-        <v>143</v>
+        <v>47</v>
       </c>
       <c r="N138" s="3">
-        <v>2405</v>
+        <v>2307</v>
       </c>
       <c r="O138" s="4" t="s">
-        <v>267</v>
+        <v>48</v>
       </c>
       <c r="P138" s="10" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="Q138" s="3" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="R138" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S138" s="3" t="s">
-        <v>178</v>
+        <v>52</v>
       </c>
       <c r="T138" s="3">
         <v>1</v>
@@ -15349,26 +15458,26 @@
         <v>53</v>
       </c>
       <c r="V138" s="3" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="W138" s="3" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="X138" s="3" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="Y138" s="3" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="Z138" s="3">
-        <v>1.3</v>
+        <v>0.6</v>
       </c>
       <c r="AA138" s="3"/>
       <c r="AB138" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC138" s="10" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="AD138" s="3"/>
       <c r="AE138" s="3"/>
@@ -15389,25 +15498,25 @@
         <v>38</v>
       </c>
       <c r="C139" s="7">
-        <v>2026062706</v>
+        <v>2026062684</v>
       </c>
       <c r="D139" s="7" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="E139" s="7" t="s">
-        <v>40</v>
+        <v>263</v>
       </c>
       <c r="F139" s="7">
-        <v>4196</v>
+        <v>4025</v>
       </c>
       <c r="G139" s="7" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="H139" s="7" t="s">
-        <v>42</v>
+        <v>170</v>
       </c>
       <c r="I139" s="7" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="J139" s="7" t="s">
         <v>376</v>
@@ -15416,28 +15525,28 @@
         <v>65</v>
       </c>
       <c r="L139" s="7" t="s">
-        <v>46</v>
+        <v>142</v>
       </c>
       <c r="M139" s="8" t="s">
-        <v>47</v>
+        <v>143</v>
       </c>
       <c r="N139" s="7">
-        <v>2305</v>
+        <v>2405</v>
       </c>
       <c r="O139" s="8" t="s">
-        <v>345</v>
+        <v>267</v>
       </c>
       <c r="P139" s="9" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="Q139" s="7" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="R139" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S139" s="7" t="s">
-        <v>52</v>
+        <v>178</v>
       </c>
       <c r="T139" s="7">
         <v>1</v>
@@ -15446,26 +15555,26 @@
         <v>53</v>
       </c>
       <c r="V139" s="7" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="W139" s="7" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="X139" s="7" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="Y139" s="7" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="Z139" s="7">
-        <v>0.4</v>
+        <v>1.3</v>
       </c>
       <c r="AA139" s="7"/>
       <c r="AB139" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC139" s="9" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="AD139" s="7"/>
       <c r="AE139" s="7"/>
@@ -15486,10 +15595,10 @@
         <v>38</v>
       </c>
       <c r="C140" s="3">
-        <v>2026062707</v>
+        <v>2026062706</v>
       </c>
       <c r="D140" s="3" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
       <c r="E140" s="3" t="s">
         <v>40</v>
@@ -15498,13 +15607,13 @@
         <v>4196</v>
       </c>
       <c r="G140" s="3" t="s">
-        <v>970</v>
+        <v>981</v>
       </c>
       <c r="H140" s="3" t="s">
         <v>42</v>
       </c>
       <c r="I140" s="3" t="s">
-        <v>980</v>
+        <v>982</v>
       </c>
       <c r="J140" s="3" t="s">
         <v>376</v>
@@ -15525,10 +15634,10 @@
         <v>345</v>
       </c>
       <c r="P140" s="10" t="s">
-        <v>981</v>
+        <v>983</v>
       </c>
       <c r="Q140" s="3" t="s">
-        <v>973</v>
+        <v>984</v>
       </c>
       <c r="R140" s="3" t="s">
         <v>51</v>
@@ -15543,16 +15652,16 @@
         <v>53</v>
       </c>
       <c r="V140" s="3" t="s">
-        <v>982</v>
+        <v>985</v>
       </c>
       <c r="W140" s="3" t="s">
-        <v>976</v>
+        <v>986</v>
       </c>
       <c r="X140" s="3" t="s">
-        <v>983</v>
+        <v>987</v>
       </c>
       <c r="Y140" s="3" t="s">
-        <v>984</v>
+        <v>988</v>
       </c>
       <c r="Z140" s="3">
         <v>0.4</v>
@@ -15562,7 +15671,7 @@
         <v>58</v>
       </c>
       <c r="AC140" s="10" t="s">
-        <v>985</v>
+        <v>989</v>
       </c>
       <c r="AD140" s="3"/>
       <c r="AE140" s="3"/>
@@ -15580,38 +15689,58 @@
         <v>139</v>
       </c>
       <c r="B141" s="7" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C141" s="7">
-        <v>2026062732</v>
-      </c>
-      <c r="D141" s="7"/>
-      <c r="E141" s="7"/>
+        <v>2026062707</v>
+      </c>
+      <c r="D141" s="7" t="s">
+        <v>990</v>
+      </c>
+      <c r="E141" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F141" s="7">
-        <v>3243</v>
+        <v>4196</v>
       </c>
       <c r="G141" s="7" t="s">
-        <v>986</v>
+        <v>981</v>
       </c>
       <c r="H141" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="I141" s="7"/>
-      <c r="J141" s="7"/>
-      <c r="K141" s="7"/>
-      <c r="L141" s="7"/>
-      <c r="M141" s="8"/>
-      <c r="N141" s="7"/>
-      <c r="O141" s="8"/>
-      <c r="P141" s="9"/>
+        <v>42</v>
+      </c>
+      <c r="I141" s="7" t="s">
+        <v>991</v>
+      </c>
+      <c r="J141" s="7" t="s">
+        <v>376</v>
+      </c>
+      <c r="K141" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L141" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M141" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="N141" s="7">
+        <v>2305</v>
+      </c>
+      <c r="O141" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="P141" s="9" t="s">
+        <v>992</v>
+      </c>
       <c r="Q141" s="7" t="s">
-        <v>987</v>
+        <v>984</v>
       </c>
       <c r="R141" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S141" s="7" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="T141" s="7">
         <v>1</v>
@@ -15620,29 +15749,29 @@
         <v>53</v>
       </c>
       <c r="V141" s="7" t="s">
-        <v>988</v>
+        <v>993</v>
       </c>
       <c r="W141" s="7" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
       <c r="X141" s="7" t="s">
-        <v>990</v>
-      </c>
-      <c r="Y141" s="7"/>
+        <v>994</v>
+      </c>
+      <c r="Y141" s="7" t="s">
+        <v>995</v>
+      </c>
       <c r="Z141" s="7">
-        <v>1.1</v>
+        <v>0.4</v>
       </c>
       <c r="AA141" s="7"/>
       <c r="AB141" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC141" s="9" t="s">
-        <v>991</v>
+        <v>996</v>
       </c>
       <c r="AD141" s="7"/>
-      <c r="AE141" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AE141" s="7"/>
       <c r="AF141" s="7"/>
       <c r="AG141" s="7"/>
       <c r="AH141" s="7"/>
@@ -15660,18 +15789,18 @@
         <v>100</v>
       </c>
       <c r="C142" s="3">
-        <v>2026062748</v>
+        <v>2026062732</v>
       </c>
       <c r="D142" s="3"/>
       <c r="E142" s="3"/>
       <c r="F142" s="3">
-        <v>3818</v>
+        <v>3243</v>
       </c>
       <c r="G142" s="3" t="s">
-        <v>992</v>
+        <v>997</v>
       </c>
       <c r="H142" s="3" t="s">
-        <v>86</v>
+        <v>323</v>
       </c>
       <c r="I142" s="3"/>
       <c r="J142" s="3"/>
@@ -15682,13 +15811,13 @@
       <c r="O142" s="4"/>
       <c r="P142" s="10"/>
       <c r="Q142" s="3" t="s">
-        <v>993</v>
+        <v>998</v>
       </c>
       <c r="R142" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S142" s="3" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="T142" s="3">
         <v>1</v>
@@ -15697,24 +15826,24 @@
         <v>53</v>
       </c>
       <c r="V142" s="3" t="s">
-        <v>994</v>
+        <v>999</v>
       </c>
       <c r="W142" s="3" t="s">
-        <v>995</v>
+        <v>1000</v>
       </c>
       <c r="X142" s="3" t="s">
-        <v>996</v>
+        <v>1001</v>
       </c>
       <c r="Y142" s="3"/>
       <c r="Z142" s="3">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="AA142" s="3"/>
       <c r="AB142" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC142" s="10" t="s">
-        <v>997</v>
+        <v>1002</v>
       </c>
       <c r="AD142" s="3"/>
       <c r="AE142" s="3" t="s">
@@ -15737,18 +15866,18 @@
         <v>100</v>
       </c>
       <c r="C143" s="7">
-        <v>2026062835</v>
+        <v>2026062748</v>
       </c>
       <c r="D143" s="7"/>
       <c r="E143" s="7"/>
       <c r="F143" s="7">
-        <v>4715</v>
+        <v>3818</v>
       </c>
       <c r="G143" s="7" t="s">
-        <v>998</v>
+        <v>1003</v>
       </c>
       <c r="H143" s="7" t="s">
-        <v>323</v>
+        <v>86</v>
       </c>
       <c r="I143" s="7"/>
       <c r="J143" s="7"/>
@@ -15759,13 +15888,13 @@
       <c r="O143" s="8"/>
       <c r="P143" s="9"/>
       <c r="Q143" s="7" t="s">
-        <v>999</v>
+        <v>1004</v>
       </c>
       <c r="R143" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S143" s="7" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="T143" s="7">
         <v>1</v>
@@ -15774,34 +15903,34 @@
         <v>53</v>
       </c>
       <c r="V143" s="7" t="s">
-        <v>1000</v>
+        <v>1005</v>
       </c>
       <c r="W143" s="7" t="s">
-        <v>1001</v>
+        <v>1006</v>
       </c>
       <c r="X143" s="7" t="s">
-        <v>1002</v>
+        <v>1007</v>
       </c>
       <c r="Y143" s="7"/>
       <c r="Z143" s="7">
-        <v>2.4</v>
+        <v>1.3</v>
       </c>
       <c r="AA143" s="7"/>
       <c r="AB143" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC143" s="9" t="s">
-        <v>1003</v>
+        <v>1008</v>
       </c>
       <c r="AD143" s="7"/>
-      <c r="AE143" s="7"/>
+      <c r="AE143" s="7" t="s">
+        <v>60</v>
+      </c>
       <c r="AF143" s="7"/>
       <c r="AG143" s="7"/>
       <c r="AH143" s="7"/>
       <c r="AI143" s="7"/>
-      <c r="AJ143" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ143" s="7"/>
       <c r="AK143" s="7" t="s">
         <v>60</v>
       </c>
@@ -15814,18 +15943,18 @@
         <v>100</v>
       </c>
       <c r="C144" s="3">
-        <v>2026062845</v>
+        <v>2026062835</v>
       </c>
       <c r="D144" s="3"/>
       <c r="E144" s="3"/>
       <c r="F144" s="3">
-        <v>5399</v>
+        <v>4715</v>
       </c>
       <c r="G144" s="3" t="s">
-        <v>1004</v>
+        <v>1009</v>
       </c>
       <c r="H144" s="3" t="s">
-        <v>209</v>
+        <v>323</v>
       </c>
       <c r="I144" s="3"/>
       <c r="J144" s="3"/>
@@ -15834,15 +15963,15 @@
       <c r="M144" s="4"/>
       <c r="N144" s="3"/>
       <c r="O144" s="4"/>
-      <c r="P144" s="4"/>
+      <c r="P144" s="10"/>
       <c r="Q144" s="3" t="s">
-        <v>1005</v>
+        <v>1010</v>
       </c>
       <c r="R144" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S144" s="3" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="T144" s="3">
         <v>1</v>
@@ -15851,28 +15980,26 @@
         <v>53</v>
       </c>
       <c r="V144" s="3" t="s">
-        <v>1006</v>
+        <v>1011</v>
       </c>
       <c r="W144" s="3" t="s">
-        <v>1007</v>
+        <v>1012</v>
       </c>
       <c r="X144" s="3" t="s">
-        <v>1008</v>
+        <v>1013</v>
       </c>
       <c r="Y144" s="3"/>
       <c r="Z144" s="3">
-        <v>0.3</v>
+        <v>2.4</v>
       </c>
       <c r="AA144" s="3"/>
       <c r="AB144" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="AC144" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD144" s="3" t="s">
-        <v>60</v>
-      </c>
+      <c r="AC144" s="10" t="s">
+        <v>1014</v>
+      </c>
+      <c r="AD144" s="3"/>
       <c r="AE144" s="3"/>
       <c r="AF144" s="3"/>
       <c r="AG144" s="3"/>
@@ -15882,6 +16009,419 @@
         <v>60</v>
       </c>
       <c r="AK144" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="145" spans="1:37">
+      <c r="A145" s="7">
+        <v>143</v>
+      </c>
+      <c r="B145" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C145" s="7">
+        <v>2026062845</v>
+      </c>
+      <c r="D145" s="7"/>
+      <c r="E145" s="7"/>
+      <c r="F145" s="7">
+        <v>5399</v>
+      </c>
+      <c r="G145" s="7" t="s">
+        <v>1015</v>
+      </c>
+      <c r="H145" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="I145" s="7"/>
+      <c r="J145" s="7"/>
+      <c r="K145" s="7"/>
+      <c r="L145" s="7"/>
+      <c r="M145" s="8"/>
+      <c r="N145" s="7"/>
+      <c r="O145" s="8"/>
+      <c r="P145" s="9"/>
+      <c r="Q145" s="7" t="s">
+        <v>1016</v>
+      </c>
+      <c r="R145" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S145" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T145" s="7">
+        <v>1</v>
+      </c>
+      <c r="U145" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V145" s="7" t="s">
+        <v>1017</v>
+      </c>
+      <c r="W145" s="7" t="s">
+        <v>1018</v>
+      </c>
+      <c r="X145" s="7" t="s">
+        <v>1019</v>
+      </c>
+      <c r="Y145" s="7"/>
+      <c r="Z145" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA145" s="7"/>
+      <c r="AB145" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC145" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD145" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE145" s="7"/>
+      <c r="AF145" s="7"/>
+      <c r="AG145" s="7"/>
+      <c r="AH145" s="7"/>
+      <c r="AI145" s="7"/>
+      <c r="AJ145" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK145" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="146" spans="1:37">
+      <c r="A146" s="3">
+        <v>144</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C146" s="3">
+        <v>2026063114</v>
+      </c>
+      <c r="D146" s="3" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E146" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F146" s="3">
+        <v>5428</v>
+      </c>
+      <c r="G146" s="3" t="s">
+        <v>1021</v>
+      </c>
+      <c r="H146" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I146" s="3" t="s">
+        <v>1022</v>
+      </c>
+      <c r="J146" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="K146" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L146" s="3" t="s">
+        <v>809</v>
+      </c>
+      <c r="M146" s="4" t="s">
+        <v>810</v>
+      </c>
+      <c r="N146" s="3">
+        <v>5804</v>
+      </c>
+      <c r="O146" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="P146" s="10" t="s">
+        <v>1023</v>
+      </c>
+      <c r="Q146" s="3" t="s">
+        <v>1024</v>
+      </c>
+      <c r="R146" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S146" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T146" s="3">
+        <v>1</v>
+      </c>
+      <c r="U146" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V146" s="3" t="s">
+        <v>1025</v>
+      </c>
+      <c r="W146" s="3" t="s">
+        <v>1026</v>
+      </c>
+      <c r="X146" s="3" t="s">
+        <v>1027</v>
+      </c>
+      <c r="Y146" s="3" t="s">
+        <v>1028</v>
+      </c>
+      <c r="Z146" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA146" s="3"/>
+      <c r="AB146" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC146" s="10" t="s">
+        <v>1029</v>
+      </c>
+      <c r="AD146" s="3"/>
+      <c r="AE146" s="3"/>
+      <c r="AF146" s="3"/>
+      <c r="AG146" s="3"/>
+      <c r="AH146" s="3"/>
+      <c r="AI146" s="3"/>
+      <c r="AJ146" s="3"/>
+      <c r="AK146" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="147" spans="1:37">
+      <c r="A147" s="7">
+        <v>145</v>
+      </c>
+      <c r="B147" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C147" s="7">
+        <v>2026063128</v>
+      </c>
+      <c r="D147" s="7"/>
+      <c r="E147" s="7"/>
+      <c r="F147" s="7">
+        <v>5457</v>
+      </c>
+      <c r="G147" s="7" t="s">
+        <v>1030</v>
+      </c>
+      <c r="H147" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I147" s="7"/>
+      <c r="J147" s="7"/>
+      <c r="K147" s="7"/>
+      <c r="L147" s="7"/>
+      <c r="M147" s="8"/>
+      <c r="N147" s="7"/>
+      <c r="O147" s="8"/>
+      <c r="P147" s="9"/>
+      <c r="Q147" s="7" t="s">
+        <v>1031</v>
+      </c>
+      <c r="R147" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S147" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T147" s="7">
+        <v>1</v>
+      </c>
+      <c r="U147" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V147" s="7" t="s">
+        <v>1032</v>
+      </c>
+      <c r="W147" s="7" t="s">
+        <v>1033</v>
+      </c>
+      <c r="X147" s="7" t="s">
+        <v>1034</v>
+      </c>
+      <c r="Y147" s="7"/>
+      <c r="Z147" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA147" s="7"/>
+      <c r="AB147" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC147" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD147" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE147" s="7"/>
+      <c r="AF147" s="7"/>
+      <c r="AG147" s="7"/>
+      <c r="AH147" s="7"/>
+      <c r="AI147" s="7"/>
+      <c r="AJ147" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK147" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="148" spans="1:37">
+      <c r="A148" s="3">
+        <v>146</v>
+      </c>
+      <c r="B148" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C148" s="3">
+        <v>2026063145</v>
+      </c>
+      <c r="D148" s="3"/>
+      <c r="E148" s="3"/>
+      <c r="F148" s="3">
+        <v>3796</v>
+      </c>
+      <c r="G148" s="3" t="s">
+        <v>1035</v>
+      </c>
+      <c r="H148" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I148" s="3"/>
+      <c r="J148" s="3"/>
+      <c r="K148" s="3"/>
+      <c r="L148" s="3"/>
+      <c r="M148" s="4"/>
+      <c r="N148" s="3"/>
+      <c r="O148" s="4"/>
+      <c r="P148" s="10"/>
+      <c r="Q148" s="3" t="s">
+        <v>1036</v>
+      </c>
+      <c r="R148" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S148" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T148" s="3">
+        <v>1</v>
+      </c>
+      <c r="U148" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V148" s="3" t="s">
+        <v>1037</v>
+      </c>
+      <c r="W148" s="3" t="s">
+        <v>1038</v>
+      </c>
+      <c r="X148" s="3" t="s">
+        <v>1039</v>
+      </c>
+      <c r="Y148" s="3"/>
+      <c r="Z148" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA148" s="3"/>
+      <c r="AB148" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC148" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD148" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE148" s="3"/>
+      <c r="AF148" s="3"/>
+      <c r="AG148" s="3"/>
+      <c r="AH148" s="3"/>
+      <c r="AI148" s="3"/>
+      <c r="AJ148" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK148" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="149" spans="1:37">
+      <c r="A149" s="7">
+        <v>147</v>
+      </c>
+      <c r="B149" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C149" s="7">
+        <v>2026063152</v>
+      </c>
+      <c r="D149" s="7"/>
+      <c r="E149" s="7"/>
+      <c r="F149" s="7">
+        <v>4191</v>
+      </c>
+      <c r="G149" s="7" t="s">
+        <v>1040</v>
+      </c>
+      <c r="H149" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I149" s="7"/>
+      <c r="J149" s="7"/>
+      <c r="K149" s="7"/>
+      <c r="L149" s="7"/>
+      <c r="M149" s="8"/>
+      <c r="N149" s="7"/>
+      <c r="O149" s="8"/>
+      <c r="P149" s="8"/>
+      <c r="Q149" s="7" t="s">
+        <v>1041</v>
+      </c>
+      <c r="R149" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S149" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T149" s="7">
+        <v>1</v>
+      </c>
+      <c r="U149" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V149" s="7" t="s">
+        <v>1042</v>
+      </c>
+      <c r="W149" s="7" t="s">
+        <v>1043</v>
+      </c>
+      <c r="X149" s="7" t="s">
+        <v>1044</v>
+      </c>
+      <c r="Y149" s="7"/>
+      <c r="Z149" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA149" s="7"/>
+      <c r="AB149" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC149" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD149" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE149" s="7"/>
+      <c r="AF149" s="7"/>
+      <c r="AG149" s="7"/>
+      <c r="AH149" s="7"/>
+      <c r="AI149" s="7"/>
+      <c r="AJ149" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK149" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06251756
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$149</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$155</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1045">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-24  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1075">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-25  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -3223,6 +3223,96 @@
   </si>
   <si>
     <t>2026-06-24 15:06:00</t>
+  </si>
+  <si>
+    <t>1T107115062501</t>
+  </si>
+  <si>
+    <t>T107</t>
+  </si>
+  <si>
+    <t>五股訓練教室027401</t>
+  </si>
+  <si>
+    <t>2026-06-25 14:34:03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">台芝湯先生表示到門市保養設備，門市告知訓練教室SC(SHUTTLE7S)無法開啟，點選HISHOP、e網都會出現【捷徑\'HISHOP.lnk\'參照的磁碟機或網路連線無法使用。請確定插入的磁碟正確，而且網路資源可以使用，然後重試。】，重啟SC仍異常。將協助更換第二顆硬碟不備份還原，請客服協助派工，還請台芝協助 PS.若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對) </t>
+  </si>
+  <si>
+    <t>THILF0T107</t>
+  </si>
+  <si>
+    <t>2026-06-25 14:37:30</t>
+  </si>
+  <si>
+    <t>2026-06-25 15:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-25 15:20:00</t>
+  </si>
+  <si>
+    <t>2026-06-26 18:37:00</t>
+  </si>
+  <si>
+    <t>更換一二顆硬碟不備份還原</t>
+  </si>
+  <si>
+    <t>蘆竹六福店</t>
+  </si>
+  <si>
+    <t>THILF02255</t>
+  </si>
+  <si>
+    <t>2026-06-25 15:03:28</t>
+  </si>
+  <si>
+    <t>2026-06-25 11:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-25 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-25 15:03:32</t>
+  </si>
+  <si>
+    <t>2026-06-25 14:20:00</t>
+  </si>
+  <si>
+    <t>2026-06-25 14:50:00</t>
+  </si>
+  <si>
+    <t>2026-06-25 15:44:27</t>
+  </si>
+  <si>
+    <t>裝潢回裝</t>
+  </si>
+  <si>
+    <t>三重金陵店</t>
+  </si>
+  <si>
+    <t>THILF03359</t>
+  </si>
+  <si>
+    <t>2026-06-25 16:31:21</t>
+  </si>
+  <si>
+    <t>2026-06-25 16:05:00</t>
+  </si>
+  <si>
+    <t>2026-06-25 16:25:00</t>
+  </si>
+  <si>
+    <t>TT01</t>
+  </si>
+  <si>
+    <t>五股訓練教室</t>
+  </si>
+  <si>
+    <t>THILF0TT01</t>
+  </si>
+  <si>
+    <t>2026-06-25 16:52:21</t>
   </si>
 </sst>
 </file>
@@ -3636,7 +3726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK149"/>
+  <dimension ref="A1:AK155"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -16374,7 +16464,7 @@
       <c r="M149" s="8"/>
       <c r="N149" s="7"/>
       <c r="O149" s="8"/>
-      <c r="P149" s="8"/>
+      <c r="P149" s="9"/>
       <c r="Q149" s="7" t="s">
         <v>1041</v>
       </c>
@@ -16407,7 +16497,7 @@
       <c r="AB149" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC149" s="8" t="s">
+      <c r="AC149" s="9" t="s">
         <v>111</v>
       </c>
       <c r="AD149" s="7" t="s">
@@ -16422,6 +16512,492 @@
         <v>60</v>
       </c>
       <c r="AK149" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="150" spans="1:37">
+      <c r="A150" s="3">
+        <v>148</v>
+      </c>
+      <c r="B150" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C150" s="3">
+        <v>2026063278</v>
+      </c>
+      <c r="D150" s="3" t="s">
+        <v>1045</v>
+      </c>
+      <c r="E150" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F150" s="3" t="s">
+        <v>1046</v>
+      </c>
+      <c r="G150" s="3" t="s">
+        <v>1047</v>
+      </c>
+      <c r="H150" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="I150" s="3" t="s">
+        <v>1048</v>
+      </c>
+      <c r="J150" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K150" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L150" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="M150" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="N150" s="3">
+        <v>2405</v>
+      </c>
+      <c r="O150" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="P150" s="10" t="s">
+        <v>1049</v>
+      </c>
+      <c r="Q150" s="3" t="s">
+        <v>1050</v>
+      </c>
+      <c r="R150" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S150" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T150" s="3">
+        <v>1</v>
+      </c>
+      <c r="U150" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V150" s="3" t="s">
+        <v>1051</v>
+      </c>
+      <c r="W150" s="3" t="s">
+        <v>1052</v>
+      </c>
+      <c r="X150" s="3" t="s">
+        <v>1053</v>
+      </c>
+      <c r="Y150" s="3" t="s">
+        <v>1054</v>
+      </c>
+      <c r="Z150" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA150" s="3"/>
+      <c r="AB150" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC150" s="10" t="s">
+        <v>1055</v>
+      </c>
+      <c r="AD150" s="3"/>
+      <c r="AE150" s="3"/>
+      <c r="AF150" s="3"/>
+      <c r="AG150" s="3"/>
+      <c r="AH150" s="3"/>
+      <c r="AI150" s="3"/>
+      <c r="AJ150" s="3"/>
+      <c r="AK150" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="151" spans="1:37">
+      <c r="A151" s="7">
+        <v>149</v>
+      </c>
+      <c r="B151" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C151" s="7">
+        <v>2026063281</v>
+      </c>
+      <c r="D151" s="7"/>
+      <c r="E151" s="7"/>
+      <c r="F151" s="7">
+        <v>2255</v>
+      </c>
+      <c r="G151" s="7" t="s">
+        <v>1056</v>
+      </c>
+      <c r="H151" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I151" s="7"/>
+      <c r="J151" s="7"/>
+      <c r="K151" s="7"/>
+      <c r="L151" s="7"/>
+      <c r="M151" s="8"/>
+      <c r="N151" s="7"/>
+      <c r="O151" s="8"/>
+      <c r="P151" s="9"/>
+      <c r="Q151" s="7" t="s">
+        <v>1057</v>
+      </c>
+      <c r="R151" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S151" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T151" s="7">
+        <v>1</v>
+      </c>
+      <c r="U151" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V151" s="7" t="s">
+        <v>1058</v>
+      </c>
+      <c r="W151" s="7" t="s">
+        <v>1059</v>
+      </c>
+      <c r="X151" s="7" t="s">
+        <v>1060</v>
+      </c>
+      <c r="Y151" s="7"/>
+      <c r="Z151" s="7">
+        <v>3</v>
+      </c>
+      <c r="AA151" s="7"/>
+      <c r="AB151" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC151" s="9" t="s">
+        <v>725</v>
+      </c>
+      <c r="AD151" s="7"/>
+      <c r="AE151" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF151" s="7"/>
+      <c r="AG151" s="7"/>
+      <c r="AH151" s="7"/>
+      <c r="AI151" s="7"/>
+      <c r="AJ151" s="7"/>
+      <c r="AK151" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="152" spans="1:37">
+      <c r="A152" s="3">
+        <v>150</v>
+      </c>
+      <c r="B152" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C152" s="3">
+        <v>2026063282</v>
+      </c>
+      <c r="D152" s="3"/>
+      <c r="E152" s="3"/>
+      <c r="F152" s="3">
+        <v>2255</v>
+      </c>
+      <c r="G152" s="3" t="s">
+        <v>1056</v>
+      </c>
+      <c r="H152" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="I152" s="3"/>
+      <c r="J152" s="3"/>
+      <c r="K152" s="3"/>
+      <c r="L152" s="3"/>
+      <c r="M152" s="4"/>
+      <c r="N152" s="3"/>
+      <c r="O152" s="4"/>
+      <c r="P152" s="10"/>
+      <c r="Q152" s="3" t="s">
+        <v>1057</v>
+      </c>
+      <c r="R152" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S152" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T152" s="3">
+        <v>1</v>
+      </c>
+      <c r="U152" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V152" s="3" t="s">
+        <v>1061</v>
+      </c>
+      <c r="W152" s="3" t="s">
+        <v>1062</v>
+      </c>
+      <c r="X152" s="3" t="s">
+        <v>1063</v>
+      </c>
+      <c r="Y152" s="3"/>
+      <c r="Z152" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA152" s="3"/>
+      <c r="AB152" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC152" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD152" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE152" s="3"/>
+      <c r="AF152" s="3"/>
+      <c r="AG152" s="3"/>
+      <c r="AH152" s="3"/>
+      <c r="AI152" s="3"/>
+      <c r="AJ152" s="3"/>
+      <c r="AK152" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="153" spans="1:37">
+      <c r="A153" s="7">
+        <v>151</v>
+      </c>
+      <c r="B153" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C153" s="7">
+        <v>2026063301</v>
+      </c>
+      <c r="D153" s="7"/>
+      <c r="E153" s="7"/>
+      <c r="F153" s="7">
+        <v>2255</v>
+      </c>
+      <c r="G153" s="7" t="s">
+        <v>1056</v>
+      </c>
+      <c r="H153" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I153" s="7"/>
+      <c r="J153" s="7"/>
+      <c r="K153" s="7"/>
+      <c r="L153" s="7"/>
+      <c r="M153" s="8"/>
+      <c r="N153" s="7"/>
+      <c r="O153" s="8"/>
+      <c r="P153" s="9"/>
+      <c r="Q153" s="7" t="s">
+        <v>1057</v>
+      </c>
+      <c r="R153" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S153" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T153" s="7">
+        <v>1</v>
+      </c>
+      <c r="U153" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V153" s="7" t="s">
+        <v>1064</v>
+      </c>
+      <c r="W153" s="7" t="s">
+        <v>1059</v>
+      </c>
+      <c r="X153" s="7" t="s">
+        <v>1060</v>
+      </c>
+      <c r="Y153" s="7"/>
+      <c r="Z153" s="7">
+        <v>3</v>
+      </c>
+      <c r="AA153" s="7"/>
+      <c r="AB153" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC153" s="9" t="s">
+        <v>1065</v>
+      </c>
+      <c r="AD153" s="7"/>
+      <c r="AE153" s="7"/>
+      <c r="AF153" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG153" s="7"/>
+      <c r="AH153" s="7"/>
+      <c r="AI153" s="7"/>
+      <c r="AJ153" s="7"/>
+      <c r="AK153" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="154" spans="1:37">
+      <c r="A154" s="3">
+        <v>152</v>
+      </c>
+      <c r="B154" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C154" s="3">
+        <v>2026063311</v>
+      </c>
+      <c r="D154" s="3"/>
+      <c r="E154" s="3"/>
+      <c r="F154" s="3">
+        <v>3359</v>
+      </c>
+      <c r="G154" s="3" t="s">
+        <v>1066</v>
+      </c>
+      <c r="H154" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I154" s="3"/>
+      <c r="J154" s="3"/>
+      <c r="K154" s="3"/>
+      <c r="L154" s="3"/>
+      <c r="M154" s="4"/>
+      <c r="N154" s="3"/>
+      <c r="O154" s="4"/>
+      <c r="P154" s="10"/>
+      <c r="Q154" s="3" t="s">
+        <v>1067</v>
+      </c>
+      <c r="R154" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S154" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T154" s="3">
+        <v>1</v>
+      </c>
+      <c r="U154" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V154" s="3" t="s">
+        <v>1068</v>
+      </c>
+      <c r="W154" s="3" t="s">
+        <v>1069</v>
+      </c>
+      <c r="X154" s="3" t="s">
+        <v>1070</v>
+      </c>
+      <c r="Y154" s="3"/>
+      <c r="Z154" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA154" s="3"/>
+      <c r="AB154" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC154" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD154" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE154" s="3"/>
+      <c r="AF154" s="3"/>
+      <c r="AG154" s="3"/>
+      <c r="AH154" s="3"/>
+      <c r="AI154" s="3"/>
+      <c r="AJ154" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK154" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="155" spans="1:37">
+      <c r="A155" s="7">
+        <v>153</v>
+      </c>
+      <c r="B155" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C155" s="7">
+        <v>2026063315</v>
+      </c>
+      <c r="D155" s="7"/>
+      <c r="E155" s="7"/>
+      <c r="F155" s="7" t="s">
+        <v>1071</v>
+      </c>
+      <c r="G155" s="7" t="s">
+        <v>1072</v>
+      </c>
+      <c r="H155" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I155" s="7"/>
+      <c r="J155" s="7"/>
+      <c r="K155" s="7"/>
+      <c r="L155" s="7"/>
+      <c r="M155" s="8"/>
+      <c r="N155" s="7"/>
+      <c r="O155" s="8"/>
+      <c r="P155" s="8"/>
+      <c r="Q155" s="7" t="s">
+        <v>1073</v>
+      </c>
+      <c r="R155" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S155" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T155" s="7">
+        <v>1</v>
+      </c>
+      <c r="U155" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V155" s="7" t="s">
+        <v>1074</v>
+      </c>
+      <c r="W155" s="7" t="s">
+        <v>1060</v>
+      </c>
+      <c r="X155" s="7" t="s">
+        <v>1052</v>
+      </c>
+      <c r="Y155" s="7"/>
+      <c r="Z155" s="7">
+        <v>1</v>
+      </c>
+      <c r="AA155" s="7"/>
+      <c r="AB155" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC155" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD155" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE155" s="7"/>
+      <c r="AF155" s="7"/>
+      <c r="AG155" s="7"/>
+      <c r="AH155" s="7"/>
+      <c r="AI155" s="7"/>
+      <c r="AJ155" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK155" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06261534
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$155</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$172</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1075">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-25  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1175">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-26  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -3313,6 +3313,309 @@
   </si>
   <si>
     <t>2026-06-25 16:52:21</t>
+  </si>
+  <si>
+    <t>14528115062601</t>
+  </si>
+  <si>
+    <t>八里鐵塔店</t>
+  </si>
+  <si>
+    <t>2026-06-26 09:51:48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06/29 10:00 與總公司宸宇確認啟動緊急叫修:門市反應訂貨3.0點選傳輸後會出現I/O error 1392，客服查看門市TM兩台、SC主檔錯誤，協助接收總公司主檔&gt;手動主檔轉入後SC主檔正確但執行SC轉TM時出現訊息:SC資料轉檔失敗，請通知總公司。檔案或目錄損毀而且無法讀取。總公司健誌副理:Computer: H4528  Description: 在磁碟區 E: 的檔案系統結構中發現損毀。請到店更換SC(SHUTTLE6S)第二顆硬碟，不要備份。....請台芝到店協助
+PS.若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對)																																
+與門市確認帳務做到06/25，與通訊健誌副理確認有收到06/25的銷售																										
+</t>
+  </si>
+  <si>
+    <t>THILF04528</t>
+  </si>
+  <si>
+    <t>2026-06-26 10:05:21</t>
+  </si>
+  <si>
+    <t>2026-06-26 10:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-26 12:33:00</t>
+  </si>
+  <si>
+    <t>2026-06-26 16:05:00</t>
+  </si>
+  <si>
+    <t>更換第二顆硬碟不備份還原完成</t>
+  </si>
+  <si>
+    <t>E2540115062601</t>
+  </si>
+  <si>
+    <t>蘆竹坑子口</t>
+  </si>
+  <si>
+    <t>2026-06-26 10:01:24</t>
+  </si>
+  <si>
+    <t>當機或無畫面</t>
+  </si>
+  <si>
+    <t>門市反應從交接這間門市後LIFE-ET4一直都無上方透明廣告看板......需請台芝到店協助(LIFE-ET上方壓克力背板遺失)</t>
+  </si>
+  <si>
+    <t>THILF02540</t>
+  </si>
+  <si>
+    <t>2026-06-26 10:08:10</t>
+  </si>
+  <si>
+    <t>2026-06-26 13:13:00</t>
+  </si>
+  <si>
+    <t>2026-06-26 13:43:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 14:08:00</t>
+  </si>
+  <si>
+    <t>安裝MMK看板完成</t>
+  </si>
+  <si>
+    <t>五股五工店</t>
+  </si>
+  <si>
+    <t>THILF02535</t>
+  </si>
+  <si>
+    <t>2026-06-26 10:38:13</t>
+  </si>
+  <si>
+    <t>2026-06-26 10:10:00</t>
+  </si>
+  <si>
+    <t>2026-06-26 10:40:00</t>
+  </si>
+  <si>
+    <t>12535115062601</t>
+  </si>
+  <si>
+    <t>2026-06-26 10:43:50</t>
+  </si>
+  <si>
+    <t>門市反應tm1 ccd掃描器(HC76-TR)無法刷讀ipsaamoney條碼，有些消費者的可以有些消費者的不行，已有將手機亮度調整到最高且掃槍也有執行校正仍異常....請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-06-26 10:46:38</t>
+  </si>
+  <si>
+    <t>2026-06-26 13:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-26 13:20:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 14:46:00</t>
+  </si>
+  <si>
+    <t>到場測試正常</t>
+  </si>
+  <si>
+    <t>12535115062602</t>
+  </si>
+  <si>
+    <t>2026-06-26 10:46:11</t>
+  </si>
+  <si>
+    <t>門市反應tm2 ccd掃描器(HC76-TR)無法刷讀ipsaamoney條碼，有些消費者的可以有些消費者的不行，已有將手機亮度調整到最高且掃槍也有執行校正仍異常....請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-06-26 10:46:46</t>
+  </si>
+  <si>
+    <t>2026-06-26 13:40:00</t>
+  </si>
+  <si>
+    <t>12535115062603</t>
+  </si>
+  <si>
+    <t>2026-06-26 10:46:24</t>
+  </si>
+  <si>
+    <t>門市反應tm3 ccd掃描器(HC76-TR)無法刷讀ipsaamoney條碼，有些消費者的可以有些消費者的不行，已有將手機亮度調整到最高且掃槍也有執行校正仍異常....請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-06-26 10:46:57</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:00:00</t>
+  </si>
+  <si>
+    <t>L516</t>
+  </si>
+  <si>
+    <t>車麗屋新莊店</t>
+  </si>
+  <si>
+    <t>THILF0L516</t>
+  </si>
+  <si>
+    <t>2026-06-26 11:03:20</t>
+  </si>
+  <si>
+    <t>2026-06-26 11:00:00</t>
+  </si>
+  <si>
+    <t>板橋福康店</t>
+  </si>
+  <si>
+    <t>THILF04046</t>
+  </si>
+  <si>
+    <t>2026-06-26 13:18:31</t>
+  </si>
+  <si>
+    <t>2026-06-26 12:35:00</t>
+  </si>
+  <si>
+    <t>2026-06-26 12:58:00</t>
+  </si>
+  <si>
+    <t>D161</t>
+  </si>
+  <si>
+    <t>板橋僑中三</t>
+  </si>
+  <si>
+    <t>THILF0D161</t>
+  </si>
+  <si>
+    <t>2026-06-26 13:20:46</t>
+  </si>
+  <si>
+    <t>2026-06-26 13:18:00</t>
+  </si>
+  <si>
+    <t>板橋僑興店</t>
+  </si>
+  <si>
+    <t>THILF04145</t>
+  </si>
+  <si>
+    <t>2026-06-26 13:40:17</t>
+  </si>
+  <si>
+    <t>2026-06-26 13:23:00</t>
+  </si>
+  <si>
+    <t>2026-06-26 13:38:00</t>
+  </si>
+  <si>
+    <t>板橋板龍店</t>
+  </si>
+  <si>
+    <t>THILF02403</t>
+  </si>
+  <si>
+    <t>2026-06-26 13:56:35</t>
+  </si>
+  <si>
+    <t>2026-06-26 13:53:00</t>
+  </si>
+  <si>
+    <t>12535115062604</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:03:39</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:03:52</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:05:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 18:03:00</t>
+  </si>
+  <si>
+    <t>取消報修</t>
+  </si>
+  <si>
+    <t>12535115062605</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:04:20</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:04:36</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:10:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 18:04:00</t>
+  </si>
+  <si>
+    <t>12535115062606</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:04:52</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:05:08</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:15:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 18:05:00</t>
+  </si>
+  <si>
+    <t>D609</t>
+  </si>
+  <si>
+    <t>板橋大興店</t>
+  </si>
+  <si>
+    <t>THILF0D609</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:13:59</t>
+  </si>
+  <si>
+    <t>2026-06-26 13:57:00</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:12:00</t>
+  </si>
+  <si>
+    <t>三重中央南</t>
+  </si>
+  <si>
+    <t>THILF04083</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:56:35</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:53:00</t>
+  </si>
+  <si>
+    <t>三重三和夜市</t>
+  </si>
+  <si>
+    <t>THILF02303</t>
+  </si>
+  <si>
+    <t>2026-06-26 15:25:32</t>
+  </si>
+  <si>
+    <t>2026-06-26 14:59:00</t>
+  </si>
+  <si>
+    <t>2026-06-26 15:20:00</t>
   </si>
 </sst>
 </file>
@@ -3726,7 +4029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK155"/>
+  <dimension ref="A1:AK172"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -16950,7 +17253,7 @@
       <c r="M155" s="8"/>
       <c r="N155" s="7"/>
       <c r="O155" s="8"/>
-      <c r="P155" s="8"/>
+      <c r="P155" s="9"/>
       <c r="Q155" s="7" t="s">
         <v>1073</v>
       </c>
@@ -16983,7 +17286,7 @@
       <c r="AB155" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC155" s="8" t="s">
+      <c r="AC155" s="9" t="s">
         <v>111</v>
       </c>
       <c r="AD155" s="7" t="s">
@@ -16998,6 +17301,1477 @@
         <v>60</v>
       </c>
       <c r="AK155" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="156" spans="1:37">
+      <c r="A156" s="3">
+        <v>154</v>
+      </c>
+      <c r="B156" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C156" s="3">
+        <v>2026063334</v>
+      </c>
+      <c r="D156" s="3" t="s">
+        <v>1075</v>
+      </c>
+      <c r="E156" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="F156" s="3">
+        <v>4528</v>
+      </c>
+      <c r="G156" s="3" t="s">
+        <v>1076</v>
+      </c>
+      <c r="H156" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="I156" s="3" t="s">
+        <v>1077</v>
+      </c>
+      <c r="J156" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K156" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L156" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="M156" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="N156" s="3">
+        <v>2405</v>
+      </c>
+      <c r="O156" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="P156" s="10" t="s">
+        <v>1078</v>
+      </c>
+      <c r="Q156" s="3" t="s">
+        <v>1079</v>
+      </c>
+      <c r="R156" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S156" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T156" s="3">
+        <v>1</v>
+      </c>
+      <c r="U156" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V156" s="3" t="s">
+        <v>1080</v>
+      </c>
+      <c r="W156" s="3" t="s">
+        <v>1081</v>
+      </c>
+      <c r="X156" s="3" t="s">
+        <v>1082</v>
+      </c>
+      <c r="Y156" s="3" t="s">
+        <v>1083</v>
+      </c>
+      <c r="Z156" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="AA156" s="3"/>
+      <c r="AB156" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC156" s="10" t="s">
+        <v>1084</v>
+      </c>
+      <c r="AD156" s="3"/>
+      <c r="AE156" s="3"/>
+      <c r="AF156" s="3"/>
+      <c r="AG156" s="3"/>
+      <c r="AH156" s="3"/>
+      <c r="AI156" s="3"/>
+      <c r="AJ156" s="3"/>
+      <c r="AK156" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="157" spans="1:37">
+      <c r="A157" s="7">
+        <v>155</v>
+      </c>
+      <c r="B157" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C157" s="7">
+        <v>2026063335</v>
+      </c>
+      <c r="D157" s="7" t="s">
+        <v>1085</v>
+      </c>
+      <c r="E157" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F157" s="7">
+        <v>2540</v>
+      </c>
+      <c r="G157" s="7" t="s">
+        <v>1086</v>
+      </c>
+      <c r="H157" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I157" s="7" t="s">
+        <v>1087</v>
+      </c>
+      <c r="J157" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="K157" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L157" s="7" t="s">
+        <v>809</v>
+      </c>
+      <c r="M157" s="8" t="s">
+        <v>810</v>
+      </c>
+      <c r="N157" s="7">
+        <v>5801</v>
+      </c>
+      <c r="O157" s="8" t="s">
+        <v>1088</v>
+      </c>
+      <c r="P157" s="9" t="s">
+        <v>1089</v>
+      </c>
+      <c r="Q157" s="7" t="s">
+        <v>1090</v>
+      </c>
+      <c r="R157" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S157" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T157" s="7">
+        <v>1</v>
+      </c>
+      <c r="U157" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V157" s="7" t="s">
+        <v>1091</v>
+      </c>
+      <c r="W157" s="7" t="s">
+        <v>1092</v>
+      </c>
+      <c r="X157" s="7" t="s">
+        <v>1093</v>
+      </c>
+      <c r="Y157" s="7" t="s">
+        <v>1094</v>
+      </c>
+      <c r="Z157" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA157" s="7"/>
+      <c r="AB157" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC157" s="9" t="s">
+        <v>1095</v>
+      </c>
+      <c r="AD157" s="7"/>
+      <c r="AE157" s="7"/>
+      <c r="AF157" s="7"/>
+      <c r="AG157" s="7"/>
+      <c r="AH157" s="7"/>
+      <c r="AI157" s="7"/>
+      <c r="AJ157" s="7"/>
+      <c r="AK157" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="158" spans="1:37">
+      <c r="A158" s="3">
+        <v>156</v>
+      </c>
+      <c r="B158" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C158" s="3">
+        <v>2026063339</v>
+      </c>
+      <c r="D158" s="3"/>
+      <c r="E158" s="3"/>
+      <c r="F158" s="3">
+        <v>2535</v>
+      </c>
+      <c r="G158" s="3" t="s">
+        <v>1096</v>
+      </c>
+      <c r="H158" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="I158" s="3"/>
+      <c r="J158" s="3"/>
+      <c r="K158" s="3"/>
+      <c r="L158" s="3"/>
+      <c r="M158" s="4"/>
+      <c r="N158" s="3"/>
+      <c r="O158" s="4"/>
+      <c r="P158" s="10"/>
+      <c r="Q158" s="3" t="s">
+        <v>1097</v>
+      </c>
+      <c r="R158" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S158" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T158" s="3">
+        <v>1</v>
+      </c>
+      <c r="U158" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V158" s="3" t="s">
+        <v>1098</v>
+      </c>
+      <c r="W158" s="3" t="s">
+        <v>1099</v>
+      </c>
+      <c r="X158" s="3" t="s">
+        <v>1100</v>
+      </c>
+      <c r="Y158" s="3"/>
+      <c r="Z158" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA158" s="3"/>
+      <c r="AB158" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC158" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD158" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE158" s="3"/>
+      <c r="AF158" s="3"/>
+      <c r="AG158" s="3"/>
+      <c r="AH158" s="3"/>
+      <c r="AI158" s="3"/>
+      <c r="AJ158" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK158" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="159" spans="1:37">
+      <c r="A159" s="7">
+        <v>157</v>
+      </c>
+      <c r="B159" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C159" s="7">
+        <v>2026063341</v>
+      </c>
+      <c r="D159" s="7" t="s">
+        <v>1101</v>
+      </c>
+      <c r="E159" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F159" s="7">
+        <v>2535</v>
+      </c>
+      <c r="G159" s="7" t="s">
+        <v>1096</v>
+      </c>
+      <c r="H159" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I159" s="7" t="s">
+        <v>1102</v>
+      </c>
+      <c r="J159" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="K159" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L159" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="M159" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="N159" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="O159" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="P159" s="9" t="s">
+        <v>1103</v>
+      </c>
+      <c r="Q159" s="7" t="s">
+        <v>1097</v>
+      </c>
+      <c r="R159" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S159" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T159" s="7">
+        <v>1</v>
+      </c>
+      <c r="U159" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V159" s="7" t="s">
+        <v>1104</v>
+      </c>
+      <c r="W159" s="7" t="s">
+        <v>1105</v>
+      </c>
+      <c r="X159" s="7" t="s">
+        <v>1106</v>
+      </c>
+      <c r="Y159" s="7" t="s">
+        <v>1107</v>
+      </c>
+      <c r="Z159" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA159" s="7"/>
+      <c r="AB159" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC159" s="9" t="s">
+        <v>1108</v>
+      </c>
+      <c r="AD159" s="7"/>
+      <c r="AE159" s="7"/>
+      <c r="AF159" s="7"/>
+      <c r="AG159" s="7"/>
+      <c r="AH159" s="7"/>
+      <c r="AI159" s="7"/>
+      <c r="AJ159" s="7"/>
+      <c r="AK159" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="160" spans="1:37">
+      <c r="A160" s="3">
+        <v>158</v>
+      </c>
+      <c r="B160" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C160" s="3">
+        <v>2026063342</v>
+      </c>
+      <c r="D160" s="3" t="s">
+        <v>1109</v>
+      </c>
+      <c r="E160" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F160" s="3">
+        <v>2535</v>
+      </c>
+      <c r="G160" s="3" t="s">
+        <v>1096</v>
+      </c>
+      <c r="H160" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="I160" s="3" t="s">
+        <v>1110</v>
+      </c>
+      <c r="J160" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K160" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L160" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="M160" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="N160" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="O160" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="P160" s="10" t="s">
+        <v>1111</v>
+      </c>
+      <c r="Q160" s="3" t="s">
+        <v>1097</v>
+      </c>
+      <c r="R160" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S160" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T160" s="3">
+        <v>1</v>
+      </c>
+      <c r="U160" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V160" s="3" t="s">
+        <v>1112</v>
+      </c>
+      <c r="W160" s="3" t="s">
+        <v>1106</v>
+      </c>
+      <c r="X160" s="3" t="s">
+        <v>1113</v>
+      </c>
+      <c r="Y160" s="3" t="s">
+        <v>1107</v>
+      </c>
+      <c r="Z160" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA160" s="3"/>
+      <c r="AB160" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC160" s="10" t="s">
+        <v>1108</v>
+      </c>
+      <c r="AD160" s="3"/>
+      <c r="AE160" s="3"/>
+      <c r="AF160" s="3"/>
+      <c r="AG160" s="3"/>
+      <c r="AH160" s="3"/>
+      <c r="AI160" s="3"/>
+      <c r="AJ160" s="3"/>
+      <c r="AK160" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="161" spans="1:37">
+      <c r="A161" s="7">
+        <v>159</v>
+      </c>
+      <c r="B161" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C161" s="7">
+        <v>2026063343</v>
+      </c>
+      <c r="D161" s="7" t="s">
+        <v>1114</v>
+      </c>
+      <c r="E161" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F161" s="7">
+        <v>2535</v>
+      </c>
+      <c r="G161" s="7" t="s">
+        <v>1096</v>
+      </c>
+      <c r="H161" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I161" s="7" t="s">
+        <v>1115</v>
+      </c>
+      <c r="J161" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="K161" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L161" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="M161" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="N161" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="O161" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="P161" s="9" t="s">
+        <v>1116</v>
+      </c>
+      <c r="Q161" s="7" t="s">
+        <v>1097</v>
+      </c>
+      <c r="R161" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S161" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T161" s="7">
+        <v>1</v>
+      </c>
+      <c r="U161" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V161" s="7" t="s">
+        <v>1117</v>
+      </c>
+      <c r="W161" s="7" t="s">
+        <v>1113</v>
+      </c>
+      <c r="X161" s="7" t="s">
+        <v>1118</v>
+      </c>
+      <c r="Y161" s="7" t="s">
+        <v>1107</v>
+      </c>
+      <c r="Z161" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA161" s="7"/>
+      <c r="AB161" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC161" s="9" t="s">
+        <v>1108</v>
+      </c>
+      <c r="AD161" s="7"/>
+      <c r="AE161" s="7"/>
+      <c r="AF161" s="7"/>
+      <c r="AG161" s="7"/>
+      <c r="AH161" s="7"/>
+      <c r="AI161" s="7"/>
+      <c r="AJ161" s="7"/>
+      <c r="AK161" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="162" spans="1:37">
+      <c r="A162" s="3">
+        <v>160</v>
+      </c>
+      <c r="B162" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C162" s="3">
+        <v>2026063344</v>
+      </c>
+      <c r="D162" s="3"/>
+      <c r="E162" s="3"/>
+      <c r="F162" s="3" t="s">
+        <v>1119</v>
+      </c>
+      <c r="G162" s="3" t="s">
+        <v>1120</v>
+      </c>
+      <c r="H162" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="I162" s="3"/>
+      <c r="J162" s="3"/>
+      <c r="K162" s="3"/>
+      <c r="L162" s="3"/>
+      <c r="M162" s="4"/>
+      <c r="N162" s="3"/>
+      <c r="O162" s="4"/>
+      <c r="P162" s="10"/>
+      <c r="Q162" s="3" t="s">
+        <v>1121</v>
+      </c>
+      <c r="R162" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S162" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T162" s="3">
+        <v>1</v>
+      </c>
+      <c r="U162" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V162" s="3" t="s">
+        <v>1122</v>
+      </c>
+      <c r="W162" s="3" t="s">
+        <v>1100</v>
+      </c>
+      <c r="X162" s="3" t="s">
+        <v>1123</v>
+      </c>
+      <c r="Y162" s="3"/>
+      <c r="Z162" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA162" s="3"/>
+      <c r="AB162" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC162" s="10" t="s">
+        <v>476</v>
+      </c>
+      <c r="AD162" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE162" s="3"/>
+      <c r="AF162" s="3"/>
+      <c r="AG162" s="3"/>
+      <c r="AH162" s="3"/>
+      <c r="AI162" s="3"/>
+      <c r="AJ162" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK162" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="163" spans="1:37">
+      <c r="A163" s="7">
+        <v>161</v>
+      </c>
+      <c r="B163" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C163" s="7">
+        <v>2026063378</v>
+      </c>
+      <c r="D163" s="7"/>
+      <c r="E163" s="7"/>
+      <c r="F163" s="7">
+        <v>4046</v>
+      </c>
+      <c r="G163" s="7" t="s">
+        <v>1124</v>
+      </c>
+      <c r="H163" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I163" s="7"/>
+      <c r="J163" s="7"/>
+      <c r="K163" s="7"/>
+      <c r="L163" s="7"/>
+      <c r="M163" s="8"/>
+      <c r="N163" s="7"/>
+      <c r="O163" s="8"/>
+      <c r="P163" s="9"/>
+      <c r="Q163" s="7" t="s">
+        <v>1125</v>
+      </c>
+      <c r="R163" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S163" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="T163" s="7">
+        <v>1</v>
+      </c>
+      <c r="U163" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V163" s="7" t="s">
+        <v>1126</v>
+      </c>
+      <c r="W163" s="7" t="s">
+        <v>1127</v>
+      </c>
+      <c r="X163" s="7" t="s">
+        <v>1128</v>
+      </c>
+      <c r="Y163" s="7"/>
+      <c r="Z163" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA163" s="7"/>
+      <c r="AB163" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC163" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD163" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE163" s="7"/>
+      <c r="AF163" s="7"/>
+      <c r="AG163" s="7"/>
+      <c r="AH163" s="7"/>
+      <c r="AI163" s="7"/>
+      <c r="AJ163" s="7"/>
+      <c r="AK163" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="164" spans="1:37">
+      <c r="A164" s="3">
+        <v>162</v>
+      </c>
+      <c r="B164" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C164" s="3">
+        <v>2026063379</v>
+      </c>
+      <c r="D164" s="3"/>
+      <c r="E164" s="3"/>
+      <c r="F164" s="3" t="s">
+        <v>1129</v>
+      </c>
+      <c r="G164" s="3" t="s">
+        <v>1130</v>
+      </c>
+      <c r="H164" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I164" s="3"/>
+      <c r="J164" s="3"/>
+      <c r="K164" s="3"/>
+      <c r="L164" s="3"/>
+      <c r="M164" s="4"/>
+      <c r="N164" s="3"/>
+      <c r="O164" s="4"/>
+      <c r="P164" s="10"/>
+      <c r="Q164" s="3" t="s">
+        <v>1131</v>
+      </c>
+      <c r="R164" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S164" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="T164" s="3">
+        <v>1</v>
+      </c>
+      <c r="U164" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V164" s="3" t="s">
+        <v>1132</v>
+      </c>
+      <c r="W164" s="3" t="s">
+        <v>1105</v>
+      </c>
+      <c r="X164" s="3" t="s">
+        <v>1133</v>
+      </c>
+      <c r="Y164" s="3"/>
+      <c r="Z164" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA164" s="3"/>
+      <c r="AB164" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC164" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD164" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE164" s="3"/>
+      <c r="AF164" s="3"/>
+      <c r="AG164" s="3"/>
+      <c r="AH164" s="3"/>
+      <c r="AI164" s="3"/>
+      <c r="AJ164" s="3"/>
+      <c r="AK164" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="165" spans="1:37">
+      <c r="A165" s="7">
+        <v>163</v>
+      </c>
+      <c r="B165" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C165" s="7">
+        <v>2026063380</v>
+      </c>
+      <c r="D165" s="7"/>
+      <c r="E165" s="7"/>
+      <c r="F165" s="7">
+        <v>4145</v>
+      </c>
+      <c r="G165" s="7" t="s">
+        <v>1134</v>
+      </c>
+      <c r="H165" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I165" s="7"/>
+      <c r="J165" s="7"/>
+      <c r="K165" s="7"/>
+      <c r="L165" s="7"/>
+      <c r="M165" s="8"/>
+      <c r="N165" s="7"/>
+      <c r="O165" s="8"/>
+      <c r="P165" s="9"/>
+      <c r="Q165" s="7" t="s">
+        <v>1135</v>
+      </c>
+      <c r="R165" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S165" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="T165" s="7">
+        <v>1</v>
+      </c>
+      <c r="U165" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V165" s="7" t="s">
+        <v>1136</v>
+      </c>
+      <c r="W165" s="7" t="s">
+        <v>1137</v>
+      </c>
+      <c r="X165" s="7" t="s">
+        <v>1138</v>
+      </c>
+      <c r="Y165" s="7"/>
+      <c r="Z165" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA165" s="7"/>
+      <c r="AB165" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC165" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD165" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE165" s="7"/>
+      <c r="AF165" s="7"/>
+      <c r="AG165" s="7"/>
+      <c r="AH165" s="7"/>
+      <c r="AI165" s="7"/>
+      <c r="AJ165" s="7"/>
+      <c r="AK165" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="166" spans="1:37">
+      <c r="A166" s="3">
+        <v>164</v>
+      </c>
+      <c r="B166" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C166" s="3">
+        <v>2026063381</v>
+      </c>
+      <c r="D166" s="3"/>
+      <c r="E166" s="3"/>
+      <c r="F166" s="3">
+        <v>2403</v>
+      </c>
+      <c r="G166" s="3" t="s">
+        <v>1139</v>
+      </c>
+      <c r="H166" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I166" s="3"/>
+      <c r="J166" s="3"/>
+      <c r="K166" s="3"/>
+      <c r="L166" s="3"/>
+      <c r="M166" s="4"/>
+      <c r="N166" s="3"/>
+      <c r="O166" s="4"/>
+      <c r="P166" s="10"/>
+      <c r="Q166" s="3" t="s">
+        <v>1140</v>
+      </c>
+      <c r="R166" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S166" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="T166" s="3">
+        <v>1</v>
+      </c>
+      <c r="U166" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V166" s="3" t="s">
+        <v>1141</v>
+      </c>
+      <c r="W166" s="3" t="s">
+        <v>1113</v>
+      </c>
+      <c r="X166" s="3" t="s">
+        <v>1142</v>
+      </c>
+      <c r="Y166" s="3"/>
+      <c r="Z166" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="AA166" s="3"/>
+      <c r="AB166" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC166" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD166" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE166" s="3"/>
+      <c r="AF166" s="3"/>
+      <c r="AG166" s="3"/>
+      <c r="AH166" s="3"/>
+      <c r="AI166" s="3"/>
+      <c r="AJ166" s="3"/>
+      <c r="AK166" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="167" spans="1:37">
+      <c r="A167" s="7">
+        <v>165</v>
+      </c>
+      <c r="B167" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C167" s="7">
+        <v>2026063387</v>
+      </c>
+      <c r="D167" s="7" t="s">
+        <v>1143</v>
+      </c>
+      <c r="E167" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F167" s="7">
+        <v>2535</v>
+      </c>
+      <c r="G167" s="7" t="s">
+        <v>1096</v>
+      </c>
+      <c r="H167" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I167" s="7" t="s">
+        <v>1144</v>
+      </c>
+      <c r="J167" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="K167" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L167" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="M167" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="N167" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="O167" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="P167" s="9" t="s">
+        <v>1103</v>
+      </c>
+      <c r="Q167" s="7" t="s">
+        <v>1097</v>
+      </c>
+      <c r="R167" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S167" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T167" s="7">
+        <v>1</v>
+      </c>
+      <c r="U167" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V167" s="7" t="s">
+        <v>1145</v>
+      </c>
+      <c r="W167" s="7" t="s">
+        <v>1118</v>
+      </c>
+      <c r="X167" s="7" t="s">
+        <v>1146</v>
+      </c>
+      <c r="Y167" s="7" t="s">
+        <v>1147</v>
+      </c>
+      <c r="Z167" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="AA167" s="7"/>
+      <c r="AB167" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="AC167" s="9" t="s">
+        <v>1148</v>
+      </c>
+      <c r="AD167" s="7"/>
+      <c r="AE167" s="7"/>
+      <c r="AF167" s="7"/>
+      <c r="AG167" s="7"/>
+      <c r="AH167" s="7"/>
+      <c r="AI167" s="7"/>
+      <c r="AJ167" s="7"/>
+      <c r="AK167" s="7"/>
+    </row>
+    <row r="168" spans="1:37">
+      <c r="A168" s="3">
+        <v>166</v>
+      </c>
+      <c r="B168" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C168" s="3">
+        <v>2026063388</v>
+      </c>
+      <c r="D168" s="3" t="s">
+        <v>1149</v>
+      </c>
+      <c r="E168" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F168" s="3">
+        <v>2535</v>
+      </c>
+      <c r="G168" s="3" t="s">
+        <v>1096</v>
+      </c>
+      <c r="H168" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="I168" s="3" t="s">
+        <v>1150</v>
+      </c>
+      <c r="J168" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K168" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L168" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="M168" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="N168" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="O168" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="P168" s="10" t="s">
+        <v>1111</v>
+      </c>
+      <c r="Q168" s="3" t="s">
+        <v>1097</v>
+      </c>
+      <c r="R168" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S168" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T168" s="3">
+        <v>1</v>
+      </c>
+      <c r="U168" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V168" s="3" t="s">
+        <v>1151</v>
+      </c>
+      <c r="W168" s="3" t="s">
+        <v>1146</v>
+      </c>
+      <c r="X168" s="3" t="s">
+        <v>1152</v>
+      </c>
+      <c r="Y168" s="3" t="s">
+        <v>1153</v>
+      </c>
+      <c r="Z168" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="AA168" s="3"/>
+      <c r="AB168" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="AC168" s="10" t="s">
+        <v>1148</v>
+      </c>
+      <c r="AD168" s="3"/>
+      <c r="AE168" s="3"/>
+      <c r="AF168" s="3"/>
+      <c r="AG168" s="3"/>
+      <c r="AH168" s="3"/>
+      <c r="AI168" s="3"/>
+      <c r="AJ168" s="3"/>
+      <c r="AK168" s="3"/>
+    </row>
+    <row r="169" spans="1:37">
+      <c r="A169" s="7">
+        <v>167</v>
+      </c>
+      <c r="B169" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C169" s="7">
+        <v>2026063389</v>
+      </c>
+      <c r="D169" s="7" t="s">
+        <v>1154</v>
+      </c>
+      <c r="E169" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F169" s="7">
+        <v>2535</v>
+      </c>
+      <c r="G169" s="7" t="s">
+        <v>1096</v>
+      </c>
+      <c r="H169" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I169" s="7" t="s">
+        <v>1155</v>
+      </c>
+      <c r="J169" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="K169" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L169" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="M169" s="8" t="s">
+        <v>327</v>
+      </c>
+      <c r="N169" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="O169" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="P169" s="9" t="s">
+        <v>1116</v>
+      </c>
+      <c r="Q169" s="7" t="s">
+        <v>1097</v>
+      </c>
+      <c r="R169" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S169" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T169" s="7">
+        <v>1</v>
+      </c>
+      <c r="U169" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V169" s="7" t="s">
+        <v>1156</v>
+      </c>
+      <c r="W169" s="7" t="s">
+        <v>1152</v>
+      </c>
+      <c r="X169" s="7" t="s">
+        <v>1157</v>
+      </c>
+      <c r="Y169" s="7" t="s">
+        <v>1158</v>
+      </c>
+      <c r="Z169" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="AA169" s="7"/>
+      <c r="AB169" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="AC169" s="9" t="s">
+        <v>1148</v>
+      </c>
+      <c r="AD169" s="7"/>
+      <c r="AE169" s="7"/>
+      <c r="AF169" s="7"/>
+      <c r="AG169" s="7"/>
+      <c r="AH169" s="7"/>
+      <c r="AI169" s="7"/>
+      <c r="AJ169" s="7"/>
+      <c r="AK169" s="7"/>
+    </row>
+    <row r="170" spans="1:37">
+      <c r="A170" s="3">
+        <v>168</v>
+      </c>
+      <c r="B170" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C170" s="3">
+        <v>2026063390</v>
+      </c>
+      <c r="D170" s="3"/>
+      <c r="E170" s="3"/>
+      <c r="F170" s="3" t="s">
+        <v>1159</v>
+      </c>
+      <c r="G170" s="3" t="s">
+        <v>1160</v>
+      </c>
+      <c r="H170" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I170" s="3"/>
+      <c r="J170" s="3"/>
+      <c r="K170" s="3"/>
+      <c r="L170" s="3"/>
+      <c r="M170" s="4"/>
+      <c r="N170" s="3"/>
+      <c r="O170" s="4"/>
+      <c r="P170" s="10"/>
+      <c r="Q170" s="3" t="s">
+        <v>1161</v>
+      </c>
+      <c r="R170" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S170" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="T170" s="3">
+        <v>1</v>
+      </c>
+      <c r="U170" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V170" s="3" t="s">
+        <v>1162</v>
+      </c>
+      <c r="W170" s="3" t="s">
+        <v>1163</v>
+      </c>
+      <c r="X170" s="3" t="s">
+        <v>1164</v>
+      </c>
+      <c r="Y170" s="3"/>
+      <c r="Z170" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA170" s="3"/>
+      <c r="AB170" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC170" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD170" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE170" s="3"/>
+      <c r="AF170" s="3"/>
+      <c r="AG170" s="3"/>
+      <c r="AH170" s="3"/>
+      <c r="AI170" s="3"/>
+      <c r="AJ170" s="3"/>
+      <c r="AK170" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="171" spans="1:37">
+      <c r="A171" s="7">
+        <v>169</v>
+      </c>
+      <c r="B171" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C171" s="7">
+        <v>2026063394</v>
+      </c>
+      <c r="D171" s="7"/>
+      <c r="E171" s="7"/>
+      <c r="F171" s="7">
+        <v>4083</v>
+      </c>
+      <c r="G171" s="7" t="s">
+        <v>1165</v>
+      </c>
+      <c r="H171" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I171" s="7"/>
+      <c r="J171" s="7"/>
+      <c r="K171" s="7"/>
+      <c r="L171" s="7"/>
+      <c r="M171" s="8"/>
+      <c r="N171" s="7"/>
+      <c r="O171" s="8"/>
+      <c r="P171" s="9"/>
+      <c r="Q171" s="7" t="s">
+        <v>1166</v>
+      </c>
+      <c r="R171" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S171" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T171" s="7">
+        <v>1</v>
+      </c>
+      <c r="U171" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V171" s="7" t="s">
+        <v>1167</v>
+      </c>
+      <c r="W171" s="7" t="s">
+        <v>1168</v>
+      </c>
+      <c r="X171" s="7" t="s">
+        <v>1169</v>
+      </c>
+      <c r="Y171" s="7"/>
+      <c r="Z171" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA171" s="7"/>
+      <c r="AB171" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC171" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD171" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE171" s="7"/>
+      <c r="AF171" s="7"/>
+      <c r="AG171" s="7"/>
+      <c r="AH171" s="7"/>
+      <c r="AI171" s="7"/>
+      <c r="AJ171" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK171" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="172" spans="1:37">
+      <c r="A172" s="3">
+        <v>170</v>
+      </c>
+      <c r="B172" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C172" s="3">
+        <v>2026063398</v>
+      </c>
+      <c r="D172" s="3"/>
+      <c r="E172" s="3"/>
+      <c r="F172" s="3">
+        <v>2303</v>
+      </c>
+      <c r="G172" s="3" t="s">
+        <v>1170</v>
+      </c>
+      <c r="H172" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I172" s="3"/>
+      <c r="J172" s="3"/>
+      <c r="K172" s="3"/>
+      <c r="L172" s="3"/>
+      <c r="M172" s="4"/>
+      <c r="N172" s="3"/>
+      <c r="O172" s="4"/>
+      <c r="P172" s="4"/>
+      <c r="Q172" s="3" t="s">
+        <v>1171</v>
+      </c>
+      <c r="R172" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S172" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T172" s="3">
+        <v>1</v>
+      </c>
+      <c r="U172" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V172" s="3" t="s">
+        <v>1172</v>
+      </c>
+      <c r="W172" s="3" t="s">
+        <v>1173</v>
+      </c>
+      <c r="X172" s="3" t="s">
+        <v>1174</v>
+      </c>
+      <c r="Y172" s="3"/>
+      <c r="Z172" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA172" s="3"/>
+      <c r="AB172" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC172" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD172" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE172" s="3"/>
+      <c r="AF172" s="3"/>
+      <c r="AG172" s="3"/>
+      <c r="AH172" s="3"/>
+      <c r="AI172" s="3"/>
+      <c r="AJ172" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK172" s="3" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06261722
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,14 +11,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$172</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$174</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1186">
   <si>
     <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-26  )</t>
   </si>
@@ -3616,6 +3616,39 @@
   </si>
   <si>
     <t>2026-06-26 15:20:00</t>
+  </si>
+  <si>
+    <t>三重文化北</t>
+  </si>
+  <si>
+    <t>THILF04312</t>
+  </si>
+  <si>
+    <t>2026-06-26 15:42:56</t>
+  </si>
+  <si>
+    <t>2026-06-26 15:23:00</t>
+  </si>
+  <si>
+    <t>2026-06-26 15:43:00</t>
+  </si>
+  <si>
+    <t>D346</t>
+  </si>
+  <si>
+    <t>三重維德店</t>
+  </si>
+  <si>
+    <t>THILF0D346</t>
+  </si>
+  <si>
+    <t>2026-06-26 16:05:43</t>
+  </si>
+  <si>
+    <t>2026-06-26 15:46:00</t>
+  </si>
+  <si>
+    <t>2026-06-26 16:06:00</t>
   </si>
 </sst>
 </file>
@@ -4029,7 +4062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK172"/>
+  <dimension ref="A1:AK174"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -18724,7 +18757,7 @@
       <c r="M172" s="4"/>
       <c r="N172" s="3"/>
       <c r="O172" s="4"/>
-      <c r="P172" s="4"/>
+      <c r="P172" s="10"/>
       <c r="Q172" s="3" t="s">
         <v>1171</v>
       </c>
@@ -18757,7 +18790,7 @@
       <c r="AB172" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="AC172" s="4" t="s">
+      <c r="AC172" s="10" t="s">
         <v>111</v>
       </c>
       <c r="AD172" s="3" t="s">
@@ -18772,6 +18805,164 @@
         <v>60</v>
       </c>
       <c r="AK172" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="173" spans="1:37">
+      <c r="A173" s="7">
+        <v>171</v>
+      </c>
+      <c r="B173" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C173" s="7">
+        <v>2026063401</v>
+      </c>
+      <c r="D173" s="7"/>
+      <c r="E173" s="7"/>
+      <c r="F173" s="7">
+        <v>4312</v>
+      </c>
+      <c r="G173" s="7" t="s">
+        <v>1175</v>
+      </c>
+      <c r="H173" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I173" s="7"/>
+      <c r="J173" s="7"/>
+      <c r="K173" s="7"/>
+      <c r="L173" s="7"/>
+      <c r="M173" s="8"/>
+      <c r="N173" s="7"/>
+      <c r="O173" s="8"/>
+      <c r="P173" s="9"/>
+      <c r="Q173" s="7" t="s">
+        <v>1176</v>
+      </c>
+      <c r="R173" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S173" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T173" s="7">
+        <v>1</v>
+      </c>
+      <c r="U173" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V173" s="7" t="s">
+        <v>1177</v>
+      </c>
+      <c r="W173" s="7" t="s">
+        <v>1178</v>
+      </c>
+      <c r="X173" s="7" t="s">
+        <v>1179</v>
+      </c>
+      <c r="Y173" s="7"/>
+      <c r="Z173" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA173" s="7"/>
+      <c r="AB173" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC173" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD173" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE173" s="7"/>
+      <c r="AF173" s="7"/>
+      <c r="AG173" s="7"/>
+      <c r="AH173" s="7"/>
+      <c r="AI173" s="7"/>
+      <c r="AJ173" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK173" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="174" spans="1:37">
+      <c r="A174" s="3">
+        <v>172</v>
+      </c>
+      <c r="B174" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C174" s="3">
+        <v>2026063403</v>
+      </c>
+      <c r="D174" s="3"/>
+      <c r="E174" s="3"/>
+      <c r="F174" s="3" t="s">
+        <v>1180</v>
+      </c>
+      <c r="G174" s="3" t="s">
+        <v>1181</v>
+      </c>
+      <c r="H174" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I174" s="3"/>
+      <c r="J174" s="3"/>
+      <c r="K174" s="3"/>
+      <c r="L174" s="3"/>
+      <c r="M174" s="4"/>
+      <c r="N174" s="3"/>
+      <c r="O174" s="4"/>
+      <c r="P174" s="4"/>
+      <c r="Q174" s="3" t="s">
+        <v>1182</v>
+      </c>
+      <c r="R174" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S174" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T174" s="3">
+        <v>1</v>
+      </c>
+      <c r="U174" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V174" s="3" t="s">
+        <v>1183</v>
+      </c>
+      <c r="W174" s="3" t="s">
+        <v>1184</v>
+      </c>
+      <c r="X174" s="3" t="s">
+        <v>1185</v>
+      </c>
+      <c r="Y174" s="3"/>
+      <c r="Z174" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA174" s="3"/>
+      <c r="AB174" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC174" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD174" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE174" s="3"/>
+      <c r="AF174" s="3"/>
+      <c r="AG174" s="3"/>
+      <c r="AH174" s="3"/>
+      <c r="AI174" s="3"/>
+      <c r="AJ174" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK174" s="3" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06301344
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$174</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$200</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1186">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-26  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1353">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-30  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -3649,6 +3649,522 @@
   </si>
   <si>
     <t>2026-06-26 16:06:00</t>
+  </si>
+  <si>
+    <t>12749115062701</t>
+  </si>
+  <si>
+    <t>淡水灰瑤子</t>
+  </si>
+  <si>
+    <t>2026-06-27 14:37:06</t>
+  </si>
+  <si>
+    <t>門市反應TM1多卡機QP3000E悠遊卡無法使用，協助TM點選版更&gt;悠遊卡機重開顯示悠遊卡通訊逾時...請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF02749</t>
+  </si>
+  <si>
+    <t>2026-06-27 14:40:14</t>
+  </si>
+  <si>
+    <t>2026-06-30 11:45:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 12:18:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 13:00:00</t>
+  </si>
+  <si>
+    <t>多卡機重啟之後更新皆為正常</t>
+  </si>
+  <si>
+    <t>12749115062702</t>
+  </si>
+  <si>
+    <t>2026-06-27 14:40:31</t>
+  </si>
+  <si>
+    <t>門市反應TM2多卡機QP3000E悠遊卡無法使用，協助TM點選版更&gt;悠遊卡機重開顯示悠遊卡通訊逾時...請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-06-27 14:41:02</t>
+  </si>
+  <si>
+    <t>2026-06-30 11:30:00</t>
+  </si>
+  <si>
+    <t>14197115062801</t>
+  </si>
+  <si>
+    <t>龜山崇優店</t>
+  </si>
+  <si>
+    <t>2026-06-28 11:31:28</t>
+  </si>
+  <si>
+    <t>門市反應TM2熱感發票機(BSC-10)頻繁顯示[熱感機正在列印中或熱感機無法連線!請稍後或檢查發票機電源、上蓋是否蓋妥!請按清除!]，已多次關機紙捲重裝重啟仍頻繁發生...請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF04197</t>
+  </si>
+  <si>
+    <t>2026-06-28 11:37:44</t>
+  </si>
+  <si>
+    <t>2026-06-29 12:35:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 13:05:00</t>
+  </si>
+  <si>
+    <t>更換發票機
+換下8155003538
+換上8155004461</t>
+  </si>
+  <si>
+    <t>12222115062901</t>
+  </si>
+  <si>
+    <t>2026-06-29 09:05:44</t>
+  </si>
+  <si>
+    <t>06/29 09:10 啟動緊急叫修:門市反應SC(SHUTTLE6S)開啟HISHOP、e網、訂貨3.0都會出現【捷徑\'HISHOP.lnk\'參照的磁碟機或網路連線無法使用。請確定插入的磁碟正確，而且網路資源可以使用，然後重試。】，重啟SC仍異常。因開啟[訂貨3.0][HiShop][E網]出現捷徑異常訊息，請更換第二顆硬碟不備份還原，並攜帶主機隨行檢測...請台芝到店協助 
+PS.若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對) 
+與門市確認帳務做到06/28，與通訊小晶確認有收到，缺少TM1.2電子存根聯</t>
+  </si>
+  <si>
+    <t>2026-06-29 09:10:12</t>
+  </si>
+  <si>
+    <t>2026-06-29 12:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 14:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 15:10:00</t>
+  </si>
+  <si>
+    <t>更換第二課硬碟無備份還原</t>
+  </si>
+  <si>
+    <t>12746115062901</t>
+  </si>
+  <si>
+    <t>2026-06-29 09:02:51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">門市反應tm1收銀機(TCX800)(抽屜顏色:白色、鑰匙孔位子(中)、鎖頭編號:無編號)抽屜無法開啟，點選開抽屜也無反應，已有將發票機關機紙捲重裝仍異常...請台芝到店協助
+</t>
+  </si>
+  <si>
+    <t>2026-06-29 09:10:46</t>
+  </si>
+  <si>
+    <t>2026-06-30 11:58:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 12:28:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 13:10:00</t>
+  </si>
+  <si>
+    <t>E4658115062801</t>
+  </si>
+  <si>
+    <t>淡水英才店</t>
+  </si>
+  <si>
+    <t>2026-06-28 19:36:38</t>
+  </si>
+  <si>
+    <t>D302</t>
+  </si>
+  <si>
+    <t>發票印字不清</t>
+  </si>
+  <si>
+    <t xml:space="preserve">門市反應tm1發票機(BSC-10)印出的兌換卷條碼到兩台tm都無法刷讀，門市已有重裝紙捲重開機簡易清潔出紙口仍異常.....須請台芝到店協助(兌換卷條碼都刷不出來)
+</t>
+  </si>
+  <si>
+    <t>THILF04658</t>
+  </si>
+  <si>
+    <t>2026-06-29 09:12:51</t>
+  </si>
+  <si>
+    <t>2026-06-30 10:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 11:10:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 13:12:00</t>
+  </si>
+  <si>
+    <t>更換發票機
+換下8155003663
+換上8155005419</t>
+  </si>
+  <si>
+    <t>1T197115062901</t>
+  </si>
+  <si>
+    <t>T197</t>
+  </si>
+  <si>
+    <t>2026-06-29 09:30:46</t>
+  </si>
+  <si>
+    <t>無電源反應、無法開機</t>
+  </si>
+  <si>
+    <t>五股訓練中心范小姐反應tm1(TCX800)無電源反應燈號未亮燈，已有拔插休息仍異常確認插座有正常過電但仍無電源反應....須請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF0T197</t>
+  </si>
+  <si>
+    <t>2026-06-29 09:34:26</t>
+  </si>
+  <si>
+    <t>2026-06-30 09:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 09:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 13:34:00</t>
+  </si>
+  <si>
+    <t>更換變壓器</t>
+  </si>
+  <si>
+    <t>D649</t>
+  </si>
+  <si>
+    <t>三重運動公園</t>
+  </si>
+  <si>
+    <t>THILF0D649</t>
+  </si>
+  <si>
+    <t>2026-06-29 09:35:33</t>
+  </si>
+  <si>
+    <t>2026-06-29 09:05:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 09:25:00</t>
+  </si>
+  <si>
+    <t>三重果菜市場</t>
+  </si>
+  <si>
+    <t>THILF02014</t>
+  </si>
+  <si>
+    <t>2026-06-29 09:56:01</t>
+  </si>
+  <si>
+    <t>2026-06-29 09:32:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 09:55:00</t>
+  </si>
+  <si>
+    <t>1D072115062901</t>
+  </si>
+  <si>
+    <t>2026-06-29 11:01:33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">門市反應TM1(TCX800)抽屜開關都會卡卡的，都需要手動拉開，抽屜外觀米白/鑰匙孔位置右邊/鑰匙孔編號716.....須請台芝到店協助	</t>
+  </si>
+  <si>
+    <t>2026-06-29 11:14:43</t>
+  </si>
+  <si>
+    <t>2026-06-29 18:10:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 18:38:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 15:14:00</t>
+  </si>
+  <si>
+    <t>到場測試功能正常</t>
+  </si>
+  <si>
+    <t>1D072115062902</t>
+  </si>
+  <si>
+    <t>2026-06-29 11:14:21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">門市反應TM2(TCX800)抽屜開關都會卡卡的，都需要手動拉開，抽屜外觀米白/鑰匙孔位置右邊/鑰匙孔編號K01.....須請台芝到店協助	</t>
+  </si>
+  <si>
+    <t>2026-06-29 11:15:01</t>
+  </si>
+  <si>
+    <t>2026-06-29 18:39:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 15:15:00</t>
+  </si>
+  <si>
+    <t>更換錢箱
+換上：81Z1004949
+換下：81Z1001036</t>
+  </si>
+  <si>
+    <t>龜山復興店</t>
+  </si>
+  <si>
+    <t>THILF05075</t>
+  </si>
+  <si>
+    <t>2026-06-29 11:50:59</t>
+  </si>
+  <si>
+    <t>2026-06-29 11:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 11:30:00</t>
+  </si>
+  <si>
+    <t>蘆竹領航店</t>
+  </si>
+  <si>
+    <t>THILF04601</t>
+  </si>
+  <si>
+    <t>2026-06-29 13:48:29</t>
+  </si>
+  <si>
+    <t>2026-06-29 13:20:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 13:45:00</t>
+  </si>
+  <si>
+    <t>蘆竹海湖店</t>
+  </si>
+  <si>
+    <t>THILF04572</t>
+  </si>
+  <si>
+    <t>2026-06-29 14:30:43</t>
+  </si>
+  <si>
+    <t>2026-06-29 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 14:29:00</t>
+  </si>
+  <si>
+    <t>蘆洲永樂店</t>
+  </si>
+  <si>
+    <t>THILF04036</t>
+  </si>
+  <si>
+    <t>2026-06-29 15:39:57</t>
+  </si>
+  <si>
+    <t>2026-06-29 15:00:00</t>
+  </si>
+  <si>
+    <t>協助回裝</t>
+  </si>
+  <si>
+    <t>中和浪漫店</t>
+  </si>
+  <si>
+    <t>THILF04573</t>
+  </si>
+  <si>
+    <t>2026-06-29 15:41:08</t>
+  </si>
+  <si>
+    <t>2026-06-29 15:40:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 15:41:23</t>
+  </si>
+  <si>
+    <t>撤店</t>
+  </si>
+  <si>
+    <t>2026-06-29 15:52:38</t>
+  </si>
+  <si>
+    <t>2026-06-29 11:10:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 15:50:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">裝潢回裝已完工，使用ADSL
+</t>
+  </si>
+  <si>
+    <t>14036115062901</t>
+  </si>
+  <si>
+    <t>2026-06-29 17:31:06</t>
+  </si>
+  <si>
+    <t>不能連線</t>
+  </si>
+  <si>
+    <t>hub(DGS1210-28)門市今日重新裝潢回裝，區經理來電反應門市複合機無法使用ping30不通，經與複合機廠商確認將8port與7port交叉測試後，ping30有通，但目前ping91不通無法連線hub確認是否未開port或鎖mac，重啟hub後仍異常....須請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-06-29 17:34:27</t>
+  </si>
+  <si>
+    <t>2026-06-29 19:30:00</t>
+  </si>
+  <si>
+    <t>2026-06-29 20:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 21:34:00</t>
+  </si>
+  <si>
+    <t>HUB重設後測試列印正常</t>
+  </si>
+  <si>
+    <t>1T104115063001</t>
+  </si>
+  <si>
+    <t>T104</t>
+  </si>
+  <si>
+    <t>2026-06-30 09:10:06</t>
+  </si>
+  <si>
+    <t>五股訓練中心范小姐反應SC(SHUTTLE7S)近期SC頻繁當機，卡在登入畫面當掉重開機後就直接黑屏，拔差休息再次開機仍異常...須請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF0T104</t>
+  </si>
+  <si>
+    <t>2026-06-30 09:19:54</t>
+  </si>
+  <si>
+    <t>2026-06-30 10:00:00</t>
+  </si>
+  <si>
+    <t>2026-07-01 13:19:00</t>
+  </si>
+  <si>
+    <t>更換主機 
+換上8114004460
+換下8114004719</t>
+  </si>
+  <si>
+    <t>D024</t>
+  </si>
+  <si>
+    <t>三重三民店</t>
+  </si>
+  <si>
+    <t>THILF0D024</t>
+  </si>
+  <si>
+    <t>2026-06-30 11:52:22</t>
+  </si>
+  <si>
+    <t>2026-06-30 10:58:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 11:20:00</t>
+  </si>
+  <si>
+    <t>三重力行店</t>
+  </si>
+  <si>
+    <t>THILF05410</t>
+  </si>
+  <si>
+    <t>2026-06-30 12:07:01</t>
+  </si>
+  <si>
+    <t>2026-06-30 11:35:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 12:00:00</t>
+  </si>
+  <si>
+    <t>12746115063001</t>
+  </si>
+  <si>
+    <t>2026-06-30 12:15:41</t>
+  </si>
+  <si>
+    <t>台芝到店tm1收銀機(TCX800)(抽屜顏色:白色、鑰匙孔位子(中)、鎖頭編號:無編號)抽屜錢箱仍異常需更換，請客服協助建叫修...請台芝協助</t>
+  </si>
+  <si>
+    <t>2026-06-30 12:26:29</t>
+  </si>
+  <si>
+    <t>2026-06-30 12:30:00</t>
+  </si>
+  <si>
+    <t>2026-07-01 16:26:00</t>
+  </si>
+  <si>
+    <t>更換錢箱
+換上：81Z1004950
+換下：81Z1000995</t>
+  </si>
+  <si>
+    <t>三重美堤店</t>
+  </si>
+  <si>
+    <t>THILF03890</t>
+  </si>
+  <si>
+    <t>2026-06-30 12:41:31</t>
+  </si>
+  <si>
+    <t>2026-06-30 12:20:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 12:40:00</t>
+  </si>
+  <si>
+    <t>板橋江子翠站</t>
+  </si>
+  <si>
+    <t>THILF02069</t>
+  </si>
+  <si>
+    <t>2026-06-30 13:01:39</t>
+  </si>
+  <si>
+    <t>2026-06-30 12:45:00</t>
+  </si>
+  <si>
+    <t>三重頂崁店</t>
+  </si>
+  <si>
+    <t>THILF04698</t>
+  </si>
+  <si>
+    <t>2026-06-30 13:11:56</t>
+  </si>
+  <si>
+    <t>2026-06-30 12:48:00</t>
   </si>
 </sst>
 </file>
@@ -4062,7 +4578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK174"/>
+  <dimension ref="A1:AK200"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -18915,7 +19431,7 @@
       <c r="M174" s="4"/>
       <c r="N174" s="3"/>
       <c r="O174" s="4"/>
-      <c r="P174" s="4"/>
+      <c r="P174" s="10"/>
       <c r="Q174" s="3" t="s">
         <v>1182</v>
       </c>
@@ -18948,7 +19464,7 @@
       <c r="AB174" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="AC174" s="4" t="s">
+      <c r="AC174" s="10" t="s">
         <v>111</v>
       </c>
       <c r="AD174" s="3" t="s">
@@ -18963,6 +19479,2260 @@
         <v>60</v>
       </c>
       <c r="AK174" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="175" spans="1:37">
+      <c r="A175" s="7">
+        <v>173</v>
+      </c>
+      <c r="B175" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C175" s="7">
+        <v>2026063463</v>
+      </c>
+      <c r="D175" s="7" t="s">
+        <v>1186</v>
+      </c>
+      <c r="E175" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F175" s="7">
+        <v>2749</v>
+      </c>
+      <c r="G175" s="7" t="s">
+        <v>1187</v>
+      </c>
+      <c r="H175" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="I175" s="7" t="s">
+        <v>1188</v>
+      </c>
+      <c r="J175" s="7" t="s">
+        <v>266</v>
+      </c>
+      <c r="K175" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L175" s="7" t="s">
+        <v>522</v>
+      </c>
+      <c r="M175" s="8" t="s">
+        <v>523</v>
+      </c>
+      <c r="N175" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="O175" s="8" t="s">
+        <v>628</v>
+      </c>
+      <c r="P175" s="9" t="s">
+        <v>1189</v>
+      </c>
+      <c r="Q175" s="7" t="s">
+        <v>1190</v>
+      </c>
+      <c r="R175" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S175" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T175" s="7">
+        <v>1</v>
+      </c>
+      <c r="U175" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V175" s="7" t="s">
+        <v>1191</v>
+      </c>
+      <c r="W175" s="7" t="s">
+        <v>1192</v>
+      </c>
+      <c r="X175" s="7" t="s">
+        <v>1193</v>
+      </c>
+      <c r="Y175" s="7" t="s">
+        <v>1194</v>
+      </c>
+      <c r="Z175" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="AA175" s="7"/>
+      <c r="AB175" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC175" s="9" t="s">
+        <v>1195</v>
+      </c>
+      <c r="AD175" s="7"/>
+      <c r="AE175" s="7"/>
+      <c r="AF175" s="7"/>
+      <c r="AG175" s="7"/>
+      <c r="AH175" s="7"/>
+      <c r="AI175" s="7"/>
+      <c r="AJ175" s="7"/>
+      <c r="AK175" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="176" spans="1:37">
+      <c r="A176" s="3">
+        <v>174</v>
+      </c>
+      <c r="B176" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C176" s="3">
+        <v>2026063464</v>
+      </c>
+      <c r="D176" s="3" t="s">
+        <v>1196</v>
+      </c>
+      <c r="E176" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F176" s="3">
+        <v>2749</v>
+      </c>
+      <c r="G176" s="3" t="s">
+        <v>1187</v>
+      </c>
+      <c r="H176" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="I176" s="3" t="s">
+        <v>1197</v>
+      </c>
+      <c r="J176" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="K176" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L176" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="M176" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="N176" s="3" t="s">
+        <v>627</v>
+      </c>
+      <c r="O176" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="P176" s="10" t="s">
+        <v>1198</v>
+      </c>
+      <c r="Q176" s="3" t="s">
+        <v>1190</v>
+      </c>
+      <c r="R176" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S176" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T176" s="3">
+        <v>1</v>
+      </c>
+      <c r="U176" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V176" s="3" t="s">
+        <v>1199</v>
+      </c>
+      <c r="W176" s="3" t="s">
+        <v>1200</v>
+      </c>
+      <c r="X176" s="3" t="s">
+        <v>1192</v>
+      </c>
+      <c r="Y176" s="3" t="s">
+        <v>1194</v>
+      </c>
+      <c r="Z176" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA176" s="3"/>
+      <c r="AB176" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC176" s="10" t="s">
+        <v>1195</v>
+      </c>
+      <c r="AD176" s="3"/>
+      <c r="AE176" s="3"/>
+      <c r="AF176" s="3"/>
+      <c r="AG176" s="3"/>
+      <c r="AH176" s="3"/>
+      <c r="AI176" s="3"/>
+      <c r="AJ176" s="3"/>
+      <c r="AK176" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="177" spans="1:37">
+      <c r="A177" s="7">
+        <v>175</v>
+      </c>
+      <c r="B177" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C177" s="7">
+        <v>2026063468</v>
+      </c>
+      <c r="D177" s="7" t="s">
+        <v>1201</v>
+      </c>
+      <c r="E177" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F177" s="7">
+        <v>4197</v>
+      </c>
+      <c r="G177" s="7" t="s">
+        <v>1202</v>
+      </c>
+      <c r="H177" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="I177" s="7" t="s">
+        <v>1203</v>
+      </c>
+      <c r="J177" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="K177" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L177" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="M177" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="N177" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="O177" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="P177" s="9" t="s">
+        <v>1204</v>
+      </c>
+      <c r="Q177" s="7" t="s">
+        <v>1205</v>
+      </c>
+      <c r="R177" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S177" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T177" s="7">
+        <v>1</v>
+      </c>
+      <c r="U177" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V177" s="7" t="s">
+        <v>1206</v>
+      </c>
+      <c r="W177" s="7" t="s">
+        <v>1207</v>
+      </c>
+      <c r="X177" s="7" t="s">
+        <v>1208</v>
+      </c>
+      <c r="Y177" s="7" t="s">
+        <v>1194</v>
+      </c>
+      <c r="Z177" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA177" s="7"/>
+      <c r="AB177" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC177" s="9" t="s">
+        <v>1209</v>
+      </c>
+      <c r="AD177" s="7"/>
+      <c r="AE177" s="7"/>
+      <c r="AF177" s="7"/>
+      <c r="AG177" s="7"/>
+      <c r="AH177" s="7"/>
+      <c r="AI177" s="7"/>
+      <c r="AJ177" s="7"/>
+      <c r="AK177" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="178" spans="1:37">
+      <c r="A178" s="3">
+        <v>176</v>
+      </c>
+      <c r="B178" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C178" s="3">
+        <v>2026063480</v>
+      </c>
+      <c r="D178" s="3" t="s">
+        <v>1210</v>
+      </c>
+      <c r="E178" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="F178" s="3">
+        <v>2222</v>
+      </c>
+      <c r="G178" s="3" t="s">
+        <v>807</v>
+      </c>
+      <c r="H178" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I178" s="3" t="s">
+        <v>1211</v>
+      </c>
+      <c r="J178" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="K178" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L178" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="M178" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="N178" s="3">
+        <v>2405</v>
+      </c>
+      <c r="O178" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="P178" s="10" t="s">
+        <v>1212</v>
+      </c>
+      <c r="Q178" s="3" t="s">
+        <v>812</v>
+      </c>
+      <c r="R178" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S178" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="T178" s="3">
+        <v>1</v>
+      </c>
+      <c r="U178" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V178" s="3" t="s">
+        <v>1213</v>
+      </c>
+      <c r="W178" s="3" t="s">
+        <v>1214</v>
+      </c>
+      <c r="X178" s="3" t="s">
+        <v>1215</v>
+      </c>
+      <c r="Y178" s="3" t="s">
+        <v>1216</v>
+      </c>
+      <c r="Z178" s="3">
+        <v>2</v>
+      </c>
+      <c r="AA178" s="3"/>
+      <c r="AB178" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC178" s="10" t="s">
+        <v>1217</v>
+      </c>
+      <c r="AD178" s="3"/>
+      <c r="AE178" s="3"/>
+      <c r="AF178" s="3"/>
+      <c r="AG178" s="3"/>
+      <c r="AH178" s="3"/>
+      <c r="AI178" s="3"/>
+      <c r="AJ178" s="3"/>
+      <c r="AK178" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="179" spans="1:37">
+      <c r="A179" s="7">
+        <v>177</v>
+      </c>
+      <c r="B179" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C179" s="7">
+        <v>2026063481</v>
+      </c>
+      <c r="D179" s="7" t="s">
+        <v>1218</v>
+      </c>
+      <c r="E179" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F179" s="7">
+        <v>2746</v>
+      </c>
+      <c r="G179" s="7" t="s">
+        <v>697</v>
+      </c>
+      <c r="H179" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I179" s="7" t="s">
+        <v>1219</v>
+      </c>
+      <c r="J179" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K179" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L179" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M179" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="N179" s="7">
+        <v>2305</v>
+      </c>
+      <c r="O179" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="P179" s="9" t="s">
+        <v>1220</v>
+      </c>
+      <c r="Q179" s="7" t="s">
+        <v>700</v>
+      </c>
+      <c r="R179" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S179" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="T179" s="7">
+        <v>1</v>
+      </c>
+      <c r="U179" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V179" s="7" t="s">
+        <v>1221</v>
+      </c>
+      <c r="W179" s="7" t="s">
+        <v>1222</v>
+      </c>
+      <c r="X179" s="7" t="s">
+        <v>1223</v>
+      </c>
+      <c r="Y179" s="7" t="s">
+        <v>1224</v>
+      </c>
+      <c r="Z179" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA179" s="7"/>
+      <c r="AB179" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="AC179" s="9" t="s">
+        <v>1148</v>
+      </c>
+      <c r="AD179" s="7"/>
+      <c r="AE179" s="7"/>
+      <c r="AF179" s="7"/>
+      <c r="AG179" s="7"/>
+      <c r="AH179" s="7"/>
+      <c r="AI179" s="7"/>
+      <c r="AJ179" s="7"/>
+      <c r="AK179" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="180" spans="1:37">
+      <c r="A180" s="3">
+        <v>178</v>
+      </c>
+      <c r="B180" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C180" s="3">
+        <v>2026063482</v>
+      </c>
+      <c r="D180" s="3" t="s">
+        <v>1225</v>
+      </c>
+      <c r="E180" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F180" s="3">
+        <v>4658</v>
+      </c>
+      <c r="G180" s="3" t="s">
+        <v>1226</v>
+      </c>
+      <c r="H180" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="I180" s="3" t="s">
+        <v>1227</v>
+      </c>
+      <c r="J180" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="K180" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="L180" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="M180" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="N180" s="3" t="s">
+        <v>1228</v>
+      </c>
+      <c r="O180" s="4" t="s">
+        <v>1229</v>
+      </c>
+      <c r="P180" s="10" t="s">
+        <v>1230</v>
+      </c>
+      <c r="Q180" s="3" t="s">
+        <v>1231</v>
+      </c>
+      <c r="R180" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S180" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T180" s="3">
+        <v>1</v>
+      </c>
+      <c r="U180" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V180" s="3" t="s">
+        <v>1232</v>
+      </c>
+      <c r="W180" s="3" t="s">
+        <v>1233</v>
+      </c>
+      <c r="X180" s="3" t="s">
+        <v>1234</v>
+      </c>
+      <c r="Y180" s="3" t="s">
+        <v>1235</v>
+      </c>
+      <c r="Z180" s="3">
+        <v>0.7</v>
+      </c>
+      <c r="AA180" s="3"/>
+      <c r="AB180" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC180" s="10" t="s">
+        <v>1236</v>
+      </c>
+      <c r="AD180" s="3"/>
+      <c r="AE180" s="3"/>
+      <c r="AF180" s="3"/>
+      <c r="AG180" s="3"/>
+      <c r="AH180" s="3"/>
+      <c r="AI180" s="3"/>
+      <c r="AJ180" s="3"/>
+      <c r="AK180" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="181" spans="1:37">
+      <c r="A181" s="7">
+        <v>179</v>
+      </c>
+      <c r="B181" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C181" s="7">
+        <v>2026063487</v>
+      </c>
+      <c r="D181" s="7" t="s">
+        <v>1237</v>
+      </c>
+      <c r="E181" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F181" s="7" t="s">
+        <v>1238</v>
+      </c>
+      <c r="G181" s="7" t="s">
+        <v>1047</v>
+      </c>
+      <c r="H181" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I181" s="7" t="s">
+        <v>1239</v>
+      </c>
+      <c r="J181" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K181" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L181" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M181" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="N181" s="7">
+        <v>2306</v>
+      </c>
+      <c r="O181" s="8" t="s">
+        <v>1240</v>
+      </c>
+      <c r="P181" s="9" t="s">
+        <v>1241</v>
+      </c>
+      <c r="Q181" s="7" t="s">
+        <v>1242</v>
+      </c>
+      <c r="R181" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S181" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T181" s="7">
+        <v>1</v>
+      </c>
+      <c r="U181" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V181" s="7" t="s">
+        <v>1243</v>
+      </c>
+      <c r="W181" s="7" t="s">
+        <v>1244</v>
+      </c>
+      <c r="X181" s="7" t="s">
+        <v>1245</v>
+      </c>
+      <c r="Y181" s="7" t="s">
+        <v>1246</v>
+      </c>
+      <c r="Z181" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA181" s="7"/>
+      <c r="AB181" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC181" s="9" t="s">
+        <v>1247</v>
+      </c>
+      <c r="AD181" s="7"/>
+      <c r="AE181" s="7"/>
+      <c r="AF181" s="7"/>
+      <c r="AG181" s="7"/>
+      <c r="AH181" s="7"/>
+      <c r="AI181" s="7"/>
+      <c r="AJ181" s="7"/>
+      <c r="AK181" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="182" spans="1:37">
+      <c r="A182" s="3">
+        <v>180</v>
+      </c>
+      <c r="B182" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C182" s="3">
+        <v>2026063489</v>
+      </c>
+      <c r="D182" s="3"/>
+      <c r="E182" s="3"/>
+      <c r="F182" s="3" t="s">
+        <v>1248</v>
+      </c>
+      <c r="G182" s="3" t="s">
+        <v>1249</v>
+      </c>
+      <c r="H182" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I182" s="3"/>
+      <c r="J182" s="3"/>
+      <c r="K182" s="3"/>
+      <c r="L182" s="3"/>
+      <c r="M182" s="4"/>
+      <c r="N182" s="3"/>
+      <c r="O182" s="4"/>
+      <c r="P182" s="10"/>
+      <c r="Q182" s="3" t="s">
+        <v>1250</v>
+      </c>
+      <c r="R182" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S182" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T182" s="3">
+        <v>1</v>
+      </c>
+      <c r="U182" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V182" s="3" t="s">
+        <v>1251</v>
+      </c>
+      <c r="W182" s="3" t="s">
+        <v>1252</v>
+      </c>
+      <c r="X182" s="3" t="s">
+        <v>1253</v>
+      </c>
+      <c r="Y182" s="3"/>
+      <c r="Z182" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA182" s="3"/>
+      <c r="AB182" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC182" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD182" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE182" s="3"/>
+      <c r="AF182" s="3"/>
+      <c r="AG182" s="3"/>
+      <c r="AH182" s="3"/>
+      <c r="AI182" s="3"/>
+      <c r="AJ182" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK182" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="183" spans="1:37">
+      <c r="A183" s="7">
+        <v>181</v>
+      </c>
+      <c r="B183" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C183" s="7">
+        <v>2026063492</v>
+      </c>
+      <c r="D183" s="7"/>
+      <c r="E183" s="7"/>
+      <c r="F183" s="7">
+        <v>2014</v>
+      </c>
+      <c r="G183" s="7" t="s">
+        <v>1254</v>
+      </c>
+      <c r="H183" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I183" s="7"/>
+      <c r="J183" s="7"/>
+      <c r="K183" s="7"/>
+      <c r="L183" s="7"/>
+      <c r="M183" s="8"/>
+      <c r="N183" s="7"/>
+      <c r="O183" s="8"/>
+      <c r="P183" s="9"/>
+      <c r="Q183" s="7" t="s">
+        <v>1255</v>
+      </c>
+      <c r="R183" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S183" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T183" s="7">
+        <v>1</v>
+      </c>
+      <c r="U183" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V183" s="7" t="s">
+        <v>1256</v>
+      </c>
+      <c r="W183" s="7" t="s">
+        <v>1257</v>
+      </c>
+      <c r="X183" s="7" t="s">
+        <v>1258</v>
+      </c>
+      <c r="Y183" s="7"/>
+      <c r="Z183" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA183" s="7"/>
+      <c r="AB183" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC183" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD183" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE183" s="7"/>
+      <c r="AF183" s="7"/>
+      <c r="AG183" s="7"/>
+      <c r="AH183" s="7"/>
+      <c r="AI183" s="7"/>
+      <c r="AJ183" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK183" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="184" spans="1:37">
+      <c r="A184" s="3">
+        <v>182</v>
+      </c>
+      <c r="B184" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C184" s="3">
+        <v>2026063501</v>
+      </c>
+      <c r="D184" s="3" t="s">
+        <v>1259</v>
+      </c>
+      <c r="E184" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F184" s="3" t="s">
+        <v>618</v>
+      </c>
+      <c r="G184" s="3" t="s">
+        <v>619</v>
+      </c>
+      <c r="H184" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I184" s="3" t="s">
+        <v>1260</v>
+      </c>
+      <c r="J184" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="K184" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L184" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M184" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="N184" s="3">
+        <v>2305</v>
+      </c>
+      <c r="O184" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="P184" s="10" t="s">
+        <v>1261</v>
+      </c>
+      <c r="Q184" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="R184" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S184" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="T184" s="3">
+        <v>1</v>
+      </c>
+      <c r="U184" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V184" s="3" t="s">
+        <v>1262</v>
+      </c>
+      <c r="W184" s="3" t="s">
+        <v>1263</v>
+      </c>
+      <c r="X184" s="3" t="s">
+        <v>1264</v>
+      </c>
+      <c r="Y184" s="3" t="s">
+        <v>1265</v>
+      </c>
+      <c r="Z184" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA184" s="3"/>
+      <c r="AB184" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC184" s="10" t="s">
+        <v>1266</v>
+      </c>
+      <c r="AD184" s="3"/>
+      <c r="AE184" s="3"/>
+      <c r="AF184" s="3"/>
+      <c r="AG184" s="3"/>
+      <c r="AH184" s="3"/>
+      <c r="AI184" s="3"/>
+      <c r="AJ184" s="3"/>
+      <c r="AK184" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="185" spans="1:37">
+      <c r="A185" s="7">
+        <v>183</v>
+      </c>
+      <c r="B185" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C185" s="7">
+        <v>2026063502</v>
+      </c>
+      <c r="D185" s="7" t="s">
+        <v>1267</v>
+      </c>
+      <c r="E185" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F185" s="7" t="s">
+        <v>618</v>
+      </c>
+      <c r="G185" s="7" t="s">
+        <v>619</v>
+      </c>
+      <c r="H185" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I185" s="7" t="s">
+        <v>1268</v>
+      </c>
+      <c r="J185" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K185" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L185" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M185" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="N185" s="7">
+        <v>2305</v>
+      </c>
+      <c r="O185" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="P185" s="9" t="s">
+        <v>1269</v>
+      </c>
+      <c r="Q185" s="7" t="s">
+        <v>620</v>
+      </c>
+      <c r="R185" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S185" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="T185" s="7">
+        <v>1</v>
+      </c>
+      <c r="U185" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V185" s="7" t="s">
+        <v>1270</v>
+      </c>
+      <c r="W185" s="7" t="s">
+        <v>1263</v>
+      </c>
+      <c r="X185" s="7" t="s">
+        <v>1271</v>
+      </c>
+      <c r="Y185" s="7" t="s">
+        <v>1272</v>
+      </c>
+      <c r="Z185" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA185" s="7"/>
+      <c r="AB185" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC185" s="9" t="s">
+        <v>1273</v>
+      </c>
+      <c r="AD185" s="7"/>
+      <c r="AE185" s="7"/>
+      <c r="AF185" s="7"/>
+      <c r="AG185" s="7"/>
+      <c r="AH185" s="7"/>
+      <c r="AI185" s="7"/>
+      <c r="AJ185" s="7"/>
+      <c r="AK185" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="186" spans="1:37">
+      <c r="A186" s="3">
+        <v>184</v>
+      </c>
+      <c r="B186" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C186" s="3">
+        <v>2026063522</v>
+      </c>
+      <c r="D186" s="3"/>
+      <c r="E186" s="3"/>
+      <c r="F186" s="3">
+        <v>5075</v>
+      </c>
+      <c r="G186" s="3" t="s">
+        <v>1274</v>
+      </c>
+      <c r="H186" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I186" s="3"/>
+      <c r="J186" s="3"/>
+      <c r="K186" s="3"/>
+      <c r="L186" s="3"/>
+      <c r="M186" s="4"/>
+      <c r="N186" s="3"/>
+      <c r="O186" s="4"/>
+      <c r="P186" s="10"/>
+      <c r="Q186" s="3" t="s">
+        <v>1275</v>
+      </c>
+      <c r="R186" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S186" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T186" s="3">
+        <v>1</v>
+      </c>
+      <c r="U186" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V186" s="3" t="s">
+        <v>1276</v>
+      </c>
+      <c r="W186" s="3" t="s">
+        <v>1277</v>
+      </c>
+      <c r="X186" s="3" t="s">
+        <v>1278</v>
+      </c>
+      <c r="Y186" s="3"/>
+      <c r="Z186" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA186" s="3"/>
+      <c r="AB186" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC186" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD186" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE186" s="3"/>
+      <c r="AF186" s="3"/>
+      <c r="AG186" s="3"/>
+      <c r="AH186" s="3"/>
+      <c r="AI186" s="3"/>
+      <c r="AJ186" s="3"/>
+      <c r="AK186" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="187" spans="1:37">
+      <c r="A187" s="7">
+        <v>185</v>
+      </c>
+      <c r="B187" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C187" s="7">
+        <v>2026063567</v>
+      </c>
+      <c r="D187" s="7"/>
+      <c r="E187" s="7"/>
+      <c r="F187" s="7">
+        <v>4601</v>
+      </c>
+      <c r="G187" s="7" t="s">
+        <v>1279</v>
+      </c>
+      <c r="H187" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I187" s="7"/>
+      <c r="J187" s="7"/>
+      <c r="K187" s="7"/>
+      <c r="L187" s="7"/>
+      <c r="M187" s="8"/>
+      <c r="N187" s="7"/>
+      <c r="O187" s="8"/>
+      <c r="P187" s="9"/>
+      <c r="Q187" s="7" t="s">
+        <v>1280</v>
+      </c>
+      <c r="R187" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S187" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="T187" s="7">
+        <v>1</v>
+      </c>
+      <c r="U187" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V187" s="7" t="s">
+        <v>1281</v>
+      </c>
+      <c r="W187" s="7" t="s">
+        <v>1282</v>
+      </c>
+      <c r="X187" s="7" t="s">
+        <v>1283</v>
+      </c>
+      <c r="Y187" s="7"/>
+      <c r="Z187" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA187" s="7"/>
+      <c r="AB187" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC187" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD187" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE187" s="7"/>
+      <c r="AF187" s="7"/>
+      <c r="AG187" s="7"/>
+      <c r="AH187" s="7"/>
+      <c r="AI187" s="7"/>
+      <c r="AJ187" s="7"/>
+      <c r="AK187" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="188" spans="1:37">
+      <c r="A188" s="3">
+        <v>186</v>
+      </c>
+      <c r="B188" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C188" s="3">
+        <v>2026063579</v>
+      </c>
+      <c r="D188" s="3"/>
+      <c r="E188" s="3"/>
+      <c r="F188" s="3">
+        <v>4572</v>
+      </c>
+      <c r="G188" s="3" t="s">
+        <v>1284</v>
+      </c>
+      <c r="H188" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="I188" s="3"/>
+      <c r="J188" s="3"/>
+      <c r="K188" s="3"/>
+      <c r="L188" s="3"/>
+      <c r="M188" s="4"/>
+      <c r="N188" s="3"/>
+      <c r="O188" s="4"/>
+      <c r="P188" s="10"/>
+      <c r="Q188" s="3" t="s">
+        <v>1285</v>
+      </c>
+      <c r="R188" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S188" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T188" s="3">
+        <v>1</v>
+      </c>
+      <c r="U188" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V188" s="3" t="s">
+        <v>1286</v>
+      </c>
+      <c r="W188" s="3" t="s">
+        <v>1287</v>
+      </c>
+      <c r="X188" s="3" t="s">
+        <v>1288</v>
+      </c>
+      <c r="Y188" s="3"/>
+      <c r="Z188" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA188" s="3"/>
+      <c r="AB188" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC188" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD188" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE188" s="3"/>
+      <c r="AF188" s="3"/>
+      <c r="AG188" s="3"/>
+      <c r="AH188" s="3"/>
+      <c r="AI188" s="3"/>
+      <c r="AJ188" s="3"/>
+      <c r="AK188" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="189" spans="1:37">
+      <c r="A189" s="7">
+        <v>187</v>
+      </c>
+      <c r="B189" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C189" s="7">
+        <v>2026063588</v>
+      </c>
+      <c r="D189" s="7"/>
+      <c r="E189" s="7"/>
+      <c r="F189" s="7">
+        <v>4036</v>
+      </c>
+      <c r="G189" s="7" t="s">
+        <v>1289</v>
+      </c>
+      <c r="H189" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="I189" s="7"/>
+      <c r="J189" s="7"/>
+      <c r="K189" s="7"/>
+      <c r="L189" s="7"/>
+      <c r="M189" s="8"/>
+      <c r="N189" s="7"/>
+      <c r="O189" s="8"/>
+      <c r="P189" s="9"/>
+      <c r="Q189" s="7" t="s">
+        <v>1290</v>
+      </c>
+      <c r="R189" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S189" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T189" s="7">
+        <v>1</v>
+      </c>
+      <c r="U189" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V189" s="7" t="s">
+        <v>1291</v>
+      </c>
+      <c r="W189" s="7" t="s">
+        <v>1277</v>
+      </c>
+      <c r="X189" s="7" t="s">
+        <v>1292</v>
+      </c>
+      <c r="Y189" s="7"/>
+      <c r="Z189" s="7">
+        <v>4</v>
+      </c>
+      <c r="AA189" s="7"/>
+      <c r="AB189" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC189" s="9" t="s">
+        <v>1293</v>
+      </c>
+      <c r="AD189" s="7"/>
+      <c r="AE189" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF189" s="7"/>
+      <c r="AG189" s="7"/>
+      <c r="AH189" s="7"/>
+      <c r="AI189" s="7"/>
+      <c r="AJ189" s="7"/>
+      <c r="AK189" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="190" spans="1:37">
+      <c r="A190" s="3">
+        <v>188</v>
+      </c>
+      <c r="B190" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C190" s="3">
+        <v>2026063589</v>
+      </c>
+      <c r="D190" s="3"/>
+      <c r="E190" s="3"/>
+      <c r="F190" s="3">
+        <v>4573</v>
+      </c>
+      <c r="G190" s="3" t="s">
+        <v>1294</v>
+      </c>
+      <c r="H190" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="I190" s="3"/>
+      <c r="J190" s="3"/>
+      <c r="K190" s="3"/>
+      <c r="L190" s="3"/>
+      <c r="M190" s="4"/>
+      <c r="N190" s="3"/>
+      <c r="O190" s="4"/>
+      <c r="P190" s="10"/>
+      <c r="Q190" s="3" t="s">
+        <v>1295</v>
+      </c>
+      <c r="R190" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S190" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T190" s="3">
+        <v>1</v>
+      </c>
+      <c r="U190" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V190" s="3" t="s">
+        <v>1296</v>
+      </c>
+      <c r="W190" s="3" t="s">
+        <v>1292</v>
+      </c>
+      <c r="X190" s="3" t="s">
+        <v>1297</v>
+      </c>
+      <c r="Y190" s="3"/>
+      <c r="Z190" s="3">
+        <v>0.7</v>
+      </c>
+      <c r="AA190" s="3"/>
+      <c r="AB190" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC190" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="AD190" s="3"/>
+      <c r="AE190" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF190" s="3"/>
+      <c r="AG190" s="3"/>
+      <c r="AH190" s="3"/>
+      <c r="AI190" s="3"/>
+      <c r="AJ190" s="3"/>
+      <c r="AK190" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="191" spans="1:37">
+      <c r="A191" s="7">
+        <v>189</v>
+      </c>
+      <c r="B191" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C191" s="7">
+        <v>2026063590</v>
+      </c>
+      <c r="D191" s="7"/>
+      <c r="E191" s="7"/>
+      <c r="F191" s="7">
+        <v>4573</v>
+      </c>
+      <c r="G191" s="7" t="s">
+        <v>1294</v>
+      </c>
+      <c r="H191" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="I191" s="7"/>
+      <c r="J191" s="7"/>
+      <c r="K191" s="7"/>
+      <c r="L191" s="7"/>
+      <c r="M191" s="8"/>
+      <c r="N191" s="7"/>
+      <c r="O191" s="8"/>
+      <c r="P191" s="9"/>
+      <c r="Q191" s="7" t="s">
+        <v>1295</v>
+      </c>
+      <c r="R191" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S191" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="T191" s="7">
+        <v>1</v>
+      </c>
+      <c r="U191" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V191" s="7" t="s">
+        <v>1298</v>
+      </c>
+      <c r="W191" s="7" t="s">
+        <v>1292</v>
+      </c>
+      <c r="X191" s="7" t="s">
+        <v>1297</v>
+      </c>
+      <c r="Y191" s="7"/>
+      <c r="Z191" s="7">
+        <v>0.7</v>
+      </c>
+      <c r="AA191" s="7"/>
+      <c r="AB191" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC191" s="9" t="s">
+        <v>1299</v>
+      </c>
+      <c r="AD191" s="7"/>
+      <c r="AE191" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF191" s="7"/>
+      <c r="AG191" s="7"/>
+      <c r="AH191" s="7"/>
+      <c r="AI191" s="7"/>
+      <c r="AJ191" s="7"/>
+      <c r="AK191" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="192" spans="1:37">
+      <c r="A192" s="3">
+        <v>190</v>
+      </c>
+      <c r="B192" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C192" s="3">
+        <v>2026063594</v>
+      </c>
+      <c r="D192" s="3"/>
+      <c r="E192" s="3"/>
+      <c r="F192" s="3">
+        <v>4036</v>
+      </c>
+      <c r="G192" s="3" t="s">
+        <v>1289</v>
+      </c>
+      <c r="H192" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="I192" s="3"/>
+      <c r="J192" s="3"/>
+      <c r="K192" s="3"/>
+      <c r="L192" s="3"/>
+      <c r="M192" s="4"/>
+      <c r="N192" s="3"/>
+      <c r="O192" s="4"/>
+      <c r="P192" s="10"/>
+      <c r="Q192" s="3" t="s">
+        <v>1290</v>
+      </c>
+      <c r="R192" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S192" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="T192" s="3">
+        <v>1</v>
+      </c>
+      <c r="U192" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V192" s="3" t="s">
+        <v>1300</v>
+      </c>
+      <c r="W192" s="3" t="s">
+        <v>1301</v>
+      </c>
+      <c r="X192" s="3" t="s">
+        <v>1302</v>
+      </c>
+      <c r="Y192" s="3"/>
+      <c r="Z192" s="3">
+        <v>4.7</v>
+      </c>
+      <c r="AA192" s="3"/>
+      <c r="AB192" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC192" s="10" t="s">
+        <v>1303</v>
+      </c>
+      <c r="AD192" s="3"/>
+      <c r="AE192" s="3"/>
+      <c r="AF192" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG192" s="3"/>
+      <c r="AH192" s="3"/>
+      <c r="AI192" s="3"/>
+      <c r="AJ192" s="3"/>
+      <c r="AK192" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="193" spans="1:37">
+      <c r="A193" s="7">
+        <v>191</v>
+      </c>
+      <c r="B193" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C193" s="7">
+        <v>2026063640</v>
+      </c>
+      <c r="D193" s="7" t="s">
+        <v>1304</v>
+      </c>
+      <c r="E193" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F193" s="7">
+        <v>4036</v>
+      </c>
+      <c r="G193" s="7" t="s">
+        <v>1289</v>
+      </c>
+      <c r="H193" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="I193" s="7" t="s">
+        <v>1305</v>
+      </c>
+      <c r="J193" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K193" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L193" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="M193" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="N193" s="7">
+        <v>3402</v>
+      </c>
+      <c r="O193" s="8" t="s">
+        <v>1306</v>
+      </c>
+      <c r="P193" s="9" t="s">
+        <v>1307</v>
+      </c>
+      <c r="Q193" s="7" t="s">
+        <v>1290</v>
+      </c>
+      <c r="R193" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S193" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="T193" s="7">
+        <v>1</v>
+      </c>
+      <c r="U193" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V193" s="7" t="s">
+        <v>1308</v>
+      </c>
+      <c r="W193" s="7" t="s">
+        <v>1309</v>
+      </c>
+      <c r="X193" s="7" t="s">
+        <v>1310</v>
+      </c>
+      <c r="Y193" s="7" t="s">
+        <v>1311</v>
+      </c>
+      <c r="Z193" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA193" s="7"/>
+      <c r="AB193" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC193" s="9" t="s">
+        <v>1312</v>
+      </c>
+      <c r="AD193" s="7"/>
+      <c r="AE193" s="7"/>
+      <c r="AF193" s="7"/>
+      <c r="AG193" s="7"/>
+      <c r="AH193" s="7"/>
+      <c r="AI193" s="7"/>
+      <c r="AJ193" s="7"/>
+      <c r="AK193" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="194" spans="1:37">
+      <c r="A194" s="3">
+        <v>192</v>
+      </c>
+      <c r="B194" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C194" s="3">
+        <v>2026063650</v>
+      </c>
+      <c r="D194" s="3" t="s">
+        <v>1313</v>
+      </c>
+      <c r="E194" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F194" s="3" t="s">
+        <v>1314</v>
+      </c>
+      <c r="G194" s="3" t="s">
+        <v>1047</v>
+      </c>
+      <c r="H194" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="I194" s="3" t="s">
+        <v>1315</v>
+      </c>
+      <c r="J194" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="K194" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L194" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="M194" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="N194" s="3">
+        <v>2401</v>
+      </c>
+      <c r="O194" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="P194" s="10" t="s">
+        <v>1316</v>
+      </c>
+      <c r="Q194" s="3" t="s">
+        <v>1317</v>
+      </c>
+      <c r="R194" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S194" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="T194" s="3">
+        <v>1</v>
+      </c>
+      <c r="U194" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V194" s="3" t="s">
+        <v>1318</v>
+      </c>
+      <c r="W194" s="3" t="s">
+        <v>1245</v>
+      </c>
+      <c r="X194" s="3" t="s">
+        <v>1319</v>
+      </c>
+      <c r="Y194" s="3" t="s">
+        <v>1320</v>
+      </c>
+      <c r="Z194" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA194" s="3"/>
+      <c r="AB194" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC194" s="10" t="s">
+        <v>1321</v>
+      </c>
+      <c r="AD194" s="3"/>
+      <c r="AE194" s="3"/>
+      <c r="AF194" s="3"/>
+      <c r="AG194" s="3"/>
+      <c r="AH194" s="3"/>
+      <c r="AI194" s="3"/>
+      <c r="AJ194" s="3"/>
+      <c r="AK194" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="195" spans="1:37">
+      <c r="A195" s="7">
+        <v>193</v>
+      </c>
+      <c r="B195" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C195" s="7">
+        <v>2026063676</v>
+      </c>
+      <c r="D195" s="7"/>
+      <c r="E195" s="7"/>
+      <c r="F195" s="7" t="s">
+        <v>1322</v>
+      </c>
+      <c r="G195" s="7" t="s">
+        <v>1323</v>
+      </c>
+      <c r="H195" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I195" s="7"/>
+      <c r="J195" s="7"/>
+      <c r="K195" s="7"/>
+      <c r="L195" s="7"/>
+      <c r="M195" s="8"/>
+      <c r="N195" s="7"/>
+      <c r="O195" s="8"/>
+      <c r="P195" s="9"/>
+      <c r="Q195" s="7" t="s">
+        <v>1324</v>
+      </c>
+      <c r="R195" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S195" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T195" s="7">
+        <v>1</v>
+      </c>
+      <c r="U195" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V195" s="7" t="s">
+        <v>1325</v>
+      </c>
+      <c r="W195" s="7" t="s">
+        <v>1326</v>
+      </c>
+      <c r="X195" s="7" t="s">
+        <v>1327</v>
+      </c>
+      <c r="Y195" s="7"/>
+      <c r="Z195" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA195" s="7"/>
+      <c r="AB195" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC195" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD195" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE195" s="7"/>
+      <c r="AF195" s="7"/>
+      <c r="AG195" s="7"/>
+      <c r="AH195" s="7"/>
+      <c r="AI195" s="7"/>
+      <c r="AJ195" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK195" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="196" spans="1:37">
+      <c r="A196" s="3">
+        <v>194</v>
+      </c>
+      <c r="B196" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C196" s="3">
+        <v>2026063680</v>
+      </c>
+      <c r="D196" s="3"/>
+      <c r="E196" s="3"/>
+      <c r="F196" s="3">
+        <v>5410</v>
+      </c>
+      <c r="G196" s="3" t="s">
+        <v>1328</v>
+      </c>
+      <c r="H196" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I196" s="3"/>
+      <c r="J196" s="3"/>
+      <c r="K196" s="3"/>
+      <c r="L196" s="3"/>
+      <c r="M196" s="4"/>
+      <c r="N196" s="3"/>
+      <c r="O196" s="4"/>
+      <c r="P196" s="10"/>
+      <c r="Q196" s="3" t="s">
+        <v>1329</v>
+      </c>
+      <c r="R196" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S196" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T196" s="3">
+        <v>1</v>
+      </c>
+      <c r="U196" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V196" s="3" t="s">
+        <v>1330</v>
+      </c>
+      <c r="W196" s="3" t="s">
+        <v>1331</v>
+      </c>
+      <c r="X196" s="3" t="s">
+        <v>1332</v>
+      </c>
+      <c r="Y196" s="3"/>
+      <c r="Z196" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA196" s="3"/>
+      <c r="AB196" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC196" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD196" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE196" s="3"/>
+      <c r="AF196" s="3"/>
+      <c r="AG196" s="3"/>
+      <c r="AH196" s="3"/>
+      <c r="AI196" s="3"/>
+      <c r="AJ196" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK196" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="197" spans="1:37">
+      <c r="A197" s="7">
+        <v>195</v>
+      </c>
+      <c r="B197" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C197" s="7">
+        <v>2026063682</v>
+      </c>
+      <c r="D197" s="7" t="s">
+        <v>1333</v>
+      </c>
+      <c r="E197" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F197" s="7">
+        <v>2746</v>
+      </c>
+      <c r="G197" s="7" t="s">
+        <v>697</v>
+      </c>
+      <c r="H197" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I197" s="7" t="s">
+        <v>1334</v>
+      </c>
+      <c r="J197" s="7" t="s">
+        <v>376</v>
+      </c>
+      <c r="K197" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L197" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M197" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="N197" s="7">
+        <v>2305</v>
+      </c>
+      <c r="O197" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="P197" s="9" t="s">
+        <v>1335</v>
+      </c>
+      <c r="Q197" s="7" t="s">
+        <v>700</v>
+      </c>
+      <c r="R197" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S197" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="T197" s="7">
+        <v>1</v>
+      </c>
+      <c r="U197" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V197" s="7" t="s">
+        <v>1336</v>
+      </c>
+      <c r="W197" s="7" t="s">
+        <v>1332</v>
+      </c>
+      <c r="X197" s="7" t="s">
+        <v>1337</v>
+      </c>
+      <c r="Y197" s="7" t="s">
+        <v>1338</v>
+      </c>
+      <c r="Z197" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA197" s="7"/>
+      <c r="AB197" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC197" s="9" t="s">
+        <v>1339</v>
+      </c>
+      <c r="AD197" s="7"/>
+      <c r="AE197" s="7"/>
+      <c r="AF197" s="7"/>
+      <c r="AG197" s="7"/>
+      <c r="AH197" s="7"/>
+      <c r="AI197" s="7"/>
+      <c r="AJ197" s="7"/>
+      <c r="AK197" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="198" spans="1:37">
+      <c r="A198" s="3">
+        <v>196</v>
+      </c>
+      <c r="B198" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C198" s="3">
+        <v>2026063683</v>
+      </c>
+      <c r="D198" s="3"/>
+      <c r="E198" s="3"/>
+      <c r="F198" s="3">
+        <v>3890</v>
+      </c>
+      <c r="G198" s="3" t="s">
+        <v>1340</v>
+      </c>
+      <c r="H198" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I198" s="3"/>
+      <c r="J198" s="3"/>
+      <c r="K198" s="3"/>
+      <c r="L198" s="3"/>
+      <c r="M198" s="4"/>
+      <c r="N198" s="3"/>
+      <c r="O198" s="4"/>
+      <c r="P198" s="10"/>
+      <c r="Q198" s="3" t="s">
+        <v>1341</v>
+      </c>
+      <c r="R198" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S198" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T198" s="3">
+        <v>1</v>
+      </c>
+      <c r="U198" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V198" s="3" t="s">
+        <v>1342</v>
+      </c>
+      <c r="W198" s="3" t="s">
+        <v>1343</v>
+      </c>
+      <c r="X198" s="3" t="s">
+        <v>1344</v>
+      </c>
+      <c r="Y198" s="3"/>
+      <c r="Z198" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA198" s="3"/>
+      <c r="AB198" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC198" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD198" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE198" s="3"/>
+      <c r="AF198" s="3"/>
+      <c r="AG198" s="3"/>
+      <c r="AH198" s="3"/>
+      <c r="AI198" s="3"/>
+      <c r="AJ198" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK198" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="199" spans="1:37">
+      <c r="A199" s="7">
+        <v>197</v>
+      </c>
+      <c r="B199" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C199" s="7">
+        <v>2026063685</v>
+      </c>
+      <c r="D199" s="7"/>
+      <c r="E199" s="7"/>
+      <c r="F199" s="7">
+        <v>2069</v>
+      </c>
+      <c r="G199" s="7" t="s">
+        <v>1345</v>
+      </c>
+      <c r="H199" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I199" s="7"/>
+      <c r="J199" s="7"/>
+      <c r="K199" s="7"/>
+      <c r="L199" s="7"/>
+      <c r="M199" s="8"/>
+      <c r="N199" s="7"/>
+      <c r="O199" s="8"/>
+      <c r="P199" s="9"/>
+      <c r="Q199" s="7" t="s">
+        <v>1346</v>
+      </c>
+      <c r="R199" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S199" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="T199" s="7">
+        <v>1</v>
+      </c>
+      <c r="U199" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V199" s="7" t="s">
+        <v>1347</v>
+      </c>
+      <c r="W199" s="7" t="s">
+        <v>1348</v>
+      </c>
+      <c r="X199" s="7" t="s">
+        <v>1194</v>
+      </c>
+      <c r="Y199" s="7"/>
+      <c r="Z199" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA199" s="7"/>
+      <c r="AB199" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC199" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD199" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE199" s="7"/>
+      <c r="AF199" s="7"/>
+      <c r="AG199" s="7"/>
+      <c r="AH199" s="7"/>
+      <c r="AI199" s="7"/>
+      <c r="AJ199" s="7"/>
+      <c r="AK199" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="200" spans="1:37">
+      <c r="A200" s="3">
+        <v>198</v>
+      </c>
+      <c r="B200" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C200" s="3">
+        <v>2026063686</v>
+      </c>
+      <c r="D200" s="3"/>
+      <c r="E200" s="3"/>
+      <c r="F200" s="3">
+        <v>4698</v>
+      </c>
+      <c r="G200" s="3" t="s">
+        <v>1349</v>
+      </c>
+      <c r="H200" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I200" s="3"/>
+      <c r="J200" s="3"/>
+      <c r="K200" s="3"/>
+      <c r="L200" s="3"/>
+      <c r="M200" s="4"/>
+      <c r="N200" s="3"/>
+      <c r="O200" s="4"/>
+      <c r="P200" s="4"/>
+      <c r="Q200" s="3" t="s">
+        <v>1350</v>
+      </c>
+      <c r="R200" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S200" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T200" s="3">
+        <v>1</v>
+      </c>
+      <c r="U200" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V200" s="3" t="s">
+        <v>1351</v>
+      </c>
+      <c r="W200" s="3" t="s">
+        <v>1352</v>
+      </c>
+      <c r="X200" s="3" t="s">
+        <v>1224</v>
+      </c>
+      <c r="Y200" s="3"/>
+      <c r="Z200" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA200" s="3"/>
+      <c r="AB200" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC200" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD200" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE200" s="3"/>
+      <c r="AF200" s="3"/>
+      <c r="AG200" s="3"/>
+      <c r="AH200" s="3"/>
+      <c r="AI200" s="3"/>
+      <c r="AJ200" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK200" s="3" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 06301733
</commit_message>
<xml_diff>
--- a/IM/202606_HL_Maintain_Report.xlsx
+++ b/IM/202606_HL_Maintain_Report.xlsx
@@ -11,14 +11,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$200</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$205</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1382">
   <si>
     <t>萊爾富 工作統計表  篩選月份：202606   (  製表日期:2026-06-30  )</t>
   </si>
@@ -4043,6 +4043,29 @@
     <t>HUB重設後測試列印正常</t>
   </si>
   <si>
+    <t>E3556115063001</t>
+  </si>
+  <si>
+    <t>2026-06-30 08:06:14</t>
+  </si>
+  <si>
+    <t>門市反應tm1 ccd掃描器(HC56II-TR)刷讀所有條碼都會感應不良不好刷導致門市都需要手輸，門市已有操作掃描器校正後仍異常....須請台芝到店協助(機台1條碼感應不良.)</t>
+  </si>
+  <si>
+    <t>2026-06-30 09:04:09</t>
+  </si>
+  <si>
+    <t>2026-06-30 13:43:00</t>
+  </si>
+  <si>
+    <t>2026-07-01 13:04:00</t>
+  </si>
+  <si>
+    <t>更換掃描槍
+換下8119008389
+換上8119012861</t>
+  </si>
+  <si>
     <t>1T104115063001</t>
   </si>
   <si>
@@ -4165,6 +4188,72 @@
   </si>
   <si>
     <t>2026-06-30 12:48:00</t>
+  </si>
+  <si>
+    <t>13601115063001</t>
+  </si>
+  <si>
+    <t>三重重富店</t>
+  </si>
+  <si>
+    <t>2026-06-30 15:09:32</t>
+  </si>
+  <si>
+    <t>門市反應LIFE-ET4當機，點選任何按鍵都無反應，已協助遠端重啟仍異常....請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF03601</t>
+  </si>
+  <si>
+    <t>2026-06-30 15:10:32</t>
+  </si>
+  <si>
+    <t>2026-06-30 16:59:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 17:19:00</t>
+  </si>
+  <si>
+    <t>2026-07-01 19:10:00</t>
+  </si>
+  <si>
+    <t>螢幕無法觸控重新插拔排線</t>
+  </si>
+  <si>
+    <t>2026-06-30 16:13:06</t>
+  </si>
+  <si>
+    <t>2026-06-30 15:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 16:00:00</t>
+  </si>
+  <si>
+    <t>改裝撤機</t>
+  </si>
+  <si>
+    <t>蘆竹華麗店</t>
+  </si>
+  <si>
+    <t>THILF04456</t>
+  </si>
+  <si>
+    <t>2026-06-30 16:56:36</t>
+  </si>
+  <si>
+    <t>2026-06-30 14:15:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 16:52:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 17:25:48</t>
+  </si>
+  <si>
+    <t>2026-06-30 17:05:00</t>
+  </si>
+  <si>
+    <t>2026-06-30 17:25:00</t>
   </si>
 </sst>
 </file>
@@ -4578,7 +4667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK200"/>
+  <dimension ref="A1:AK205"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -21157,7 +21246,7 @@
         <v>38</v>
       </c>
       <c r="C194" s="3">
-        <v>2026063650</v>
+        <v>2026063645</v>
       </c>
       <c r="D194" s="3" t="s">
         <v>1313</v>
@@ -21165,17 +21254,17 @@
       <c r="E194" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F194" s="3" t="s">
+      <c r="F194" s="3">
+        <v>3556</v>
+      </c>
+      <c r="G194" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="H194" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="I194" s="3" t="s">
         <v>1314</v>
-      </c>
-      <c r="G194" s="3" t="s">
-        <v>1047</v>
-      </c>
-      <c r="H194" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="I194" s="3" t="s">
-        <v>1315</v>
       </c>
       <c r="J194" s="3" t="s">
         <v>376</v>
@@ -21184,28 +21273,28 @@
         <v>65</v>
       </c>
       <c r="L194" s="3" t="s">
-        <v>142</v>
+        <v>326</v>
       </c>
       <c r="M194" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="N194" s="3">
-        <v>2401</v>
+        <v>327</v>
+      </c>
+      <c r="N194" s="3" t="s">
+        <v>328</v>
       </c>
       <c r="O194" s="4" t="s">
-        <v>144</v>
+        <v>175</v>
       </c>
       <c r="P194" s="10" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="Q194" s="3" t="s">
-        <v>1317</v>
+        <v>153</v>
       </c>
       <c r="R194" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S194" s="3" t="s">
-        <v>178</v>
+        <v>79</v>
       </c>
       <c r="T194" s="3">
         <v>1</v>
@@ -21214,26 +21303,26 @@
         <v>53</v>
       </c>
       <c r="V194" s="3" t="s">
+        <v>1316</v>
+      </c>
+      <c r="W194" s="3" t="s">
+        <v>1194</v>
+      </c>
+      <c r="X194" s="3" t="s">
+        <v>1317</v>
+      </c>
+      <c r="Y194" s="3" t="s">
         <v>1318</v>
       </c>
-      <c r="W194" s="3" t="s">
-        <v>1245</v>
-      </c>
-      <c r="X194" s="3" t="s">
-        <v>1319</v>
-      </c>
-      <c r="Y194" s="3" t="s">
-        <v>1320</v>
-      </c>
       <c r="Z194" s="3">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="AA194" s="3"/>
       <c r="AB194" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC194" s="10" t="s">
-        <v>1321</v>
+        <v>1319</v>
       </c>
       <c r="AD194" s="3"/>
       <c r="AE194" s="3"/>
@@ -21251,30 +21340,50 @@
         <v>193</v>
       </c>
       <c r="B195" s="7" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C195" s="7">
-        <v>2026063676</v>
-      </c>
-      <c r="D195" s="7"/>
-      <c r="E195" s="7"/>
+        <v>2026063650</v>
+      </c>
+      <c r="D195" s="7" t="s">
+        <v>1320</v>
+      </c>
+      <c r="E195" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F195" s="7" t="s">
+        <v>1321</v>
+      </c>
+      <c r="G195" s="7" t="s">
+        <v>1047</v>
+      </c>
+      <c r="H195" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I195" s="7" t="s">
         <v>1322</v>
       </c>
-      <c r="G195" s="7" t="s">
+      <c r="J195" s="7" t="s">
+        <v>376</v>
+      </c>
+      <c r="K195" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L195" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="M195" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="N195" s="7">
+        <v>2401</v>
+      </c>
+      <c r="O195" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="P195" s="9" t="s">
         <v>1323</v>
       </c>
-      <c r="H195" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="I195" s="7"/>
-      <c r="J195" s="7"/>
-      <c r="K195" s="7"/>
-      <c r="L195" s="7"/>
-      <c r="M195" s="8"/>
-      <c r="N195" s="7"/>
-      <c r="O195" s="8"/>
-      <c r="P195" s="9"/>
       <c r="Q195" s="7" t="s">
         <v>1324</v>
       </c>
@@ -21282,7 +21391,7 @@
         <v>51</v>
       </c>
       <c r="S195" s="7" t="s">
-        <v>52</v>
+        <v>178</v>
       </c>
       <c r="T195" s="7">
         <v>1</v>
@@ -21294,33 +21403,31 @@
         <v>1325</v>
       </c>
       <c r="W195" s="7" t="s">
+        <v>1245</v>
+      </c>
+      <c r="X195" s="7" t="s">
         <v>1326</v>
       </c>
-      <c r="X195" s="7" t="s">
+      <c r="Y195" s="7" t="s">
         <v>1327</v>
       </c>
-      <c r="Y195" s="7"/>
       <c r="Z195" s="7">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="AA195" s="7"/>
       <c r="AB195" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC195" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD195" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>1328</v>
+      </c>
+      <c r="AD195" s="7"/>
       <c r="AE195" s="7"/>
       <c r="AF195" s="7"/>
       <c r="AG195" s="7"/>
       <c r="AH195" s="7"/>
       <c r="AI195" s="7"/>
-      <c r="AJ195" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ195" s="7"/>
       <c r="AK195" s="7" t="s">
         <v>60</v>
       </c>
@@ -21333,15 +21440,15 @@
         <v>100</v>
       </c>
       <c r="C196" s="3">
-        <v>2026063680</v>
+        <v>2026063676</v>
       </c>
       <c r="D196" s="3"/>
       <c r="E196" s="3"/>
-      <c r="F196" s="3">
-        <v>5410</v>
+      <c r="F196" s="3" t="s">
+        <v>1329</v>
       </c>
       <c r="G196" s="3" t="s">
-        <v>1328</v>
+        <v>1330</v>
       </c>
       <c r="H196" s="3" t="s">
         <v>42</v>
@@ -21355,7 +21462,7 @@
       <c r="O196" s="4"/>
       <c r="P196" s="10"/>
       <c r="Q196" s="3" t="s">
-        <v>1329</v>
+        <v>1331</v>
       </c>
       <c r="R196" s="3" t="s">
         <v>51</v>
@@ -21370,13 +21477,13 @@
         <v>53</v>
       </c>
       <c r="V196" s="3" t="s">
-        <v>1330</v>
+        <v>1332</v>
       </c>
       <c r="W196" s="3" t="s">
-        <v>1331</v>
+        <v>1333</v>
       </c>
       <c r="X196" s="3" t="s">
-        <v>1332</v>
+        <v>1334</v>
       </c>
       <c r="Y196" s="3"/>
       <c r="Z196" s="3">
@@ -21409,58 +21516,38 @@
         <v>195</v>
       </c>
       <c r="B197" s="7" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C197" s="7">
-        <v>2026063682</v>
-      </c>
-      <c r="D197" s="7" t="s">
-        <v>1333</v>
-      </c>
-      <c r="E197" s="7" t="s">
-        <v>40</v>
-      </c>
+        <v>2026063680</v>
+      </c>
+      <c r="D197" s="7"/>
+      <c r="E197" s="7"/>
       <c r="F197" s="7">
-        <v>2746</v>
+        <v>5410</v>
       </c>
       <c r="G197" s="7" t="s">
-        <v>697</v>
+        <v>1335</v>
       </c>
       <c r="H197" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="I197" s="7" t="s">
-        <v>1334</v>
-      </c>
-      <c r="J197" s="7" t="s">
-        <v>376</v>
-      </c>
-      <c r="K197" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="L197" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="M197" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="N197" s="7">
-        <v>2305</v>
-      </c>
-      <c r="O197" s="8" t="s">
-        <v>345</v>
-      </c>
-      <c r="P197" s="9" t="s">
-        <v>1335</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="I197" s="7"/>
+      <c r="J197" s="7"/>
+      <c r="K197" s="7"/>
+      <c r="L197" s="7"/>
+      <c r="M197" s="8"/>
+      <c r="N197" s="7"/>
+      <c r="O197" s="8"/>
+      <c r="P197" s="9"/>
       <c r="Q197" s="7" t="s">
-        <v>700</v>
+        <v>1336</v>
       </c>
       <c r="R197" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S197" s="7" t="s">
-        <v>94</v>
+        <v>52</v>
       </c>
       <c r="T197" s="7">
         <v>1</v>
@@ -21469,34 +21556,36 @@
         <v>53</v>
       </c>
       <c r="V197" s="7" t="s">
-        <v>1336</v>
+        <v>1337</v>
       </c>
       <c r="W197" s="7" t="s">
-        <v>1332</v>
+        <v>1338</v>
       </c>
       <c r="X197" s="7" t="s">
-        <v>1337</v>
-      </c>
-      <c r="Y197" s="7" t="s">
-        <v>1338</v>
-      </c>
+        <v>1339</v>
+      </c>
+      <c r="Y197" s="7"/>
       <c r="Z197" s="7">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="AA197" s="7"/>
       <c r="AB197" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC197" s="9" t="s">
-        <v>1339</v>
-      </c>
-      <c r="AD197" s="7"/>
+        <v>111</v>
+      </c>
+      <c r="AD197" s="7" t="s">
+        <v>60</v>
+      </c>
       <c r="AE197" s="7"/>
       <c r="AF197" s="7"/>
       <c r="AG197" s="7"/>
       <c r="AH197" s="7"/>
       <c r="AI197" s="7"/>
-      <c r="AJ197" s="7"/>
+      <c r="AJ197" s="7" t="s">
+        <v>60</v>
+      </c>
       <c r="AK197" s="7" t="s">
         <v>60</v>
       </c>
@@ -21506,38 +21595,58 @@
         <v>196</v>
       </c>
       <c r="B198" s="3" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C198" s="3">
-        <v>2026063683</v>
-      </c>
-      <c r="D198" s="3"/>
-      <c r="E198" s="3"/>
+        <v>2026063682</v>
+      </c>
+      <c r="D198" s="3" t="s">
+        <v>1340</v>
+      </c>
+      <c r="E198" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="F198" s="3">
-        <v>3890</v>
+        <v>2746</v>
       </c>
       <c r="G198" s="3" t="s">
-        <v>1340</v>
+        <v>697</v>
       </c>
       <c r="H198" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I198" s="3"/>
-      <c r="J198" s="3"/>
-      <c r="K198" s="3"/>
-      <c r="L198" s="3"/>
-      <c r="M198" s="4"/>
-      <c r="N198" s="3"/>
-      <c r="O198" s="4"/>
-      <c r="P198" s="10"/>
+        <v>86</v>
+      </c>
+      <c r="I198" s="3" t="s">
+        <v>1341</v>
+      </c>
+      <c r="J198" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="K198" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L198" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M198" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="N198" s="3">
+        <v>2305</v>
+      </c>
+      <c r="O198" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="P198" s="10" t="s">
+        <v>1342</v>
+      </c>
       <c r="Q198" s="3" t="s">
-        <v>1341</v>
+        <v>700</v>
       </c>
       <c r="R198" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S198" s="3" t="s">
-        <v>52</v>
+        <v>94</v>
       </c>
       <c r="T198" s="3">
         <v>1</v>
@@ -21546,36 +21655,34 @@
         <v>53</v>
       </c>
       <c r="V198" s="3" t="s">
-        <v>1342</v>
+        <v>1343</v>
       </c>
       <c r="W198" s="3" t="s">
-        <v>1343</v>
+        <v>1339</v>
       </c>
       <c r="X198" s="3" t="s">
         <v>1344</v>
       </c>
-      <c r="Y198" s="3"/>
+      <c r="Y198" s="3" t="s">
+        <v>1345</v>
+      </c>
       <c r="Z198" s="3">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="AA198" s="3"/>
       <c r="AB198" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC198" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD198" s="3" t="s">
-        <v>60</v>
-      </c>
+        <v>1346</v>
+      </c>
+      <c r="AD198" s="3"/>
       <c r="AE198" s="3"/>
       <c r="AF198" s="3"/>
       <c r="AG198" s="3"/>
       <c r="AH198" s="3"/>
       <c r="AI198" s="3"/>
-      <c r="AJ198" s="3" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ198" s="3"/>
       <c r="AK198" s="3" t="s">
         <v>60</v>
       </c>
@@ -21588,18 +21695,18 @@
         <v>100</v>
       </c>
       <c r="C199" s="7">
-        <v>2026063685</v>
+        <v>2026063683</v>
       </c>
       <c r="D199" s="7"/>
       <c r="E199" s="7"/>
       <c r="F199" s="7">
-        <v>2069</v>
+        <v>3890</v>
       </c>
       <c r="G199" s="7" t="s">
-        <v>1345</v>
+        <v>1347</v>
       </c>
       <c r="H199" s="7" t="s">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="I199" s="7"/>
       <c r="J199" s="7"/>
@@ -21610,13 +21717,13 @@
       <c r="O199" s="8"/>
       <c r="P199" s="9"/>
       <c r="Q199" s="7" t="s">
-        <v>1346</v>
+        <v>1348</v>
       </c>
       <c r="R199" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S199" s="7" t="s">
-        <v>94</v>
+        <v>52</v>
       </c>
       <c r="T199" s="7">
         <v>1</v>
@@ -21625,13 +21732,13 @@
         <v>53</v>
       </c>
       <c r="V199" s="7" t="s">
-        <v>1347</v>
+        <v>1349</v>
       </c>
       <c r="W199" s="7" t="s">
-        <v>1348</v>
+        <v>1350</v>
       </c>
       <c r="X199" s="7" t="s">
-        <v>1194</v>
+        <v>1351</v>
       </c>
       <c r="Y199" s="7"/>
       <c r="Z199" s="7">
@@ -21652,7 +21759,9 @@
       <c r="AG199" s="7"/>
       <c r="AH199" s="7"/>
       <c r="AI199" s="7"/>
-      <c r="AJ199" s="7"/>
+      <c r="AJ199" s="7" t="s">
+        <v>60</v>
+      </c>
       <c r="AK199" s="7" t="s">
         <v>60</v>
       </c>
@@ -21665,18 +21774,18 @@
         <v>100</v>
       </c>
       <c r="C200" s="3">
-        <v>2026063686</v>
+        <v>2026063685</v>
       </c>
       <c r="D200" s="3"/>
       <c r="E200" s="3"/>
       <c r="F200" s="3">
-        <v>4698</v>
+        <v>2069</v>
       </c>
       <c r="G200" s="3" t="s">
-        <v>1349</v>
+        <v>1352</v>
       </c>
       <c r="H200" s="3" t="s">
-        <v>42</v>
+        <v>86</v>
       </c>
       <c r="I200" s="3"/>
       <c r="J200" s="3"/>
@@ -21685,15 +21794,15 @@
       <c r="M200" s="4"/>
       <c r="N200" s="3"/>
       <c r="O200" s="4"/>
-      <c r="P200" s="4"/>
+      <c r="P200" s="10"/>
       <c r="Q200" s="3" t="s">
-        <v>1350</v>
+        <v>1353</v>
       </c>
       <c r="R200" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S200" s="3" t="s">
-        <v>52</v>
+        <v>94</v>
       </c>
       <c r="T200" s="3">
         <v>1</v>
@@ -21702,23 +21811,23 @@
         <v>53</v>
       </c>
       <c r="V200" s="3" t="s">
-        <v>1351</v>
+        <v>1354</v>
       </c>
       <c r="W200" s="3" t="s">
-        <v>1352</v>
+        <v>1355</v>
       </c>
       <c r="X200" s="3" t="s">
-        <v>1224</v>
+        <v>1194</v>
       </c>
       <c r="Y200" s="3"/>
       <c r="Z200" s="3">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="AA200" s="3"/>
       <c r="AB200" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="AC200" s="4" t="s">
+      <c r="AC200" s="10" t="s">
         <v>111</v>
       </c>
       <c r="AD200" s="3" t="s">
@@ -21729,10 +21838,417 @@
       <c r="AG200" s="3"/>
       <c r="AH200" s="3"/>
       <c r="AI200" s="3"/>
-      <c r="AJ200" s="3" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ200" s="3"/>
       <c r="AK200" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="201" spans="1:37">
+      <c r="A201" s="7">
+        <v>199</v>
+      </c>
+      <c r="B201" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C201" s="7">
+        <v>2026063686</v>
+      </c>
+      <c r="D201" s="7"/>
+      <c r="E201" s="7"/>
+      <c r="F201" s="7">
+        <v>4698</v>
+      </c>
+      <c r="G201" s="7" t="s">
+        <v>1356</v>
+      </c>
+      <c r="H201" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I201" s="7"/>
+      <c r="J201" s="7"/>
+      <c r="K201" s="7"/>
+      <c r="L201" s="7"/>
+      <c r="M201" s="8"/>
+      <c r="N201" s="7"/>
+      <c r="O201" s="8"/>
+      <c r="P201" s="9"/>
+      <c r="Q201" s="7" t="s">
+        <v>1357</v>
+      </c>
+      <c r="R201" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S201" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T201" s="7">
+        <v>1</v>
+      </c>
+      <c r="U201" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V201" s="7" t="s">
+        <v>1358</v>
+      </c>
+      <c r="W201" s="7" t="s">
+        <v>1359</v>
+      </c>
+      <c r="X201" s="7" t="s">
+        <v>1224</v>
+      </c>
+      <c r="Y201" s="7"/>
+      <c r="Z201" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA201" s="7"/>
+      <c r="AB201" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC201" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD201" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE201" s="7"/>
+      <c r="AF201" s="7"/>
+      <c r="AG201" s="7"/>
+      <c r="AH201" s="7"/>
+      <c r="AI201" s="7"/>
+      <c r="AJ201" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK201" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="202" spans="1:37">
+      <c r="A202" s="3">
+        <v>200</v>
+      </c>
+      <c r="B202" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C202" s="3">
+        <v>2026063763</v>
+      </c>
+      <c r="D202" s="3" t="s">
+        <v>1360</v>
+      </c>
+      <c r="E202" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F202" s="3">
+        <v>3601</v>
+      </c>
+      <c r="G202" s="3" t="s">
+        <v>1361</v>
+      </c>
+      <c r="H202" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I202" s="3" t="s">
+        <v>1362</v>
+      </c>
+      <c r="J202" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="K202" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L202" s="3" t="s">
+        <v>809</v>
+      </c>
+      <c r="M202" s="4" t="s">
+        <v>810</v>
+      </c>
+      <c r="N202" s="3">
+        <v>5801</v>
+      </c>
+      <c r="O202" s="4" t="s">
+        <v>1088</v>
+      </c>
+      <c r="P202" s="10" t="s">
+        <v>1363</v>
+      </c>
+      <c r="Q202" s="3" t="s">
+        <v>1364</v>
+      </c>
+      <c r="R202" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S202" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T202" s="3">
+        <v>1</v>
+      </c>
+      <c r="U202" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V202" s="3" t="s">
+        <v>1365</v>
+      </c>
+      <c r="W202" s="3" t="s">
+        <v>1366</v>
+      </c>
+      <c r="X202" s="3" t="s">
+        <v>1367</v>
+      </c>
+      <c r="Y202" s="3" t="s">
+        <v>1368</v>
+      </c>
+      <c r="Z202" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA202" s="3"/>
+      <c r="AB202" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC202" s="10" t="s">
+        <v>1369</v>
+      </c>
+      <c r="AD202" s="3"/>
+      <c r="AE202" s="3"/>
+      <c r="AF202" s="3"/>
+      <c r="AG202" s="3"/>
+      <c r="AH202" s="3"/>
+      <c r="AI202" s="3"/>
+      <c r="AJ202" s="3"/>
+      <c r="AK202" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="203" spans="1:37">
+      <c r="A203" s="7">
+        <v>201</v>
+      </c>
+      <c r="B203" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C203" s="7">
+        <v>2026063780</v>
+      </c>
+      <c r="D203" s="7"/>
+      <c r="E203" s="7"/>
+      <c r="F203" s="7">
+        <v>4098</v>
+      </c>
+      <c r="G203" s="7" t="s">
+        <v>578</v>
+      </c>
+      <c r="H203" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I203" s="7"/>
+      <c r="J203" s="7"/>
+      <c r="K203" s="7"/>
+      <c r="L203" s="7"/>
+      <c r="M203" s="8"/>
+      <c r="N203" s="7"/>
+      <c r="O203" s="8"/>
+      <c r="P203" s="9"/>
+      <c r="Q203" s="7" t="s">
+        <v>579</v>
+      </c>
+      <c r="R203" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S203" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T203" s="7">
+        <v>1</v>
+      </c>
+      <c r="U203" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V203" s="7" t="s">
+        <v>1370</v>
+      </c>
+      <c r="W203" s="7" t="s">
+        <v>1371</v>
+      </c>
+      <c r="X203" s="7" t="s">
+        <v>1372</v>
+      </c>
+      <c r="Y203" s="7"/>
+      <c r="Z203" s="7">
+        <v>1</v>
+      </c>
+      <c r="AA203" s="7"/>
+      <c r="AB203" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC203" s="9" t="s">
+        <v>1373</v>
+      </c>
+      <c r="AD203" s="7"/>
+      <c r="AE203" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF203" s="7"/>
+      <c r="AG203" s="7"/>
+      <c r="AH203" s="7"/>
+      <c r="AI203" s="7"/>
+      <c r="AJ203" s="7"/>
+      <c r="AK203" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="204" spans="1:37">
+      <c r="A204" s="3">
+        <v>202</v>
+      </c>
+      <c r="B204" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C204" s="3">
+        <v>2026063787</v>
+      </c>
+      <c r="D204" s="3"/>
+      <c r="E204" s="3"/>
+      <c r="F204" s="3">
+        <v>4456</v>
+      </c>
+      <c r="G204" s="3" t="s">
+        <v>1374</v>
+      </c>
+      <c r="H204" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="I204" s="3"/>
+      <c r="J204" s="3"/>
+      <c r="K204" s="3"/>
+      <c r="L204" s="3"/>
+      <c r="M204" s="4"/>
+      <c r="N204" s="3"/>
+      <c r="O204" s="4"/>
+      <c r="P204" s="10"/>
+      <c r="Q204" s="3" t="s">
+        <v>1375</v>
+      </c>
+      <c r="R204" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S204" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="T204" s="3">
+        <v>1</v>
+      </c>
+      <c r="U204" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V204" s="3" t="s">
+        <v>1376</v>
+      </c>
+      <c r="W204" s="3" t="s">
+        <v>1377</v>
+      </c>
+      <c r="X204" s="3" t="s">
+        <v>1378</v>
+      </c>
+      <c r="Y204" s="3"/>
+      <c r="Z204" s="3">
+        <v>2.6</v>
+      </c>
+      <c r="AA204" s="3"/>
+      <c r="AB204" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC204" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="AD204" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE204" s="3"/>
+      <c r="AF204" s="3"/>
+      <c r="AG204" s="3"/>
+      <c r="AH204" s="3"/>
+      <c r="AI204" s="3"/>
+      <c r="AJ204" s="3"/>
+      <c r="AK204" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="205" spans="1:37">
+      <c r="A205" s="7">
+        <v>203</v>
+      </c>
+      <c r="B205" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C205" s="7">
+        <v>2026063799</v>
+      </c>
+      <c r="D205" s="7"/>
+      <c r="E205" s="7"/>
+      <c r="F205" s="7">
+        <v>3601</v>
+      </c>
+      <c r="G205" s="7" t="s">
+        <v>1361</v>
+      </c>
+      <c r="H205" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I205" s="7"/>
+      <c r="J205" s="7"/>
+      <c r="K205" s="7"/>
+      <c r="L205" s="7"/>
+      <c r="M205" s="8"/>
+      <c r="N205" s="7"/>
+      <c r="O205" s="8"/>
+      <c r="P205" s="8"/>
+      <c r="Q205" s="7" t="s">
+        <v>1364</v>
+      </c>
+      <c r="R205" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S205" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T205" s="7">
+        <v>1</v>
+      </c>
+      <c r="U205" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V205" s="7" t="s">
+        <v>1379</v>
+      </c>
+      <c r="W205" s="7" t="s">
+        <v>1380</v>
+      </c>
+      <c r="X205" s="7" t="s">
+        <v>1381</v>
+      </c>
+      <c r="Y205" s="7"/>
+      <c r="Z205" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA205" s="7"/>
+      <c r="AB205" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC205" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD205" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE205" s="7"/>
+      <c r="AF205" s="7"/>
+      <c r="AG205" s="7"/>
+      <c r="AH205" s="7"/>
+      <c r="AI205" s="7"/>
+      <c r="AJ205" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK205" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>